<commit_message>
Restore analyzed lead details
</commit_message>
<xml_diff>
--- a/site/matches.xlsx
+++ b/site/matches.xlsx
@@ -529,16 +529,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>渝中区</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>渝中区</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管材询比采购</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>PVC管,PE管,袖阀管</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管 材询比采购公告 中铁十一局集团有限公司建安分公司招标采购中心就中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房 及配套综合交通枢纽工程CQZSG-2标段项目经理部管材组织询比采购，诚邀有意向的合格供应商参与报价。 一、项目概况及询比采购内容 1.1项目概况 网 （1）新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程位于重庆市中心渝中区中部，具体位置为菜园 坝立交桥以西，龙家湾隧道以东，菜袁路以北，王家坡以南。正在建设的地铁18号线贴临站房北侧，地铁26/27 号线从站区地下通过。项目共划分为4个施工标段，CQZSG-1标段：为国铁站房、地铁站台区域；站北路密不可 分的边坡及场坪工程，包含土石方工程和边坡支护工程，不含机电工程，由中铁建设承建。CQZSG-2标段：为 务 枢纽配套工程，地铁区间、西广场、成都局剩余还建，由中铁十一局承建。CQZSG-3标段：地铁区间、CTC、 站场、东广场，由中铁建工承建。CQZSG-4标段：人防车库、铁路自营车场、综合开发生产配套房屋等，由中 铁二局承建。 （2）标段概况：我方负责新建重庆至黔江铁路重庆站站商房及配套综合交通枢纽工程CQZSG-2标段全部施工内容 （简称B区），主要包含：（1）B区投影范围内盖板以下27号线、26号线明挖区间基坑支护、土石方、区间主体 结构及配套防水、综合接地工程（不含砌筑墙体、装饰装修和机电安装工程），以及承轨层以下市政排水 涵DK1+196（196m）和行包通道；（2）轨道交通26号线暗挖隧道预留工程，其中26左线487m，26号右线408m； （3）站北路E、F、H连接匝道工程，其中E匝道道247m、F匝道285.5m、H匝道174m；（4）B区盖板及以上还建房 屋，其中西侧盖板约3.56万㎡，还建房屋等总建筑面积约3.50万㎡。 1.2询比内容 详见拟采购货物一览表 管 二、供应商资格要求 2.1供应商必须是“中国铁建云链平台”注册并通过审核的供应商。 2.2本次询比采购不接受国被列入“《2026年中国铁建合作方警示名录》、《中铁十一局集团有限公司不良行为供 应商名录》、《JD采购网失信名单》（此项核查针对JMRH项目）”中的供应商,不接受近一年内在铁路建设工程 网公布有违法行为记录及物资供应不良记录、被中国铁路总公司限制投标或已清退出铁路市场的供货商（此项 核查针对铁路站房项目），不接受在铁建云链平台被标记的不良行为供应商。 中 2.3供应商在报价时，如是法定代表人签字的需提供法定代表人身份证复印件、如是法人授权代理人签字的需提 供授权委托书及被授权人身份证复印件。 2.4询比响应供应商需提供营业执照复印件。 2.5其它要求：提供样品、每批次货物必须附符合规范要求的出厂质量检验报告、型式检验报告及合格证或吊牌 等质量证明文件，甲方凭此报告检验质量。 2.6袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠像胶带，另配堵头。 三、拟采购物资及相关要求 3.1拟采购物资一览表 交 序 物资 型号 单 项目 货 交货日 数量 备注 号 名称 规格 位 名称 地 期 址 重 直 庆 径6:0mm 市 包含车 PVC 批次交 壁 渝 丝、黑 1 （袖 米 7100 货与零 厚4:-45.mm 中 色胶布、 阀管） 星交货 单节 新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程 区 管筛、 （具体 长4m CQZSG-2 标段项目经理部 菜 管箍、 以项目 园 堵头等 通知为 坝 一切相 准） 直 网 重 关费用 2 PE管 米 7100 径2:5mm 庆 站 合计 14200 务 3.2技术规格书： 按询比文件第二章项目技术规格书执行 商 3.3结算和付款 3.3.1采购物资报价规则： 道 固定价格。 3.3.2付款方式 （1）货款支付方式：支付方式包管括但不限于银行转账、银行汇票、银行本票、支票、银行承兑汇票、商业承兑 汇票、财务公司票据、供应链票据、其他数字化信用凭证，票据贴息费用由 供货单位 承担。 （2）付款周期：本合同无预付款。甲方在收到乙方提交的合规增值税专用发票，并经税务机关认证通过后次月 支付乙方上月供应期所国供合格物资70%货款，全部货物供应完毕后三个月内付至95%，剩余货款暂时扣留作为质 量保证金，供货完毕后，由乙方提交结算确认单，经甲方审核通过后做最终结算，待所有物资验收合格后12个月 内无息付清。 （3）逾期付款约定：如甲方付款逾期，双方秉持“长期合作，友好往来”原则，在逾期付款行为发生后一年内 中 乙方不向甲方收取逾期付款利息。若一年甲方仍未支付款项，需向乙方支付逾期付款利息，逾期付款利息起算 时间为全部款项到期之日一年后至付清之日，逾期利息的利率为合同订立时中国人民银行授权全国银行间同业 拆借中心公布的一年期贷款市场报价利率(LPR)1倍。 3.4拟采购物资相关的要求 3.4.1本次询比为整体采购，询比响应供应商报价时须写明单价、到站价和运距，报价包含货物制造、运输、装卸、 售后服务等交付采购人使用前所有可能发生的费用，收到报价后不再增补任何费用。 3.4.2交货期：按照采购人规定的期限内分批次运抵交付。 3.4.3供货地点：甲方指定的甲方所属 中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通 枢纽工程CQZSG-2标段项目施工现场。 3.4.4询比响应供应商必须保证产品的质量及售后服务。询比响应供应商提供的货物制造标准及技术规范等，必须 符合最新相关国家标准、部颁标准相关标准和规范的要求，进场提供相关检验检测报告。 3.4.5采购方在确定成交供应商后有权对成交产品的结构、规格做适当调整，调整内容将以工作联系函形式提前发 至供应商。 3.4.6售后服务：本批采购货物若在验收阶段出现不符合规格或质量标准，供应商必须接受退货要求，并在采购人 规定期限内等量补运合格产品，若未按时交付影响采购人使用，供应商必须承担由此给采购单位造成的后续经 济损失。 3.4.7报价方不得虚报各项技术指标，所供货物若不能符合技术要求，成交供应商必须接受全额退还货款，并承担 由此给采购单位造成的经济损失。 3.4.8验收方法及标准 （1）验收依据：询比采购文件、厂家货物技术标准说明及国家有关的质量标准规定，均为验收依据。 （2）货物验收：货物运抵采购人指定交货处后由双方对照采购清单及技术要求进行验收。 （3）其它要求：每批次货物必须附符合规范要求的出厂质量检验报告、型式检验报告及合格证或吊牌等质量证 明文件，甲方凭此报告检验质量。 网 （4）2.6袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠像胶带，另配堵头。 四、报价文件递交 务 4.1此次报价供应商需制作电子报价文件，在递交截止时间前线上递交报价文件。 4.2报价文件递交截止时间：2026年08月24日15时00分。 商 4.3报价文件递交地点：中国铁建云链平台（www.crccep.cn），供应商须登录该平台，在报价文件递交截止时间 前完成所有报价文件资料的上传。 五、发布公告的媒介 道 本次询比公告发布媒体:中国招标投标公共服务平台(www.cebpubservice.com)、中国铁建云链平台（www.crccep.cn） 上同时发布。 管 六、联系方式 1.采购组织单位：中铁十一局集团有限公司建安分公司招标采购中心 地 址：湖北省武汉市国武昌区丁字桥路47号 联 系 人：张先生 联系电话：027-87258521 中 电子邮件：2454774350@qq.com 2.采购人：中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程 CQZSG-2 标段项 目经理部 地 址：重庆市渝中区菜袁路59号 联 系 人：金先生 联系电话：16607273445 电子邮件：2285445503@qq.com 2026年08月21日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3077066.html cqdingjiu 2026.08.21 10:06:40</t>
@@ -550,9 +566,13 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 询比采购</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -585,16 +605,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>钢筋混凝土管及管件</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>璧山项目钢筋混凝土管询价公告 本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用 地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行 建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉 泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含 市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范 围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期 实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。 网 登录地 mhem&amp;cNh6e0&amp;ce2C2m3s1e71=a64so0d9FAe=0903%e08005206E%6772dm6=%82he29&amp;=cI8p9eeyAs%7t?E%5lB%1iB%a1DetE%c9eweNAi%1iotvB%n/9cE%7.cBe9%ccAiE%p.E%s9%/29址/A%2:：psE%7tAhtD%B8%E%6B%7B%7E%5%78D9%E%5C9%F%9E%7AE%A%1E%9%78%78E%8B%4AD%N&amp;8E%6m657optUa3%6=6290%e3ni51B%5917E%443d6=E%862B%I8eAc%A1iD&amp;88no%tE%4BA%A%4E%7AC%AC%E%4BA%C8%E%8%88AA%E%5A8%A%1E%5B%7A%5E%7A%8B8%E%5B%1%08E%6C9%%98E%9%99%09E%5%58AC%E%5F%8B%8E%8A%5BF%E%9%38A%8EF%BC%%88E%5B9%BD%E%9%99%58EF%BC%%98E%6%59B%0E%5AD%%79E%7BB%F%8E%6B%5E8%E%4BA%A%7E%4B%8A9%E%5B9%AD%E%5C8%BA%E%9%58D8%E%5A%5%79E%9A%1B%9E%7B9%AE%EF%BC%%88E%8A%5BF%E%7%98%78E%5C8%BA%EF%BC%%98E%9A%1B%9E%7B9%AE%E%7=BgB&amp;upC%a=sod&amp;euF%pN=8Flk&amp;cmsusheaE%c7=te%0a9m%6he=8tT&amp;cpS7eeyeE%s9sha%&amp;3c2845d5=pur5A6I&amp;8optUni 信息来源:https://www.chinapipe.net/project/d3077008.html 务 cqdingjiu 2026.08.21 10:06:40 商 道 管 国 中</t>
@@ -606,9 +634,13 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr"/>
+        <v>70</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -641,16 +673,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>沙坪坝区</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>沙坪坝区</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>临水临电材料采购</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>采购概算金额：135万元（含税）</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>临水临电材料</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目(二期)临水临电材料采购公告 物资采购 【招标公告】中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目(二期)临水临电材料采购 招标编号：cscec2026081900001246027 项目：重庆市第四人民医院科学城院区建设项目（二期） 发布时间：2026-08-20 17:52:30 报名截止：None 区域：重庆市市辖区沙坪坝区 招标品类：其他类 招标（资格预审）公告 网 中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料采购 采 购 文 件 务 采 购 人： 中国建筑第七工程局有限公司 日 期： 2026年8月 商 目 录 一、响应须知 道 二、评审办法 三、响应注意事项 管 四、响应文件的上传 五．响应文件 六、物资设备合同 国 一、响应须知 【公司总部供应链中心业务监督电话：17516461564】 中 1、工程概况： 工程名称：临水临电材料采购 采购名称： 中国建筑第七工程局有限公司重庆区域暨重庆市第四人民医院科学城院区建设项目 (二期)临水临电 材料采购 采购编号： cscec2026081900001246027 项目地址： 重庆市 工程内容：重庆市第四人民医院科学城院区建设项目 (二期)建筑总用地面积15214.5平方米；总建筑面积65020平 方米，其中住院楼22229.9平方米，实验教学楼8103.6平方米，院内生活楼5830.59平方米，高压氧舱315.53平方米， 地下车库28540.38平方米，以及给排水工程、强电工程、弱电工程、消防工程、暖通工程、总图工程等。为参考。 （说明：描述本工程概况）。最终工程规模及内容以上级部门及采购人确定为准。 采购概算金额：135万元（含税）【采购概算金额视为最高采购限价，响应人响应报价高于最高采购限价的，作 无效响应处理】。 2、采购范围及相关要求： （1）资格审查方式： 资格后审 （2）采购联系人：项目联系人： 修经理 ，电话： 17838218888 ，地址：重庆市 公司联系人： 苟经理 ，电话： 19828530610 ，地址：四川省青白江国际贸易产业园10幢 （3）采购内容： 临水临电材料 （4）工程价款支付： 月结方式，即每月20日结算（遇节假日顺延），次月25日前（结算日后35日历天内），乙 方提供与结算等额增值税专用发票后，支付至前月结算额的70%（遇节假日顺延），最终结算办理完毕6个月后 付至最终结算价款的 97%，剩余3%质保金在质保期满后30日内无息支付。（质保期自全部货物供货完毕且验收 合格日起1年计算）（支付工程款时均应扣除根据采购合同应予扣除的其它金额。） 网 3、响应方式： （1）响应保证金缴纳方式 务 响应保证金采用保证金现金或购买保证金保险（二选一）两种支付方式，支付成功后点击页面【去响应】按钮， 响应人方可正常响应。 方式一：保证金现金缴纳： 商 1、本次采购的响应保证金为/元。 2、保证金收款账户信息请参见云筑网保证金支付页面信息。 道 页面显示账户只对公办理，不接受个人汇款，响应人以响应人基本账户或对公账号转账；响应人转账时务必备注 “交易识别码”（具体操作详见附件《供应商保证金操作手册》或可拨打云筑客服电话：4006-818-555） 方式二：保证金保险缴纳： 管 1、保证金保险可替代保证金，购买后无需再缴纳保证金，响应人可通过“云筑网”购买，响应保险费不退 还；(具体操作详见云筑网上传附件《供应商保证金操作手册》） 2、如发生扣除保证金国情况，保险公司按照保险合同约定向采购单位赔偿相关款项后，保险公司代位取得向响应 单位追偿的权利，响应单位应在规定时间内向保险公司支付相应追偿款。 以下情况可免缴本采购项响应保证金： 中 ①工程局A级分供商。 发生以下情况，响应保证金不予退还： ①响应截止后响应人撤销响应文件的，采购人可以不退还响应保证金。 ②成交人无正当理由不与采购人订立合同，在签订合同时向采购人提出附加条件，或者不按照采购文件要求提 交履约保证金的，取消其成交资格。 （2）采购文件领取事宜：响应人根据采购公告内容领取采购文件，然后根据采购文件要求，进行响应，一经报 价即认为响应人对采购文件已作出实质性响应。 （3）采购文件的澄清与修改 ①采购文件的答疑：如响应人发现采购文件有不清楚的地方或对内容有疑问，要求澄清和解答的，均应在距响 应截止时间2天前向采购人提出答疑，采购人应解答响应人提出的问题。 ②采购人允许响应人在响应截止日期之前对云筑网响应进行修改，但必须在响应截止时间之前完成云筑网响应， 逾期未响应的，则视为无效响应。 （4）（4）响应文件递交事宜 采用云筑网电子响应。 4、评审： （1）评审方法：本次采购拟选出 1 名成交人，区段划分：（如选2个及以上，应明确划分各成交人分供范围及工 程量，成交人按照最终排名顺序享有优先选择权）。采用经评审的（原则上应选择合理低价法），在响应文件 能够满足采购文件实质性要求的响应人中，评审出响应价格合理低价的响应人，但响应价格低于其成本的除外， 具体由采购评审小组在评审会上商定。 （2）响应人有下列情形之一的，取消成交资格： ①成交人在成交后拒签合同； 网 ②成交人未按约定缴纳履约保证金。 采购人： 中国建筑第七工程局有限公司 务 采购时间：2026年8月 二、评 审 办 法 （一）、评审依据 商 1、采购文件 2、响应文件 道 3、评审办法 （二）、评审小组 管 1、评审小组成员：（评审小组应由5人及以上单数评审专家组成，项目负责人必须参与评审。与分供商存在利害 关系的应回避。） 2、小组成员负责根据国评审办法及标准开展评审工作。 3、与响应人有利害关系的，不得进入评审小组。 （三）、评审原则 中 （1）采取经评审的合理低价法：从满足采购文件实质性要求的响应人中，选择合理报价中最低者（不合理低价 除外）为成交分供商。 （四）、初步评审 有效分供商（资审通过并参与有效报价的分供商）数量不少于N（拟选分供商数量）+2家。（询比采购和竞价采 购要求，其他采购方式参照采购管理办法，下同） 出现以下情形的，响应无效。 1、未按要求缴纳响应保证金的。 2、未按要求完成线上响应的。 3、未响应采购文件的实质性要求和条件的。 4、响应人提供虚假资料、隐瞒误导采购的。 5、响应人以他人名义响应或者以其他方式弄虚作假，骗取成交的。 6、响应人ip重复、涉嫌弄虚作假或串通交易行为的。 7、采购文件或法律规定的其它情形。 （五）、详细评审 1、评审：以云筑网填报数据为准。 2、排名：对进入详细评审的响应人响应报价进行汇总后，按响应报价由低到高进行综合排名。 若出现响应人响应报价相同时，按其年度供应商考评评级高低优先排序，若仍相同，可再选用以下进行情况排序 （根据情况自行排序）。 网 ①近三年工抵房金额； ②具有绿色节能环保材料设备； 务 ③云筑网显示的该响应人响应时间等。 1）、采购概算金额（见采购公告）视为最高采购限价，响应人响应报价高于采购概算金额的，作无效响应处理。 响应人响应报价低于成本的，经评审小组评审确定后，作无效响应处理。 商 2）、在评审过程中，评审小组可以要求响应人对所提交的响应文件中含义不明确、表述不一致或者有明显笔误、 文字和计算错误的内容作出必要的澄清、说明或者补正，该澄清、说明和补正属于响应文件的组成部分，须经 采购授权代表书面署名确认，不得改变响应文件的实质性内容，且须经评审小组一致同意。评审小组不接受响 应人主动提出的澄清、说明或补正。 道 3）、经以上评审，有效响应人数量仍须满足“有效分供商（资审通过并参与有效报价的分供商）数量不少于N （拟选分供商数量）+2家”，否则本次采购按废止处理（成交单位数量为“N”）。 管 4）、废止后重新发起采购，需经调查核实后，视具体调查核实结果决定是否准予原响应人参与新发起的采购响 应。 （六）、确定成交候选单位 国 多轮次公开竞争报价：（说明：如需要(应视采购标的物及响应报价情况)进行多轮次公开竞争报价的，应按详细 评审的排名顺序确定一定比例(首轮最高价不得进入二次报价)的有效响应人进行后续轮次报价，总轮次不超过3轮 （竞价采购）。 中 报价规则：响应人提交的首轮报价作为后续报价基准；后续轮次总报价不得高于前轮报价，若设置参考价，单 项报价不得高于参考单价。否则该轮报价无效；最终轮次报价提交后不得撤回或修改（以系统记录为准）。 晋级规则：每轮报价截止后，采购人按报价从低到高排序；出现相同报价时，依次比较：（1）资源库等级；（2） （参考上述第五条第2点，以优质优价为原则，优先选用具备相应能力的本级及上级A级分供商） 成交机制：最终按末轮有效报价的从低到高排序；当最低报价出现多家时，可自主决定成交人。 最终按照排名顺序拟定有效响应人作为成交候选单位，具体成交候选单位数量由评审小组根据采购文件确定。 成交候选单位经审批后作为最终成交单位。 成交候选人放弃成交、因不可抗力不能履行合同、不按照采购文件要求提交履约保证金，或者被查实存在影响 成交结果的违法行为等情形，不符合成交条件的，采购人可以按照评审小组提出的成交候选人名单排序依次确 定其他成交候选人为成交人，也可以重新采购。 （七）、其他事项 1、因响应人原因造成其自身未响应采购要求及未能成交等情况，由响应人自行承担相应责任及损失，与采购人 无关。 2、本采购文件中的合同范本即实际签约合同范本，双方均不允许以任何理由更改合同内容。 三、响应注意事项 1、若响应人对采购文件中之任何内容有不理解之处，须立即联系采购人，以便在响应截止日期之前能予以解释。 2、采购人不保证一定要接受最低价成交，不论响应结果如何响应人的响应文件均不退回，且不对未成交单位做 任何解释。 3、响应人在响应之前，对本采购项的分包条件均已了解，响应即认为已详细了解。 4、采购人对响应人进行考察时，响应人应提供便利条件。 5、本次采购的最终解释权在采购人。 网 四、响应文件的上传 1需上传的响应附件（未上传视为不响应采购文件）有： 务 1.1.《响应函》 1.2.《响应承诺函》 1.3.法定代表人身份证明（格式）； 商 1.4.授权委托书（格式）（若若为法定代表人响应则可不提供）； 1.5.报价清单明细（盖章版） 道 1.6金融工具支付方式及优惠措施 1.7.响应保证金汇款凭证扫描件或免缴证明（云筑网平台缴纳的无须提供）（若需） 管 六、响应文件格式 一、封面（格式） 国 中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料采购响应文件 响应内容：临水临电材料采购 中 （编号：cscec2026081900001246027） 响应人：（盖章） 法定代表人 或授权代理人（签字盖章）： 响 应 函 致：中国建筑第七工程局有限公司 1、经勘察了本工程现场,并仔细研究了响应须知、合同协议条款、合同条件、采购图纸、工程规范、地质勘察报 告、工程量清单、响应答疑、及其他有关采购文件后，我公司愿以我公司云筑网所上传的含税综合单价，并按 采购文件所要求的条件承包在规定工期内完成重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料的施 工、竣工并补充其任何缺陷。 2、我公司保证本工程质量必须：达到符合工程所需材料质量验收标准、设计、合同及有关工程施工及验收规范 的要求标准。 3、一旦我公司的云筑网响应内容被接纳，我公司将在收到成交通知书后按贵公司的要求开始施工，我公司保证 于承诺的工期内或双方议定的工期内完成并交付本合同中规定的整项工程。 4、我公司同意在本区段的正式建设工程施工合同签署之前，云筑网响应将始终对我公司具有约束力，并可随时 被贵公司接受。 5、我公司知道：云筑网报价及云筑网响应的其他部分构成我公司向贵公司的要约，贵公司如发出成交通知书则 成交通知书及云筑网响应、采购文件将构成约束我们双方的合同，如果我公司在接到成交通知书后，没有按贵 公司要求的时间签署正式合同或坚持提出附加条件，那么我公司同意贵公司有权另选成交单位并向我公司追讨 有关损失。 6、我公司知道，贵公司并无义务必须接受所收到的价格最低的或其他任何响应书。 7、云筑网响应内容已考虑了贵公司向我公司发出的关于采购文件的相关答疑，网补充通知（如有的话） 8、云筑网响应效力优先于同时提交的任何响应文件的其他组成部分。 响应人： （盖章） 务 日 期： 年 月 日 响应承诺书 商 致：中国建筑第七工程局有限公司 我系有幸参与贵公司 重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料的响应，我公司经研究决定， 在此郑重承诺： 道 1、我公司在响应过程中已完全了解并掌握了采购内容、合同条件及施工现场等情况。确保云筑网响应报价操作 为本公司自己操作，如响应后发生非本公司操作的情形，本公司承担相应违约责任。 管 2、我公司已经详细阅读该采购文件所有内容，充分领会并完全接受采购文件所述响应人应尽的实质性的权利与 义务。我公司保证不会对采购文件产生不利于双方友好合作关系和将增加贵公司采购范围内经济支出的重大误 解。 3、我公司确认，贵公国司发出的采购文件所有内容为不可割裂的整体。 4、我公司保证成交后不会对成交价格提出任何异议，更不会以任何理由要求贵公司针对成交范围的价款要求额 外补偿。不会以不了解采购文件、合同文件为由或曲解、片面理解采购文件、合同文件或割裂采购文件、合同 文件，断章取义，向贵公司提出任何补偿要求。 中 5、在本合同的履约过程中，如因我公司的供货或质量原因导致贵司损失，我公司保证承担因此而给贵公司带来 的所有经济上的损失。 6、我公司将本工程作为重点项目对待，保证不会出现供货能力不能满足施工需要的现象。为满足本工程业主及 贵公司在质量、进度、安全、环保上的要求，我公司将采取一切措施保证物资设备生产、供应、租赁，运输等 均满足贵公司的要求，并保证不会因此而向贵公司提出增加任何补偿要求。 7、我公司承诺无论本工程最终的成本状况如何，将不会违背合同基本原则而向贵公司要求增加或补偿合同文件 约定以外的任何费用。 8、我公司认为，贵公司可以就物资设备采购数量或租赁时长进行调整，并且此种调整不构成我公司的索赔理由。 响应人：（盖章） 法定代表人或 其授权代理人：（签字或盖章） 日 期： 年 月 日 响应人名称：【全称】 单位性质： 地 址： 成立时间：年月日 经营期限： 姓名：性别：年龄：职务：系（响应人名称）的法定代表人。 网 特此证明。 响应人：（盖单位章） 务 年月日 授权委托书 商 本人（姓名）系（响应人名称）的法定代表人，现委托（姓名）为我方代理人。代理人根据授权，以我方名义 签署、澄清、说明、补正、递交、撤回、修改中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建 设项目 (二期)临水临电材料采购（采购项目名称）响应文件、签订合同和处理有关事宜，其法律后果由我方承担。 道 委托期限：本授权书于年月日签字生效，至本次采购期结束为止。授权期限内无特殊情况不变更合法授权代理 人。 代理人无权转委托。 管 特此声明。 响应人：（盖章） 国 法定代表人：（签字） 身份证号： 中 授权代理人：（签字） 身份证号： 联系方式： 日期： 年 月 日 备注：法定代表人和委托代理人必须在授权书上亲笔签名，不得使用印章、签名章或其他电子制版签名,同时附 法定代表人和授权代理人身份证复印件（正反面，加盖公章） 报价清单明细 不 含 含 不含 计量单 税 税 含税 备 序号 材料名称 规格型号 数量 税 税合 税额 位 率 单 合价 注 单 价 价 价 1 镀锌钢管 DN100*4.0 米 500 2 镀锌钢管 DN150*4.5 米 250 3 镀锌钢管 DN65*3.25 米 650 4 镀锌钢管 DN50*3.25 米 800 5 PE管 DN100*1.6MPA 米 450 6 PPR管 DN50*1.6MPA 米 400 7 闸阀 DN100 个 22 8 闸阀 DN250 个 10 9 截止阀 DN50 个 42 网 10 截止阀 DN25 个 60 11 蝶阀 DN100 个 6 12 消防箱 800×1000×250mm 台 20 务 功率30kw,扬程144m，流 13 加压泵（变频控制） 台 1 量55m/h 14 橡塑保温材料 DN100*20mm 米 620 商 15 橡塑保温材料 DN150*30mm 米 280 16 橡塑保温材料 DN65*20mm 米 700 17 压线钳 CO-1000 个 1 道 18 污水泵 380V4KW=25米 台 12 19 污水泵 380V5KW=30米 台 7 20 热熔机 63-160 台 1 管 21 电工胶布 / 卷 200 22 高压自粘带 / 卷 120 23 水泵控制箱 / 个 8 国 24 PE聚乙烯管 DE110*1.6MPA m 560 25 PE聚乙烯管 DE75*1.6MPA m 420 26 PE聚乙烯管 DE63*1.6MPA m 480 中 27 PE聚乙烯管 DE32*1.6MPA m 750 28 PE球阀 DN25 个 6 29 PE球阀 DN50 个 6 30 PE球阀 DN100 个 5 31 镀锌桥架 200*100*1.2mm 米 1200 32 PVC排水管 DE300*5.0 m 180 33 PVC排水管 DE200*5.0 m 380 34 PVC排水管 DE160*4.0 m 486 35 PVC排水管 De110*4.0 米 560 36 PVC排水管 DE75*3.0 m 420 37 PVC排水管 DE50*2.0 m 660 38 PVC排水管 DE32*2.0 m 380 39 PPR给水管 De90*1.6MPA 米 440 40 PPR给水管 DE75*1.6MPA 米 360 41 PPR给水管 DE63*1.6MPA 米 450 42 PPR给水管 De50*1.6MPA 米 435 43 PPR给水管 De40*1.6MPA 米 315 44 PPR给水管 DE32*1.6MPA 米 520 45 PPR给水管 De25*1.6MPA 米 680 46 PPR给水管 De20*1.6MPA 米 370 47 橡塑保温板 平板×20mm m 15 48 橡塑保温板 平板×30mm m 28 49 保温胶 3公斤/桶 桶 25 网 50 PPR给水管接头 De75 个 30 51 PPR给水管弯头 De75 个 20 52 PPR给水管三通 De75 个 22 务 53 PPR给水管接头 De63 个 20 54 PPR给水管弯头 De63 个 15 55 PPR给水管三通 De63 个 15 商 56 PPR给水管接头 De50 个 17 57 PPR给水管弯头 De50 个 22 58 PPR给水管三通 De50 个 17 道 59 PPR给水管接头 De40 个 14 60 PPR给水管弯头 De40 个 22 61 PPR给水管三通 De40 个 17 管 62 PPR给水管接头 De32 个 14 63 PPR给水管弯头 De32 个 14 64 PPR给水管三通 De32 个 17 国 65 PPR给水管接头 De25 个 22 66 PPR给水管弯头 De25 个 17 67 PPR给水管三通 De25 个 14 中 68 PPR给水管接头 De20 个 25 69 PPR给水管弯头 De20 个 17 70 PPR给水管三通 De20 个 22 71 PPR内丝直接 De25 个 17 72 PPR内丝直接 De20 个 84 73 球墨铸铁井盖 700*800*40T 套 22 74 球墨铸铁井盖 1000*1000*20T 套 20 75 球墨铸铁雨箅子 400*600*30 块 1750 76 球墨铸铁雨箅子 350*500*30 块 1200 77 高分子成品排水沟 300*300*1000 米 850 78 高压洗车机 380v/3KW 套 5 79 高压洗车机 380v/5.5KW 套 3 80 HDPE双壁波纹管 DN300 米 360 81 HDPE双壁波纹管 DN200 米 410 82 HDPE双壁波纹管 DN400 米 340 83 HDPE双壁波纹管 DN800 米 260 84 玻璃钢化粪池 20m 个 1 85 玻璃钢化粪池 50m 个 1 86 不锈钢消防水箱 12m 个 1 87 一级配电柜 2000*1200*500*630A 台 1 88 二级配电柜 800*600*210*250A 台 8 89 铜芯电缆线 YC3*16+2*10 米 60 90 铜芯电缆线 YC3*10+2*6 米 70 网 91 铜芯电缆线 YC3*6+2*4 米 70 92 铜芯电缆线 YC3*10 米 100 93 铜芯电缆线 YC3*6 米 100 务 94 铜芯电缆线 YC3*4 米 100 95 铜芯电缆线 YC3*2.5+2*1.5 米 100 96 聚录乙烯铝芯电缆 YJLV-22-4*185+1*95 米 50 商 97 聚录乙烯铝芯电缆 YJLY-4*25+1*16 米 90 98 聚录乙烯铝芯电缆 YJLY-4*35+1*16 米 100 99 聚录乙烯铝芯电缆 YJY-4*50+1*25 米 90 道 100 聚录乙烯铝芯电缆 YJLY-4*70+1*35 米 72 101 网线 Cat5e 米 100 102 铜芯电线 BV-2.5 米 400 管 103 铜芯电线 BV-4 米 300 104 铜芯电线 BV-6 米 200 105 铝芯电缆线 YJLV3*10 米 100 国 106 透明塑壳断路器 3P32A 米 34 107 透明塑壳断路器 3P63A 米 28 108 透明塑壳断路器 4P100A 米 26 中 109 透明塑壳断路器 4P160A 米 22 110 透明塑壳断路器 4P250A 米 20 111 透明塑壳断路器 4P400A 米 8 112 低压铝芯电缆 YJLV-4*300+1 米 20 113 低压铝芯电缆 YJLV-4*150+1 米 50 114 铝芯铠装电缆 YJLV-22-4*95+1*50 米 60 115 铜铝线鼻 300mm2 个 20 116 铜铝线鼻 150mm2 个 36 117 铜铝线鼻 95mm2 个 24 118 铜铝线鼻 50mm2 个 20 合计 0.00 0.00 0.00 1、综合单价：包括但不限于材料费、保险费、风险费、包装费、装车费、过桥过路费、管理费、检验费、技术 指导费、货到工地负责卸货堆入至指定地点等所有费用。本合同单价一次包死，在合同履行过程中不再做任何 调整。本合同的总价为暂估价，用方有权调整合同中材料计划或材料数量，材料数量和规格的调整，不影响本 合同单价及其他条款的执行。 2、计量方式：查看检测报告合格证，以实际验收通过数量计量。 3、付款比例：月结方式，即每月20日结算（遇节假日顺延），次月25日前（结算日后35日历天内），乙方提供 与结算等额增值税专用发票后，支付前月结算额的70%（遇节假日顺延）；供货完毕，验收合格，材料相关资料 （包括不限于合格证、质检报告等）移交甲方，且最终结算办理完毕6个月后付至最终结算价款的 97%；剩余3% 质保金在质保期满后30日内无息支付。质保期自全部货物供货完毕且竣工验收合格日起1年计算，支付工程款时 均应扣除根据采购合同应予扣除的其它金额。 4、付款方式： （1）现金支付:采用现金转账的模式支付； （2）非现金支付:包括不限于(1)金融工具支付:银行承兑汇票，商业承兑汇票，网应付账款保理，银行信用证，中 建财务公司承兑汇票。(2)工抵房支付。 5、响应报价表中所列数量的变动，丝毫不会降低或影响合同条款的效力。 务 6、整个合同执行期内，若遇市场价格下行，甲方有权做出价格调整，乙方应接受并重新签订补充协议确认价格。 若乙方无法接受新的低价，甲方有权重新选择其他能够响应该价格的供应商进行供货，乙方无条件同意。 响应人（加盖公章）： 商 法定代表人或授权代理人（签字）： 日 期：年月 道 金融工具支付方式及优惠措施 管 1、金融工具支付： 可接受金融工具支付比例累计为%，其中： ① 可接受的国银行承兑汇票比例%；贴息响应人自行承担。 ② 可接受的商业承兑汇票比例%；贴息响应人自行承担。 金融支付 ③ 可接受的应付账款保理比例 %；贴息响应人自行承担。 中④ 可接受的银行信用证比例%；贴息响应人自行承担。 ⑤ 可接受的中建财务公司承兑汇票比例为%；贴息响应人自行承担。 2、资产支付 资产支付 可接受比例为合同额的%。 3、优惠付款比例：按按照采购文件的付款比例，我方可优惠%。 4、如响应人提供其他由于采购条件的承诺，请逐项列示。 响应人（加盖公章）： 法定代表人或授权代理人（签字）： 日 期：年月 响应保证金汇款凭证扫描件或免缴证明（若需） 响应人（加盖公章）： 法定代表人或授权代理人（签字）： 日 期：年月 六、物资设备采购合同 合同编号：______________________ 物资采购与供应合同 （通用） 项目名称：【 重庆市第四人民医院科学城院区建设项目 (二期) 】 网 甲 方：【 】 乙 方：【 】 务 签订时间：【 】 签订地点：【 】 商 目录 1. 工程概况及供货范围 道 2. 企业性质 3. 合同价款 2 管 4. 质量要求 5. 供货时间及地点 6. 交货与验收 国 7. 结算方式及时间 8. 支付 中 9. 发票 10. 双方责任 11. 不可抗力 12. 权利瑕疵 13. 保密 14. 违约与赔偿 15. 联络与送达 16. 争议解决 17. 补充条款 18. 其他 物资采购与供应合同 甲方（买受人）：【中建七局安装工程有限公司 】 乙方（出卖人）：【 】 根据《中华人民共和国民法典》及有关规定，为明确双方权利、义务和责任，经双方协商一致，就甲方承包的 【高新LIVE（咸阳高新区租赁住房）建设项目】工程所用【 水电管材】采购与供应事宜签订本合同条款，愿共 同遵守。 1. 网 1.1 工程名称：【高新LIVE（咸阳高新区租赁住房）建设项目 】 1.2 工程地点：【陕西省咸阳市星火大道】 务 本合同供货范围为：【高新LIVE（咸阳高新区租赁住房）建设项目 】的【水电管材】供应（以下简称为“本合 同标的物”）。 1.3本合同标的物的数量为暂定量，乙方按附件1《计划采商购与供应物资清单》所列品种和规格供货，最终以经甲 方验收合格的实际数量为准。 2. 企业性质 道 乙方企业规模：大型 □中型 □小型 □微型企业 以上企业规模由乙方根据（1）工信部官网：“中小企业规模类型测试网址https://baosong.miit.gov.cn/ScaleTest。 （2）工信部微信小程序：“中小企业规模类型自测”两种渠道自测确定。 管 乙方应保证其企业规模的真实性。如乙方提供信息不实，经甲方查证后，将按照《中国建筑股份有限公司分供 商资源管理办法》中的《不良行为分供商禁用处理标准》第19项对乙方严格实施禁用管理。 合同价款 国 3.1 本合同采用第【 】种价格形式： （1）固定综合单价包干，价格不可调整。 中 3.2 本合同价款为各项货款之和，合同价款（含增值税）暂定：（大写）【 】（￥【 】元），其中不含税价款为 （大写）【 】（￥【 】元），增值税为（大写）【 】（￥【 】元），税率为【 】%。最终甲乙双方以实际验收 的数量结算。 3.3 本合同约定的不含税价款不因国家税率变化而变化，在合同履行期间，如遇国家的税率调整，则价税合计的 合同价款或货款相应调整，以开具发票时间为准。 3.4 本合同不含税价款仅指不包含增值税，除增值税外的其他全部税费（包括但不限于城市建设维护税、教育费 附加及地方教育费附加、个人所得税、合同印花税、企业所得税、车船使用税以及国家和地方规定的所有税费） 均包含在不含税价款中。 3.5 本合同标的物的计价、结算和支付货币均为人民币。 3.6 本合同标的物的计量单位为中华人民共和国法定公制计量单位（除技术规范标准另有规定外）。 3.7 本合同标的物的不含税单价，指运抵本工程施工现场甲方指定交货地点的综合单价，包括但不限于货物费、 加工费、包装费、人工搬运费（由乙方自行协调，甲方只进行指定场地和材料验收工作）、运输费、出厂检测费 （包括但不限于到场后的第三方检测费用）、装卸费、码放费、现场倒运费用，保险费、仓储费、驻厂监造费、 运输造成的道路污染的清理及维修费用、除增值税以外的税金、乙方合理的利润、管理费、市场价格波动带来 的风险、向有关部门缴纳的各项费用以及政策性文件所规定的各项应有费用等乙方履行本合同规定义务的全部 价款与费税。除本合同第3.1条约定的因素外，不含税单价不因政府政策变动、市场环境改变、税率调整等而调 整。 3.8 除合同条款另有约定外，本合同标的物的不含税单价已包含专利、专有技术以及技术秘密的使用费。 质量要求 4.1 乙方应在交货同时向甲方提供本合同标的物制造商出具的书面质量保证书。 4.2 本合同所采购与供应的物资，应符合现行中华人民共和国国家标准及行业或地方标准，行业标准或地方标准 高于国家标准的，执行行业标准或地方标准。各项技术性能指标经本工程所在地具有相应检测资质的专业机构 或单位检测中心检验必须符合相关标准要求。合同执行过程中，若出现新的国家标准、行业标准、地方标准， 则以更新后的标准为准。 网 4.3 乙方的物资供应与管理应符合国家有关环保法律、法规和甲方ISO14001环境体系及OHSMS18001职业安全健康 管理体系标准。 4.4 本合同标的物的质量保证期为最后一批货物验收合格之日起满【180】日。 务 4.5在合同履行期及质量保证期内，乙方无条件地向甲方提供缺陷产品的免费维修、更换等服务。针对甲方提出 的书面要求，乙方必须在3日内给予书面答复。如有必要，乙方在3日内指派专人到现场解决，因此产生的所有费 用均由乙方承担。 商 4.6 如缺陷产品经乙方进行免费维修和更换后仍无法达到甲方要求的质量标准时，甲方有权终止合同。终止合同 后，乙方需向甲方赔偿由于乙方问题造成的损失及其连带损失。如乙方借故推脱或拒绝甲方提出的维修、更换 等服务请求，甲方有权自行采购同等货物替代或委托第三方维修，实际发生的更换等或维修费用，从应支付给 乙方的任一期货款中扣除，并保留进一步索赔道的权利，乙方不得提出异议。维修或更换物资的质量保证期相应 延长6个月。 4.7 如因乙方产品质量导致工程出现质量问题，由此给甲方造成的一切损失由乙方承担。 管 4.8 其他质量要求：/。 供货时间及地点 5.1 供货方式：□按批次国供货 □一次性供货 5.2 通知方式：供货时间及数量以甲方书面通知为准，甲方可以选择通过电子邮件、微信、QQ等方式将物资采购 订单发送至乙方。紧急情况下，甲方可口头通知乙方发货，手续后补，乙方应予以确认。 中 5.3 供货地点：乙方负责送货至施工现场，卸至甲方指定的卸货地点【高新LIVE（咸阳高新区租赁住房）建设项 目】。乙方不得雇佣甲方在班人员及设备装卸货物。运输、装卸过程中发生的安全事故责任，乙方自行承担。 5.4 根据工程项目施工需要，甲方对所采购物资的数量和送货时间如有变更，应及时书面通知乙方，乙方按变更 后的数量和送货时间供货，货物单价不因货物数量和送货时间的变更而变化。 5.5 乙方应确保已经知悉货物运输的交通状况、交货卸车环境以及政府的交通管制政策措施，不得以此等理由要 求增加费用、减免责任、提出索赔、要求延长或变更供货期限。 交货与验收 6.1交货 6.1.1 除另有规定和协议要求外，乙方提供的全部货物须采用国家、企业、行业标准要求包装，具有足够的强度 及安全起吊标识，保证货物能够经受多次搬运、装卸、长途及短途运输的要求，并采取良好的防潮、防震、防 腐蚀、防爆及防止其它损坏的必要保措施。包装物的回收按以下第【 2】项方式执行：（1）不回收；（2）包装 物由乙方在交货时回收；（3）其它方式：【 /】。 6.1.2 装箱单应注明货物的名称、规格、型号、数量、质量、生产商、发货地、供货人、收货人、交货地、承运 人等，并在显著位置标明装卸警示标志。 6.1.3 乙方运抵甲方指定现场的物资，交货单据上应详细列明当次供应物资的名称、品牌、产地、生产厂家、规 格型号、计量单位、数量。 6.1.4 乙方应向甲方提交本合同标的物的技术文件，包括材质报告（物资质量检验报告）和出厂检验报告（合格 证），以及按照工程竣工验收规定及甲方要求，提供所有相关符合要求的资料。 6.1.5 乙方在首次供货前需提供样品，乙方须在样品和样品资料上加盖单位公章，样品经双方指定人员签字确认 后予以封存，在提交文件上注明与合同文件约定不同之处。 6.2.1 乙方须随货提供载有数量、规格等内容的送货单，否则，甲方有权对本批次货物不予验收确认，由此导致 的违约责任由乙方承担。乙方送货到交货地点后，甲方指定验收人员对产品的规格、尺寸偏差、外观、数量及 质量证明资料等进行查验。若产品的以上各项符合合同约定，则双方人员共同在收领单上签字确认。 6.2.2 甲乙双方在交货现场以 【 点数】方式进行数量验收。乙方应对在甲方工地网现场的验收数据进行确认。 6.2.3 进行数量验收的同时，甲方可以按照封存样品标准进行尺寸、外观质量验收，尺寸和外观质量符合要求方 可卸车，否则不得卸车。 务 6.2.4 外观质量符合要求的， 甲方可打开包装进行质量、性能检验或及时按规定取样送本工程所在地具有相应检 测资质的专业机构或单位进行检测。抽检未发现不合格产品不视为乙方供应产品全部合格，甲方有权随时将乙 方所供货物送到有检测资质的第三方进行检测。如检测合格，检测费用由甲方承担；如检测不合格，甲方可全 部退货，检测费用由乙方承担，并承担由此给甲方造成的一切损失。 商 6.2.5 甲方及工程监理（业主）的收货验收仅作为感观合格的依据，不能免除乙方对货物品牌真实性、内在质量 及使用功能所负的责任。如甲方、本工程建设单位或监理单位提出异议，乙方需参照有关标准规范，结合现场 情况解决。 道 6.2.6 若发现不合格产品，乙方必须及时（接到甲方通知后【 3】小时内），从甲方项目现场运走不合格品，甲方 不负有保管义务，不对不合格产品的损毁灭失承担人和责任，若超过【 12】小时乙方仍未运走的，甲方收取场 地租赁费（根据货物合理确定）【 1.0】万元/天，且不合格品的储存、装卸、运输等所有相关费用及风险由乙方 承担。 管 6.2.7 如因乙方产品问题造成甲方工期、质量、劳务等损失，全部责任均由乙方承担。乙方对甲方所提出的质量 问题有不同意见的，双方可送至双方共同选定的具有法定资质的检测机构检测，所产生的费用及责任由责任方 承担。 国 6.2.8 本合同的标的物所有权自【卸货完毕且经甲方验收合格】起转移。 结算方式及时间 中 7.1 过程结算：甲乙双方按以下第【 1】条约定的时间办理过程结算。 （1）每月20日结算（遇节假日顺延），每季度最后一个月的25日后支付当期货款额的70%（遇节假日顺延，乙 方提供与结算等额增值税专用发票），供货完毕，验收合格，材料相关资料（包括不限于合格证、质检报告等） 移交甲方，且最终结算办理完毕6个月后付至最终结算价款的 97%，余款3%（不计息）待质保期满无质量问题后 无息付清。（质保期为供货完毕且验收合格后2年）（支付工程款时均应扣除根据采购合同应予扣除的其它金额。 ）； （2）按节点结算，具体结算节点为：【 】。 7.2 最终结算：全部供货完毕后【 6个月后】日内，乙方应向甲方提供完整的结算资料，甲方在收到完整的结算 资料后【 5 】日内进行审核。 7.3 结算依据：包括但不限于物资采购与供应合同、乙方合法等额有效增值税发票（含税务机关代开）、产品合 格报告、项目授权人员验收单、送货单等有效材料。 7.4 乙方未按照约定的期限和甲方要求提供结算资料，或未委派专人与甲方办理结算，或提供的结算资料不齐全、 提供虚假资料的，经甲方催告后10个工作日内，乙方仍未按要求提供结算资料的，甲方有权不予办理结算并暂停 支付材料款，同时甲方可根据本合同、现有结算资料及乙方实际履约情况单方办理结算，确定结算价格，结算 对甲乙双方具有法律约束力。 支付 支付/√不支付预付款 8.1.1 预付款金额（或占合同价款的比例）：【 /】。 8.1.2 预付款的支付时间：【 /】，在乙方提交等额银行保函及增值税专用发票后，甲方向乙方支付预付款。 8.1.3 扣回预付款的时间、比例：【 /】。 8.1.4 乙方提交的银行保函有效期至预付款抵扣完为止，若预付款保函到期日前，预付款无法抵扣完毕，则乙方 应于预付款保函到期日前不少于10日及时办理保函延期，否则甲方有权暂停支付未抵扣完部分的货款。 网 / 8.2.1 货款支付，按以下第【 3】条约定的时间和比例支付。 务 （1）月度付款：甲方在次月的25日支付上月月度结算货款的【 / 】%。双方办理完毕最终结算后【 / 】（条款说 明：建议不超过60日，如超过60日，应当按照行业规范、交易习惯合理约定付款期限并及时支付款项）个日历天 内付至总结算货款（且不超含税合同价款）的【 / 】%。余款【 /】%作为质保金，在质保期届满后28日内付清； 或由乙方提供等同余款金额的质保保函（仅接受金融机构出具的无条件见索即付保函，质保保函格式以开函金 融机构标准格式为准），则双方办理完毕最终结算后【 /商】（条款说明：建议不超过60日，如超过60日，应当按 照行业规范、交易习惯合理约定付款期限并及时支付款项）个日历天内付清。 （2）节点付款：按节点支付（条款说明：此处需具体罗列每个付款节点及各节点对应的付款比例，节点结算完 成后约定支付期限应在60日内，如超过60日，道应当按照行业规范、交易习惯合理约定付款期限并及时支付款项）， 余款【 /】作为质保金，在质保期满后28日内付清，或由乙方提供等同余款金额的质保保函（仅接受金融机构出 具的无条件见索即付保函，质保保函格式以开函金融机构标准格式为准），则在最后一个付款节点付清。每次 付款前乙方应提供结算值【100%】的发票，否则甲方可拒绝付款。 管 （3）其他支付方式【每月20日结算（遇节假日顺延），每季度最后一个月的25日后支付当期货款额的70%（遇 节假日顺延，乙方提供与结算等额增值税专用发票），供货完毕，验收合格，材料相关资料（包括不限于合格 证、质检报告等）移交甲方，且最终结算办理完毕6个月后付至最终结算价款的 97%，余款3%（不计息）待质保 期满无质量问题后无息付清。（质保期为供货完毕且验收合格后2年）（支付工程款时均应扣除根据采购合同应 予扣除的其它金额。）国】 （4）甲方依合同约定确认的进度款仅为中期付款依据，不作为竣工结算的依据，且不视为对因变更调整的合同 价款、索赔的价款或费用以及其他约定的追加合同价款的确认。 中 8.2.2 甲乙双方协商一致同意本合同采用【银行转账支票、网银转账、银行承兑汇票、银行保理、商业承兑汇票、 国内信用证、应收账款电子凭证、抵房抵款及其他】常规支付方式的付款方式。付款过程中产生的贴息费用及 手续费由【乙方】承担。乙方委托专职收款人办理收付款业务，收款人必须取得授权 8.3 乙方指定以下帐户为收款帐户，甲方所有款项均需通过该帐户支付。如乙方变更收款帐户，应提前十五天以 上书面通知甲方，否则造成资金的损失由乙方自行承担，与甲方无关。 账户名：【 】 开户行：【 】 账 号：【 】 发票 9.1 乙方在向甲方请款时，应根据甲方确认的应支付金额开具合法、有效、完整、准确的增值税（请勾选：□专 用□普通）发票，计税方法为【□一般计税方法 □简易计税方法】，双方发票信息如下： 名 称 纳税人身份 □一般纳税人 □小规模纳税人（请勾选） 甲方 纳税人识别号 地 址、电 话 开户行及账号 名 称 纳税人身份 □一般纳税人 □小规模纳税人（请勾选） 网 纳税人识别号 乙方 地 址、电 话 开户行及账号 务 联 行 号 该开户行为乙方在税务局已备案的乙方单位账户。 9.2 任何一方如上述信息发生变更，应提前10日以书面方商式通知另一方。如一方未按本合同规定通知而使另一方 遭受损失的，应予以赔偿。 9.3 每次乙方在甲方付款前必须提供符合国家现行税法规定的合法有效等额增值税发票，甲乙双方一致确认提供 发票为主合同义务而非附随义务，若乙方未按要求提供发票，甲方有权暂停付款。乙方应在开票之日起7天内将 道 发票送达甲方指定人员【 刘磊】，甲方指定人员签收发票的日期为发票的送达日期。 9.4 乙方开具的增值税专用发票应保证信息完整、内容规范，如乙方未提供发票或提供的发票不合规、不及时、 无法认证，甲方有权拒绝付款，且不视为甲方付款逾期，乙方无权要求甲方支付利息、违约金或赔偿损失，也 管 不得以此为由中止履行合同约定的义务。 9.5若乙方由一般纳税人身份变为小规模纳税人身份的，或者计税方法发生变化的，或者政策法规等规范性文件 发生变化的，并导致甲方可抵扣的进项税额减少或被税务机关要求补缴税款的，则减少的进项税额或补缴的税 款应由乙方承担，甲方国有权从将支付的任何一笔款项中扣除。 9.6 增值税税率变化：合同执行过程中如果遇到国家税务政策调整，增值税税率发生变化的，按新的税率执行， 不含税价不变，仅调整增值税税率的原则进行相应调整。 中 若乙方提供的发票不符合要求的，发包人有权拒收增值税发票，并有权暂停支付相应款项，乙方不得以此为由 中止履行合同的义务。如因乙方不能按期提供发票或提供的发票不符合要求而导致付款延期的，由其自行承担 后果，发包人不承担任何责任。 9.8若乙方迟延提供发票的，每日应按暂定合同总价的0.05%向甲方支付违约金，但迟延违约金累计支付不超过90 日；若乙方迟延提供发票超过90日且已跨年的，视为乙方未提供发票，乙方除应支付前述迟延违约金外，还应另 行向甲方支付以下款项： （1）相当于合同暂定总价1%的违约金； （2）甲方因未收到发票所产生的税款损失， 损失金额按以下公式计算：赔偿损失金额=未提供发票对应的增值税税额*（1+增值税附加税率）+未提供发票金额 *甲方企业所得税税率。 9.9乙方保证开具的发票已经依法足额纳税，支付每笔款项前，乙方需提供发票对应税期的增值税纳税申报表和 完税证明。 9.10乙方承诺其提供的发票真实合法，若发包人认证后出现走逃失联、被列为异常纳税人等违规行为，导致发包 人不能认证抵扣或者认证抵扣后被税务机关要求进项转出情形，应在72小时内补开合规发票，否则按以下方法计 算应赔偿发包人损失，应赔偿损失金额=进项转出税额*（1+增值税附率)+不合规发票金额*发包人企业所得税税 率，逾期未赔偿的，甲方有权从结算金额或者履约保证金中扣除。 9.11乙方主张已开具发票的，应提供：①税务系统发票开具记录 ；②采购方签收凭证或者发票邮寄物流凭证。无 法完整提供两项证据的视为未开票。 10.双方责任 10.1 双方现场代表 10.1.1甲方现场代表为【 】，其职务为【 】 ，其授权签署文件的范围为：【签发监管项目的各类文函、工程变更 指令、索赔文件的报出、违约处罚决定文件等】。 10.1.2甲方收货代表：【 】，联系电话【 】。甲方指定收货代表仅有对乙方送货单中货物的数量及乙方提供的单 据是否齐全子以确认的权利，对货物单价、质量、货款以及总结算单没有确认的权利。 10.1.3乙方应将物资按合同约定时间运至甲方指定地点，并经甲方指定收货代表和甲方工程项目所属其他1人及以 上在甲方指定的收领单上签字验收确认后有效。 网 10.1.4 甲方未经授权的任何人员和项目印章均无权从事下列行为：【（1）签订本合同的补充协议或签署其他合 同类文件，包括但不限于采购合同、分包合同、租赁合同；（2）签署任何借贷、担保性质的文件，包括但不限 于借条、保函、保证书、承诺书；（3）签署代他人清偿债务的文件，签署任何放弃债权的文件；（4）签署任何 对总承包合同进行修改和补充的文件;（5）收取现金及任何款项；（6）签署合同价款的变更、结算及支付确认 务 文件；（7）签署任何劳动关系确认文件、工资发放承诺文件。】 10.1.5 甲方授权人员的职权/职责范围、授权签署文件范围均不可转授权，任何形式的转授权、代签行为，甲方均 不予认可且不承担任何法律责任。 商 10.1.6 乙方确认已完全明白和理解甲方对甲方人员及项目印章的上述授权范围，超出甲方授权范围的行为属于无 权代理行为，对甲方无效，甲方不承担任何法律责任。乙方应谨慎审查相关文件的签署主体资格和权限，对于 无权代理人签署的相关文件，乙方应及时与甲方核实。 道 10.1.7 乙方现场代表为【 】，其职务为【 】，其授权范围为：【全面代表乙方履行本合同，并有权代表乙方签署、 确认履约过程中形成的工程变更、价款确认、经济索赔、违约处罚决定及物资丢失损坏赔偿文件；签署确权文 件及结算书；签收甲方发出的各类文函、工程变更及其他文件等。】 管 10.1.8 双方更换各自代表时，应及时书面通知对方，以确保物资顺利交接。 10.1.9 甲方禁止项目部及任何人员以甲方、甲方分公司、甲方项目部的名义对外借款或者支取任何款项，如乙方 或乙方有关人员以任何形式将款项出借或支付或返还给甲方项目部及任何人员，则不论该等款项是否实际用于 甲方工程，均与甲方无国关，该行为均属于乙方与相关人员个人之间的经济关系，乙方无权向甲方主张任何权利。 10.1.10 未经甲方书面授权不得擅自与建设方及有关部门发生工作上的联系，严禁在对外任何事务中签署甲方单 位名称或带有甲方简称中任何“【中国建筑】”“【中建】”“【中建XX局】”“【XX局】”等字样的落款， 每发现一次中乙方承担2万元的违约金并赔偿所有直接或间接损失。 10.2卫生、环境与安全保护 10.2.1 甲乙双方须贯彻执行国家、地方政府相关部门发布的有关卫生法律、法规，以及甲方发布的规章制度，积 极配合政府部门的检查，对于提出的要求按所属责任立刻整改，确保瘟疫和传染疾病防控的管理落实到位。 10.2.2 乙方保证在运输和卸货过程中应采取相应的环保措施，符合国家环保要求。车辆在进入项目现场要保证不 沾泥土和脏物，车辆出入项目现场必须在项目大门内现场洗车。乙方在卸货过程中保证噪声不超过以下标准 （白天小于或等于【 】dB、夜间小于或等于【 】dB）。乙方保证乙方人员以及车辆进入本工地现场，应遵守现 场的一切卫生环保、文明施工的规定，因违反环保要求所造成的一切罚款由乙方承担。 10.2.3 甲乙双方必须贯彻执行国家和政府、行业主管部门颁布实施的有关安全生产的法律、法规及有关规定。乙 方车辆及人员进出工地现场时必须接受甲方安全检查。乙方因供货造成安全生产责任事故的，责任由乙方承担。 乙方必须对自身出入工地现场的人员进行安全交底，并为其配备安全防护用品，因乙方原因造成的各种人员伤 害及经济损失由乙方自行承担，并赔偿甲方及其它方因此造成的一切损失。 10.3 售后服务 10.3.1 如所供货物为专业性较高的产品，乙方应免费为甲方或工程业主提供操作及维修人员的培训服务，培训内 容应包括：基本原理、操作使用、维修保养等。 10.3.2 对于工程中的剩余或未使用到的货物在不严重影响外观、质量和功能的情况下甲方有权退货，退货原则上 以合同约定的含税单价为准，确因商品特殊的（比如定制等），价格由双方协商，协商不一致的，按照附件1 《计划采购与供应物资清单》中的含税单价（考虑甲方已支付费用、乙方承担运费等情况下，原则上不低于【 】%）【 】%退货，退货数量以实际数量为准。 不可抗力 11.1 不可抗力是指合同当事人在签订合同时不可预见，在合同履行过程中不可避免且不能克服的自然灾害和社会 性突发事件，包括地震、海啸、瘟疫、骚乱、戒严、暴动、战争等情形。 11.2 不可抗力事件发生后，乙方应立即通知甲方现场代表并迅速采取措施，尽量减少损失，并在24小时内向甲方 通报受害情况，提供必要证明。不可抗力持续发生，乙方应每日报告一次受害情况，直到不可抗力结束。甲方 应对受害处理提供必要的条件，并负责处理工作的组织、指挥。不可抗力发生后网，乙方未采取有效措施控制灾 害而发生的损失由乙方承担。 11.3 不可抗力引起的后果，由甲乙双方应各自承担其人员伤亡及财产损失，履行合同的期限相应延长。 务 不可抗力发生后，双方均应采取措施尽量避免和减少损失的扩大，任何一方没有采取有效措施导致损失扩大的， 应对扩大的损失承担责任。 因一方迟延履行合同义务，在迟延履行期间遭遇不可抗力的，不能免除迟延履行方的违约责任。 商 11.4 因单次不可抗力导致合同无法履行连续超过【30】天或累计超过【60】天的，甲方有权解除合同。合同解除 后，双方应就合同履行情况及结算与付款等善后事宜达成补充协议。 权利瑕疵 道 12.1 涉及到知识产权（专利权）标记的产品，乙方应提供知识产权（或专利权）及其权属的有效证明材料。乙方 承诺其提供的物资不侵犯他人的知识产权（或专利权），若乙方提供物资侵犯他人知识产权（或专利权）导致 他人向甲方索赔的，乙方承担由此给甲方造成的一切损失，包括但不限于甲方处理此纠纷发生的律师费、诉讼 管 费、仲裁费、差旅费等一切损失。此外，乙方应向甲方支付合同价款【5】%的违约金。甲方针对上述一切损失 有权从乙方结算货款中扣除或依法追索。 12.2 乙方所供物资应不存在任何权属纠纷及抵押、查封等权利限制情形，如乙方所供物资存在权属纠纷或任何权 利限制情形导致甲方遭国受损失，乙方应赔偿甲方全部损失。 保密 13.1 除法律规定或合同另有约定外，未经乙方同意，甲方不得将乙方提供的技术秘密及声明需要保密的资料信息 中 等商业秘密泄露给第三方。 13.2 除法律规定或合同条款另有约定外，未经甲方书面同意，乙方不得将甲方提供的图纸、文件以及声明需要保 密的资料信息等商业秘密泄露给第三方。 13.3 任何一方违反上述约定，应负责赔偿守约方因此造成的一切损失。 违约与赔偿14.1甲方应按照合同约定及时向乙方支付合同价款，若因甲方资金不到位，乙方同意给予甲方【 30 】 日的宽限期，宽限期内不视为甲方违约。超过宽限期仍未支付的，乙方可向甲方主张自宽限期结束后的违约金； 违约金以逾期支付的价款为基数，自宽限期结束之日起至甲方支付逾期价款之日止，按照中国人民银行同期活 期存款利率向乙方计付，向乙方计付，逾期支付违约金的上限为逾期支付金额的【 / 】%（不超过3%）。在我方 支付逾期付款利息后，分供商不可就此向我方再主张逾期付款的违约责任。（条款说明：乙方为中小企业时， 甲方前述条款支付期限+本条宽限期整体不得超过60日）。14.2 除本合同中规定的不可抗力外，其他不论任何原 因，乙方若不能按约定期限足额足量送至甲方指定现场存货地点，甲方向乙方收取逾期运达物资货款（含增值 税）每日【3】％的违约金，自逾期之日起计算至乙方实际送达之日止，延迟或供货不足超过【3】日时，甲方有 权单方面终止合同。14.3 未经甲方书面同意自行停止供应本合同约定的货物，均视为乙方违约，乙方除承担因此 给甲方造成的一切损失外，乙方另支付合同价款的【5】%作为违约金。 14.4若乙方提供的货物为非合同约定的厂家或品牌的产品，或提供的是假冒他人品牌的产品，甲方有权立即终止 合同，乙方必须支付合同价款【2】倍的违约金给甲方，如乙方所供产品已安装至工程项目，则乙方除承担违约 金外，还必须承担拆除、工程维修、工作面清理和重新安装产生的所有费用等，如违约金不足以弥补因此给甲 方造成的所有损失，包括一切直接损失和间接损失，则超出部分，甲方有权向乙方追偿。乙方提供的货物为合 同约定的厂家及品牌产品，但货物质量不合格或不符合约定的技术要求时，可由乙方负责更换质量合格和符合 约定技术要求的产品，同时承担合同价款【5】%的违约金，并承担因违约造成的各项损失，甲方也可直接要求 解除合同，乙方承担因此给甲方造成的所有损失。乙方提供的合同标的物因品牌、质量等原因导致甲方被项目 业主或总包方罚款或追究违约责任，乙方应向甲方相应承担赔偿责任。 14.5 本合同履行过程中，如果乙方不能按时交货，应在交货前48小时内以书面形式通报甲方，甲方视情况确定是 否同意变更供货时间。如甲方不同意变更供货时间，可自行采购部分或全部货物。甲方在自行采购和接收该违 约部分货物时实际发生的所有额外费用及因此给甲方造成的损失，从甲方应支付给乙方的任一期货款中扣除， 甲方同时保留进一步索赔的权利。 14.6甲方提出索赔通知后，乙方应在【28】日内答复，如果在【28】日内未答复，视为乙方已接受该索赔，同时 甲方保留进一步要求赔偿的权利。 网 14.7 乙方在进出场时乙方不得私自运送甲方现场物资出场，一经发现，乙方向甲方支付所涉及物资原值【2】倍 的违约金，情节严重的交由司法机关处理。 务 14.8 由于乙方自身原因（如：不按约定开立银行账户、未及时提交报量资料或不按合同配合甲方进行款项支付 等），导致货款或工程款延期支付，甲方不承担延期付款利息及违约金，乙方不得因此停止供货；乙方擅自停 供的视为乙方违约，乙方承担因此给甲方造成的所有责任及损失。 14.9 如果出现合同为可调价合同，甲乙双方调价达不成一致商情形；或者出现合同为不可调价合同，乙方提出调价， 甲乙双方达不成一致情形，则甲方有权选择其他供应商，甲方不承担任何违约责任。 14.10 若乙方因14.5和14.9款原因停止供货，或未完成全部供货、或主张解除合同等不履行合同的情形，乙方剩余 款项的支付不适用本合同8.2条款，甲乙双方应道就剩余款项的支付签订书面补充协议，重新明确支付条款，甲方 不承担任何违约责任。 14.11 其他违约与赔偿要求：【 /】。 管 联络与送达 甲方：收件人【 】，联系电话【 】，电子邮箱【 】，地址【 】。 乙方：收件人【 】，联国系电话【 】，电子邮箱【 】，地址【 】。 15.2 一方通过电子邮箱发送文件的，文件到达对方邮箱即视为送达，送达时间为电子邮件到达对方邮箱地址时间； 一方通过信函邮寄送达的，则信函寄出后的第三个工作日或收件人实际签收日（以先到的时间为准）视为送达； 一方选择直中接送达的，则递交时视为送达。 15.3 邮件邮寄至上述地址被拒收或无人签收，亦视为已经送达，由此增加的费用和（或）延误的期限由拒绝接收 一方承担。 15.4 双方承诺，因本协议的履行或争议解决，上述联系人和联系方式为有效的联系方式，各项通知均应当向上述 联系人、联系方式送达。在诉讼、仲裁中，上述联系人、联系方式亦为有效的送达地址，向上述地址的送达即 为有效送达，即使发生拒收、退信等事件。 上述联系信息发生变更的，变更方应当即时通知对方；在对方收到变更通知之前，对方当事人或者仲裁、司法 机构已经向原联系人、联系方式进行的通知，视为有效通知。 争议解决 16.1 因本合同引起或与之相关的任何争议、纠纷或权利主张，则必须先行向对方发出书面和解申请书，并告知对 方争议、纠纷或权利主张之事实及依据、联系人及联系方式，在对方收到上述通知之日起 3 个月为双方和解期限。 在和解期限内，若双方达成和解协议的，双方的权利义务按照和解协议履行；若未达成和解协议的，任何一方 采用下列第【 】种争议解决方式，并自行承担本方发生的律师费、差旅费、保函费等相关费用∶ （1）向仲裁委员会申请仲裁 周口仲裁委员会（开庭地点：郑州） 郑州仲裁委员会 武汉仲裁委员会 北京仲裁委员会 上海仲裁委员会 中国国际经济贸易仲裁委员会 R成都仲裁委 （2）向【 】人民法院提起诉讼。 网 1.因本合同引起的或与本合同有关的任何争议，如仲裁委员会，则按照其仲裁规则进行仲裁。仲裁裁决是终局的， 对双方均有约束力。 务 2.双方承诺：任何一方向仲裁委员会申请仲裁的，双方均自愿放弃向对方主张仲裁费用和实际发生的其他费用， 包括但不限于鉴定费用、评估费用、审计费用等；双方均自愿放弃向对方主张补偿因办理案件支出的合理费用， 包括但不限于律师费、保全费、差旅费、公证费等。 3.双方约定：仲裁案件无论标的额大小、复杂程度如何，商均适用普通程序，即由三名仲裁员组成仲裁庭审理，以 确保案件公正审理。 4.调解期限：争议应先行和解协商解决，设定3-6个月和解期（可根据情况调整），且和解期限不计入仲裁审理 期限。任何一方若未履行上述和解程序而直接道提请至争议解决机构的，则需要向对方承担签约合同价【10】%的 违约金；如一方出现上述情形，另一方提起反诉或反请求，则提起反诉或反请求的一方不承担违约金。 17.禁止债权转让条款甲乙双方确认，若发生下列任一情形，即视为乙方重大违约，乙方需向甲方支付合同总价 （建议10%） %的违约金，且甲方有权视违约程度单方解除本合同，同时乙方应赔偿甲方因此遭受的全部损失 管 （包括但不限于直接损失、间接损失、维权产生的律师费、诉讼费、保全费等）。具体情形如下： （1）未经甲 方事先书面同意，乙方擅自将其在本合同项下对甲方享有的全部或部分债权进行转让、质押或以其他方式处分 给任何第三方的； （2）因乙方与乙方债权人存在债务纠纷，导致该乙方债权人以甲方为被告或被申请人提起代 位权诉讼、仲裁或采取其他司法/仲裁手段的； （3）未经甲方事先书面同意，乙方以自身名义或委托任何第三 方，就本合同相关事项国对甲方的关联单位（包括但不限于业主单位、建设单位、 发包方）提起代位权诉讼、仲 裁或采取其他司法/仲裁手段的； （4）其他性质同上述条款规定的情形。18.补充条款 /】 中 其他 19.1 本合同采用下列第【 2 】种签订方式： （1）本合同自双方签字并盖章后生效，一式【叁】份，甲方执 【贰】份，乙方执【壹】份，每份具有同等法律 效力。 （2）本合同采用电子签章签署生效。根据《中华人民共和国民法典》、《电子签名法》等相关法律、法规，双 方一致认可在【 】平台（网址：【 】）使用电子印章签署合同为其真实意思表示，且确保在该平台注册时，使 用的企业信息和个人相关信息真实有效，并且自觉遵守国家法律法规和甲方在该平台的合同签约流程。甲乙双 方使用电子签章方式签署的合同，只有通过验证生效的电子原件具有法律效力，未经电子印章服务平台公司提 供书面证明材料的电子合同打印版不能作为法律依据。如因乙方使用不当给甲方造成损失，乙方愿自行承担由 此造成的全部经济损失和法律责任。 19.2未尽事宜经双方协商一致后，可签订补充协议，与本合同具有同等法律效力。 19.3对于因本合同产生的任何争议或投诉，乙方可通过【 】（条款说明：根据各公司情况填写投诉平台或者联系 方式）进行提交。甲方将在收到乙方的投诉后，对乙方的投诉进行初步审查，并尽快与乙方取得联系以进一步 了解详情。因不可抗力或第三方原因导致无法按时处理投诉的情况，甲方将尽快通知乙方，并尽力协调解决问 题。 19.4本合同条款（包括但不���于免责条款、责任限制条款等）均经双方充分协商，双方已就全部条款内容达成一 致意见，不存在单方预先拟定且未予协商的情形。 附件： 附件1：《计划采购与供应物资清单》 附件2：《法人授权委托书》 附件3：《廉政合同书》 （以下无正文） 甲 方：【盖章】 乙 方：【盖章】 网 法定代表人：【签字】 法定代表人：【签字】 委托代理人：【签字】 委托代理人：【签字】 务 地 址：【 】 地 址：【 】 电 话：【 】 电 话：【 】 商 电子信箱：【 】 电子信箱：【 】 附件1 道 计划采购与供应物资清单 人民币：元 管 计量 暂定 单价 暂定含税 序号 物资名称 规格型号 品牌/产地 生产厂家 备注 单位 数量 不含税单价 增值税 含税单价 货款金额 价税合计 暂定合同价款人民币大写： 国 以上数量为暂定项目，最终以双方签字确认的采购结算单为准 中 附件2 中国建筑 项目管理表格 表格编号 法人授权委托书 CSCEC-WZ-HN003 （甲方）： 本授权委托书声明：本的法定代表人，授权委托我公司的 为我公司代理人，代表我公司与贵公司工程对涉及投标报价，物资合同、补充协议的签订、履行，物资结算、收款等业务进行签字确认，由在上述授权范围签字的所有文书，我公 司均予认可，由此产生的一切经济法律责任由我公司承担。 代理期限为前述代理人对上述业务发生第一次签字确认之日起至本工程结算完成之日止。代理人无转委托权。 特此委托。 代理人（签字/按指纹）：身份证号码： （供应商）法定代表人签字： （供应商盖章）： 日期： 附件3 廉政合同书 甲方：【 】 乙方：【 】 为确保甲方对业主的承诺，高效、优质共同完成施工任务，争创优质工程，保证合同双方能够高效廉洁地履行， 维护双方合法权益，经双方协商，特订立如下廉政合同书。 第一条 甲乙双方的权利和义务 1.甲乙双方应本着“公开、公平、公正、诚信、透明”的原则开展工作，自觉遵守党和国家、工程项目所在省、 市、区工程建设有关法律法规以及廉政建设的各项规定。 2.甲乙双方应建立健全廉政教育制度，开展经常性教育活动，积极宣贯“合规诚信 自律清正”的廉洁从业核心理 念，加强廉政教育。 3.加强相互监督，发现对方有违反廉政合同书规定的行为，应及时提醒对方纠正。 第二条 甲方的责任 网 甲方工作人员不得有以下行为： （1）为乙方多结算工程量、多签证、多付工程款等，并向乙方索要或接受贿赂、回扣、礼金、有价证券（卡）、 务 贵重物品和好处费等; （2）在乙方报销任何应由甲方或个人支付的费用; （3）参加有可能影响公正执行公务的超标准宴请和娱乐商、健身等活动; （4）接受乙方提供的通讯工具、交通工具和高档办公用品; （5）要求、暗示或接受乙方为个人住房装修道、婚丧嫁娶、配偶子女工作的安排以及出国（境）、旅游提供的方 便; （6）向乙方介绍或推荐配偶、子女、亲属参与的工程施工合同有关的设备、材料、工程分包、劳务等; 管 （7）向乙方推荐分包单位或要求乙方购买合同规定以外的材料、机具设备等; （8）因乙方拒绝本人的不合理要求，而故意刁难乙方。 第三条 乙方的责任 国 乙方应当通过正常途径开展业务，不得有以下行为： （1）为多结算工程量、多签证、多收工程款等，向甲方及其管理人员行贿或馈赠礼金、有价证券（卡）、贵重 中 礼品; （2）为甲方及其工作人员报销应由甲方单位或个人支付的任何费用; （3）安排甲方人员参加超标准宴请、娱乐活动及带有黄、赌性质的娱乐活动; （4）为甲方人员购置或提供通讯工具、交通工具和高档办公用品等; （5）乙方向甲方工作人员及其家属或者亲友介绍从事与甲乙双方工程有关的工程分包及材料设备、周转工具的 供应、租赁等经营活动。 第四条 违约责任 1.如甲方工作人员有违反本廉政合同书的行为，由甲方纪委查处，追究相应的党纪、政务责任，涉嫌犯罪的，移 交司法机关追究刑事责任；对实名举报的，甲方要立即调查，并采取有效措施保障乙方的合法权益，防止报复 事件发生。 2.如乙方单位或个人有违反本廉政合同书的行为，甲方视情节对乙方处以合同额0.5%—1%的罚款，情节较重并给 甲方造成损失的，乙方另需赔偿甲方直接经济损失，并取消乙方工程分包资格。 第五条 甲方接受举报的途径 1. 受理电话：【 】 2. 受理地址：【 】 3. 受理部门：【 】 4. 受理邮箱：【 】 第六条 本廉政合同书作为采购合同的一部分，具有同等法律效力，本协议与采购合同同日生效，至甲乙双方工 程合同履约完止。 甲方： 乙方： 网 法定代表人： 法定代表人： 授权委托人： 授权委托人： 务 签订时间： 年 月 日 请查看报价网 商 址：https://xy.yzw.cn/sj/bid-detail?tenderId=&amp;source=3&amp;tenderCode=cscec2026081900001246027&amp;tenantId=cscec 信息来源:https://www.chinapipe.net/project/d3076919.html cqdingjiu 2026.08.21 10:06:42 道 管 国 中</t>
@@ -664,7 +712,11 @@
       <c r="O4" t="n">
         <v>0</v>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -697,16 +749,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>本项目工程总投资金额：约3140万元；本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>高标准农田建设工程</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 务 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 商 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎道石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 管 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟262m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混国凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 中 2.3 本项目工程总投资金额：约3140万元； 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 网 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 务 2.7 其他： / 商 3.政府采购工程 道 3.1 是否属于政府采购工程：是 □否 管 3.2 是否专门面向中小企业预留：是 国 专门面向中小企业预留的实施方式： 中 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要网提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 务 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 商 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 道 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 管 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 国 开户银行: 开户银行: 账 号: 账 号: 中 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005499 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421353 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891814619 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001038 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00385 信息来源:https://www.chinapipe.net/project/d3076880.html cqdingjiu 2026.08.21 10:06:45</t>
@@ -718,9 +786,13 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>重庆, 高标准农田建设工程, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -735,7 +807,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -753,16 +825,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(二标段)，包括田块整治、灌溉与排水、田间道路、地力提升和其他工程。</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>本项目总投资金额约3140万元，其中二标段1022万元，三标段735万元。</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>主要产品包括混凝土生产路、泥结碎石生产路、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土排水沟、混凝土</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(二标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 务 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 商 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟2道62m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 2.3 本项目工程总投资金额：约3140万元； 管 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）施工图所示范围的所 有内容为准，详见发布国的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分中： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 网 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 务 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （忠县）下载招标文件、工程量清单、电子图纸等资料。商参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（忠县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源 交易监督网、重庆市公共资源交易网（忠县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数字证 书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的，责任 自负。 道 5.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提 问”栏提出疑问，提问时间从本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 管 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 中忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 忠县发展和改革委员会 电 话: 023-54450483 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421361 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00386 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005423 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891832091 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001039 信息来源:https://www.chinapipe.net/project/d3076879.html 网 cqdingjiu 2026.08.21 10:06:45 务 商 道 管 国 中</t>
@@ -776,7 +856,11 @@
       <c r="O6" t="n">
         <v>0</v>
       </c>
-      <c r="P6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -809,16 +893,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>田块整治工程、灌溉与排水工程、田间道路工程、地力提升工程、其他工程</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>项目总投资金额约3140万元，本次招标项目合同估算金额一标段1167万元</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>高标准农田建设工程</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(一标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）已由 忠县发展和改革委 员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来 自 业主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具 备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 务 2.项目概况与招标范围 商 2.1 建设地点： 忠县马灌镇、三汇镇、永丰镇。 道 2.2 项目概况与建设规模：忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）：田块整治 工程：水田整治50.67亩、水田区域撂荒地整治79亩、旱地区域撂荒地整治62.83亩；灌溉与排水工程：新 建200m蓄水池5座、新建500m蓄水池1座、泵站1座；田间道路工程：新建2.5m混凝土生产路12325m、改 建2.5m混凝土生产路8549m、新建2.5m泥结碎石生产路1223m、新建3.0m混凝土生产路576m、改建3.0m混凝土生 管 产路648m、改建3.0m混凝土生产路（拆除原1.5m宽路）266m、改建3.5m混凝土机耕路1662m；地力提升工程：施 有机肥136.48亩；其他工程：公示牌1座、工号牌213块。 国 2.3 本项目工程总投资金额：约3140万元； 中 本次招标项目合同估算金额：一标段1167万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 网 方式一：本项目整体面向中小企业。 务 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 商 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 道 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 管 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 国 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 中 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及CA数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-10 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 网 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 务 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段） 商 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082000104 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005469 道 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421379 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00387 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891884496 管 信息来源:https://www.chinapipe.net/project/d3076876.html cqdingjiu 2026.08.21 10:06:46 国 中</t>
@@ -830,9 +930,13 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
+        <v>95</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>重庆, 高标准农田建设工程, 投资金额, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -865,16 +969,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>永川区</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>永川区</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>农村供水管网巩固提升改造工程</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>供水管网</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
           <t>永川区农村供水管网巩固提升改造工程(东部片区)答疑补遗文件 永川区农村供水管网巩固提升改造工程（东部片区） 补遗文件（01） 各潜在投标人： 现将“永川区农村供水管网巩固提升改造工程（东部片区）”招标文件补遗通知如下，本次发布的补遗文件中 的所有内容与招标文件具有同等法律效力，如与招标文件、答疑补遗文件（01）网不一致时，以本补遗文件为准。 请各潜在投标人自行下载本补遗文件，不管下载与否，都视为全部知晓其全部内容。 一、本招标项目招标文件第二章投标人须知前附表第1.4.1项第1条第（3）款中“具备建设行政主管部门颁发的有 效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由建设行政主管部门颁发的有效的安全生产 务 考核合格证书。”修改为： “（3）具备建设行政主管部门颁发的有效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由水 行政主管部门颁发的有效的安全生产考核合格证书”。 商 二、本招标项目招标文件第二章投标人须知前附表第1.4.1项中第3条“业绩要求”修改为： “投标人自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成过1个单项合同 输配水管网长度不少于100km的水利工程施工道业绩。 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 管 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 三、本招标项目招标文国件第二章投标人须知前附表第1.4.1项中第5条中的“5.3项目经理业绩要求”修改为： “投标人拟派的项目经理自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成 过1个单项合同输配水管网长度不少于100km的水利工程施工业绩，并在该业绩中担任项目经理。 中 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 四、本招标项目的投标文件递交的截止时间（投标截止时间）调整为2026年9月4日9时30分（北京时间），开标 时间及投标保证金递交截止时间相应顺延。 招标人：重庆市永川区惠永水务有限公司 招标代理机构：重庆永川政鑫综合能源有限公司 2026年8月20日 信息来源:https://www.chinapipe.net/project/d3076870.html cqdingjiu 2026.08.21 10:06:46</t>
@@ -886,9 +1006,13 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>重庆, 农村供水管网, 巩固提升改造, 东部片区, 管材招标</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -921,16 +1045,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>长寿区</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>长寿区</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>新改建及修复DN300mm-DN1200mm排水管道20.187公里，其中新改建管道15.21公里，修复管道4.977公里，Ⅲ、Ⅳ级结构性及功能性缺陷修复453处。</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>项目业主为重庆市长寿区住房和城乡建设服务中心，建设资金来自财政资金，项目出资比例为100%。</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>DN300mm-DN1200mm排水管道</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
           <t>长寿区海棠、石堰、龙河片区污水管网建设项目(二期)招标公告 长寿区海棠、石堰、龙河片区污水管网建设项目（二期）招标公告 1.招标条件 本招标项目长寿区海棠、石堰、龙河片区污水管网建设项目已由重庆市长寿区发展和改革委员会以长改发投 〔2024〕169号文批准建设，项目业主为重庆市长寿区住房和城乡建设服务中心，建设资金来自财政资金，项目 出资比例为100%，招标人为重庆长寿乡村建设集团有限公司。项目已具备招标条件，现对该项目的施工进行公 开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：长寿区海棠镇、龙河镇、新市街道、云台镇。 2.2 项目概况与建设规模：新改建及修复DN300mm-DN1200mm排水管道20.187公里，其中新改建管道15.21公里， 务 修复管道4.977公里，Ⅲ、Ⅳ级结构性及功能性缺陷修复453处。 2.3 本次招标项目合同估算金额：4139.45万元。 2.4 招标范围：详见招标人提供的本工程的施工图图纸、图商说、设计变更以及工程量清单所明确的全部工程内容。 2.5 工期要求：270日历天。 缺陷责任期要求：24个月。 道 3.政府采购工程 3.投标人资格要求 管 3.1 本次招标要求投标人须具备以下条件： 3.1.1 本次招标要求投标人具备的资质条件：建设行政主管部门颁发的有效的市政公用工程施工总承包三级及以 上资质； 国 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 中 3.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（长寿区） （https://www.cqggzy.com/changshouweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需 在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网 导航栏“主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登 记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn）和重庆市公共资源交易网（长寿区） （https://www.cqggzy.com/changshouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公 告发布至2026-08-25 15:00:00前。 4.3招标人应于2026-08-28 18:00:00前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn）和重庆市公共资源交 易网（长寿区）（https://www.cqggzy.com/changshouweb/）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-14 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn）和重庆市公共资源交易网（长寿区） （https://www.cqggzy.com/changshouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源 交易监督网上发布。] 7.联系方式 招 标 人: 重庆长寿乡村建设集团有限公司 代理机构: 中新创达咨询有限公司 地 址: 重庆市长寿区桃源大道3号一号商务楼5-6楼 地 址: 邮 编: 邮 编: 项目负责人: 刘老师 项目负责人: 钟亮 网 电 话: 023-40233279 电 话: 19132912275 传 真: 传 真: 电子邮箱: 电子邮箱务: 开户银行: 开户银行: 账 号: 账 号: 商 监督部门: 重庆市长寿区发展和改革委员会 电 话: 023-40245080 2026年08月20日 长寿区海棠、石堰、龙河片区污水管网建设道项目（二期） 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公 中国农业银行股份有限公司重庆自由贸易 312601010400083780000033561 司 管试验区分行 重庆联合产权交易所集团股份有限公 中国建设银行股份有限公司重庆渝中支行 6232813760003317764 司 重庆联合产权交易所集国团股份有限公 重庆银行股份有限公司七星岗支行 15010202900420146632392 司 信息来源:https://www.chinapipe.net/project/d3076848.html cqdingjiu 20中26.08.21 10:06:46</t>
@@ -944,7 +1084,11 @@
       <c r="O9" t="n">
         <v>0</v>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -977,16 +1121,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>渝万高铁站前1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~D1K47+550.4，正线长度33.01km，中标造价31.73亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁301孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负责DK0+000~DK57+136段小型构件预制。</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>中标造价31.73亿元</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>刺丝滚笼,塑钢模板,泄水管</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部刺丝滚笼、塑钢模板、泄水管询价采购公告 中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 刺丝滚笼、塑钢模板、泄水管询价采购公告 询价编号： ZT1105-XJ-2026-590 尊敬的 各潜 在供应商 : 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与 中铁十一局集团有限公司重庆至万州高铁站 前 1标项目经理部 ZT1105-XJ-2026-590， 刺丝滚笼、塑钢模板、泄水管 的报价。 一、 项目概况 务 渝万高铁站前 1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~ D1K47+550.4，正线长度 33.01km，中标造 价 31.73 亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁 301 孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负 责DK0+000~DK57+136段小型构件预制。合同工期54.7月商，开工日期为2022年11月01日，竣工日期为2027 年04 月30日。 二、 询价内容 道 本次 计划对刺丝滚笼、塑钢模板、泄水管 进行询价，询价内容如下： 询价物资一览表 管 计 序 物资 量 包件号 规格型号 数量 备注 号 名称 单 位 国 刺丝 1 GL-01 2.5mm 6m0.5m 米 6500 半径 ≥225mm，包括刀片刺绳、挂丝、连接卡、支架 滚笼 防护 中 栅栏 2 GL-01 用立 50X30X765X2.5mm 套 500 含抱箍、螺栓等配件 柱支 架 平 塑钢 3 MB-01 350X300mm 方 19.2 400*400,1个挡水沿，配固定手柄 模板 米 平 塑钢 4 MB-01 350X300mm 方 19.2 400*400,2个挡水沿，配固定手柄 模板 米 平 塑钢 5 MB-01 300X300mm 方 75.6 2个挡水沿，配固定手柄 模板 米 平 塑钢 6 MB-01 300X300mm 方 75.6 1个挡水沿，配固定手柄 模板 米 7 SSG-01 管篦 PVC250X200x10mm 个 220 材质硬聚氯乙烯 PVC，详见附图 PVC 8 SSG-01 泄水 135X38mm 块 220 材质硬聚氯乙烯 PVC，详见附图 管盖 U型 9 SSG-01 125mm 个 900 详见附图 管卡 UPV 材质硬聚氯乙烯 PVC，两端接头采用阴阳螺纹连接详见 10 SSG-01 C排 125X8mm螺纹 米 2870 附图 水管 UPV 11 SSG-01 C弯 DN125X8mm90° 个 240 材质硬聚氯乙烯 PVC，详见附图 管 UPV 网 125X125X110mm弹性密 12 SSG-01 C三 个 120 材质硬聚氯乙烯 PVC，详见附图 封圈异径斜三通 通 无压 埋地 务 排污 排水 用硬 13 SSG-01 DN125 个 150 材质硬聚氯乙烯 PVC，详见附图 聚氯 商 乙烯 管 T 型接 头 道 合 计 管 说明： 1. 表中数量为计划数量，实际 采购 过程中可能有所调整，最终结算按照实际 采购 数量结算。 2.收货地点：中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部 三、 技术质量 及报价国 要求 1. 此次 询价物资 各项技术性能要 符合 甲方 的要求，质量满足甲方项目部正常使用的要求，保证 产品 的质量合 格。 具体要求或图纸见询价文件技术规格书。 。 中 2 .报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、 结算及付款方式 每个月 15 日为双方价款结算日期（即上月 16 日至当月 15 日内），结算前双方要在对帐确认单上签字认可，乙 方按双方确认的金额开具增值税专用发票，并自发票开具之日起 7日内传递给甲方。甲乙双方在增值税专用发票 传递过程中必须留取相应的交接签证手续。自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发 票认证完成之日起第6个月，支付至本次结算金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内， 累计支付总额不超结算总金额的75%，剩余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理 末次结算后第二年，支付金额应大于等于尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总 额的15%；办理末次结算后第四年，全部付清）。 五、 报价 人资格要求 1.营业范围要求：在中华人民共和国境内依法注册，具有询价物资生产或供应经验的生产商或代理商，并且具有 合法有效的营业执照。 2.生产能力要求： 生产商须具备 询价 物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定 。 代理商需出具制造厂出具签字盖章的授权函。 3.财务能力要求：报价人为增值税一般纳税人或小规模纳税人，有依法纳税的良好记录。 4.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8月至今） 国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；每种物资全指标技术参数性能满足 国家和行业最新标准的各项规定。 5.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年8月至今）企业或企业法定代表人有人民法院生效判决、裁定 认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接受 通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合作 方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 6.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★7 .下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、 报价人需要提供的资料 1. 营业执照复印件、 法人身份证复印件、 开户许可证、商授权委托书 、 报价表 和报价人资格要求中所需的证明资 料， 所有资料需加盖公司鲜章。 2. 产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、 询价 报名截止 时间 管 有意参加本次询价采购的报价人 须在铁建云链平台 （ https:// www.crccep. cn） 完成供应商注册，并 于 202 6 年 8 月 20 日 9时 00 分 至 202 6 年 8 月 24 日 9时 00 分在网上 完成报名工作。 八、 询价 截止 时间 国 凡有意参加本次询价采购的报价人，请于 202 6 年 8 月 24 日 14 时 00分 前 提交报价。截止时间前未完成 报价 文 件传输的，视为放弃 报价 。 供应商报价必须严格按照《 报价表 》格式进行报价。 中 九、 联系方式 采购 组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村 71号 联系人：胡先生 联系电话： 13983336494 （提供平台服务支持） 采购人名称：中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 地址： 重庆市万州区双河口街道檬兴路万州现代综合物流中心信息交易大厅（中铁十一局） 联系人： 唐大伟 联系电话： 18323391938（提供采购服务支持、保证金退还） 中铁十一局集团有限公司物资设备集中采购管理中心 第五分中心 2026 年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076805.html cqdingjiu 2026.08.21 10:06:47 网 务 商 道 管 国 中</t>
@@ -998,9 +1158,13 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>重庆, 万州, 高铁站前, 刺丝滚笼, 塑钢模板, 泄水管, 询价采购</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1033,16 +1197,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>垫江县</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>垫江县</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目，主要内容包括河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m，化粪池2座；产业基地水肥一体化改造45亩等。</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>项目总投资金额为642.89万元，本次招标项目合同估算金额约为5014864.52元。</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>水利水电工程施工</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 1.招标条件 本招标项目 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 已由 垫江县发展和 改革委员会 以 垫江发改委发〔2026〕20号 文批准建设，项目业主为 垫江县太平镇人民政府，建设资金来 自 大中型后扶资金及自筹资金 ，项目出资比例为 100% ，招标人为垫江县太平镇人民政府。项目已具备招 标条件，现对本项目施工进行公开招标，评标办法采用经评审的最低投标价法。网 务 2.项目概况与招标范围 商 2.1 建设地点：垫江县太平镇桂花村 道 2.2 项目概况与建设规模：主要为河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m， 化粪池2座；产业基地水肥一体化改造45亩等。 管 2.3 本项目工程总投资金额：642.89万元 国 本次招标项目合同估算金额：约5014864.52元 中 2.4 招标范围：本工程施工图纸所含全部的施工内容，具体以招标人发布的工程量清单为准。 2.5 工期要求：工期为360日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：□是 否，因专门面向中小企业预留无法确保充分供应、充分竞争，根据 《政府采购促进中小企业发展管理办法》第六条第(三)“按本办法规定预留采购份额无法确保充分供应、充分竞 争，或者存在可能影响政府采购目标实现的情形”的规定，本项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 网 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的水利水电工程施工总承包三级 务 及以上资质。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相商应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 道 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 管 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com国/dianjiangweb/)、重庆市公共资源交易监督网下载招标文件、工程量清单、电子图纸等资 料。参与投标的投标人需在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共 资源交易监督网完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督网导航栏“主体信息”页面中“市场主体信息 登记”、“中CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流 程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督 网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-24 17:00:00前。 5.3招标人应于2026-08-28 17:00:00前在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重 庆市公共资源交易监督网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交 易监督网发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 垫江县太平镇人民政府 代理机构: 重庆皓辰建设工程咨询有限公司 重庆市渝北区金开大道1228号大雅金开国际1 地 址: 重庆市垫江县太平镇牡丹路191号 地 址: 栋9-2 邮 编: 邮 编: 项目负责人: 余老师 项目负责人: 雷雨得 电 话: 13996889839 电 话: 023-86018770 18580880860 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 网 2026年08月19日 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 务 户名 开户行 投标保证金账号 垫江县公共资源交易中心 中国农业银行重庆垫江支行 316301010400077950000005966 垫江县公共资源交易中心 中国银行重庆垫江支行 111616885778VA00139 商 垫江县公共资源交易中心 重庆农村商业银行垫江支行 2501010120010009065000128 垫江县公共资源交易中心 工商银行重庆垫江支行营业部 9558853100016843371 垫江县公共资源交易中心 重庆银行垫江支行 820101040000584-101195 道 附件：垫江县2026年度大中型水库移民后期扶持项目-.zip https://www.cqggzy.com/trade/014001/dac54522-3264-4eac-ae47-f434567ce374?categoryNum=014001001007 信息来源:https://www.chinapipe.net管/project/d3076788.html cqdingjiu 2026.08.21 10:06:47 国 中</t>
@@ -1054,9 +1234,13 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 水利, 移民, 后期扶持</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1089,16 +1273,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>新建水厂1座（新建2000m³茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管径DN20~DN250，管材为涂塑钢管。</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>合同预估金额：5000万元</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>涂塑钢管</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
           <t>万州区新田等6个镇乡农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区新田等6个镇乡农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建水厂1座（新建2000m3茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管 主要建设内容 径DN20~DN250，管材为涂塑钢管。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 备注 称 式 发布时间 所 额(万元) 商 万州区新田 万州区新田 重庆市万 招标项目 等6个镇乡农 等6个镇乡农 公开招 州区公共 1 村饮水质量提 2026-08 5000.00 村饮水质量 标 资源交易 升项目道施工总 提升项目 中心 承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076721.html 管 cqdingjiu 2026.08.21 10:06:48 国 中</t>
@@ -1110,9 +1310,13 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 商机</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1145,16 +1349,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>新建50m³蓄水池4口、取水池2座；新建50m³/d-100m³/d水厂2座；改造100m³/d-300m³/d水厂5座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设施。</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>合同预估金额：3000万元</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>DN25-DN250涂塑钢管</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
           <t>万州区大周等4个镇乡街道农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区大周等4个镇乡街道农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建50m3蓄水池4口、取水池2座；新建50m3/d-100m3/d水厂2座；改造100m3/d-300m3/d水厂5 主要建设内容 座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设 施。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 商 备注 称 式 发布时间 所 额(万元) 万州区大周 万州区大周 重庆市万 招标项目 等4个镇乡街 等4个镇乡街 公开招 州区公共 1 道农村饮水 道农村饮道水质 2026-08 3000.00 标 资源交易 质量提升项 量提升项目施 中心 目 工总承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3076720.html cqdingjiu 2026.08.21 10:06:49 国 中</t>
@@ -1166,9 +1378,13 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>重庆, 农村饮水质量提升项目, 管材招标, 合同预估金额</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1201,16 +1417,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>采购项目资金为企业自筹。</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>纤维编绕拉挤电缆保护套管(BWFRP100/2.0，79158米)</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
           <t>二航科工新燕尾山项目纤维编绕拉挤电缆保护套管采购询价通知公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目询比采购 公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目已具备采 购条件，现公开邀请供应商参加询比采购活动。 网 1. 采购项目简介 1.1 采购项目名称：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机 电工程项目。 务 1.2采购方案编号：FA00000674478。 1.3 采购人：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程 项目经理部。 商 1.4 采购代理机构：中交二航局科工（武汉）有限公司。 1.5 采购项目资金：企业自筹。 道 1.6 采购项目概况：新燕尾山隧道工程位于重庆市内环吉庆隧道北侧，四横线分流道鹿角隧道南侧，西接白居 寺大桥，东接内环快速路，并向东延伸接渝黔复线高速，其所在的道路系统呈东西布置，为主城区南部片区重 要干道。本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目 管 全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程 包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。 2.采购范围及相关要求 国 2.1 采购范围：纤维编绕拉挤电缆保护套管（BWFRP100/2.0，79158米）。 2.2 交货期：以甲方实际订单要求为准。 中 2.3 交货地点：重庆市巴南区新燕尾山项目甲方指定位置。 2.4 物资质量标准：满足国家法律法规、标准、规范、设计参数及技术规格书要求。 3.供应商资格要求 3.1 供应商应依法设立且满足如下要求： （1）资质要求：在中华人民共和国境内依法注册，具有独立法人资格、具有采购物资生产或供应经验的企业， 并且具有合法、有效的“三证合一”的营业执照,代理商需提供制造商授权委托书。 （2）财务要求：必须是经税务部门注册登记核准的一般纳税人，有依法纳税的良好记录，提供近三年的财务报 告。 （3）业绩要求：同类产品销售业绩不少于2个，并具备与本招标项目需求相适应的供货能力。 （4）信誉要求：本项目投标截止期前未被“信用中国”、“中国政府采购网”、中国交建物资采购管理信息系 统网站列入失信被执行人、违法案件当事人、违法失信行为记录名单。 （5）其他要求：提供运输方案及生产周期。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他： / 。 4.供应商报名 4.1有意参加询比采购活动的单位，请于2026年 8 月 20 日 11 时 00 分至2026 网 年 8 月 25 日 11 时 00 分（北京时间、下同），登录“中交招采网”（网 址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 务 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 商 5. 供应商报价 5.1 报价结束（递交响应文件截止）时间：2026年 8 月 25 日 11 时 00 分。 道 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的 电子响应文件，采购人将拒收。 5.3电子采购的供应商报价文件由线上电子报价表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 管 子报价表的数据为准。 6. 开标 6.1开标时间：与报价结国束时间相同。 6.2开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标，现场开标地点/。 7. 发布公告的媒介 中 本询比采购公告在中交招采网上发布。 8. 评审办法 本项目评审办法采用 经评审的最低价法 。 9. 合同主要条款 9.1 付款条件：无预付款，到货后办理结算，双方办理完结算手续、卖方提供符合合同要求的正式发票给买方 后60天，买方支付该批材料价值80%的货款，完工结算后支付至97%，剩余3%为质保金，质保期2年，两年后供 应方申请返还3%（无息）；银行转账、承兑、18个月供应链金融混合支付方式。 9.2履约保证金的递交： （1）□不要求递交 （2）要求递交 保证金金额：2万元 ； 保证金形式：银行转账、银行保函等电子保函；其他形式：无 。 10. 成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”（网址：https://zjzcw.iccec.cn）发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联 系4006765885中标服务费请按7咨询。 10.1收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； 务 （3）在1000万元（含）至3000万元之间的，每次收取1000元； （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 10.2支付流程 （1）通知推送：中标结果发布后，系统自动道推送缴费通知（含应缴金额及支付链接）； （2）费用查询：供应商登录“中交招采网-服务管理”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网- 服务管理－发票下载”模块获取。 11.监督机构 国 监督机构名称：中交二航局科工（武汉）有限公司纪委监察部 举报电话：中027-82796466 举报邮箱：sneb_kggs@ccccltd.cn 12.其他 投标保证金采用银行转账形式的需转至中交二航局科工（武汉）有限公司账户（账 号：42001186108053006379-0006开户行：建行武汉长江支行，行号：105521000053），并备注二航科工燕尾山机 电照明项目纤维编绕管投标保证金。 13.联系方式 采购 人：中交二航局科工（武汉）有限公司 采购代理机构：中交二航局科工（武汉）有限公司 地 址：武汉市新洲区双柳街星谷大道158号地 址：武汉市新洲区双柳街星谷大道158号 邮政编码：430400 邮政编 码：430400 联系人：李鑫 联系人：毕明 月 电 话：18186145302 电 话：17853118573 电子邮件：18186145302@ccccltd.cn 电子邮件：bimingyue@ccccltd.cn 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076715.html cqdingjiu 2026.08.21 10:06:50 网 务 商 道 管 国 中</t>
@@ -1222,9 +1446,13 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 光纤电缆保护套管</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1257,16 +1485,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>巴南区</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>巴南区</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>天然气表后管道安装工程</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告 重庆巴南天然气有限责任公司 重庆国际生物城配套公寓项目天然气表后管道安装工程 变更公 告 公告编号： RQBGGG202608200006 本公司于2026年08月19日发布的重庆国际生物城配套公寓项目天然气表后管道安装工程公告（编 号：RQCGXY202608170010），现做出如下变更： 网 1、对采购文件第一卷“采购需求“中墙体管道暗埋的具体内容进行明确。墙体管道暗埋应包含墙体开槽，输送 用不锈钢波纹管及钢制槽板的安装，墙体恢复，暗埋管道视频记录。 2、对由响应供应商提供的钢制槽板的规格进行明确。钢制槽板为U型开口槽，采用热镀锌Q235B钢板，钢板厚度 务 不得小于1.2mm，尺寸不得小于U40*30*1.2（宽40mm,高30mm,壁厚1.2mm热镀锌） 3、对由响应供应商提供的F型不锈钢三通，材质可以选用黄铜进行替代。 4、采购文件第二卷“技术规范及要求“中增加T/CECS633-2019 《燃气用户工程不锈钢波纹软管技术规程》。 以上内容在合同中也同步进行调整。 商 除上述变更外，原公告其余内容仍有效。 道 重庆巴南天然气有限责任公司 管 2026-08-20 信息来源:https://www.chinapipe.net/project/d3076704.html cqdingjiu 2026.08.21 10:国06:50 中</t>
@@ -1278,9 +1522,13 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>重庆, 天然气表后管道安装工程, 变更公告</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1313,16 +1561,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>合川区</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>合川区</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米，螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清淤2627米。</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>合同预估金额为1708.44万元</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>排水管道、检查井、紫外线修复设备、螺旋缠绕修复材料、树脂修复材料、不锈钢快速锁修复设备</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>合川区中南片区污水管网工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 合川区中南片区污水管网工程（一期） 名称 招标 网 法人 或招 标人 重庆市合川区住房和城乡建设委员会 名称 （盖 务 章） 项目 批准 文件 合川发改投〔2025〕19 号 商 及文 号 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新 主要 建D300排水管道38米；紫外光修复 D300-D道800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 建设 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42 内容 米；完成 D300-D1000管道清障189米、清淤2627米。 拟 招 招标文 合同预 招标 管 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 国 重 庆 市 合川 合 招标 区中 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300- 川 项目 中 南片 D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 公 区 区污 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 开 公 1 2026-09 1708.44 水管 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米， 招 共 网工程 不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清 标 资 （一 淤2627米。 源 期） 交 易 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076543.html cqdingjiu 2026.08.21 10:06:50</t>
@@ -1334,9 +1598,13 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>重庆, 污水管网工程, 管网修复, 新建工程, 排水管道, 检查井, 紫外线修复, 螺旋缠绕修复, 树脂修复, 不锈钢快速锁修复</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1369,16 +1637,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>本次采购项目涉及球墨铸铁管及管件的供应，具体包括样品的规格和数量要求。</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>球墨铸铁管及管件</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>重庆市自来水有限公司球墨铸铁管及管件2026-2027(2年)采购项目(第二次)答疑补遗文件 重庆市自来水有限公司球墨铸铁管及管件2026-2027（2年）采购项目（第二次）答疑 提问1：样品20CM长含承口吗？如果含承口20CM那就太短，标识LOGO无法体现完整建议≥20CM 答1：球墨铸铁管样品含承口，样品长度≥20CM 网 务 招标人：重庆市自来水有限公司 招标代理机构：重庆水务集团公用工程咨询有限公司 商 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d30道76446.html cqdingjiu 2026.08.21 10:06:50 管 国 中</t>
@@ -1390,9 +1666,13 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>重庆, 球墨铸铁管, 管件, 采购项目</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1425,16 +1705,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>大足区</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>大足区</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>大足区中心城区和龙水镇市政公共排水设施的运维(材料)。</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>大足区中心城区和龙水镇市政公共排水设施运维(材料)更正一号公告 一、更正项 更正项 更正子项 更正前内容 更正后内容 网上投标 网上投标截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 递交投标响应文件 线下递交投标（响应）文件开始时间 2026-08-20 14:30:00 2026-08-25 14:30:00 递交投标响应文件 线下递交投标（响应）文件截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 网 开标 开标时间 2026-08-20 15:00:00 2026-08-25 15:00:00 招标采购（附件） 附件 务 二、补遗更正说明 清单限价重新做调整，开标时间已更正，详见更正文件内容 商 三、联系方式 采购执行方： 道 单位名称：重庆誉双项目管理有限公司 联系人：陈老师 联系电话：13996336872 采购需求方： 管 单位名称：重庆市大足区茂泰市政工程有限公司 联系人：谢老师 联系电话：18523539371 信息来源:https://www.chinapipe.net/project/d3076319.html 国 cqdingjiu 2026.08.21 10:06:50 中</t>
@@ -1446,9 +1742,13 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1481,16 +1781,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>璧山区</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>璧山区</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6.都市农文旅配套建设1000平方米。</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>合同预估金额为9182.25万元</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>温度调控系统、水肥一体化设备、人工补光系统、二氧化碳补施系统、智能环境控制系统、作业物流装备</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>璧山区2026年大路街道三台村智慧设施农业建设项目招标计划表 重庆市工程建设项目招标计划表 项目 璧山区2026年大路街道三台村智慧设施农业建设项目 名称 招标 法人 或招 网 标人 中农良品（重庆）生态农业有限公司 名称 （盖 章） 项目 批准 务 文件 及文 号 主要 1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流 建设 装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6. 内容 都市农文旅配套建设1000平方米。 商 招 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 道 璧 山 区2026 重 年 庆 大 市 路 公 招标 街 管 共 项目 道 资 三 公 源 台 项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米； 2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、 开 交 1 村 二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套； 3.项目后勤及仓储配套（含装修）5000平方米； 4.土方回填及场地平整53000平 2026-09 9182.25 招 易 智 方米； 5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米； 6.都市农文旅配套建设1000平方米。 标 中 慧 心 设 国 璧 施 山 农 分 业 中 建 心 设 项 目 中 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076777.html cqdingjiu 2026.08.21 10:06:51</t>
@@ -1502,9 +1818,13 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>重庆, 智慧设施农业, 招标计划, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1537,16 +1857,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>长寿区</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>长寿区</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>本项目包括但不限于新建混凝池-三沉池，还建格栅池，厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统，原斜管沉淀池改造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰），拆除原有污泥池，新增临时污泥储罐务并还建污泥池，污泥堆场临时改建及恢复，实施技改期间的临时排放工程，进行基础的自控改造。</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>企业自筹，出资比例为100%</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>污水处理设备</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>长寿区江南街道污水处理厂更新改造工程项目公告 长寿区江南街道污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目长寿区江南街道污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源为企业 自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：长寿区江南街道污水处理厂更新改造工程包括但不限于以下内容新建混凝池-三沉池；还建格栅池； 厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统；原斜管沉淀池改 造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰）。拆除原有污泥池，新增临时污泥储罐 务 并还建污泥池；污泥堆场临时改建及恢复；实施技改期间的临时排放工程；进行基础的自控改造。 2.2 比选范围：长寿区江南街道污水处理厂更新改造工程施工图范围中的所有工作内容，包括但不限于土建工 程、设备及安装工程、工艺管道工程、电气工程、临排工程等内容，具体以比选人提供的图纸、技术规范、设 备需求清单、答疑资料、澄清资料、其他补遗资料等相关商内容为准。 2.3 建设地点：重庆市长寿区江南街道。 2.4 工期：110日历天（实际开工日期以监理工道程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 3. 参选人资格要求 管 3.1 本次比选要求参选人具备以下条件： （1）独立法人资格； （2）建设行政主管部国门颁发的有效的市政公用工程施工总承包二级及以上资质； 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 中 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月 27 日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务 大厦5楼。 5.2 比选截止时间：2026年8月 27 日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 网 联系人：曹老师 电话：023-71618725 务 代理机构：重庆招标采购（集团）有限责任公司 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 商 联系人：高老师 电话：023-67706841 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 管 信息来源:https://www.chinapipe.net/project/d3076456.html cqdingjiu 2026.08.21 10:06:51 国 中</t>
@@ -1558,9 +1894,13 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 污水处理厂</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1593,16 +1933,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>潼南区</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>潼南区</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>本项目包括两个子项目：一是潼南区新胜镇污水处理厂的更新改造，主要内容是新增一体化污水处理设备基础，更新现有污水处理系统设备，升级处理系统，新建风机房-配电室防尘防渗地坪；二是潼南区双江镇污水处理厂的更新改造，内容包括将原有斜管沉淀池改建为好氧池，新建竖流沉淀池，更新老旧及故障设备，新建储药加药区和一体化危废储存间，完善污水处理配套设施。</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>本项目资金来源为企业自筹，出资比例为100%。</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>污水处理设备、一体化设备、沉淀池、好氧池、竖流沉淀池、储药加药区、一体化危废储存间、污水处理配套设施</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>潼南区新胜镇、双江镇污水处理厂更新改造工程项目项目公告 潼南区新胜镇、双江镇污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目潼南区新胜镇、双江镇污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源 为企业自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：潼南区新胜镇污水处理厂更新改造工程，主要建设内容为新增200m?/d一体化污水处理设备基础； 更新现有污水处理系统设备，提高现有沉淀池二沉池、三沉池液位；升级处理系统（干化池改建为污泥池，新 增叠螺脱水机，改建污泥堆场及雨棚）；新建风机房－配电室防尘防渗地坪。潼南区双江镇污水处理厂更新改 务 造工程，主要建设内容为将原有斜管沉淀池改建为好氧池，新建3座竖流沉淀池，配套安装相关设备；更新污水 处理系统中老旧及故障设备；新建储药加药区与一体化危废储存间，完善污水处理配套设施。 2.2 比选范围：潼南区新胜镇、双江镇污水处理厂更新改造工程施工图范围中的工作内容（一体化设备采购及 相关安装工作除外），包括但不限于土建工程、附属工程商（包括但不限于绿化工程、工艺管线工程、电气及自 控工程、临排清淤工程等）、一体化污水处理设备基础、标准化建设、配套设备材料采购及安装工程等内容， 其中一体化设备采购及相关安装工作不在本次比选范围内；具体以比选人提供的图纸、技术规范、工程量清单、 答疑资料、澄清资料、其他补遗资料等相关内容为准。 道 2.3 建设地点：潼南区新胜镇、双江镇。 2.4 工期：120日历天（实际开工日期以监理工程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 管 3. 参选人资格要求 3.1 本次比选要求参选人具备以下条件： 国 （1）独立法人资格； （2）建设行政主管部门颁发的有效的市政公用工程施工总承包二级及以上资质； 中 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月27日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务大厦5 楼。 5.2 比选截止时间：2026年8月27日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 网 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 务 联系人：陈老师 电话：023-42756696 商 代理机构：重庆招标采购（集团）有限责任公司 道 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 联系人：高老师 管 电话：023-67706841 重庆水务电子商务平台国咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3076454.html cqdingjiu 2026.08.21 10:06:51 中</t>
@@ -1614,9 +1970,13 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 污水处理厂更新改造</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1631,7 +1991,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>房建</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1649,16 +2009,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>采购预算 409674.71元</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>市政水源</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 采购需求单位(全称) 重庆医科大学附属第二医院总务科 项目名称 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程 项目内容 给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源 采购预算 409674.71元 网 拟采购供应商全称 东部自来水分公司 配套业务用房第二市政水源从重庆水资源产业股份有限公司东部自来水分公司管辖范围 单一来源采购理由 的管网具体接入，属于市政管网施工，具有特殊要求。 务 公示时间 2026年8月19日-2026年8月25日 联系人及联系电话 刘老师 023-63693215 注：1.以上陈述是否真实，欢迎社会各界监督，公示时间商至少5个工作日； 2.公示期内无异议的，采购管理处将进行该项目采购；有异议请将意见反映采购人。 信息来源:https://www.chinapipe.net/project/d30道76334.html cqdingjiu 2026.08.21 10:06:51 管 国 中</t>
@@ -1670,9 +2038,13 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1705,16 +2077,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>黔江区</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>黔江区</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>本项目服务内容为G319黔江区正阳至城西段改建工程管线探测工作。</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>管线探测工作</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>中铁二院工程集团有限责任公司G319黔江区正阳至城西段改建工程管线探测工作线上询价采购公告 中铁二院工程集团有限责任公司G319黔江区正阳至城西 段改建工程管线探测工作线上询价采购 ZTEYCQ-XJ-2026-019 网 采购单位: 中铁二院工程集团有限责任公司 发布时间: 2026-08-19 16:10 报价截止时间: 务 2026-08-21 17:00 招标方联系人: 杨先生 招标方联系电话: 商 13883021521 招标方邮箱: 监督方联系人: 李先生 道 监督方联系电话: 15823237919 监督方邮箱: 保证金: 0元 管 结算与发票信息: 详情 交货信息: 详情 国 其他说明事项: 标的明细 流水号：询2026081900304 中 计量单 技术标准及要 序号 标的名称 数量 交货期 送货地址 位 求 G319黔江区正阳至城西段 合同签订后5天内完成 西南区-重庆市-市辖 1 1 项 详见询价文件 改建工程管线探测工作 本项目服务内容。 区-黔江区-项目地点 信息来源:https://www.chinapipe.net/project/d3076309.html cqdingjiu 2026.08.21 10:06:51</t>
@@ -1726,9 +2114,13 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类, 匹配程度, 匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1761,16 +2153,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>本项目主要涉及室外蒸汽管道φ219x6mm的安装，管道材质为20#，地上敷设，蒸汽管道运行压力1.08MPa，管道设计压力1.2MPa。蒸汽管道系统包括从锅炉房分汽缸到6#和8#车间分汽缸的所有蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温工作。还包括钢结构桁架工程的采购、运输、制作、安装、防腐工作，以及管道附件及控制系统的采购、运输、安装、接线等工作。此外，还需要进行调试与验收，确保蒸汽管道系统能够正常使用并备案。</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>项目总投资额为580.643717万元，全部为企业自筹资金。</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸、钢结构桁架、阀门、压力表、温度表、流量计、电动/气动执行机构、配套仪表电缆、桥架、保护管</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 1.招标条件 本招标项目乌江涪陵榨菜绿色智能化生产基地(一期)已由重庆市涪陵区发展和改革委员会以重庆市企业投资项目 备案证2020-500102-13-03-000003 批准建设，项目业主为重庆市涪陵榨菜集团股份有限公司，建设资金来自企业 自筹，项目出资比例为100% ，招标人为重庆市涪陵榨菜集团股份有限公司。项目已具备招标条件，现对乌江 涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 2.1 建设地点： 重庆市涪陵区马鞍街道人和社区 。 网 2.2 项目概况与建设规模：建筑面积约369384.27㎡。本项目蒸汽管道主要为室外蒸汽管道φ219x6mm，管道材质： 20#地上敷设，由14#锅炉房分汽缸分别接至6#和8#智能化车间分汽缸，蒸汽管道运行压力1.08MPa，管道设计压 力1.2MPa。 务 2.3 本次招标项目合同估算金额：580.643717万元。 2.4 招标范围： 商 （1）蒸汽管道系统本体：从锅炉房分汽缸后（含分气缸阀门）至6#车间、8#车间分气缸处，所有蒸汽管道、管 件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温（含保温层及保 护层）工作。 道 （2）钢结构桁架工程：负责本项目范围内所有钢结构架空桁架（管廊）的采购、运输、制作、安装、防腐工作。 （3）管道附件及控制系统：负责本工程范围内所有阀门、压力表、温度表、流量计、电动/气动执行机构以及配 套仪表电缆、桥架、保护管的采购、运输、安装、接线。负责与DCS/PLC系统接口的接线与联动调试。 管 （4）调试与验收：组织并确保整个蒸汽管道系统（含分气缸后段末端管道、桁架及其安全附件）通过项目所在 地特种设备安全监察管理部门实施的安装监督检验。负责报检、配合现场检验、整改、出具深化图纸并由设计 单位审核盖章、特种设备法定报检取证的全部费用，包括但不限于：施工前办理安装告知，设计院盖章审核， 施工中接受并通过安装国监督检验，最终负责取得《压力管道安装监督检验证书》与《特种设备使用登记证》， 确保蒸汽管道投入使用并备案，提交全套法定检验报告。 （5）土建工作部分 中 1）管架和桁架基础的施工，包括但不限于钢结构桁架的混凝土独立基础的土方开挖、浇筑、养护及回填恢复。 2）管道穿墙/板孔洞的开挖、封堵与修复。 3）室内外地面的开挖（包括但不限于疏水井、沟槽开挖、通行地沟、设备基础开挖）与恢复（包括但不限于土 方回填、渣土弃运、地面硬化）。 4）桁架及设备接地线的施工，包括但不限于接地极制作、接地干线敷设，并与厂区主接地网可靠连接，接地电 阻测试合格。 具体详见施工图、招标文件、工程量清单、答疑补遗等资料。 2.5 工期要求： 60 日历天 缺陷责任期要求： 24 个月 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：投标人应同时具备以下(1)、(2)项资质： （1）具备建设行政主管部门颁发的有效的建筑工程施工总承包二级及以上资质； （2）具备有效的《中华人民共和国特种设备生产许可证》（许可子项目：工业管道安装GC2级及以上）。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 网 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 务 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（涪陵区） （https://www.cqggzy.com/fulingweb/）下载招标文件、工程商量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网（涪陵区道）（https://www.cqggzy.com/fulingweb/）本项目招标公告网页下 方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-23 17:00:00前。 4.3招标人应于2026-08-24 18:00:00前在重庆市公共资源交易网（涪陵区）（https://www.cqggzy.com/fulingweb/）发 布澄清。 5.投标文件递交的内容 管 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-09 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（涪陵区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 中重庆市涪陵榨菜集团股份有限公司 代理机构: 中招国际招标有限公司 重庆两江新区黄山大道中段53号5-1（双 地 址: 重庆市涪陵区江北街道办事处二渡村一组 地 址: 鱼座A栋5楼） 邮 编: 408000 邮 编: 项目负责人: 徐老师 项目负责人: 寿云凤 电 话: 13212467016 电 话: 023-68881331-9032 传 真: 传 真: 电子邮箱: bsd2me@126.com 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市涪陵区发展和改革委员会 电 话: 023-72203687 2026年08月19日 乌江 涪陵 榨菜 绿色 智能 化生 产基地 (一 期)6#、 8#车 网 间蒸 汽管 道安 装工 务 程 中 中 国 国 重 银 重 商民 重 庆 行 庆 生 庆 涪 股 涪 银 涪 陵 份 陵 行 陵 重 投 公 有 道公 股 公 庆 标 共 限 共 份 共 银 开 保 户 资 公 资 有 资 行 户 证 110292140553VA00154 9902001860445897 430102029007791845-275 名 源 司 源 限 源 涪 行 金 交 重 交 公 交 陵 账 管 易 庆 易 司 易 支 号 有 涪 有 重 有 行 限 陵 限 庆 限 公 马 公 涪 公 国 司 鞍 司 陵 司 支 支 行 行 中 信息来源:https://www.chinapipe.net/project/d3076300.html cqdingjiu 2026.08.21 10:06:51</t>
@@ -1782,9 +2182,13 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="inlineStr"/>
+        <v>95</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>重庆, 蒸汽管道, 安装工程, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1817,16 +2221,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>完成重庆国际生物城配套公寓项目（民用1020户）天然气表后管道定制化服务。（含安装燃气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个，其它配套管件及辅材，墙体管道暗埋等）</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>天然气表后管道定制化服务</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程询比采购公告 采购公告 公告编号： RQXYGG202608190057 一、采购项目基本情况 采购人：重庆巴南天然气有限责任公司 网 采购项目编号：RQCGXY202608170010 采购项目名称：重庆国际生物城配套公寓项目天然气表后管道安装工程 务 采购内容和范围：完成重庆国际生物城配套公寓项目 （民用1020户）天然气表后管道定制化服务。（含安装燃 气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个， 其它配套管件及辅材，墙体管道暗埋等） 二、供应商资格要求 商 1. 资质要求:资质要求： 1.响应供应商为中华人民共和国境内合法注册的独立法人或其他组织，具有独立承担民事责任能力，具有独立订 立合同的权利。 道 2.响应供应商应具备市政公用工程施工总承包三级及以上资质、具备有效的安全生产许可证。 3.响应供应商应为本项目配备项目负责人一名，持有市政公用工程或机电工程专业二级建造师及以上资质，且为 本单位在职人员并提供社保证明。 4.响应供应商应为本项目配备专职安全员一名，持有安全生产考核合格C证，且为本单位在职人员并提供社保证 管 明。 5.项目负责人及专职安全员社保证明期限须包含2026年5月至2026年7月。提供的社保证明，须体现上述人员的姓 名、身份证号（或社保号）、单位名称、本单位参保时间（或起始参保时间），并带有社保部门公章或社保部 门的有效电子印章。 2. 信用要求:6.信用要求国： （1）响应供应商（含联合体响应的成员单位）未被“国家企业信用信息公示系统” 网站（www.gsxt.gov.cn）列 入严重违法失信企业名单（如：提供网站查询界面截图）； （2）响应供应商（含联合体响应的成员单位）未被 “信用中国”网站（www.creditchina.gov.cn）列入严重失信 主体名单（中如：提供网站查询界面截图）。 三、采购文件的获取 采购文件在 华润守正采购交易平台 发布，不再另行线下提供纸质采购文件，凡有意参与者请自行登录守正平台 查看和下载采购文件。 四、响应文件的提交 响应文件提交 / 报价截止时间： 2026-08-25 08:00:00 （北京时间，若有变化另行通知）。 响应文件提交 / 报价方式：在响应文件提交 / 报价截止时间前，通过 华润守正采购交易平台 提交电子响应文件或 报价，逾期提交将被拒收。 五、采购人联系方式 联系人：何俊 电话：15178855716 邮箱：1460553040@qq.com 六、采购明细 行号 采购内容 需求数量 单位 补充说明 1 重庆国际生物城配套公寓项目天然气表后管道定制化服务 1 元/次 具体内容详见采购文件 七、答疑澄清、通知 答疑澄清、通知等文件一经在 华润守正采购交易平台 发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注 华润守正采购交易平台 发布的相关信息，并及时查阅和处理。 八、服务费交纳 网 本项目向成交人收取服务费,供应商收到预成交通知书和服务费交款通知书10日内,向平台运营方(华润守正招标有 限公司)支付服务费,经确认无误后由采购人发送成交通知书。平台运营方在收到服务费后向成交人开具服务费发 票。 收费标准：项目总成交金额＜50万元的采购项目，免收服务费。项目总成交金额≥50万元的采购项目，按成交金 务 额的0.15%向成交人收取（金额四舍五入，精确到分）。单项目总收费封顶100000元。其他说明：（1）总价采购， 收费基数为成交金额；单价、费率采购，收费基数为预算金额。（2）单项目存在多个成交人情形的，按总成交 金额计算收费总额，各成交人按成交比例分摊；项目总成交金额50万以上，但单个成交人成交金额少于50万仍按 比例收取服务费。 商 退款说明：成交通知书发布后,平台提供相关服务已完成,成交人已交纳服务费不予退还。 多成交人服务费收取示例： 以某项目总成交金额100万为例,A、B、C多成交人情形,总服务费为0.15万, 供应商A成交金额为50万,A服务费为0.075万; 供应商B成交金额为30万,B服务费为0.045万; 道 供应商C成交金额为20万,C服务费为0.03万。 九、其它事项 管 1.本公告在 华润守正采购交易平台 ( https://www.szecp.com.cn/ )上公开发布。 2.本项目采购通过守正平台线上进行，供应商需注册 华润守正采购交易平台 ，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 国 3.如对采购项目有异议，请登录 华润守正采购交易平台 ,通过异议菜单提出。 2026年08月19日 中 信息来源:https://www.chinapipe.net/project/d3076125.html cqdingjiu 2026.08.21 10:06:52</t>
@@ -1838,9 +2250,13 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>重庆, 天然气表后管道安装工程, 管材招标</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1873,16 +2289,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)建设。</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>项目资金来自业主自筹，项目出资比例为100%。本次招标项目货物采购估算金额约为330万元。</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>非金属管道管件阀门</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)非金属管道管件阀门采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）非金属管道管件阀门采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约 330 万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采 购”包括不限于非金属管道管件阀门所含设计、制造、试验、出厂检验、防腐、运输（含保护、包装及运输、 货到现场车板交货）、保险（交货验收前）、指导安装、调试、备件及专用工具、税费、技术资料和图纸及质 保期内的各种备品、备件的供应及相关的技术服务、产品质量证明书及原材料检测报告等。（详见“第五章货 物需求一览中表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 2.6 交货期： 2.6.1合同签订后3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向买方提交完整的技术资料，以供设计院开展相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）投标人具备有效的《中华人民共和国特种设备生产许可证》压力管道管子-B级及以上资质、压力管道管 件B2级及以上资质； （3）投标人具备塑料管道管子、管件的型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4. 招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年 8 月19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 网 5.投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月10 日上午09时30分，地点在重庆市公共资源交易中心开标厅（地 址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见一、二楼大厅显示屏。 务 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 商 本次招标公告在中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 道 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 管 联 系 人：张先生 电 话：023-40717888 国 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区五里店五简路2号重庆咨询大厦A栋20楼2001室 中 项目负责人：彭文婷 电 话： 023-67703002 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购 户名 开户行 投标保证金账号 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000631258 支行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303372 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630010400 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000002549 贸易试验区分行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835014652 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146619529 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764260665 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020038958 信息来源:https://www.chinapipe.net/project/d3076119.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
@@ -1894,9 +2318,13 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 资金, 产品</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1929,16 +2357,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)，包括衬氟管道及管件的采购。</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>项目资金来自业主自筹，项目出资比例为100%。货物采购估算金额约为225万元。</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>衬氟管道及管件</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)衬氟管道及管件采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）衬氟管道及管件采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约225万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）衬氟管道及管件采购一批” 包括但不限于制造、涂漆、包装、运输、配合验收工作、检验检测、产品质量证明书等。（详见“第五章货物 （材料）需求一览表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 中 2.6 交货期： 2.6.1合同签订后 3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向招标方提交完整的技术资料，以供设计院开展设备相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）具备有效的《中华人民共和国特种设备生产许可证》-压力管道元件制造-元件组合装置。 （3）具有防腐管道元件特种设备型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4、招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年8 月 19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 5、投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月 10 日上午09时30分，地点在重庆市公共资源交易中心开标厅 （地址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见网一、二楼大厅显示屏。 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 务 本次招标公告在 中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 商 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 道 联 系 人：张先生 电 话：023-40717888 管 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区国五里店五简路2号重庆咨询大厦A栋20楼2001室 项目负责人：彭文婷 电 话： 023-67703002 中 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630011190 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835003139 坝支行 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000000834 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146638621 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051302432 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000620855 支行 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020013554 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764235261 信息来源:https://www.chinapipe.net/project/d3076111.html cqdingjiu 2026.08.21 10:06:52</t>
@@ -1950,9 +2386,13 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>重庆, 废盐综合利用, 离子膜烧碱, 衬氟管道, 管件采购</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1985,16 +2425,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>蒸汽管道改造</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>蒸汽管道</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
           <t>重庆市益康环保工程有限公司永川分公司蒸汽管道改造项目询价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3076108.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
@@ -2006,9 +2454,13 @@
         </is>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>重庆, 蒸汽管道, 改造项目, 询价采购</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2041,16 +2493,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>南岸区</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>南岸区</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>包括改造市政混接点194个，改造管网8582米，缺陷管网开挖修复1355米，非开挖修复8679米。</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>总投资概算未明确具体金额，但合同预估金额为6600万元。</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>排水管网改造</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>南岸区融侨大道、江南大道片区2023年排水管网改造项目(三标段)招标计划表 重庆市工程建设项目招标计划表 项目名 南岸区融侨大道、江南大道片区 2023年排水管网改造项目（三标段） 称 网 招标法 人或招 重庆市南岸区城市建设发展（集团）有限公司 标人名称 （盖章） 务 项目批 准文件 南岸发改〔2024〕304《南岸区融侨大道、江南大道片区2023年排水管网改造项目总投资概算的批复》 及文号 主要建 包括改造市政混接点194个，改造管网8582米，商管径d300~d1500;缺陷管网开挖修复1355米，管 设内容 径d300~d600;非开挖修复8679米，管径d300~d1200。 招标文件 拟交 合同预估 招标内 招标 序号 招标项目名称 计划发布 易场 金额(万 备注 道容 方式 时间 所 元) 51处雨 污混错 重庆 招标项 接点位 管 市公 目 改 南岸区融侨大道、江南大道片区 2023年排 公开 共资 1 造，1082 2026-08 6600.00 水管网改造项目（三标段） 招标 源交 个管网 易中 三四级 国 心 缺陷修 复。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 中 信息来源:https://www.chinapipe.net/project/d3076097.html cqdingjiu 2026.08.21 10:06:52</t>
@@ -2062,9 +2530,13 @@
         </is>
       </c>
       <c r="O29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>重庆, 排水管网改造, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2097,16 +2569,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>永川区</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>永川区</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、综合楼、生产建（构）筑物以及附属建筑物等。</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>项目合同额1.7亿元</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>钢筋混凝土排水管</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购公告 永川三教水厂项目 已具备采购条件，现公开邀请供应商参加询比采购活动。 1.采购项目简介 1.1 采购项目名称：中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购。 1.2 采购方案编号：FA00000663117。 网 1.3 采购人：中交一公局重庆工程有限公司。 1.4 采购代理机构：/。 务 1.5 采购项目资金：已落实 1.6 采购项目概况： 商 永川三教水厂项目：项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建 净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、 综合楼、生产建（构）筑物以及附属建筑物等。项目合同额1.7亿元，工期450天。 道 项目地址：重庆市永川区。 2.采购范围及相关要求 管 2.1 采购范围：钢筋混凝土排水管。 2.2 交货期：2026年9月-2026年12月。 2.3 交货地点：重庆市永国川区项目指定地点。 2.4 物资质量标准：满足《混凝土和钢筋混凝土排水管》（GB/T 11836-2023）的相关要求。 3.供应商资格要求 中 3.1 供应商应依法设立且满足如下要求： （1）资质要求：本次询比采购要求供应商须是在中华人民共和国境内依法注册，具有合法有效的营业执照、税 务登记、组织机构代码等证件，具有独立法人资格、具有采购物资生产经营范围的生产商或代理商（销售商）。 （2）财务要求：供应商必须是经税务部门注册登记核准的纳税人，有依法纳税的良好记录。 （3）业绩要求：无。 （4）信誉要求：无不良履约记录、未列入工程所在地质量监督部门和中国交建、中交一公局集团企业黑名单。 因质量原因被交通部质监站通报，正在进行整改的生产厂家和产品不得参与投标。生产商或代理商（销售商） 具有良好的社会信誉，近3年内没有与骗取合同有关的犯罪或严重违法行为而引起的诉讼和仲裁；近3年不曾在合 同中严重违约或被逐；财产未被接管或冻结，企业未处于禁止或取消投标状态；在最高人民法院、信用中国 （www.creditchina.gov.cn）或各级信用信息共享平台查询拟入库单位无不良行为记录。 （5）其他要求：无。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他：无。 4.供应商报名 4.1 有意参加询比采购活动的单位，请于2026年8月19日15时00分至2026年8月26日17时00分（北京时间，下同，法 定公休日、节假日不休），登录“中交招采网”（网址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 网 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 务 5.供应商报价 5.1 报价结束（递交响应文件截止）时间为2026年8月26日17时00分。 商 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的电 子响应文件，采购人将拒收。 5.3电子采购的供应商响应文件由线上电子报价道表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 子报价表的数据为准。 6.开标 管 6.1 开标时间：与报价结束时间相同。 6.2 开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标。 国 7.发布公告的媒介 本询比采购公告在 “中交招采网” 上发布。 中 8.评审办法 本项目评审办法采用 经评审的最低价法 。 9.合同主要条款 9.1 付款条件：按月结算，上月11日至本月10日为一个结算对账期，乙方必须按照甲方要求开具合规的增值税专 用发票，无发票不予付款。结算完成后1个月内支付已结算金额的70%，剩余30%货款在结算完成后3个月内支付。 付款方式为银行转账，甲方有权采用票据支付或者供应链支付的方式支付货款，因此产生的费用包含在综合单 价中，乙方不得因此调价和索赔。如遇业主支付不及时，乙方应予理解。 9.2 履约保证金的递交： （1）R不要求递交 （2）要求递交，保证金金额：/，保证金形式：/，其他形式：/ 。 10.监督机构 监督机构名称： 中交一公局重庆工程有限公司审计部 11.成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联系400-676-5885，中标服务费请按7咨询。 11.1 收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； （3）在1000万元（含）至3000万元之间的，每次收取1000元； 务 （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 11.2 支付流程 （1）通知推送：中标结果发布后，系统自动推送缴费通知（含应缴金额及支付链接）； 道 （2）费用查询：供应商登录“中交招采网—供应商协同—服务费”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网— 供应商协同—服务费—发票查询”模块获取。 12.其他 国 / 。 13.联系方式 中 采 购 人：中交一公局重庆工程有限公司 地 址：重庆市江北区创富路5号 邮 编：361021 联 系 人：汪仁宽 电 话：13527572392 电子邮件：1176245792@qq.com 项目联系人及电话： 序号 项目名称 联系人 联系电话 1 永川三教水厂项目 高博 17788661005 中交一公局重庆工程有限公司 2026年8月19日 物资信息 序号 设备物资名称 设备物资说明 税率 单位 网 1 钢筋混凝土排水管 2000mm Ⅲ级 承插口 13% 米 信息来源:https://www.chinapipe.net/project/d3076078.html 务 cqdingjiu 2026.08.21 10:06:52 商 道 管 国 中</t>
@@ -2118,9 +2606,13 @@
         </is>
       </c>
       <c r="O30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 钢筋混泥土排水管, 永川三教水厂项目</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2153,16 +2645,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>重庆市大渡口区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防护工程施工劳务招标。</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>项目出资比例为100%，资金已落实。</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>施工劳务</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr">
         <is>
           <t>中国铁路成都局集团有限公司重庆市大渡口区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防护工程施 工劳务招标招标公告 重庆市大渡口区萤石及配套企业 35 千伏专用变电站项目穿越渝贵等铁路防护工程施工劳务招标公告 招标编号：DXNZBCQ-GC-2026-13 1. 招标条件 本建设项目重庆市大渡口区萤石及配套企业 35 千伏专用变电站项目穿越渝贵等网铁路防护工程施工劳务招标已由 《中国铁路成都局集团有限公司关于重庆市大渡 口 区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防 护工程施工图设计的复函》（科信技审〔2025 〕115号）批准建设，建设单位为重庆建桥置业有限公司，建设资 金使用外委资金，项 目出资比例为100%，资金已落实。招标人为中国铁路成都局集团有限公司重庆工务段。本 项目已具备法定招标条件，现进行公开招标，特邀请有意向的投标人参加投标。 务 2. 项目概况与招标范围 2.1 项目概况 商 2.1.1建设地点：渝贵线K38+838、南疏Ⅰ线K10+808、川黔线K1+622、川黔线K3+781、兴珞上行线K38+619、兴珞 下行线K38+635、小西线K1+633、南疏Ⅱ线K11+257。 2.1.2建设规模：重庆市大渡 口区萤石及配套企道业35千伏专用变电站项目穿越渝贵等铁 路防护工程，本项目工分为5个交叉工点。工点一采用明挖直埋方式下穿渝贵铁路新白沙沱长江多线特大桥第14孔 （渝贵线K38+838）；工点二采用顶进套管方式下穿南疏 Ⅰ 线K10+808（ 已停用）、川黔线K3+781（ 已停用 ）； 工点三采用明挖直埋方式下穿兴珞线陈家湾双线特大桥（上行线K38+619、下行线K38+635）；工点四采用顶进 管 套管方式下穿。 2.2 招标范围：重庆市大渡口区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防护工程施工劳务招标。 即涉铁部分第第三章桥涵，第六章通信、信号、信息及灾害监测，第十章大型临时设施和过渡工程，第十一章 其他费用中的安全生产国费以及非涉铁部分。 2.3标段划分：本项目施工招标划分为1个标段。 2.4计划工期：240日历天，计划开工日期：2026年10月8日，计划竣工日期：2027年6月4日。 中 2.5 其他说明：___/___。 3. 投标人资格要求 3.1本次招标要求投标人为在中华人民共和国境内合法注册的独立法人，具备有效的营业执照、施工企业资质和 安全生产许可证等，并在人员、设备、资金等方面具备相应的施工能力。资格要求如下： 3.1.1 标段编号：全标段 （1）资质要求：施工劳务企业资质。 （2）业绩要求：近3年内完成过铁路营业线类似项目业绩。 （3）项目负责人要求:具有工程师及以上职称，2 年及以上类似铁路营业线项目管理工作经验， 良好的职业道德， 且未在其他在建工程项目任职。 （4）本标段不接受联合体投标申请。 （投标人资格要求详见招标公告附件） 3.2 各投标人可就上述标段中的 1 个标段进行投标。 3.3投标人未在“信用中国”网站（www.creditchina.gov.cn）中被列入失信被执行人名单，投标人未在国家企业信 用信息公示系统（www.gsxt.gov.cn）中被列入严重违法失信企业名单，投标人未被列入铁路工程建设失信行 为“黑名单”，投标人及其法定代表人、拟委派的项目经理在近3年不曾有行贿犯罪记录； 其他信誉要求：未被取消或暂停投标资格、不存在辖内失信的情形、不存在最近一期国铁集团施工企业评价为D 级且在整改期内的情形。 4. 招标文件的获取 4.1凡有意参加投标者，请于2026年08月20日00时00分至2026年08月25日00时00，在重庆龙头寺旅游集散中心（重 庆市两江新区天宫殿街道昆仑大道56号附1号5楼办公室）持单位介绍信获取招标网文件。 4.2招标文件每套售价0元，售后不退。 4.3其他：凡有意参加投标者可通过网上登记获取招标文件，将获取招标文件材料扫描件（PDF格式）发送 务 至dxncq_bgs@163.com邮箱登记，由招标代理人通过电子邮件方式向有意参加投标者发送招标文件。 5. 投标文件的递交 5.1投标文件递交时间为2026年09 月10 日08时30分至2026年商09月10 日09时00分，递交比选申请文件的截止时间（比 选截止时间，下同）为2026年09月10日09时00分，地点为重庆龙头寺旅游集散中心（重庆市两江新区天宫殿街道 昆仑大道56号附1号5楼开标室）。 5.2逾期送达的或者未送达指定地点或者不按照道招标文件要求密封的投标文件，招标代理人不予受理。 6. 发布公告的媒介 本次招标公告在国铁采购平台（https://cg.95306.cn）发布。 管 7. 联系方式 招 标 人：中国铁路成都局集团有限公司 招标代理机构：成都大西南铁路监理 国 重庆工务段 有限公司 地 址：重庆市九龙坡区黄桷坪街道铁 地 址：成都市金牛区站西桥西街305 中 路3村161号 号府河路苑9栋14楼 邮 编： / 邮 编：610081 法定代表人： 法定代表人 或其委托代理人： 或其委托代理人： 联 系 人： 任女士 联 系 人：汤女士 电 话： 17393148353 电 话：023-61896910 传 真： / 传 真： / 电子邮箱： / 电子邮箱：dxncq_bgs@163.com 网 址： / 网 址： / 开户银行： / 开户银行： / 账 号： / 账 号： / 2026年08月19日 附件： 获取招标文件信息表 申请人名称： （加盖公章） 项目名称：（按公告名称填写） 获取招标文件起止时间：（按照公告时间填写） 项目编号：（按照公告填写） 单位名称 经办人 联系电话 电子邮箱 标段 资料提交时间 备注 网 注：须附经办人介绍信、身份证复印件、单位营业执照复印件。 信息来源:https://www.chinapipe.net/project/d3075989.html cqdingjiu 2026.08.21 10:06:53 务 商 道 管 国 中</t>
@@ -2176,7 +2676,11 @@
       <c r="O31" t="n">
         <v>0</v>
       </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2209,16 +2713,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>云阳县</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>云阳县</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>合同预估金额：9100.00万元</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>污水管网</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr">
         <is>
           <t>长江流域云阳青龙段污水管网一体化建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 长江流域云阳青龙段污水管网一体化建设项目 招标法人或 招标人名称 云阳县青江环境综合整治有限公司 网 （盖章） 项目批准文 云阳发改资环【2025】55号 件及文号 务 主要建设内 新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。 容 招标方 招标文件计 拟交易场 合同预估金额 序号 招标项目名称 招标内容 备注 式 划发布时间 所 (万元) 商 长江流域云阳 新建污水管网55.5千米， 重庆市公 青龙段污水管 其中DN200管网12千 公开招 共资源交 1 网一体化建设 米、DN300管网24千 2026-08 9100.00 标 易中心云 项目EPC总承 米、DN40道0管网19.5千 招标项目 阳分中心 包 米等。 新建污水管网55.5千米， 长江流域云阳 重庆市公 其中DN200管网12千 青龙段污水管 公开招 共资源交 2 管米、DN300管网24千 2026-08 140.00 网一体化建设 标 易中心云 米、DN400管网19.5千 项目监理 阳分中心 米等监理。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 国 信息来源:https://www.chinapipe.net/project/d3075867.html cqdingjiu 2026.08.21 10:06:53 中</t>
@@ -2230,9 +2750,13 @@
         </is>
       </c>
       <c r="O32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 污水管网, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2265,16 +2789,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3站5区间的土建）：高龙大道站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子站区间、石家院子站～终点区间、7/17号线联络线区间。采购范围为雨污水排水迁改工程。</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>建设资金来源已落实，但具体资金数额未明确。</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>雨污水排水迁改工程</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
           <t>中国电建水电四局华中公司重庆轨道交通17号线一期5标项目雨污水排水迁改工程施工劳务分包采购项目公开询 比采购公告 询比采购公告 采购编号： PC-0104-26J6-FP0895 一、采购条件 受中国水利水电第四工程局有限公司重庆轨道交通17号线一期5标项目委托，中水电四局华中（武汉）工程有限 公司以公开询比方式采购重庆轨道交通17号线一期5标雨污水排水迁改工程项目网，建设资金来源已落实。目前项 目已具备采购条件，现进行公开询比采购。 二、项目概况、采购范围 务 1、项目概况：重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3 站5 区间的土建）：高龙大道 站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子 站区间、石家院子站～终点区间、7/17号线联络线区间。 2、采购范围： 商 （1）雨污水排水迁改工程 （2）工程招标范围工作内容：17号线一期5标道中高龙大道站、斑竹林站及高斑竖井位于城市既有道路下方，设计 采用明挖法施工。为保证市政排水管网的正常使用，在明挖施工前需对既有管网进行临时迁改，车站结构施工 后进行恢复。施工PE钢带管长度2387米、B型排水管长度2799m、钢筋混凝土管127米，检查井239座劳务部分。 （3）施工内容详见工程量清单，以及为完成此项工程而做的一切工作。 管 3、计划工期:计划开工日期：2026年9月25日（具体时间以采购人通知为准），计划完工日期：2027年 12 月25 日； 合同工期总日历天数为457天。 4、质量要求：符合《国给水排水管道工程施工及验收规范》（GB 50268）、《混凝土结构工程施工质量验收规范》 （GB 50204）、《城镇道路工程施工与质量验收规范》（CJJ 1-2008）以及项目所在地最新的相关法规、标准和 图集。工程质量全面达到设计要求和标准，其中：验收合格率 100%，优良率达 90%以上，工程综合验收质量评 定达优良标准。 中 5、付款方式：采用银行转账/支票支付工程价款，月度结算完成具备付款条件后30天内工程进度款支付比例约定 为扣除各项保证金及费用后应付价款不低于65%；清算完成并签订《退场协议》后30天内工程进度款支付比例约 定为扣除各项保证金及费用后应付价款不低于80%；清算完成并签订《退场协议》后一年内工程进度款支付比例 约定为扣除响应人缺陷责任等相关费用后应付价款不低于90%；清算完成并签订《退场协议》，办理完成保证金 退还手续后两年内，工程进度款支付比例约定为扣除响应人缺陷责任等相关费用后应付价款的100%。 6、其他：无。 三、响应人资格要求 响应人必须满足以下全部资格要求： （1）资质要求：施工劳务不分等级 （2）主要人员要求:授权委托人（如有）及项目经理、专职安全员应提供社保和劳动合同。其中劳动合同至少提 供首、末两页，并且包含有关人员的详细信息;社保证明应提供响应截止时间前三个月的社保缴纳记录。 （3）安全三类人员要求:应提供企业主要负责人安全A证、项目经理B证、专职安全员C证。 （4）响应人具有良好的银行资信和商业信誉，没有处于被责令停业，财产被接管、冻结、破产状态。 （5）响应人应具有 雨污水排水迁改 工程的施工业绩，在近 5年内(2021年7月-2026年7月内签订)的施工合同不少 于 1 个，且签订单项合同金额均在 100 万元以上（应附成交通知书和（或）合同扫描件）。 （6）其它要求:无。 （7）本次采购不接受联合体响应。 四、采购文件的获取 凡满足本公告规定资格要求并有意参加的响应人，请于2026年8月22日10时00分前在中国电建采购招标数智化平台 （https://bid.powerchina.cn/bidweb/#/login，以下简称“数智化平台”）获取采购文件，采购文件免费提供。 五、响应文件的递交 1、响应文件递交的截止时间（响应截止时间，下同）为2026年8月26日10时30分网（北京时间），响应人应在截止 时间前通过数智化平台递交电子响应文件。 2、本次采购将通过数智化平台全程在线开展，电子响应文件的加密、提交等流程须响应人在线进行操作。响应 人须提前办理数字证书用于在线递交响应文件，办理方式详见数智化平台首页，并严格按照要求进行在线操作， 务 因操作流程失误造成的递交失败将由响应人自行承担后果。 3、开启由“数智化平台”在响应截止时间后自动对响应文件进行解密，响应人及时关注开启结果。 4、响应截止时间如有变动，采购人将及时通知已获取采商购文件的响应人。 六、发布公告的媒介 本次询比采购公告同时在中国电建阳光采购网道（https://bid-zb.powerchina.cn）上发布。 七、评审办法 采用综合评估法。 管 八、联系方式 采 购 人： 中水电四局华中（武汉）工程有限公司 国 地 址： 湖北省武汉市江岸区塔子湖东路健美街30号立城中心商务楼13、14层 邮 编： 430014 中 联 系 人： 王飞 电 话： 15827222587 电子邮箱： 107830343@qq.com 九、提出异议的渠道和方式 单位名称： 中水电四局华中（武汉）工程有限公司 电 话： 17708178186 电子邮箱： sjhzgsjw@163.com 十、纪检监督机构 响应人或者其他利害关系人认为本次采购活动存在违规违纪行为的，可以书面形式向中国水利水电第四工程局 有限公司中水电四局华中（武汉）工程有限公司纪委办公室（联系方式：17708178186）提出投诉。 2026年8月 19 日 报价网址:https://bid.powerchina.cn/notice/detail?id=2409510708 信息来源:https://www.chinapipe.net/project/d3075750.html cqdingjiu 2026.08.21 10:06:53 网 务 商 道 管 国 中</t>
@@ -2286,9 +2818,13 @@
         </is>
       </c>
       <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>重庆, 轨道交通, 雨污水排水迁改, 施工劳务分包</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2321,16 +2857,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>本项目涉及预制钢筋砼管、成品混凝土仿木栏杆等材料的采购。</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>建设资金为国债资金，项目出资比例为100%。具体预算金额未在文本中明确列出。</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>预制钢筋砼管,成品混凝土仿木栏杆</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr">
         <is>
           <t>万州区2026年超长期特别国债高标准农田建设项目拟进行预制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜的 信息公告 1.采购条件 1.1本项目万州区2026年超长期特别国债高标准农田建设项目工程已由 重庆市万州路桥建设有限公司承建，项目 业主为重庆市万州区农业技术与机械推广中心，代建业主为重庆市万州区农业发展有限公司，建设资金为国债 资金，项目出资比例为 100% ，承包人为重庆市万州路桥建设有限公司。项目已具备施工条件，现对该项目的预 制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜发布信息公告。 网 2.项目概况与采购范围 2.1建设地点：重庆市万州区走马镇、瀼渡镇、罗田镇、余家镇、高梁镇、分水镇、柱山乡等7个镇乡。 务 2.2本项目材料采购拟进行比选情况如下： 罗田镇谷山片区材料采购费暂定金额约： 17.5万元； 余家镇桥亭片区材料采购费暂定金额约： 17.99万元； 商 柱山乡山田片区材料采购费暂定金额约： 26.32 万元； 走马镇凉风片区材料采购费暂定金额约： 15.道66万元； 瀼渡镇高村片区材料采购费暂定金额约： 17.72 万元； 分水镇大冲片区材料采购费暂定金额约： 47.12 万元； 管 高梁镇茨坪片区材料采购费暂定金额约： 10.7万元； （以上片区片区金额为暂定金额，最终比选限价金额以比选文件为准）。 国 2.3计划采购周期： 以合同签订为准 日历天。 2.4采购范围：本项目各片区所包含的预制钢筋砼管、成品混凝土仿木栏杆等材料。 中 3.供应商资格要求 3.1本次材料采购要求供应商具备独立企业法人，具有本次所需材料生产能力的厂家或经销商等，其经营范围和 权限应满足本次所需材料的要求，并依法取得国家行政主管部门颁发的有效工商营业执照(建筑材料销售或水泥 制品制造、水泥制品销售等相关营业资格），所提供产品必须满足各项检测要求，达到国家现行标准规定的合 格标准。具有良好的商业信誉和充分的供应保障能力，具备相应售后服务能力。要求竞选人为一般纳税人，可 开具13%税率增值税专用发票，提供一般纳税人认定证明。 3.2本次供应商单位优先选择万州本地企业。 3.3本次 不接受 联合体竞选。 4. 报名要求 4.1报名时间：2026年8月 19日9:00起至 8月21日17:00止。 4.2报名地点：重庆市万州路桥建设有限公司经营部（重庆市万州区天城东路278号）。 4.3报名时，须提交有效的营业执照(有效工商营业执照((建筑材料销售或水泥制品制造、水泥制品销售等相关营 业资格）)，前述证书均为复印件并加盖单位公章。法定代表人参加报名的不需要授权委托书，只需要提供法定 代表人身份证明；非法定代表人参加报名的除提供法定代表人身份证明外还须提供授权委托书、委托代理人身 份证明。 4.4 本项目材料采购需提前报名。经资格预审合格后，通知资格预审合格的供应商，到承包人单位领取相关文件。 4.5本项目材料采购设七个片区进行比选，为保证比选公平、公正、有效，规定同一参选单位报名片区上限为2个， 且最终仅限中选一个片区。 5.联系方式 承包人：重庆市万州路桥建设有限公司 地 址：重庆市万州区天城东路278号 网 联系人： 张红娟 电 话：15923491915 务 邮 箱： 商 重庆市万州路桥建设有限公司 2026年8月19日 道 信息来源:https://www.chinapipe.net/project/d3075512.html cqdingjiu 2026.08.21 10:06:53 管 国 中</t>
@@ -2342,9 +2894,13 @@
         </is>
       </c>
       <c r="O34" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>重庆, 预制钢筋砼管, 成品混凝土仿木栏杆, 国债资金, 高标准农田建设</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2377,16 +2933,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>酉阳土家族苗族自治县</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>酉阳土家族苗族自治县</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水管道)公开招标采购。</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>污水管道</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水 管道)招标采购流标公告 发布单位：中国铁建/中铁十一局/六公司 发布时间：2026-08-19 10:40:49 投标截至时间：2026-08-18 10:00:00 内容： 各投标人： 网 中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资（污水 管道）公开招标采购（采购编号： CR1106-JC-2026-26-02）评标工作，已于北京时间2026年08月18日10:00整，在 铁建云链（https://www.crccep.com）线上平台公开开标。评审委员会根据招标文件载明的评审办法完成评审工作， 现将评审结果公示如下： 务 一、招标公告发布日期及媒体 招标公告发布日期：2026年07月27日至2026年08月01日 商 招标公告媒体：铁建云链（https://www.crccep.com） 二、拟中标信息 道 公开招标采购编号：CR1106-JC-2026-26-02 包件号：WSGD-01 序号 供应商名称 推荐排序 管 1 无 1 国 以上包件有效投标不足三家，本次招标做流标处理。 三、公示时间 中 自2026年08月19日始，至2026年08月22日止。在公示期间，所有竞标人和其他利害关系人如对公示的评审结果有 异议，可以向相关监督部门举报，逾期将不再受理。举报人必须由其法定代表人或者授权代表签字并盖章，其 他组织或者个人举报的，必须由其主要负责人或者本人签字，并附有效身份证明复印件。举报人如实反映情况 受法律保护。 公示期满，如无异议，即时生效。 监督竞诉受理部门： 中铁十一局集团第六工程有限公司招采中心 联系电话：18671041790 信息来源:https://www.chinapipe.net/project/d3075461.html cqdingjiu 2026.08.21 10:06:53</t>
@@ -2398,9 +2970,13 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 酉阳县, 污水管网, 新建改造工程</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2433,16 +3009,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>详见附件。</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>镀锌管件</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t>协同创新区-四期房建三标段镀锌管件物资竞价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3075420.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
@@ -2454,9 +3038,13 @@
         </is>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 商机</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2489,16 +3077,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>渝北区</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>渝北区</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>长江一级支流溉澜溪流域(新华水库混流箱涵)污水收集效能提升工程(渝北区)施工答疑补遗文件</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr">
         <is>
           <t>长江一级支流溉澜溪流域(新华水库混流箱涵)污水收集效能提升工程(渝北区)施工答疑补遗文件 长江一级支流溉澜溪流域（新华水库混流箱涵）污水收集效能提升工程（渝北区）施工答疑文件 各潜在投标人： 现将“长江一级支流溉澜溪流域（新华水库混流箱涵）污水收集效能提升工程（渝北区）施工”公开招标项目 答疑文件发布。本答疑文件是在招标文件的基础上作出的澄清、说明或补正，与招标文件具有同等法律效力， 若相关内容与原招标文件不一致时，一律以本答疑文件内容为准。 网 一、答疑部分： 问题一：1、我公司于2026年进行了优势合并整合，现准备使用合并前公司项目业绩作为本次我司投标的投标人 业绩证明，并提供上级主管单位出具的相关吸收合并文件或两家公司签订的吸收合并协议，请问是否可视为满 务 足招标业绩要求？ 2、我单位为中型企业，其控股股东为大企业，但我单位不属于大企业的分支机构，也不存在与大企业的负责人 为同一人的情形。鉴于此种情况，我单位应提供《中小企业声明函（工程类）》还是《中小企业承担合同份额 承诺函》？ 商 回复：1. 满足，但还需满足招标文件对业绩的其他要求。最终由评标委员会根据投标人提供的证明材料并结合 招标文件要求进行评审； 道 2. 贵司其控股股东为大企业，故需提供中小企业承担合同份额承诺函。 问题二：本项目有无业主专家参与评标？ 管 回复：该项目评标委员会由招标人按法律法规及相关规定依法组建。 问题三：请明确是否有业主专家 是否异地评标 回复：1. 该项目评标委国员会由招标人按法律法规及相关规定依法组建。 2.本项目是异地评标。 问题四：1、财务报告可以不提供财务报表附注吗? 中 2、投标函附录中，工期、分包、工程质量、缺陷责任期等要求可以统一填写"达到招标文件要求"吗? 3、招标文件第八章投标文件格式中(二)承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要提供其 他格式之外的其他承诺? 4、是否有业代专家参与评标，不要模糊的回答什么依法组建评标委员会。请明确回复有或者没有。 5、本项目是否异地评标？ 6、业绩竣工验收证明材料中有单位盖的项目部章是否认可呢？ 回复：1. 可以不提供财务报表附注。 2. 可以统一填写"达到招标文件要求"。 3. 投标人自行核实招标文件要求提供的承诺要求，如有需要，还需补充提供招标文件第八章投标文件格式中 （二）承诺部分之外的其他承诺。 4. 该项目评标委员会由招标人按法律法规及相关规定依法组建。 5. 本项目是异地评标。 6. 不认可。 问题五：请问**公司现在被人民法院列为被执行人且有1000多万股权冻结到2028年，因为不能履行保函的见索即 付，拒绝赔付。 相关业主方在招标文件补遗通知中直接将**公司列入担保公司回避名单，拒绝**公司所出具的保函。由此可 见**公司的信用资质、履约能力、根本无能力是存在很大问题的。请问以**公司目前的被执行和不履行投标担保 责任的情况是否符合招标文件的要求? 回复：纸质投标保函的开立人应当是具有相应资格的银行、保险机构、融资担保公司，其信用资质、履约能力、 担保能力、赔付流程、安全保密等应符合工程保函业务条件。纸质投标保函应合网法合规，符合招投标行政监督 部门、行业主管部门和金融监管部门的相关规定，满足招标文件约定要求。投标人应选择在渝依法设立总部或 者设有分支机构的金融机构开具纸质投标保函。投标人对所提交的纸质投标保函的真实性、合法性、有效性负 责。以纸质投标保函形式交纳投标保证金是否符合招标文件要求，由评标委员会评标时，根据招标文件要求进 行独立评审，并作出相应评审判断。 务 问题六：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 回复：经核实，招标文件（PDF签章版）中投标文件格式商与重庆市电子招投标系统投标文件制作软件中格式一致。 可能因重庆市电子招投标系统投标文件制作软件中的格式页边距与招标文件（PDF签章版）不一致的原因导致格 式显示不一致，该情形不影响投标人编制投标文件。若重庆市电子招投标系统投标文件制作软件导出的投标文 件格式与招标文件（PDF签章版）的投标文件格式不一致，以重庆市电子招投标系统投标文件制作软件导出的投 标文件格式为准。 道 问题七：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖 章，请问需要提供联合体协议书吗？ 管 回复：若投标人提供的公司业绩为epc业绩，且合同协议书或工程竣工验收合格的证明材料或业主证明能证明该 投标人承担的工作为施工任务的，则不需要提供联合体协议书；若投标人提供的公司业绩为epc业绩，但合同协 议书或工程竣工验收合格的证明材料或业主证明不能证明该投标人承担的工作为施工任务的，则需要提供联合 体协议书。 国 问题八：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可 以不填(空白)，对此有无要求？ 回复：投标中文件中下划线上、空格处、表格中无需要填写或无法填写内容的，填“/”或“无”均可。 问题九：公园施工业绩符合吗？ 回复：公园概念太宽泛，无法判定该施工业绩是否属市政工程，请投标人自行核实，并按招标文件要求提供施 工业绩证明材料，其是否满足要求应由评标委员会根据证明材料具体内容进行判定。 问题十：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需 要提供其他格式之外的其他承诺？ 回复：投标人自行核实招标文件要求提供的承诺要求，如有需要，还需补充提供招标文件第八章投标文件格式中 （二）承诺部分之外的其他承诺。 问题十一：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收， 请问我公司业绩满足业绩要求吗？ 回复：不满足。 问题十二：可以用自己做的材料购买协议、劳务协议、设备租赁协议作为低价说明证明材料吗？ 回复：投标人投标总报价低于招标文件规定的对应的异常低价警戒线的，应提供报价合理性说明，并提供必要 的证明材料。证明材料由投标人自行提供，但提供的说明不得降低或者改变原设计方案、技术工艺、施工标准， 不得影响项目的质量、安全、工期、结算等正常履约。 问题十三：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 回复：按照招标文件要求“提供：会计师事务所或审计机构出具的合法有效的财务审计报告及财务报表，财务 报表须至少包括现金流量表、资产负债表、利润表”。 问题十四：业绩要求的竣工时间是指竣工验收时间吗？ 回复：本项目业绩要求所指竣工时间，即为工程竣工验收合格证明载明的竣工验收时间。 问题十五：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知 书发出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面网通知相关金融机构本项目准 予提前注销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 回复：纸质投标保函原件上未加盖“正本”字样的，不因此否决投标，但投标人应确保提交的保函为唯一正本。 若因保函真伪问题导致的一切不利后果由投标人自行承担。 务 问题十六：燃气管道安装施工业绩满足吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 商 问题十七：请问招标人是否委派业主专家参与评标吗？ 回复：该项目评标委员会由招标人按法律法规及相关规定依法组建。 道 问题十八：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 回复：根据招标文件“投标人的工程量清单单项报价不得为零报价（招标人提供的工程量清单单项最高限价中 金额为零的除外）或者负数报价”，招标人提供的工程量清单单项最高限价中金额为零的，该项清单综合单价 管 报价可以为0。 问题十九：自来水厂或者净水厂施工业绩满足业绩要求吗？ 回复：满足，但还需满国足招标文件对业绩的其他要求。 问题二十：财务报告可以不提供财务报表附注吗？ 回复：可以不提供财务报表附注。 中 问题二十一：老旧小区室外环境改造施工业绩符合吗？ 回复：不满足。 问题二十二：有人提出一个无关问题。 回复：无关问题不予回复。 问题二十三：任一清单的综合单价低于警戒线，就要提供说明吗？ 回复：本招标项目单项报价未设置异常低价警戒线。 问题二十四：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 问题二十五：本项目是异地评标吗？ 回复：本项目是异地评标。 问题二十六：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、 注册证及在本单位注册的证明文件替代？ 回复：不满足。 问题二十七：污水处理厂提标改造施工业绩满足吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 问题二十八：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 回复：可以填“达到招标文件的要求”。 问题二十九：财政部 国务院国资委 金融监管总局2023年9月14日发布的《关于加网强审计报告查验工作的通知》 中要求会计师事务所应当按照规定将其承办《中华人民共和国注册会计师法》第十四条规定审计业务出具的报告 （以下简称审计报告）上传注册会计师行业统一监管平台（以下简称统一监管平台）并申请赋码。本项目投标 人提供的财务报告需要赋码和提供深度查询截图吗？ 务 回复：投标人提供的财务报告不需要赋码和提供深度查询截图。 问题三十：有人提出一个无关问题。 回复：无关问题不予回复。 商 问题三十一：我公司业绩合同金额3600万元及以上，但是竣工报告业绩金额小于3600万元，请问是否满足业绩要 求？ 道 回复：按招标文件执行。“当上述业绩证明材料中针对同一指标存在不一致时，以工程竣工验收合格的证明材 料为准”。 问题三十二：专业分包业绩满足业绩要求吗？ 管 回复：专业分包业绩可满足业绩要求，但还需满足招标文件对业绩的其他要求。 问题三十三：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养 老保险证明材料复印件国递交吗？ 回复：不需要。 问题三十四：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要 中 求”吗？ 回复：可以统一填写“达到招标文件要求”。 问题三十五：市政桥梁施工业绩满足业绩要求吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 问题三十六：有人提出一个无关问题。 回复：无关问题不予回复。 问题三十七：本项目委派业主专家吗？ 回复：该项目评标委员会由招标人按法律法规及相关规定依法组建。 特别提示：本通知与招标文件具有同等法律效力，若招标文件与本通知不一致时，一律以本通知为准。 招标人：重庆水务环境控股集团管网有限公司 招标代理机构：重庆市工程管理有限公司 2026年8月19日 信息来源:https://www.chinapipe.net/project/d3075975.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
@@ -2512,7 +3116,11 @@
       <c r="O37" t="n">
         <v>0</v>
       </c>
-      <c r="P37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2545,16 +3153,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>新建一体化提升泵站及管道约5000m，投资约800万元。</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>投资约800万元</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>施工</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr">
         <is>
           <t>中化重庆涪陵化工搬迁后污水处理厂建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 中化重庆涪陵化工搬迁后污水处理厂建设项目 招标法人或 招标人名称 重庆市涪陵交通旅游建设投资集团有限公司 网 （盖章） 项目批准文 涪发改委发[2019] 505号 件及文号 务 主要建设内 新建一体化提升泵站及管道约5000m，投资约800万元。 容 招标 招标 招标文件计 拟交易 合同预估 序号 招标项目名称 备注 内容 方式 划发布时间 场所 金额(万元) 商 本招标计划与2026年5 月25日发布的招标项目 中化重庆涪陵 重庆市 名称为“中化重庆涪陵 招标项目 化工搬迁后污 涪陵区 公道开 化工搬迁后污水处理厂 1 水处理厂建设 施工 2026-09 公共资 800.00 招标 建设项目（场外连接管 项目（场外干 源交易 网）”的招标计划，除 管部分） 中心 招标项目名称调整外， 其余内容完全一致。 管 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075591.html cqdingjiu 2026.08.21 10:国06:54 中</t>
@@ -2566,9 +3190,13 @@
         </is>
       </c>
       <c r="O38" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 商机</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2601,16 +3229,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>綦江区</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>綦江区</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造，包括配电柜、风机、污水提升泵、在线监测等设备的更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>上级补助和业主自筹，项目出资比例为100%，本项目工程总投资金额约1327.40万元</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>污水处理设施设备</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr">
         <is>
           <t>綦江区污水处理厂设施设备更新改造工程(二期)招标公告 1.招标条件 本招标项目 綦江区污水处理厂设施设备更新改造工程（二期） 已由 重庆市綦江区发展和改革委员会 以 重庆市企业投资备案证（项目代码：2502-500110-04-01-844057） 批准建设，项目业主为 重庆南州城市管 理服务有限公司 ，建设资金来自 上级补助和业主自筹 ，项目出资比例为 100% ，招标人为 重庆南州 城市管理服务有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审的最低 投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 綦江区 2.2 项目概况与建设规模：对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造， 务 包括配电柜、风机、污水提升泵、在线监测等设备更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污 水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。 2.3 本项目工程总投资金额： 约1327.40万元 商 2.4 招标范围： 本项目设计施工图和招标文件、答疑、补遗、工程量清单等资料所涉及的全部内容。 2.5 工期要求： 180日历天 道 缺陷责任期要求： 24个月 2.6 标段划分（如有）： / 管 2.7 其他： / 3.政府采购工程 国 3.1 是否属于政府采购工程：否 4.投标人资格要求 中 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（綦江区） （https://www.cqggzy.com/qijiangweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（綦江区）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间 从本公告发布至2026-08-22 18:00:00前。 5.3招标人应于2026-09-11 18:00:00前在重庆市公共资源交易网（綦江区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（綦江区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆南州城市管理服务有限公司 代理机构: 永卓国际工程技术有限公司 地 址: 重庆市綦江区红星美凯龙生活广场3幢19-3 地 址: 两江新区网泰山大道东段98号2幢10-12号 邮 编: 邮 编: 项目负责人: 赵老师 项目负责人: 廖淼 电 话: 023-48690537 电 话: 务023-60391733 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 商开户银行: 账 号: 账 号: 监督部门: 道 电 话: 2026年08月18日 綦江区污水处理厂设施设备更新改造工程（二期） 管 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051287453 中国农业银行股份有限公司重庆自由贸 重庆联合产权交易所集国团股份有限公司 312601010400083780000031123 易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146631326 信息来源:https://www.chinapipe.net/project/d3075589.html 中 cqdingjiu 2026.08.21 10:06:54</t>
@@ -2622,9 +3266,13 @@
         </is>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>重庆, 綦江区, 污水处理厂, 设施设备更新改造, 管材招标</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2657,16 +3305,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>南岸区</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>南岸区</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统，对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平台。</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>概算批复工程建安费2975.27万元。</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>农村供水管网、智慧加压泵站、水厂升级改造、智能控制系统、加药系统、金属防腐工程、入户管道、入户水表、监测计量基础设施。</t>
+        </is>
+      </c>
       <c r="M40" t="inlineStr">
         <is>
           <t>南岸区峡口、迎龙片区农村供水保障提升工程招标计划表 重庆市工程建设项目招标计划表 项目 南岸区峡口、迎龙片区农村供水保障提升工程 名称 招标 网 法人 或招 标人 重庆市江南城市建设发展（集团）有限公司 名称 务 （盖 章） 项目 批准 商 文件 南岸发改﹝2026﹞156号 及文 号 本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体 主要 化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统， 建设 对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平 内容 台。概算批复工程建安费2975.27万元。 管 拟 招 招标文 合同预 招标 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 国 所 南岸 重 区峡 庆 口、 中 市 迎龙 朱家岩水厂升级改造工程：对全厂老旧设备进行设备更新；对全 公 片区 公 厂进行智慧化改造，增加高级工艺控制系统；对厂区建筑和构筑 共 农村 开 1 物修缮；优化加药系统投加模式，增加精确加药系统；对全厂部 2026-08 资 1600.00 供水 招 分老旧管道进行更换；金属防腐工程，对金属设备和管道的防锈 源 保障 标 刷漆工作。 交 提升 招标 易 工程 项目 中 （一 心 标段） 南岸 重 区峡 庆 口、 市 迎龙 公 片区 管网工程：延伸、改造峡口镇、迎龙镇等4个乡镇 46 公里 公 共 农村 DN40~DN300 配水主支管，36公里 DN20入户管道，新建3座一体 开 2 2026-08 资 1300.00 供水 化智慧加压泵房，入户水表改造 1752 户，并配套建设监测计量 招 源 保障 基础设施。 标 交 提升 易 工程 中 （二 心 标段） 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075572.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
@@ -2678,9 +3342,13 @@
         </is>
       </c>
       <c r="O40" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>重庆, 农村供水保障提升工程, 管材招标, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2713,16 +3381,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>北碚区</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>北碚区</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水主要建设内容管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网附属设施。</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>合同预估金额为8457万元</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>供水管网</t>
+        </is>
+      </c>
       <c r="M41" t="inlineStr">
         <is>
           <t>北碚区东阳天府片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区东阳天府片区农村供水提升工程 招标法人或招 标人名称（盖 重庆北碚文旅产业发展有限公司 网 章） 项目批准文件 及文号 务 工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水 主要建设内容 管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网 附属设施。 招标项目名 招标内 招标方 招标文件计划 拟交易场 合同预估金 序号 商 备注 称 容 式 发布时间 所 额(万元) 北碚区东阳 招标项目 重庆市公 天府片区农 施工招 公开招 1 2026-08 共资源交 8457.00 村供水提升 标 道标 易中心 工程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075569.html 管 cqdingjiu 2026.08.21 10:06:55 国 中</t>
@@ -2734,9 +3418,13 @@
         </is>
       </c>
       <c r="O41" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 农村供水提升工程, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2769,16 +3457,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供水管网68.5km及其附属设施。</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>合同预估金额：8741.00万元</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>供水管网及相关附属设施</t>
+        </is>
+      </c>
       <c r="M42" t="inlineStr">
         <is>
           <t>北碚区澄江片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区澄江片区农村供水提升工程 招标法人或招标 重庆北碚文旅产业发展有限公司 人名称（盖章） 网 项目批准文件及 文号 改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供 主要建设内容 务 水管网68.5km及其附属设施。 招标项目名 招标文件计划 合同预估金 序号 招标内容 招标方式 拟交易场所 备注 称 发布时间 额(万元) 招标项目 北碚区澄江 商重庆市公共 1 片区农村供 施工招标 公开招标 2026-08 资源交易中 8741.00 水提升工程 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 道 信息来源:https://www.chinapipe.net/project/d3075568.html cqdingjiu 2026.08.21 10:06:55 管 国 中</t>
@@ -2790,9 +3486,13 @@
         </is>
       </c>
       <c r="O42" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 商机</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2807,7 +3507,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2825,16 +3525,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>主要改造及延伸配水管188.2千米，新建加压泵站4座，新建计量监测设施建设以及配套电气工程。</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>预算金额为3137.22万元</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>管道、加压泵站、计量监测设施、电气设备</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr">
         <is>
           <t>涪陵区江东街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区江东街道农村供水保障能力提升工程（二期） 名称 招标 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 项目 网 批准 文件 涪陵发改〔2026〕471号 及文 号 主要 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 建设 以及配套电气工程。 务 内容 招 标 合 文 同 招 件 预 招标 标 招标方 计 拟交易 备 序号 招标项目名商称 估 项目 内 式 划 场所 注 金额 容 发 (万 布 元) 时 间 重 道 庆 市 涪 陵 公 区 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 开 公 1 涪陵区江东街道农村供水保障能力提升工程（二期） 2026-09 3137.22 管以及配套电气工程。 招 共 标 资 源 交 易 中 心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075558.html cqdingjiu 2026.08.21 10:06:55 中</t>
@@ -2846,9 +3562,13 @@
         </is>
       </c>
       <c r="O43" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2863,7 +3583,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2881,16 +3601,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>改造荣桂水厂老化、破损、生锈的输水管道7.36公里。马武水厂增设废水回收及污泥浓缩系统1套。荣桂水厂增设废水回收及污泥浓缩系统1套。新建配水管道总长0.74公里；改造配水管道总长139.42公里。新建1座微型集成泵房及改造1座泵站(原牌坊泵站)。新增管网监测设施40套。</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>预估合同金额为3236.36万元人民币</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>输水管道、废水回收及污泥浓缩系统、配水管道、微型集成泵房、泵站、管网监测设施</t>
+        </is>
+      </c>
       <c r="M44" t="inlineStr">
         <is>
           <t>涪陵区龙桥街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 涪陵区龙桥街道农村供水保障能力 项目名称 提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水 名称（盖 有限公司 章） 网 项目批准 文件及文 涪陵发改〔2026〕466号 号 改造荣桂水厂老化、破损、生锈的 务 输水管道7.36公里。马武水厂增设 废水回收及污泥浓缩系统1套。荣 桂水厂增设废水回收及污泥浓缩系 主要建设 统1套。新建配水管道总长0.74公里； 商 内容 改造配水管道总长139.42公里。新 建1座微型集成泵房及改造1座泵 站(原牌坊泵站)。新增管网监测设 施40套。 道 招标 合同 招 文件 预估 标 招标方 拟交易 备 招标项目 序号 招标项目名称 计划 金 内 式 场所 注 管 发布 额(万 容 时间 元) 改造荣桂水厂老化、 破损、生锈的输水管 国 道7.36公里。马武水厂 增设废水回收及污泥 重庆 浓缩系统1套。荣桂水 市涪 厂增设废水回收及污 公 陵区 中 涪陵区龙桥街道农村供水保障能力 泥浓缩系统1套。新建 开 1 2026-09 公共 3236.36 提升工程 配水管道总长0.74公里； 招 资源 改造配水管道总 标 交易 长139.42公里。新建1 中心 座微型集成泵房及改 造1座泵站(原牌坊泵 站)。新增管网监测设 施40套。 本计划表所列招标项目信息均为暂 备注 定，最终以实际招标时的信 信息来源:https://www.chinapipe.net/project/d3075556.html cqdingjiu 2026.08.21 10:06:55</t>
@@ -2902,9 +3638,13 @@
         </is>
       </c>
       <c r="O44" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>涪陵区龙桥街道, 农村供水保障能力提升工程, 输水管道, 废水回收及污泥浓缩系统, 配水管道, 微型集成泵房, 泵站, 管网监测设施</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2919,7 +3659,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2937,16 +3677,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>整治De315原水管长1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>合同金额1489.90万元</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>管材、水泵、加压泵站、废水处理系统、电气工程</t>
+        </is>
+      </c>
       <c r="M45" t="inlineStr">
         <is>
           <t>涪陵区百胜镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区百胜镇农村供水保障能力提升工程 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕465号 及文 号 务 主要 建设整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。 内容 招 拟 标 招招标文 合同预 交 序项 标件计划 估金 备 招标内容 易 号目 方发布时 额(万 注 场 名 商 式间 所 元) 称 涪 陵 区 重 百 庆 胜 市 招标 镇 涪 项目 农 道 陵 村 公 区 供整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1开 公 1 2026-09 1489.90 水套及配套电气工程。 招 共 保 标 资 障 源 能 交 力 易 提 中 管 升 心 工 程 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075553.html 国 cqdingjiu 2026.08.21 10:06:55 中</t>
@@ -2958,9 +3706,13 @@
         </is>
       </c>
       <c r="O45" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>涪陵区百胜镇, 农村供水保障能力提升工程, 管材招标, 重庆</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2993,16 +3745,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>对清溪水厂原取水口进行改造。改造清溪厂输水管道长6.38公里。清溪水厂新建3000m³/d集成水厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04公里。四合村泵站增加1套备用加压泵。新增管网监测设施35套。</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>合同预估金额：2888.89万元</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>集成水厂、输水管道、配水管道、加压泵、管网监测设施</t>
+        </is>
+      </c>
       <c r="M46" t="inlineStr">
         <is>
           <t>涪陵区清溪镇农村供水保障能力提升工程招标计划 重庆市工程建设项目招标计划表 项目名称 涪陵区清溪镇农村供水保障能力提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕467号 务 号 对清溪水厂原取水口进行改造。改造清溪水厂输水管道长6.38公里。清溪水厂新建3000m3/d集成水 主要建设 厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04 内容 公里。四合村泵站增加1套备用加压泵。新商增管网监测设施35套。 招标项目 招标方 招标文件计 拟交易场 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 所 (万元) 对清溪水厂原道取水口进行 改造。改造清溪水厂输水 管道长6.38公里。清溪水厂 涪陵区清 新建3000m3/d集成水厂1套， 重庆市涪 招标项目 溪镇农村 增设废水回收及污泥浓缩 公开招 陵区公共 管 1 供水保障 2026-09 2888.89 系统1套。新建配水管道总 标 资源交易 能力提升 长2.46公里。改造配水管道 中心 工程 总长145.04公里。四合村泵 站增加1套备用加压泵。新 国 增管网监测设施35套。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075552.html 中 cqdingjiu 2026.08.21 10:06:55</t>
@@ -3014,9 +3782,13 @@
         </is>
       </c>
       <c r="O46" t="n">
-        <v>0</v>
-      </c>
-      <c r="P46" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3031,7 +3803,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3049,16 +3821,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>改造11000m³/d(旺水垭6000m³/d和二水厂5000m³/d)原水处理系统及辅助设施，主要包括加氯系统、加药系统、清水池、絮凝池、重力无阀滤池、污水处理回收池、二水厂泵房设备等及其他辅助设施。更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km，新建应急泵站至百汇大桥配水管9km；百汇至观将泵站4.5km；共计37.3km。</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>合同预估金额3427.27万元</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>管材</t>
+        </is>
+      </c>
       <c r="M47" t="inlineStr">
         <is>
           <t>涪陵区珍溪镇农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区珍溪镇农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕476号 及文号 (一)改造11000m3/d(旺水垭6000m3/d和二水厂5000m3/d)原水处理系统及辅助设施，主要有加氯系统、 加药系统、清水池、絮凝池、重力无阀滤池、商污水处理回收池、二水厂泵房设备等及其他辅助设施。 主要建 (二)更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪 设内容 湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km， 新建应急泵站至百汇大桥配水管9km：百汇至观将泵站4.5km；共计37.3km。 道 招标项目 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 场所 (万元) (一)改造11000m3/d(旺水 垭6000m3/d和二水厂5000m3/d) 管 原水处理系统及辅助设施，主 要有加氯系统、加药系统、清 水池、絮凝池、重力无阀滤池、 污水处理回收池、二水厂泵房 涪陵国区珍 设备等及其他辅助设施。(二) 重庆市 招标项 溪镇农村 更换旺水垭水厂至张家塘配水 涪陵区 目 供水保障 公开招 1 管13.5km，张家塘至滴水配水 2026-09 公共资 3427.27 能力提升 标 管长3.3km，全长16.8km；滴水 源交易 中工程（一 至洪湖配水管长0.3km；更换八 中心 期） 一水库至旺水垭水厂引水 管1.7km，更换珍溪二水厂至珍 溪大桥配水管5km，新建应急 泵站至百汇大桥配水管9km： 百汇至观将泵站4.5km；共 计37.3km。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075551.html cqdingjiu 2026.08.21 10:06:56</t>
@@ -3070,9 +3858,13 @@
         </is>
       </c>
       <c r="O47" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 供水, 改造</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3087,7 +3879,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3105,16 +3897,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>新建及整治输配水管网总长124.26千米，新建加压泵站5座，新建高位水箱4座（总容积354立方米），武陵山水厂新建废水处理系统1套及配套电气工程等。</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>合同预估金额1861.77万元</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>输配水管网、加压泵站、高位水箱、废水处理系统、电气工程</t>
+        </is>
+      </c>
       <c r="M48" t="inlineStr">
         <is>
           <t>涪陵区武陵山镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区武陵山镇农村供水保障能力提升工程 名称 招标 网 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 务 （盖 章） 项目 批准 商 文件 涪陵发改〔2026〕468号 及文 号 主要 道 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高位水箱4座（总容积 354立方米），武 建设 陵山水厂新建废水处理系统1套及配套电气工程等。 内容 招 管 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 国 称 涪 陵 区 中 重 武 庆 陵 市 山 招标 涪 镇 项目 陵 农 公 区 村 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高 开 公 1 供 位水箱4座（总容积 354立方米），武陵山水厂新建废水处理系统1套 2026-09 1861.77 招 共 水 及配套电气工程等。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075549.html cqdingjiu 2026.08.21 10:06:56</t>
@@ -3126,9 +3934,13 @@
         </is>
       </c>
       <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>涪陵区武陵山镇, 农村供水保障能力提升工程, 重庆, 输配水管网, 加压泵站, 高位水箱, 废水处理系统, 电气工程</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3143,7 +3955,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3161,16 +3973,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>建设配水管网总长34.80km，新建加压泵站2座、改造已成泵站2座、新建加氯加药间1座、新建高位水箱7座、新建计量监测设施以及配套电气工程。</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>合同预估金额3503.77万元</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>配水管网、加压泵站、加氯加药间、高位水箱、计量监测设施、电气工程</t>
+        </is>
+      </c>
       <c r="M49" t="inlineStr">
         <is>
           <t>涪陵区江东街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区江东街道农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕470 号 及文号 主要建 建设配水管网总长 34.80km，新建加压泵站 2 座、改造已成泵站 2 座、新建加氯加药间 1 座、新建高位 设内容 水箱 7 座、新建计量监测设施以及配套电气工程商。 招 招标文件 拟交 合同预估 序 招标项 标 备 招标内容 计划发布 易场 金额(万 号 目名称 方 注 道 时间 所 元) 式 涪陵区 重庆 招标项 江东街 市涪 目 建设配水管网总长 34.80km，新建加压泵站 2 座、 公 道农村 陵区 管 改造已成泵站 2 座、新建加氯加药间 1 座、新建高 开 1 供水保 2026-09 公共 3503.77 位水箱 7 座、新建计量监测设施以及配套电气工 招 障能力 资源 程。 标 提升工程 交易 （一期） 中心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075548.html cqdingjiu 20中26.08.21 10:06:56</t>
@@ -3182,9 +4010,13 @@
         </is>
       </c>
       <c r="O49" t="n">
-        <v>0</v>
-      </c>
-      <c r="P49" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>重庆, 农村供水保障能力提升工程, 配水管网, 加压泵站, 加氯加药间, 高位水箱, 计量监测设施, 电气工程</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3217,16 +4049,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>详见附件。</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>内外涂环氧消防复合钢管管件</t>
+        </is>
+      </c>
       <c r="M50" t="inlineStr">
         <is>
           <t>中国电建水电五局二公司重庆轨道交通17号线一期7标内外涂环氧消防复合钢管管件采购项目公开竞价采购(二次 挂网)变更公告(一) 详见附件。 信息来源:https://www.chinapipe.net/project/d3075376.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
@@ -3238,9 +4078,13 @@
         </is>
       </c>
       <c r="O50" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3273,16 +4117,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>本次修复选择开挖换管：开挖约80米，2孔110波纹管、2孔蜂窝管，新建两通信手控井。</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>项目资金已落实。</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>通信管道</t>
+        </is>
+      </c>
       <c r="M51" t="inlineStr">
         <is>
           <t>2026年石柱分公司黄水镇黄连大道通信管道建设招标公告 ZB_ZHAOBIAOGONGGAO_START 本询比项目为 2026年石柱分公司黄水镇黄连大道通信管道建设 （标段 编号： CQBBFA202604170051 ），采购人为 中国电信股份有限公司石柱分公司 ，采购代理机构为 。项目 资金已落实。 具备采购条件，现进行公开询比，特邀请有意向的且具有提供标的物能力的潜在供应商（以下简 称供应商）参加询比响应。 1.项目概况与采购内容 1.1项目概况： 2026年石柱分公司黄水黄连大道通信管道修复项目主要针对黄水网黄连大道受损通信管道进行修 复80米 本次集中询比合同有效期为： 2026.9-2026.12 1.2采购内容 及标包划分情况： 务 1.2.1 本次询比的规模、货物名称、数量及主要技术参数、交货期及交货地点具体如下：黄水镇黄连大道80米通 信管道修复。 序号 标包名称 产品名称 规格型号 数量 交货地点 交货期 商 2026年石柱分公司黄水 黄水镇黄连 1 镇黄连大道通信管道建 管道建设 新建2孔110波纹管、 新建2孔蜂窝管 80 2026.12.20 大道 设 道 本项目 不划分标包 。 ${ } ${ 本项目允许供应商同时成交的最多标包数为 0 个。 } 本项目将按照最新的《中国电信供应商不良行为管 理规则》执行供应商不良行为处理结果，请重点关注处理结果适用的供应商主体、被处理产品、处理范围、禁 限期、处理措施等关键内容，请务必登录中国电信阳光采购网（https://caigou.chinatelecom.com.cn）查阅《中国 管 电信供应商不良行为管理规则》。 本项目根据《中国电信供应商不良行为管理规则》选择适用备选处理措施 （但涉及生产安全责任事故的处理结果不适用备选措施）。 1.2.2成交供应商数量： 1 个，每个成交供应商对应的份额如下 ： [请在此处自行编辑与采购方案相同的成交原则] 国 ${ 1.2.2成交供应商数量如下： [ 请在此处自行编辑与采购方案相同的有效供应商及成交供应商数量原则相关表格 ] 每个成交供应商对应的份额如下: [请在此处自行编辑与采购方案相同的份额分配原则] } 1.3本项目 设置最高 响应限价 。 设置最高响应限价，最高响应限价为不含税31000元人民币/计算方法，供应商响应报价高于最高 响应限价的，其响应将被否决 供应商响应报价高于最高响应限价的，其响应 将被否决。 ${ } 2.供应商中资格要求 2.1供应商基本资格要求 2.1.1 供应商 应为 中华人民共和国境内 法律上和财务上独立的法人或依法登记注册的其他组织，合法运作并 独立于采购人和采购代理机构。 供应商应具有良好的银行资信和商业信誉。法人下属不具备法人资格的分支机 构参与响应的，应提供所属法人针对本项目或覆盖本项目的经营事项的有效授权。 2.1.2 供应商 的法定代表人或负责人为同一人或者存在控股、管理关系的不同 供应商 ，不得参加同一标包响应或 者未划分标包的同一询比项目响应。 ${ 2.1.3 } ${ 2.1.3 } 2.1.4 本次询比 不接受 联合体响应。 ${如 供应商 为联合体，应满足下列要求： （1） 联合体各方必须按询比文件提供的格式签订联合体协议书，明确联合体牵头人和各方的权利义务； （2）由同一 专业的单位组成的联合体，按照资质等级较低的单位确定资质等级； （3）联合体各方不得再以自己名义单独或 加入其他联合体在同一标包或者未划分标包的同一询比项目中响应。 ${ （4） 。} } 2.1.5 本次询比 不接受代理商响应。 ${ （1）产品制造商注册地在中华人民共和国境外（与中华人民共和国有正常贸易与往来的国家或地区）及香港、 澳门、台湾地区且必须使用代理商响应和签订销售合同的；（2）产品制造商为注册地在中华人民共和国境内的 外资企业（包括香港、澳门、台湾地区资本）或者由外国投资者（包括香港、澳门、台湾地区）享有绝对控制权 （最大或最多表决权）的企业且必须使用代理商响应和签订销售合同的。代理商响应的，应满足下列要求 ： } ${ （1） ${ （2） 供应商与产品制造商 的代理合作关系迄今为止应已持续 0 年（含）以上。 } ${ （3） } } ${ 2.1.6 与供应商有产品代工制造关系的制造商不得参加同一标包响应或者未划分标包的同一询比项目响 应。 } 2.1.7 供应商须提供2022年1月1日至本项目发布公告之日的同类项目（通信管道施工类）证明材料， 合同累计金额不低于3万元（含税） 2.2供应商不得存在下列情形之一 （1） 为采购人不具有独立法人资格的附属机构（单位）； （2） 被依法暂停或取消 投标/ 响应资格的； （3） 被责令停产停业、暂扣或者吊销许可证、暂扣或者吊销执照； （4） 进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （5） 在最近三年内（自 2022年04月01日 起）被相关行业主管部门或司法机关认定有骗取 中标/成交 、严重 违约、重大工程质量或者安全问题的； 网 （6） 在最近五年内（自 2022年06月01日 起）被判处单位行贿罪，且行贿行为与采购活动相关的（以“中国 裁判文书网”的生效判决为准）； （7） 在最近五年内（自 2022年06月01日 起）被判处合同诈骗罪的（以“中国裁判文书网”的生效判决为 务 准）； （8） 被最高人民法院在“信用中国”网站（www.creditchina.gov.cn）或各级信用信息共享平台中列入失信被执 行人名单，已执行完毕或不再执行的除外； 商 （9） 为本询比项目提供过设计、编制技术规范和其他文件的咨询服务 ； （10） 为本工程项目的相关监理人，或者与本工程项目的相关监理人存在隶属关系或者其他利害关系； 道 （11） 为本询比项目的代建人 ； （12） 为本询比项目的采购代理机构 ； 管 （13） 与本询比项目的监理人或代建人或采购代理机构同为一个法定代表人 ； （14） 与本询比项目的监理人或代建人或采购代理机构存在控股或参股关系 ； （15） 被工商行政管理国机关在国家企业信用信息公示系统中列入严重违法失信企业名单的； （16） 中国电信在职员工违规担任供应商法定代表人并参与采购活动的； （17） 中国电信集团有限公司/中国电信股份有限公司中层及以上管理人员违反有关领导人员配偶、子女及其配 中 偶经商办企业行为管理规定，其配偶、子女及其配偶经商办企业参与采购活动的； （18） 中国电信领导人员离职或退休后三年内违反《国有企业领导人员廉洁从业若干规定》等相关规定任职、 投资入股的私营企业、外资企业和中介机构，参与其原任职单位采购活动的； ${ （19） } （19） 其他按照中国电信供应商不良行为处理结果及《中国电信供应商不良行为管理规则》的结 果执行规则，应对供应商及其响应产品在本项目中执行禁止采购处理措施的； （20） 法律法规、询比文件限定的其他情形。 ${ 供应商 是代理商的，本条所指的 供应商 也包括其所代理的制造商。 } ${ 联合体响应的，联合体成员均不得 存在上述任一情形。 } 2.3产品资格要求 2.3.1 产品 应是来自中华人民共和国 ${或是与中华人民共和国有正常贸易与往来的国家或地区} 的 成熟稳定的 产品 。 ${ 2.3.2 产品 。 } ${ 2.3.3 产品 。 } ${ 2.3.4 。 } ${ 2.3.5 。 } 2.3.6 产品应符合中国电信相关技术要求， 并满足以下关键技术指标： （1） 序号 技术指标 具体要求 1 开挖深度 埋深≥0.8m（道路≥1.2m） 2 施工规格 本次修复选择开挖换管：开挖约80米，2孔110波纹管、2孔蜂窝管，新建两通信手控井 ${ 2.3.7 产品 业绩要求： 。 } ${ 2.3.8 。 } ${ 2.4 产品制造商资格要求 2.4.1 制造商应提供合法有效的登记 （或注册）证明文件，应具有良好的银行资信和商业信誉。 } ${ 2.4.2 } ${ 2.4.2 } ${ 2.4.3 } ${ 2.4.4 } ${ 2.4.5 } ${ 2.5现场考察 } ${ 2.6评价检测 } 2.7 法律法规规定的其他要求。 3.资格审查方法 本项目将进行资格后审，资格审查标准和内容见询比文件第三章“评审办法”，凡未通过资格后审的供应商， 其响应将被否决 。 网 4.询比文件的获取 4.1询比文件获取时间: 2026年08月25日 00时00分00秒 至 2026年09月01日 00时00分00秒 （北京时间，下同）。 4.2询比文件获取方式：登录“中国电信阳光采购网（https://caigou.c务hinatelecom.com.cn）”后，通过“招投标-采 购文件领取”模块或通过“电子采购入口”跳转中国电信电子采购系统，进入本项目进行询比文件登记申领， 未在系统注册的供应商须先进行注册，注册方法详见本公告“ 7 供应商注册”。 4.3询比文件费用： 本项目不收取文件费用。 ${每套售价商 0 元人民币，售后不退。支付要求： } 5.响应文件的递交 5.1响应文件递交截止时间（即响应截止时间）为： 2026年09月02日 00时00分00秒 道 5.2 电子响应文件的提交方式：登录中国电信阳光采购网（https://caigou.chinatelecom.com.cn）后，通过“招投 标-我的项目”模块或通过“电子采购入口”跳转中国电信电子采购系统，选择本项目进行响应文件提交，供应 商应在响应文件提交截止时间之前通过电子采购系统完成加密电子响应文件的上传。供应商未在电子采购系统 进行询比文件申领登记或电子响应管文件未按照要求加密的，将无法通过电子采购系统提交电子响应文件 。 5.3 本项目将于响应文件提交截止同一时间通过中国电信电子采购系统开启响应文件， 采购人/采购代理机构 邀 请响应供应商的法定代表人或者其委托代理人准时参加 。 国 ${ 6.样品的递交 6.1样品递交的时间、地点：于 递交至 。 } 7. 供应商注册 7.1 中国电信阳光采购网注册 未注册过的潜在供应商，须通过中国电信阳光采购网（https://caigou.chinatelecom.com.cn）首页“立即注册”模 中 块完成注册后，方可申领本项目询比文件。 7.2 CA证书办理 参加询比响应的潜在供应商须提前办理CA证书，并确保CA证书在使用时有效。CA证书办理流程详见中国电信 阳光采购网首页“操作指引-CA办理”。 7.3 技术支撑联系方式 服务热线：4000111884 服务邮箱：zb_support@chinatelecom.cn（电子采购系统技术支撑） ctsc@chinatelecom.cn（CA证书办理技术支撑） 8. 发布公告的媒介 本询比公告在 中国电信阳光采购网（https://caigou.chinatelecom.com.cn） 、中国招标投标公共服务平台 （http://www.cebpubservice.com/） 上发布，其他媒介转载无效。 9. 联系及异议接收方式 9.1 联系方式 采 购 人: 中国电信股份有限公司石柱分公司 采购代理机构: 地 址： 重庆市石柱县城南路6号 地 址： 无 邮 编： 邮 编： 无 联 系 人： 马卫平 联 系 人： 无 电 话： 17365204567 电 话： 无 电子邮件： 17365204567@189.cn 电子邮件： 无 网 址： www.chinatelecom.com.cn或“/” 网 址： 无 网 开户银行： 无 账 号： 无 9.2 异议接收方式 务 登录中国电信阳光采购网（https://caigou.chinatelecom.com.cn）后，通过“招投标-采购异议-提出异议”模块提出。 采购代理机构： 商 2026年08月25日 信息来源:https://www.chinapipe.net/project/d30道75344.html cqdingjiu 2026.08.21 10:06:56 管 国 中</t>
@@ -3296,7 +4148,11 @@
       <c r="O51" t="n">
         <v>0</v>
       </c>
-      <c r="P51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3329,16 +4185,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>重庆站站房CQZSG-4标项目蓝色PVC袖阀管(外径60mm)询价采购公告</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>蓝色PVC袖阀管，外径60mm，壁厚4.5-5mm PVC管</t>
+        </is>
+      </c>
       <c r="M52" t="inlineStr">
         <is>
           <t>重庆站站房CQZSG-4标项目蓝色PVC袖阀管(外径60mm)询价采购公告 ZTEJWZ-JZ-2026-询027（一） 采购单位:重庆站站房CQZSG-4标段项目经理部 发布时间:2026-08-18 19:06 报价截止时间:2026-08-21 10:00 招标方联系人:刘健 网 招标方联系电话:13540650091 招标方邮箱: 务 监督方联系人:纪委 监督方联系电话:028-87653066 商 监督方邮箱: 保证金:0.0元 道 结算与发票信息: 结算方式：上月21日至本月的20日为一个结算周期，当月20日为本月的结算截止日期。结算时根据甲方检验合格 及双方共同签认的凭证计算当月实际收货数量。 管 支付条件：结算完成后，甲方在收到乙方开具的正式的增值税专用发票后第1个月支付该批物资结算金额的70%， 第12个月支付20%，剩余10%在第18-24月内按月均衡支付。 发票种类：增值税专用国发票 发票抬头：中铁二局集团有限公司 税号：9151中0100MA61RKR7X3 其他要求： 交货信息: 交货方式:点数验收 收货人:刘健 收货人联系方式:13540650091 其他说明事项: 流水号：询2026081800458 交 标的 规格 计量 标的编号 数量 技术标准及要求 货 送货地址 名称 型号 单位 期 蓝色PVC袖阀管，外 西南区-重庆市-市辖区-渝中区-重 袖阀 径60mm，壁 庆市菜园坝立交以西，龙家湾隧道 0950999183764 - 23188.0 米 管 厚4.5-5mm PVC管，承压 以东，菜袁路以北，王家坡以南的 不小于5MPa,节长4m 地块内，原重庆站。 报价网址:http://www.crecgec.com 信息来源:https://www.chinapipe.net/project/d3075317.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
@@ -3350,9 +4214,13 @@
         </is>
       </c>
       <c r="O52" t="n">
-        <v>0</v>
-      </c>
-      <c r="P52" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3385,16 +4253,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>新建、更换配水管网396.72km（dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>合同金额：3611.91万元</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管</t>
+        </is>
+      </c>
       <c r="M53" t="inlineStr">
         <is>
           <t>涪陵区蔺市街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（一期） 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕474号 及文 号 主要 务 建设新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。 内容 拟 招招标文 合同预 招标 交 序 标件计划 估金 备 项目招标内容 易 号 方发布时 额(万 注 名称 场 式间 元) 所 商 重 庆 涪陵 市 区蔺 招标 市街 涪 项目 道农 陵 公 区 村供 新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收 开 公 1 水保 2026-09 3611.91 及污泥浓缩处理系统。 招 共 障能 道 标 资 力提 源 升工程 交 （一 易 期） 中 心 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075278.html 管 cqdingjiu 2026.08.21 10:06:57 国 中</t>
@@ -3406,9 +4290,13 @@
         </is>
       </c>
       <c r="O53" t="n">
-        <v>0</v>
-      </c>
-      <c r="P53" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 商机</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3441,16 +4329,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>改造李渡街道15个村（社区）配水主支管道，更换配水主管网193.71千米（DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治3座，新建测控井78座。</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>项目批准文件：涪陵发改[2026]469号</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管</t>
+        </is>
+      </c>
       <c r="M54" t="inlineStr">
         <is>
           <t>涪陵区李渡街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区李渡街道农村供水保障能力提升工程 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕469号 及文 号 商 主要 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套 建设 附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建测控井78座。 内容 招 拟 标 道 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 管 涪 陵 区 重 李 庆 渡 市 街 国 招标 涪 道 项目 陵 农 公 区 村 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂 开 公 1 供 塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建 2026-09 2372.74 招 共 水中测控井78座。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075277.html cqdingjiu 2026.08.21 10:06:57</t>
@@ -3462,9 +4366,13 @@
         </is>
       </c>
       <c r="O54" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 改造, 配水主支管道, 更换配水主管网, 抗菌耐磨涂塑钢管, PE管, 泵站改造, 集成泵站, 蓄水池整治, 测控井</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3497,16 +4405,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管主要建设有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>合同预估金额为2182.77万元</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>PE管、衬塑钢管、水泵、不锈钢水箱、减压阀、排污阀</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
           <t>涪陵区珍溪镇农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目名称 涪陵区珍溪镇农村供水保障能力提升工程（二期） 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕477号 务 号 (一)本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管 主要建设 有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵 内容 站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水 箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。 招标项目名 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 称 式 划发布时间 场所 (万元) 道 (一)本项目对珍溪镇23个 村(社区)安装配水管网660km 及配套附属设施，其 中：1.De160~De40的PE管 管 有232km；2.连接各村社 涪陵区珍溪 重庆市 的De32~De20的PE管有381km； 招标项目 镇农村供水 涪陵区 3.219~32的衬塑钢 公开招 1 保障能力提 2026-09 公共资 2182.77 管47km。(二)购置安装泵 标 升工国程（二 源交易 站14座(一用一备共计28台水 期） 中心 泵)，其中新建泵站10座、更 换泵站4座及配套电力设施; 新建不锈钢水箱2座等。(三) 中 购置安装(0~25kg)减压阀61 个;排污阀(25kg）3个。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075275.html cqdingjiu 2026.08.21 10:06:57</t>
@@ -3518,9 +4442,13 @@
         </is>
       </c>
       <c r="O55" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>涪陵区, 珍溪镇, 农村供水, 提升工程, PE管, 衬塑钢管, 水泵, 不锈钢水箱, 减压阀, 排污阀</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3553,16 +4481,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长105.307km（dn20-dn40PE管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建1座改造3座；新建测控井52座。</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>合同预估金额：2652.89万元</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>净水设备、PE管、抗菌耐磨涂塑钢管</t>
+        </is>
+      </c>
       <c r="M56" t="inlineStr">
         <is>
           <t>涪陵区蔺市街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（二期） 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕475号 及文 号 商 主要 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 105.307km（dn20-dn40PE 建设 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座；新建测控井 52座。 内容 拟 招 招标文 合同预 招标 交 序 道 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 重 庆 涪陵 管 市 区蔺 涪 招标 市街 陵 项目 道农 公 区 村供 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 开 公 1 水保 105.307km（dn20-dn40PE 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座； 2026-09 2652.89 国 招 共 障能 新建测控井 52座。 标 资 力提 源 升工程 交 （二 易 期） 中 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075274.html cqdingjiu 2026.08.21 10:06:57</t>
@@ -3574,9 +4518,13 @@
         </is>
       </c>
       <c r="O56" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3609,16 +4557,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1，该管道为自流管道，位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水厂的正常收水及运行，需对该段管道进行改造。</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>项目资金来自企业自筹</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>DN600混凝土管，检查井</t>
+        </is>
+      </c>
       <c r="M57" t="inlineStr">
         <is>
           <t>重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目项目公告 重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称）比选公告 1.比选条件 本比选项目重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称），比选人为重庆市排 网 水有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。中标后合同与重庆市豪洋水务 建设管理有限公司签订。现对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 2.项目概况与比选范围 务 2.1 建设地点：重庆市巴南区 2.2 项目概况：本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1,该管道为自流管道， 位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道 为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现 象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水 厂的正常收水及运行，需对该段管道进行改造。 道 2.3 比选范围：拆除现状管道为DN600混凝土管，同时需拆除并新建9座检查井。 2.4 工期要求：30日历天，以甲方通知进场时间为准。 管 2.5缺陷责任期要求：24个月 3.投标人资格要求 国 3.1 本次比选要求投标人须具备以下条件： 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质。 中 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 项内容。 3.2 本次比选接受不联合体投标。 4.比选文件的获取 4.1 投标人于2026年8月 18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子 版，以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都 视为投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的 一切后果由投标人自行负责。各投标单位应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行供应商注册，填写相关信息，审批过后成为 平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价、递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，将被否决投标。 4.4 比选文件每份售价800元，售后不退。投标单位在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标 文件。 5.投标文件的递交 5.1 电子投标文件递交时间：2026年8月24日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月24日14时00分至14时30分（北京时间），地点：重庆水务招标采购中心 （重庆市两江新区嘉华路36号重庆水务大厦5楼）。 5.3 投标截止时间：2026年 8月24日14时30分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆市排水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝中区长江滨江路126号 地 址：重庆市两江新区嘉华路36号重庆水务大厦 道 联 系 人： 黄老师 联 系 人： 黄晓华 电 话： 023-67767416 电 话： 18523396416 管 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3075272.html 国 cqdingjiu 2026.08.21 10:06:57 中</t>
@@ -3630,9 +4586,13 @@
         </is>
       </c>
       <c r="O57" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>重庆, 排水公司, 污水处理厂, 管网改造, DN600混凝土管, 检查井</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3665,16 +4625,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>潼南区</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>潼南区</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>改建潼南城区输水主管网约39.63km及配套相应阀门阀件等，对城区供水管网上商老旧阀门阀件、设施设备进行更换，合理增设部分计量及压力监控、水质监控等。</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>合同预估金额：918.00万元</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>城区配套阀门阀件改造工程</t>
+        </is>
+      </c>
       <c r="M58" t="inlineStr">
         <is>
           <t>重庆市潼南城区老旧供水管网改造工程招标计划 重庆市工程建设项目招标计划表 项目名称 重庆市潼南城区老旧供水管网改造工程 招标法人或招 标人名称（盖 重庆市潼南自来水有限公司 网 章） 项目批准文件 及文号 务 主要建设内容 改建潼南城区输水主管网约39.63km及配套相应阀门阀件等 招标方 招标文件计 拟交易场 合同预估 序号 招标项目名称 招标内容 备注 式 划发布时间 所 金额(万元) 对城区供水管网上商 重庆市潼南城 老旧阀门阀件、设 区老旧供水管 重庆市潼 招标项目 施设备进行更换， 网改造工程 公开招 南区公共 1 保障供水管网稳定 2026-09 918.00 （城区配套阀 标 资源交易 运行合道理增设部分 门阀件改造工 中心 计量及压力监控、 程） 水质监控等。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3075266.html cqdingjiu 2026.08.21 10:06:58 国 中</t>
@@ -3686,9 +4662,13 @@
         </is>
       </c>
       <c r="O58" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3721,16 +4701,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>开州区</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>开州区</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>该项目涉及硬化生产便道、建设防旱池和蓄水池、建造育苗大棚和小棚、安装水源处理和水肥一体化设施、新建设备管理房以及完善蔬菜基地配套设施等内容。</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>工程总投资335万元。</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>工程设计服务</t>
+        </is>
+      </c>
       <c r="M59" t="inlineStr">
         <is>
           <t>关于为【重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购】公开选取【工程设计】 机构的公告 我单位在重庆市网上中介超市公开选取工程设计中介服务机构，现将相关事项公告如下： 该项目为直接选取项目，由采购人从报名的中介服务机构中直接选定一家中介服务机构进行项目服务。 项目 重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购 名称 网 采购 重庆市开州区河堰镇人民政府 人 投资 审批 否 务 项目 是否 破产 商 业务 否 服务 项目 采购 道 所需 中介 其他 服务 事项 管 所需 服务 工程设计 类型 项目实施地点为国河堰镇清泉社区，项目建设内容为：硬化2米宽生产便道5.5千米，100方防旱池1口，50方 服务 蓄水池1口，标准自动化育苗大棚1个，蔬菜小棚20个，水源处理设施1套，水肥一体化配套设施1套，新 内容 建50平方米设备管理房，完善蔬菜基地配套设施等。工程总投资335万元。选取此项目设计单位（含预算 编制服务）。 中 中介 机构 资质（资格）要求 要求 资质 （资 1、报名单位提供有效的营业执照，资质证书（资质丙级或丙级以上），具备从事项目设计服务工作； 2、 格） 具有独立承担民事责任的能力； 3、具有良好的商业信誉和健全的财务会计制度； 4、具有履行合同所必 要求 需的专业技术能力； 5、有依法缴纳税收和社会保障资金的良好记录。 说明 其他 要求 无 说明 服务 时限 无要求，按照合同双方自行约定 说明 服务 3.1%费率 金额 金额 按文件要求执行 说明 选取 直接选取 方式 需规 避机 构 规避 原因 选取 2026-08-20 16:00:00 （选取时间到达后不接受报名，建议中介机构至少在选取开始半小时前完成报名。） 时间 采购 人业 网 务咨 重庆市开州区河堰镇人民政府（18716685679） 询电 话 采购 务 需求 26清泉社区项目设计服务采购说明.pdf 书下 载 商 2026-08-18 信息来源:https://www.chinapipe.net/project/d3075198.html 道 cqdingjiu 2026.08.21 10:06:58 管 国 中</t>
@@ -3742,9 +4738,13 @@
         </is>
       </c>
       <c r="O59" t="n">
-        <v>0</v>
-      </c>
-      <c r="P59" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3777,16 +4777,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>开州区</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>开州区</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米，务周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>项目总投资金额：500万元，本次招标项目合同估算金额：446.278921万元</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>柑橘基地改造提升项目</t>
+        </is>
+      </c>
       <c r="M60" t="inlineStr">
         <is>
           <t>重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目招标公告 1.招标条件 本招标项目重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目已由重庆市开州区发展和改革委员会以开州 发改审〔2026〕357号批准建设，项目业主为重庆市开州区长沙镇人民政府，建设资金来自开州区2026年中央和 市级提前批财政衔接推进乡村振兴补助资金，项目出资比例为 100% ，招标人为重庆市开州区长沙镇人民 政府。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：开州区长沙镇桔香村 2.2 项目概况与建设规模：1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输 线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米， 务 周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。 2.3 本项目工程总投资金额： 500万元 本次招标项目合同估算金额： 446.278921万元 商 2.4 招标范围：招标人发布的由重庆中煜华资工程技术有限公司设计的《重庆市开州区2026年长沙镇桔香村柑橘 基地改造提升项目》施工图及图纸说明、招标文件(含补遗)及工程量清单、答疑资料、澄清资料范围内所涉及的 工作内容，具体以招标人发布的工程量清单及道施工图为准。 2.5 工期要求： 150日历天 缺陷责任期要求： 12个月 管 2.6 标段划分（如有）： / 2.7 其他： / 国 3.政府采购工程 3.1 是否属于政府采购工程：是 中 3.2 是否专门面向中小企业预留：否，按照《政府采购促进中小企业发展管理办法》第六条第(三)“按照本办法 规定预留采购份额 无法确保充分供应、充分竞争，或者存在可能影响政府采购目标实现的情形”的规定，故本 项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包叁级及以 上资质或市政公用工程施工总承包叁级及以上资质或水利水电工程施工总承包叁级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）下载招 标文件、工程量清单、电子图纸等资料。参与投标的投标人需在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）完成市 场主体信息登记以及CA数字证书办理，办理方式请参见 重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、 重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）导航栏“主体信息”页面中“市场主 体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完 成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告 发布至2026-08-21 17:00:00前。 5.3招标人应于2026-08-25 23:59:59前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源 交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）发布澄清。 6.投标文件递交的内容 网 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-21 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 务 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交 易监督网上发布。] 商 8.联系方式 招 标 人: 重庆市开州区长沙镇人民政府 代理机构: 重庆毅仁建设项目管理有限公司 重庆市开州区文峰街道天鹅湖社区富厚街158号附10 地 址: 重庆市开州区长沙镇山花街1号 地 址: 道号 邮 编: 邮 编: 项目负责人: 丁敬余 项目负责人: 谭毅 电 话: 15826368887 管电 话: 13452653126 传 真: 传 真: 电子邮箱: 1415705480@qq.com 电子邮箱: 开户银行: 国 开户银行: 账 号: 账 号: 监督部门:中重庆市开州区公共资源交易管理局 电 话: 023-52218977 2026年08月17日 重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目 户名 开户行 投标保证金账号 重庆市开州区公共资源交易中心 重庆农村商业银行股份有限公司开州支行 3401010120010012772000200 中国农业银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 314401010400104500000006031 业部 中国工商银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 9558853100005824176 业部 重庆市开州区公共资源交易中心 重庆银行股份有限公司开州支行 680101040007547-100984 重庆市开州区公共资源交易中心 中国银行股份有限公司重庆开州支行 108865555576VA00149 信息来源:https://www.chinapipe.net/project/d3075199.html cqdingjiu 2026.08.21 10:06:58</t>
@@ -3798,9 +4814,13 @@
         </is>
       </c>
       <c r="O60" t="n">
-        <v>0</v>
-      </c>
-      <c r="P60" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>重庆, 柑橘基地改造, 水肥一体化系统, 运输线, 排灌站, 生产便道, 无人机, 小型挖机, 智慧平台</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3833,16 +4853,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>万盛区</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>万盛区</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>万盛城区老旧供水管网更新改造工程答疑及补遗。</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>供水管网</t>
+        </is>
+      </c>
       <c r="M61" t="inlineStr">
         <is>
           <t>万盛城区老旧供水管网更新改造工程答疑及补遗(一) 万盛城区老旧供水管网更新改造工程 答疑及补遗（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程答疑及补遗（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。? 问题2：本项目是否采用异地评标方式？ 答：是 。 商 问题3：本项目是否有业主代表，如有，请明确业主代表数量。 答：是，本项目评标委员会共7人，其中在重道庆市综合评标专家库随机抽取5人，招标人代表2人 。 问题4：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 答：可以。 管 问题5：污水处理厂提标改造及附属管道施工业绩满足吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 国 问题6：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可以 不填(空白)，对此有无要求？ 答：无要求。? 中 问题7：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖章， 请问需要提供联合体协议书吗？ 。 答： 根据招标文件第二章“投标人须知前附表”1.4.1 第3条业绩要求中：“注：（2）投标人提供的业绩为联 合体业绩的，其在该业绩中的工作分工应与本项目承担的工作一致。”要求，故需要提供联合体协议书。 问题8：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要求”吗？ 答：填写“达到招标文件的要求”或按照招标文件相关条款填写具体内容均可 。 问题9：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 答：投标人的工程量清单单项报价不得为零报价(招标人提供的工程量清单单项最高限价中金额为零的除外)或者 负数报价，否则由评标委员会作否决投标处理。 问题10：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知书发 出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面通知相关金融机构本项目准予提前注 销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 答：需要。但不将加盖正本作为评审因素。 问题11：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收，请 问我公司业绩满足业绩要求吗？ 答：不满足。? 问题12：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 答：可以 。 问题13：业绩要求的竣工时间是指竣工验收时间吗？ 答：是的。 网 问题14：重庆市电子招投标系统投标文件-报价部分“己标价工程量清单”-“投标总价”页面招标人名称需要填 写吗？ 务 答：由投标人自行决定是否填写，是否填写不作为评审因素。 问题15：请问招标人是否委派业主专家参与评标吗？ 答：是，本项目评标委员会共7人，其中在重庆市综合评商标专家库随机抽取5人，招标人代表2人。 问题16：自来水厂或者净水厂含管道施工业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需道满足招标文件要求。? 问题17：有没有人行贿专家，有的话我们就不参加了。 答：本项目评标委员会由招标人按法律法规及相关规定依法组建。 管 问题18：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要 提供其他格式之外的其他承诺？ 答：请各潜在投标人仔国细阅读招标文件，并按招标文件要求提供相应承诺。 问题19：财务报告可以不提供财务报表附注吗？ 答：可以。 中 问题20：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题21：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、注册证 及在本单位注册的证明文件替代？ 答：退休证等材料不能替代养老保险证明，按招标文件执行。? 问题22：本项目是异地评标吗？ 答：是。 问题23：现在除了没有警戒线和技术方案的低价项目评标专家不被围猎，哪个项目不围猎评标专家，请问招标人 如何保证公平？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题24：没有低价警戒线怎么保证中高价呢？ 答：本项目未设置低价警戒线，通过综合评估法对各潜在投标人进行评审。分值由技术、商务、报价组成，综 合实力优良的投标人合理中高价可依靠综合得分优势参与竞争，同时招标文件履约追责条款约束投标人理性报 价，保障合理报价竞争环境。 问题25：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养老保险 证明材料复印件递交吗？ 答：现场递交纸质保函原件的人员不作要求 。 问题26：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 网 答：电子投标系统中锁定不可修改的格式（如封面、投标函）直接填空即可，其他投标文件格式以加盖公章的 招标文件PDF文件为准。? 问题27：专业分包业绩满足业绩要求吗？ 务 答：不满足。 问题28： 市政道路包含给水管网施工业绩满足业绩要求吗？ 商 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题29：技术负责人在资格审查部分中提供了工程类高级及以上职称证后，在商务部分中再提供工程类高级及以 上职称证可以加分吗？ 道 答：可以。 问题30：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 管 全是万盛的公司中的！业主、专家全是你们自己人吧？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 国 二、补遗 1、本次重新发布本项目的工程量清单，在《重庆市公共资源交易网》(綦江区) （https://www.cqggzy.com/qijiangweb/）网上发布，请投标人自行下载。 中 招 标 人：重庆市万盛经济技术开发区城市管理局 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 信息来源:https://www.chinapipe.net/project/d3074975.html cqdingjiu 2026.08.21 10:06:58</t>
@@ -3854,9 +4890,13 @@
         </is>
       </c>
       <c r="O61" t="n">
-        <v>0</v>
-      </c>
-      <c r="P61" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>重庆, 供水管网, 更新改造</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3871,7 +4911,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3889,16 +4929,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>巴南区</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>巴南区</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>为解决片区内涝问题，在李家沱街道、花溪街道改建d400-d800雨水管网9665m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管；改建d1000-d1400雨水管网664m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管；改建d1500-d2000雨水管网426m，管材采用III级钢筋混凝土管；改建d2100-d2600雨水管网1000m，管材采用III级钢筋混凝土管；修复雨水管网5345m，增加智能感知设备6套。</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>本次招标项目工程费估算金额：11061.83万元，勘察设计合同估算金额：334.544万元。</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>雨水管网、高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管、智能感知设备</t>
+        </is>
+      </c>
       <c r="M62" t="inlineStr">
         <is>
           <t>重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 1.招标条件 本招标项目 重庆市巴南区土桥片区内涝积水整治工程已由重庆市巴南区发展和改革委员会以巴南发改审 发[2025]33号文批准建设，项目业主为重庆市巴南区住房和城乡建设委员会，代建业主为重庆市巴南公路建设有 限公司，建设资金来自区级财政资金统筹，项目出资比例为 100%，招标人为重庆市巴南公路建设有限公司。 项目已具备招标条件，现对该工程的勘察设计进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 2.1 建设地点：重庆市巴南区花溪街道、李家沱街道 务 2.2 项目概况与建设规模：为解决片区内涝问题，在李家沱街道、花溪街道改建 d400-d800 雨水管网 9665m，管材 采用高密度聚乙烯(HDPE)缠绕结构壁管 B型管；改建 d1商000-d1400雨水管网 664m，管材采用高密度聚乙 烯(HDPE)缠绕结构壁管 B 型管、III 级钢筋混凝土管；改建 d1500-d2000 雨水管网 426m，管材采用III 级钢筋混凝 土管;改建 d2100-d2600 雨水管网 1000m，管材采用 III 级钢筋混凝土管；修复雨水管网 5345m，增加智能感知设 备6 套。 道 2.3 本项目工程总投资金额：13477.10万元 管 本次招标项目工程费估算金额：11061.83万元 国 本次招标项目勘察设计合同估算金额：334.544万元 中 2.4 招标范围：主要包括勘察、施工图设计（包含高边坡、深基坑）和相应阶段的勘察工作，以及提供施工现场 全过程技术服务，并配合业主办理相关手续等，具体范围为： （1）勘察部分：完成本项目范围内的勘察工作，包括但不限于排水管网排查、1:500地形图测量、地质钻勘、管 线内窥、物探、综合管线测量，市政管网错混接点测量及调查等工作，解决区域地下空间臭气问题，勘察成果 需达到重庆市城市建成区排水管网排查技术导则的要求，并配合业主完成对应的成果审查等事宜。 （2）设计部分：包括不限于完成本项目的施工图设计、施工期间交通组织设计、桥梁（涉轨）安全论证方案及 施工期间至竣工验收阶段，质量保修阶段的设计配合服务，配合办理施工图审查相关手续及竣工验收阶段、质 量保修阶段的设计服务等工作以及协助招标人完成各项审批手续办理等工作。 2.5 勘察设计服务期限：30日历天 2.6 标段划分（如有）：/ 2.7 其他：/ 3.政府采购工程 3.投标人资格要求 3.1 本次招标要求投标人须具备以下条件： 网 3.1.1 本次招标要求投标人具备的资质条件： 务 投标人应同时具有建设行政主管部门颁发的下列勘察和设计两类资质： 商 I、投标人应具备下列勘察资质之一： 道 ①工程勘察综合甲级资质。 管 ②工程勘察专业类（岩土工程）专业甲级资质和工程勘察专业类（工程测量）甲级资质； 国 II、投标人应具备下列设计资质之一： 中 ①工程设计综合甲级资质； ②工程设计市政行业甲级资质； ③工程设计市政行业(燃气工程、轨道交通工程除外)甲级资质； ④工程设计市政行业(排水工程)甲级资质。 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的勘察设计能力，详见招标文件第二章投标人须知 前附表第1.4.1项内容。 3.2 本次招标接受联合体投标。联合体投标的，应满足下列要求：联合体组成单位数量不超过2家，由负责设计 任务的单位作为联合体牵头人。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件及其附件、澄 清、修改、补充通知、最高限价通知等资料。参与投标的投标人需在重庆市公共网资源交易网完成市场主体信息 登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息 登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程 电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 务 布至2026-08-23 12:00:00前。 4.3招标人应于2026-08-26 17:00:00前在重庆市公共资源交易网发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-24 09:30，投标人应当在投标截止时间前，通过互 商 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督道网、重庆市公共资源交易网、重庆市公共资源交易网（巴南区） 发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 重庆市巴南公路建设有限公司 代理机构: 重庆云远项目管理有限公司 管 地 址: 重庆市巴南区龙洲大道265号 地 址: 重庆市九龙坡区渝隆大厦28楼 邮 编: 邮 编: 项目负责人: 牟老师 项目负责人: 李强 国 电 话: 023-66238079 电 话: 023-68434996 传 真: 传 真: 电子邮箱: 电子邮箱: 中 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 2026年08月18日 重庆市巴南区土桥片区内涝积水整治工程勘察设计 户名 开户行 投标保证金账号 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000001675 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051304894 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020041267 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764210157 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000682897 支行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835000509 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146639123 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630018252 信息来源:https://www.chinapipe.net/project/d3074953.html cqdingjiu 2026.08.21 10:06:58 网 务 商 道 管 国 中</t>
@@ -3910,9 +4966,13 @@
         </is>
       </c>
       <c r="O62" t="n">
-        <v>0</v>
-      </c>
-      <c r="P62" t="inlineStr"/>
+        <v>95</v>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 雨水管网, 高密度聚乙烯, HDPE, 钢筋混凝土管</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3945,16 +5005,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>涪陵作业区涪陵压气站空压机、阀门等设备、消防泵房消防管道、循环水管道油漆出现锈蚀情况，为保证设施安全运行，对站场设备、消防管道及附属钢结构进行打磨除锈、油漆防腐。</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>管道、设备防腐</t>
+        </is>
+      </c>
       <c r="M63" t="inlineStr">
         <is>
           <t>重庆管道公司2026年涪陵压气站管道、设备防腐项目-非招标公告 公告发布时间: 2026年08月18日09时02分19秒 一、概述 1.2.1项目概况：涪陵作业区涪陵压气站空压机、阀门等设备、消防泵房消防管道、循环水管道油漆出现锈蚀情况， 为保证设施安全运行，对站场设备、消防管道及附属钢结构进行打磨除锈、油漆防腐。 二、采购项目与标段 交货期限: 开工之日起90日内完工 网 质保期限(月): 标段 序号 标段名称 标段描述 编号 重庆管道公司2026年涪陵 涪陵作业区涪陵压气站空压务机、阀门等设备、消防泵房消防管道、循 1 1 压气站管道、设备防腐项 环水管道油漆出现锈蚀情况，为保证设施安全运行，对站场设备、消 目 防管道及附属钢结构进行打磨除锈、油漆防腐。 三、供应商资格要求 商 *1、响应人资质要求（1）响应人必须是依照中华人民共和国法律在国内注册，具备合格有效的营业执照的法人、 其他组织；与采购人存在利害关系可能影响询比采购公正性的法人、其他组织或者个人，不得参加响应。单位 负责人为同一人或者存在控股、管理关系的不同单位，不得参加同一标段响应或者未划分标段的同一询比项目 响应。（2）响应人须具备防水防腐保温工程专业承包二级及以上资质。*2、信誉要求响应人在响应文件提交截 止当日不存在以下情况：（1）响应人被“国道家企业信用信息公示系统”网站（www.gsxt.gov.cn）列入严重违法 失信企业名单（响应文件提交截止时间前已移出的除外）。（2）响应人被“信用中国”网站 （www.creditchina.gov.cn）列入严重失信主体名单（响应文件提交截止时间前已移出的除外）。（3）响应人或其 法定代表人、负责人、拟委任的项目经理被“中国执行信息公开网”（http://zxgk.court.gov.cn/shixin/）列入失信 被执行人名单（响应文件提交截止时间前已移出的除外），响应文件中需提供有效身份证号供查询。（4）响应 管 人、拟委任的项目经理被“全国建筑市场监管公共服务平台”网站（https://jzsc.mohurd.gov.cn/home）列入黑名单 （响应文件提交截止时间前已移出的除外）。上述（1）-（4）条以评审当日评审小组从官网查询信息为准。（5） 被国家管网集团或西南管道公司暂停、取消投标资格或业务承揽资格。（6）法律、行政法规规定的其他不允许 参与投标的情况。 国 四、询比文件的获取 4.1 有意向参加项目者，于2026年08月20日09时05分22秒前，登录数字供应链平台进行项目报名。 中 4.2 报名成功后于2026年08月18日09时01分42秒至2026年08月24日09时05分22秒，登录数字供应链平台进行项目下 载询比文件。 五、响应文件的递交 5.1 请于2026年08月24日11时00分00秒前，登录数字供应链平台递交项目响应文件。 5.2 逾期将无法进行递交响应文件，采购人将不予受理。 5.3 供应商在递交响应文件前，应按照有关规定提供人民币0万元项目保证金。 六、响应文件的开启 6.1 响应文件的开启时间2026年08月24日11时06分00秒 6.1 响应文件的开启地点供应链系统上 七、采购人信息 地址： 邮编： 联系人：舒建华 联系电话：18581824001 电子邮件：shujh@pipechina.com.cn 传真： 开户银行： 账户名： 账号： 信息来源:https://www.chinapipe.net/project/d3074904.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
@@ -3968,7 +5044,11 @@
       <c r="O63" t="n">
         <v>0</v>
       </c>
-      <c r="P63" t="inlineStr"/>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3983,7 +5063,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4001,16 +5081,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>安装部分包括材料验收、运输及履带式挖掘机及人工布管、管道管件安装、新旧管道的碰口、安装DN400直埋球阀1座、管道和商焊口的除锈及防腐、管道下沟后15KV电火花检测、管道的清管、强度及严密性试验、警示带敷设和线路标志桩（砖）安装、监检手续等。土建部分包括清表、扫线、平整场地、沟槽、基坑、阀井砌筑、回填土方、余方弃置、人工开挖人行道（花台）、公路及路面恢复、其他线缆穿跨越工道程施工、交通组织、水工保护等。</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>燃气管线工程</t>
+        </is>
+      </c>
       <c r="M64" t="inlineStr">
         <is>
           <t>重庆燃气集团股份有限公司输配分公司大渡口调压站至二郎调压站次高压燃气管线工程(大渡口段)公告 采购 公告 公告编号： RQXYGG202608130064 一、采购项目基本情况 网 采购人：重庆燃气集团股份有限公司输配分公司 采购项目编号：RQCGXY202608130040 务 采购项目名称：大渡口调压站至二郎调压站次高压燃气管线工程（大渡口段） 采购内容或范围：安装部分： ①材料验收（甲供材料：阀门、管材、弯头、标志桩等）、运输及履带式挖掘机及人工布管； ②管道管件安装， 新旧管道的碰口；③安装DN400直埋球阀1座； ④管道和商焊口的除锈及防腐； ⑤管道下沟后15KV电火花检测； ⑥管道的清管，强度及严密性试验；⑦警示带敷设和线路标志桩（砖）安装； ⑧监检手续等。 土建部分： ①清表； ②扫线、平整场地； ③沟槽、基坑、阀井砌筑； ④回填土方； ⑤余方弃置； ⑥人工开挖人行道（花 台），公路及路面恢复； ⑦其他线缆穿跨越工道程施工，交通组织； ⑧水工保护等。 （具体内容详见施工图纸和 工程量清单） 公告发布时间 ：2026-08-18 14:39:10 管 二、采购人联系方式 联系人：王瑶 电话：023-67502265 国 邮箱：wangyao232@crcgas.com 三、采购明细 中 行号 采购内容 需求数量 单位 补充说明 拟邀请单位 大渡口调压站至二郎调压站次高压燃气管线 重庆燃气安装工程有限责任公 1 1 项目 无 工程(大渡口段) 司 四、服务费交纳 本项目不收取服务费。 五、 其他 事项 1.本公告在华润守正 采购交易 平 台（ https://www.szecp.com.cn/ ）上公开 发布。 2. 本项目采购通过守正平台线上进行，供应商需注册华润守正 采购交易 平台，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 3 .答疑澄清、通知等文件一经在华润守正 采购交易 平台发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注华润守正 采购交易 平台发布的相关信息，并及时查阅和处理。 4 .若有参与意向 ， 请于 2026-08-22 00:00:00前联系采购人 （联系方式见公示内容）反馈。 5 .若有异议 ， 请于 2026-08-22 00:00:00前提出异议 。 信息来源:https://www.chinapipe.net/project/d3074793.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
@@ -4022,9 +5110,13 @@
         </is>
       </c>
       <c r="O64" t="n">
-        <v>0</v>
-      </c>
-      <c r="P64" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4057,16 +5149,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>2026-2027年度用户供水管道安装及管网抢（维）修服务</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>项目资金来自企业自筹，合同估算金额约280万元</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>供水管道安装及管网抢（维）修服务</t>
+        </is>
+      </c>
       <c r="M65" t="inlineStr">
         <is>
           <t>石柱公司2026-2027年度用户供水管道安装及管网抢(维)修工程(第二次)项目公告 石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（比选公告 1.比选条件 本比选项目石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（项目名称），比选人 为重庆石柱水利水电实业开发有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。现 对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 建设地点：比选人指定地点 务 2.2 项目概况与建设规模：2026-2027年度用户供水管道安装及管网抢（维）修服务 2.3 本次比选项目合同估算金额：约280万元 商 2.4 比选范围：完成石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程包括公司供水范围内用户 各类管道及管件安装、水表安装及更换、阀门安装等、并完成配套土建工程、零星签证等工程量清单所列项目、 管网抢维修和公司所属生产单元零星项目，具体内容详见第五章 工程量清单。 道 2.5 工期要求：1年 缺陷责任期要求：24个月 管 3.投标人资格要求 3.1 本次比选要求投标人须具备以下条件： 国 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质； 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 中 项内容。 3.2 本次比选不接受联合体投标。 4.比选文件的获取 4.1 投标人于2026年08月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价1000 元，售后不退。投标人在递交纸质投标文件时支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年08月24日10时00分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年08月24日09时30分至10时00分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼）。 5.3 投标截止时间：2026年08月24日10时00分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆石柱水利水电实业开发有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市石柱土家族自治县都督大道11号 地 址：重庆市两江新区嘉华路36号重庆水务大厦1018 联 系 人：王老师 联 系 人：颜老师 道 电 话：13658292968 电 话：023-67901915 重庆水务电子商务平台咨询电话：管023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074720.html cqdingjiu 2026.08.21 10:06:59 国 中</t>
@@ -4078,9 +5178,13 @@
         </is>
       </c>
       <c r="O65" t="n">
-        <v>0</v>
-      </c>
-      <c r="P65" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>重庆, 供水管道安装, 管网抢修, 企业自筹, 280万元</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4113,16 +5217,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>万盛城区老旧供水管网更新改造工程涉及3PE防腐钢管的采购，其管道部分壁厚需符合国标标准并达到设计要求。</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>项目详情中未提及具体资金情况。</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>3PE防腐钢管</t>
+        </is>
+      </c>
       <c r="M66" t="inlineStr">
         <is>
           <t>万盛城区老旧供水管网更新改造工程(甲供材料)答疑(一) 万盛城区老旧供水管网更新改造工程（甲供材料） 答疑（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程（甲供材料）答疑（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。 问题2：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 全是万盛的公司中的！业主、专家全是你们自己人吧？ 商 答：本项目招标文件严格按照《重庆市工程建设项目货物采购招标文件示范文本（2026年版）》编制，且本项目 评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题3：3PE管道部分壁厚是多少呢？ 道 答：本项目采购的3PE防腐钢管的管道部分壁厚须符合国标标准并达到设计要求。 招 标 人：重庆市万盛经济技术开发区城市管理局 管 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 国 信息来源:https://www.chinapipe.net/project/d3074712.html cqdingjiu 2026.08.21 10:06:59 中</t>
@@ -4134,9 +5246,13 @@
         </is>
       </c>
       <c r="O66" t="n">
-        <v>0</v>
-      </c>
-      <c r="P66" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 3PE防腐钢管, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4169,16 +5285,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>本项目涉及普通防腐钢管及管件的采购，包括各种规格的钢高频焊管和钢螺旋焊管，以及相应的管件如钢套筒、钢制标准接头等。</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>项目资金来自企业自筹，出资比例为100%。</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>钢高频焊管,钢螺旋焊管,钢套筒,钢制标准接头,钢制渐缩,钢制三通,钢制双盘短管,钢制弯头</t>
+        </is>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>重庆中法供水2026年普通防腐钢管及管件采购项目(第三次)项目公告 重庆中法供水2026年普通防腐钢管及管件采购项目（第三次）比选公告 1.比选条件 本比选项目重庆中法供水2026年普通防腐钢管及管件采购项目（第三次），比选人为重庆中法供水有限公司，比 选项目资金来自企业自筹，出资比例为100%，项目已具备比选条件。现对本项目进行公开比选，诚邀有兴趣的 潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 普通防腐钢管及管件采购清单： 务 序号 存货编码 材料名称 规格型号 单位 数量 最高单价限价（元） 1 10400177 钢高频焊管 D89*4 5 米 61.92 2 10400181 钢高频焊管 D108*5 300 米 88.89 商 3 10400182 钢高频焊管 D159*5 5 米 132.18 4 10400206 钢高频焊管 D159*6 5 米 152.13 5 10400290 钢螺旋焊管 DN219*6 5 米 196.68 道 6 10400291 钢螺旋焊管 DN219*8 5 米 244.80 7 10400292 钢螺旋焊管 DN325*8 5 米 361.28 8 10400293 钢螺旋焊管 DN377*8 5 米 423.12 管 9 10400294 钢螺旋焊管 DN426*8 5 米 475.89 10 10400295 钢螺旋焊管 DN426*10 5 米 574.29 11 10400297 钢螺旋焊管 DN529*8 5 米 595.76 国 12 10400298 钢螺旋焊管 DN529*10 5 米 718.91 13 10400299 钢螺旋焊管 DN630*10 5 米 861.50 14 10400300 钢螺旋焊管 DN720*10 5 米 987.95 中 15 10400301 钢螺旋焊管 DN820*10 5 米 1133.08 16 10400302 钢螺旋焊管 DN920*10 5 米 1279.51 17 10400304 钢螺旋焊管 DN1020*10 5 米 1424.64 18 10400305 钢螺旋焊管 DN1020*12 5 米 1652.24 19 10400306 钢螺旋焊管 DN1220*10 5 米 1709.70 20 10400307 钢螺旋焊管 DN1220*12 5 米 1982.83 21 10400308 钢螺旋焊管 DN1420*12 5 米 2375.96 22 10400309 钢螺旋焊管 DN1420*14 5 米 2697.83 23 10400332 钢螺旋焊管 DN1120*10 5 米 1574.96 24 10400342 钢螺旋焊管 DN1020*14 5 米 1879.02 25 10400322 钢螺旋焊管（特加强） DN820*10 5 米 1133.08 26 10200490 钢套筒 D159*500cm 5 个 159.00 27 10200491 钢套筒 D219*500cm 5 个 240.00 28 10200492 钢套筒 D273*500cm 5 个 300.00 29 10200493 钢套筒 D325*500cm 5 个 361.00 30 10200494 钢套筒 D377*500cm 5 个 436.00 31 10200495 钢套筒 D426*500cm 5 个 482.00 32 10200589 钢套筒 D159*1000cm 5 个 226.00 33 10200590 钢套筒 D219*1000cm 5 个 1627.00 34 10200591 钢套筒 D273*1000cm 5 个 2501.00 35 10200592 钢套筒 D325*1000cm 5 个 488.00 36 10200593 钢套筒 D377*1000cm 5 个 591.00 网 37 10200598 钢套筒 D426*1000cm 5 个 833.00 38 10200155 钢制标准接头 D108 5 个 91.00 39 10200156 钢制标准接头 D159 5 个 160.06 务 40 10200157 钢制标准接头 D219 5 个 319.41 41 10200158 钢制标准接头 D273 5 个 396.63 42 10200159 钢制标准接头 D325 5 个 475.96 商 43 10200160 钢制标准接头 D426 5 个 619.87 44 10200161 钢制标准接头 D529 5 个 779.22 45 10200162 钢制标准接头 D630 5 个 1068.44 道 46 10200163 钢制标准接头 D720 5 个 1214.46 47 10200164 钢制标准接头 D820 5 个 1428.34 48 10200165 钢制标准接头 D920 5 个 1600.14 管 49 10200169 钢制标准接头 D1220 5 个 2297.57 50 10200170 钢制标准接头 D1420 5 个 3027.02 51 10200171 钢制标准接头 D1020 5 个 2194.19 国 52 10300309 钢制大小头 DN65*DN50 5 个 14.74 53 10200667 钢制渐缩 D108＞57 3 个 21.06 54 10200668 钢制渐缩 D108＞89 3 个 26.00 中 55 10200695 钢制渐缩 D159＞108 3 个 40.72 56 10200671 钢制渐缩 D219＞159 3 个 68.09 57 10200672 钢制渐缩 D219＞108 3 个 80.03 58 10201605 钢制渐缩 219*125 3 个 75.82 59 10200694 钢制渐缩 D273＞108 3 个 129.87 60 10200673 钢制渐缩 D273＞159 3 个 94.07 61 10200674 钢制渐缩 D273＞219 3 个 84.94 62 10200675 钢制渐缩 D325＞108 3 个 184.63 63 10200676 钢制渐缩 D325＞159 3 个 143.91 64 10200680 钢制渐缩 D325＞219 3 个 131.98 65 10200677 钢制渐缩 D325＞273 3 个 124.25 66 10200684 钢制渐缩 D426＞325 3 个 285.01 67 10200685 钢制渐缩 D529＞325 3 个 617.76 68 10200679 钢制渐缩 D529＞426 3 个 547.56 69 10200659 钢制渐缩 D630＞325 3 个 756.00 70 10200687 钢制渐缩 D630＞426 3 个 728.00 71 10201539 钢制渐缩 D630＞529 3 个 722.00 72 10200690 钢制渐缩 D720＞630 3 个 848.00 73 10200691 钢制渐缩 D720＞529 3 个 842.00 74 10200682 钢制渐缩 D820＞720 3 个 913.00 75 10200692 钢制渐缩 D920＞720 3 个 1053.00 76 10201519 钢制渐缩 D920*820 3 个 1064.00 77 10200652 钢制渐缩 D1020＞820 3 个 1305.00 网 78 10200693 钢制渐缩 D1020＞920 3 个 1322.00 79 10201738 钢制渐缩 1220*820 3 个 1806.00 80 10201507 钢制渐缩 1220＞1020 3 个 1834.00 务 81 10201624 钢制三盘三通 D108⊥108 3 个 224.64 82 10200371 钢制三盘三通 DN200⊥100 3 个 435.24 83 10200373 钢制三盘三通 DN200⊥200 3 个 599.51 商 84 10201531 钢制三通 108*108 3 个 58.97 85 10200285 钢制三通 219*108 3 个 187.43 86 10201341 钢制双盘短管 89*400mm 3 个 139.00 道 87 10201342 钢制双盘短管 89*800mm 3 个 178.31 88 10201340 钢制双盘短管 108*300mm 3 个 158.65 89 10201299 钢制双盘短管 DN108*500mm 3 个 185.33 管 90 10201300 钢制双盘短管 DN108*1000mm 3 个 258.34 91 10201301 钢制双盘短管 DN108*1500mm 3 个 329.94 92 10201332 钢制双盘短管 159*300mm 3 个 251.32 国 93 10201339 钢制双盘短管 159*750mm 3 个 348.19 94 10201303 钢制双盘短管 DN159*1000mm 3 个 402.95 95 10201304 钢制双盘短管 DN159*1500mm 3 个 508.25 中 96 10201305 钢制双盘短管 DN219*500mm 3 个 463.32 97 10201306 钢制双盘短管 DN219*1000mm 3 个 672.52 98 10201307 钢制双盘短管 DN219*1500mm 3 个 876.00 99 10201312 钢制双盘短管 DN219*750mm 3 个 581.26 100 10201338 钢制双盘短管 273*1250mm 3 个 1010.88 101 10201458 钢制双盘渐缩 108*57 3 个 109.51 102 10201469 钢制双盘渐缩 108*89 3 个 117.94 103 10201514 钢制双盘渐缩 159*108 3 个 185.33 104 10201748 钢制双盘渐缩 200*80 3 个 294.84 105 10201462 钢制双盘渐缩 219*108 3 个 256.93 106 10201513 钢制双盘渐缩 219*159 3 个 280.80 107 10201465 钢制双盘渐缩 D273＞108 3 个 339.77 108 10201467 钢制双盘渐缩 D273＞219 3 个 388.91 109 10201770 钢制双盘渐缩 D273＞159 3 个 365.04 110 10201461 钢制双盘渐缩 325*219 3 个 477.36 111 10301108 钢制弯头 89*90° 3 个 28.78 112 10200702 钢制弯头 D108×90° 100 个 43.52 113 10200701 钢制弯头 D159×90° 3 个 84.24 114 10200705 钢制弯头 D219*90° 3 个 231.66 115 10200706 钢制弯头 D273*90° 3 个 300.46 116 10200709 钢制弯头 D325*90° 3 个 418.39 117 10200711 钢制弯头 D426*90° 3 个 744.12 118 10200712 钢制弯头 D529*90° 3 个 1352.05 网 119 10200764 钢制弯头 D570*90° 3 个 1474.20 120 10200714 钢制弯头 D630*90° 3 个 1535.98 121 10200715 钢制弯头 D720*90° 3 个 1742.36 务 122 10200717 钢制弯头 DN720*90°*12mm 3 个 1989.47 123 10200720 钢制弯头 D920*90° 3 个 2935.30 124 10200722 钢制弯头 D820*90° 3 个 2325.23 商 125 10200762 钢制弯头 D1020*90° 3 个 4829.55 126 10200723 钢制弯头 D1220*90° 3 个 6039.80 127 10200724 钢制弯头 D1420*90° 3 个 8297.00 道 注：管材按照米数进行报价，管件按照件数进行报价。 2.2 供货数量、时间和批次：根据工程实际进度与比选人的要求进行供货，以实际供货量为准，供货时间达到商 务条款的规定。 管 2.3 交货地点：比选人指定的施工现场。 2.4 供货期：两年。 国 3.投标人资格要求 3.1 本次比选允许投标人以投标货物的下列身份参加投标： 中 ?制造商 3.1.1 投标人为制造商应符合以下要求： 投标人必须是依法设立的，并在中国注册的，具有独立法人地位的企业。 【提供有效的营业执照】 3.2 投标人2025年的年度财务状况不亏损。 【提供由会计师事务所或审计机构出具的无保留意见的财务审计报告及会计报表，财务报表至少包括现金流量 表、资产负债表、利润表】 3.3 投标产品的制造商须通过质量ISO9001、环境ISO14001、职业健康体系ISO45001认证。 【提供有效的证书】 3.4 投标人须提供2023年1月1日至投标截止日止（以合同签订时间为准）,签订的30万元及以上的钢管及管件产品 购销合同至少1个。 【提供采购合同、不低于前述金额50％的发票，合同与发票的项目名称须一致】 注：①若投标人开具的发票上未能体现具体项目，需附上税务出具的发票清单（清单上需显示采购项目为钢管 及管件产品）。 ②若提供的合同为年度合同未体现具体金额，但实际供货金额达到30万元及以上，应提供与该合同对应的30万元 及以上的钢管及管件产品发票作为佐证。 3.5 投标人须为所投投标产品制造商，此次所提供的普通防腐钢管及管件必须是自己工厂所制造的产品，不得外 购他人产品。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函及工商部门出具的本产品商标或品牌证明文件】 3.6 投标产品过水部分涉及的涂料须提供行政主管部门出具的有效的“卫生许可网批件”及卫生疾控中心出具的卫 生检测报告。 【提供行政主管部门出具的有效的“卫生许可批件”及卫生疾控中心出具的卫生检测报告】 务 3.5 根据本次采购清单及技术规范的要求，投标人须承诺具备相关的技术手段和措施、保证产品设计使用寿命 20 年以上。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 商 3.6 投标人须承诺保证5年内不得停产同型号的投标产品。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 道 3.7 办事机构和库房【比选人有权对中标人的办事机构及库房进行实地核查，若发现与提供资料不符，将视为提 供虚假资料，按相关规定取消其中标资格，其投标保证金不予退还。】 投标人承诺：收到中标通知书后30日内提供租赁合同或产权证明，并提供重庆库房卫星定位图片。 管 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 【卫星定位图片：手机打开地图，搜索该地址、进行标注，然后截图或者电脑打开地图（地图软件不限），搜 索该地址、选择卫星模国式、进行标注、然后截图均可。】 3.8 符合第五章“技术要求”普通防腐钢管及管件技术要求。 【根据技术要求提供技术响应表，并根据技术条款要求提供对应的检测报告等。】 中 3.9 售后服务承诺【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】： 1）货物交付及付款方式要求，满足第四部分合同协议书第3条及第10条；供货单位应确保产品的及时供应，承诺 因产品供应不及时造成的一切损失均由供货单位负责赔偿。 2）有完整的售后服务方案、培训计划并在合同签订后为比选人免费提供培训服务。 3）售后服务承诺书，满足第四部分合同协议书第11条；承诺质保期后提供2年及以上定期免费巡查、保养计划。 4）承诺接到分派的工单1小时内联系用户约定维修时间，在24小时内处理完毕工单，且让用户满意。若工单超时、 未在规定时间内告知比选人维修时间或工单处理未让用户满意造成返单的，按比选人制度进行处罚。 3.10 投标人承诺不得存在下列情形之一： 1）被人民法院列入失信被执行人名单且在被执行期内； 2）被国家、重庆市（含市或任意区县）有关行政部门行政处罚，且在处罚期限内； 3）投标截止日前两年内（指2024年1月1日至投标截止日止），投标人或其法定代表人被人民法院判定犯行贿罪 的； 4）投标截止日前五年内（指2021年1月1日至投标截止日止），投标人与重庆中法供水有限公司有违约情况或终 止合同情况的。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 3.11 投标截止日前五年内（指2021年1月1日至投标截止日止），投标人无在我司因产品及服务等对公司生产、经 营、安全造成不良影响的记录；若投标人出现过供水通报事项，因产品质量问题对生产、安全造成影响，存在 合同违约等问题，不予参加本次项目投标。 【按照第六章 三、资格审查部分“无不良记录承诺函”提供承诺函，若经验证承诺函不属实，将对中标人作否 决投标处理。】 网 3.12 投标样品要求： 3.12.1 投标人需提供以下规格型号数量的样品： 务 【①钢螺旋焊管 DN219*8 壹件 ②钢制弯头 D108*90°壹件】，提供的样品应满足第五章技术要求规定。样品为 投标人免费提供，管材样品不低于20CM，不计入采购清单内。 3.12.2 投标样品同投标文件一并递交。每件样品上分别标明样品的投标人、生产厂家、品牌、名称、规格、型号等 （格式自拟），投标样品必须密封装箱，且在密封包装外商贴样品一览表（格式自拟），注明提供样品的投标人、 生产厂家、品牌、名称、规格、型号、数量等。 3.12.3 投标人的样品在开标当日递交至样品区（样品区地点：开标当日咨询比选代理机构），中标人的投标样品 不退还，其余投标人的样品在中标公示期满后道5个工作日内退还，如不领取，投标样品按废品处理。 3.12.4 上述对投标样品的密封和标识要求是为便于评标，请投标人积极配合，未按上述要求对投标样品进行密封 和标识的，不作否决投标处理，但由此造成的其他后果由投标人自行承担。 管 3.13 若投标人违反重庆中法供水有限公司《供应商负面清单管理办法》规定且在处罚期内的，按否决投标处理 （评标委员会根据比选公告后附“供应商负面清单”进行评审）。 3.14 本次比选不接受联合体投标。 国 特别说明： （1） 本比选文件要求提供的所有检测报告须为近2年内的检测报告（2024年1月1日-投标截止日），此要求不包 括卫生许可批件及其检测报告。 中 （2） 上述所须提交的相关证明材料复印件均应加盖投标单位法人章并装入投标文件资格审查部分中。上述有一 条不满足则投标文件由评标委员会作否决投标处理。 （3） 比选人有权对投标人提供的以上资料进行核实，若发现存在弄虚作假，取消其投标、中标资格，投标人承 担因此造成的相关责任并赔偿相应损失。 4.比选文件的获取 4.1 投标人于2026年8月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价 500 元，售后不退。投标人在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年8月26日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月26日14时00分至14时30分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼。导航：重庆水务大厦东门）。 5.3 投标截止时间：2026年8月26日14时30分（北京时间）。 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 网 6.发布公告的媒介 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 务 7.联系方式 比 选 人：重庆中法供水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝北区悦来镇悦来水厂 地 址：重庆市两商江新区嘉华路36号重庆水务大厦10楼1018 联 系 人：陈老师 联 系 人：周洲 电 话：023-67585971 电 话：18602396399 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074673.html 管 cqdingjiu 2026.08.21 10:06:59 国 中</t>
@@ -4192,7 +5316,11 @@
       <c r="O67" t="n">
         <v>0</v>
       </c>
-      <c r="P67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>未识别到明确匹配关键词</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4225,16 +5353,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>南岸区</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>南岸区</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展水土保持监管测工作。</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>供水管网</t>
+        </is>
+      </c>
       <c r="M68" t="inlineStr">
         <is>
           <t>南岸区茶园片区乡镇老旧供水管网更新改造工程更正公告 南岸区茶园片区乡镇老旧供水管网更新改造工程更正公 告 发布日期： 2026年8月18日 网 首次公示日期： 2026年8月14日 更正日期： 2026年8月18日 采购人名称： 重庆市江南城市建设发展（集团）有限公司务 采购人地址： 重庆市南岸区米兰路51号电子信息标准化厂房2号楼 联系人： 赵老师 商 电话： 023-62820331 采购代理机构名称： 重庆多杰数字科技咨询服务有限公司 采购代理机构地址： 重庆市重庆市经开区重庆市经开区长生桥镇江峡路8号13-1幢1楼 道 经办人名称： 李佩奇、戴沛轩、李倩 联系电话： 023-67648437 本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展 更正事项： 水土保持监管测工作。 https://www.gec123.com/notices/detail/1665701682723590144 信息来源:https://www.c国hinapipe.net/project/d3074669.html cqdingjiu 2026.08.21 10:07:01 中</t>
@@ -4246,9 +5390,13 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>0</v>
-      </c>
-      <c r="P68" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>重庆, 管材招标, 商机</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4281,16 +5429,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治县。合同金额28.01亿元，合同工期73个月，主要工程包括新方斗山隧道、石板坡隧道、城北隧道、刘家坪隧道、刘家店子1号大桥工程、刘家店子2号大桥、城北大桥、冉家湾大桥，采用移动模架和支商架法现浇施工，正线铺无砟道床43.808Km。</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>合同金额28.01亿元</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>排水钢管Φ200*6m</t>
+        </is>
+      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t>中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部排水钢管询价采购公告 中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 排水钢管询价采购公告 询价编号：ZT1105-XJ-2026-561-1 尊敬的各潜在供应商: 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与中铁十一局集团有限公司宜涪高铁重庆段站 前3标项目经理ZT1105-XJ-2026-561-1，排水钢管材料的报价。 一、项目概况 务 中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治（县）。合同金额28.01亿元，合同工期73个月， 开工日期：2024年12月，竣工日期：2030年12月。主要工程：新方斗山隧道(10660m)、石板坡隧道(4148m)、城北 隧道(3228m)、刘家坪隧道(2077m);刘家店子1号大桥工程(224.096m)、刘家店子2号大桥(232.099m)、城北大 桥(330.241m)、冉家湾大桥(355.245m),采用移动模架和支商架法现浇施工，其中24米移动模架施工6孔；32米支架法 施工5孔，移动模架施工28孔;正线铺无砟道床43.808Km。 二、询价内容 道 本次计划对排水钢管、GG-01材料进行询价，询价内容如下： 询价物资一览表 管 序号 包件号 物资名称 规格型号 计量单位 数量 备注 1 GG-01 排水钢管 Φ200*6m 米 3000 Q235B，壁厚6mm 合计 3000 国 说明：1.表中数量为计划数量，实际采购过程中可能有所调整，最终结算按照实际采购数量结算。 2.收货地点：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 中 三、技术质量及报价要求 1. 此次排水钢管、GG-01各项技术性能：Q235B 碳素结构钢无缝钢管，符合 GB/T8163 标准。质量需满足甲方项 目部正常使用的要求，保证产品的质量合格，满足试验室检测所有要求，详见技术规格书。 2.报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、结算及付款方式 自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发票认证完成之日起第6个月，支付至本次结算 金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内，累计支付总额不超结算总金额的75%，剩 余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理末次结算后第二年，支付金额应大于等于 尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总额的15%；办理末次结算后第四年，全部 付清）。 五、报价人资格要求 1.营业范围要求：在中华人民共和国境内依法注册、符合项目经营范围，具有询价物资生产或供应经验 的生产商或代理商，并且具有合法有效的营业执照。 2.生产能力要求：生产商须具备询价物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定。代 理商需出具制造厂出具签字盖章的授权函。 3.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8 月至今）国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；需满足排水钢管的相关所 有要求。 4.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年12月至今）企业或企业法定代表人有人民法院生效判决、裁 定认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接 受通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合 作方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 5.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★6.下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、报价人需要提供的资料 1.营业执照复印件、法人身份证复印件、开户许可证、授商权委托书、报价表和报价人资格要求中所需的证明资料， 所有资料需加盖公司鲜章。 2.生产厂家资质，产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、询价报名截止时间 管 有意参加本次询价采购的报价人须在铁建云链平台（https://www.crccep.cn）完成供应商注册，并于2026年8月18 日9时00分至2026年8月21日9时00分在网上完成报名工作。 八、询价截止时间 国 凡有意参加本次询价采购的报价人，请于 2026年8月21日14时00分 前提交报价。截止时间前未完成报价文件传 输的，视为放弃报价。 供应商报价必须严格按照《报价表》格式进行报价。 中 九、联系方式 采购组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村71号 采购人名称：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 地址：重庆市石柱土家族自治县金彰工业园区C区中铁十一局项目部 联系人：罗先生 联系电话：18580400001（提供采购服务支持） 中铁十一局集团有限公司 物资设备集中采购管理中心第五分中心 2026年8月18日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3074654.html cqdingjiu 2026.08.21 10:07:01 网 务 商 道 管 国 中</t>
@@ -4302,9 +5458,13 @@
         </is>
       </c>
       <c r="O69" t="n">
-        <v>0</v>
-      </c>
-      <c r="P69" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>重庆, 排水钢管, 询价采购</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4337,16 +5497,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热交换机组采购。</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>项目详细内容无法识别</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>冷却塔、分集水器、水板式热交换机组</t>
+        </is>
+      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t>中铁建设集团(重庆)建设有限公司重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热 交换机组采购竞价补遗公告二 各 投标单位 ： 根据参加报名的潜在投标单位数量不满足招标方充分竞价要求的情况，此次重庆协同创新区供冷供热能源站及 配套系统工程冷却塔、分集水器、水板式热交换机组采购竞价资格预审报名截止日期将延期至 8月19日（周三） 上午9:00。 特此说明。 网 中铁建设集团（重庆）建设有限公司 2026年8月17日 务 信息来源:https://www.chinapipe.net/project/d3074650.html cqdingjiu 2026.08.21 10:07:01 商 道 管 国 中</t>
@@ -4358,9 +5526,13 @@
         </is>
       </c>
       <c r="O70" t="n">
-        <v>0</v>
-      </c>
-      <c r="P70" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>重庆协同创新区, 供冷供热能源站, 冷却塔, 分集水器, 水板式热交换机组, 采购竞价</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4393,16 +5565,32 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>城口县</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>城口县</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>在城口县东安镇新建一座污水处理站，铺设不同直径的污水管道共计29.3公里，包括dn110、dn160、dn200、DN300、DN400等规格的污水管道，以及DN200压力管道7.4公里，建设配套泵站2座和化粪池56座、隔油池32座。</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>合同预估金额为3400万元人民币。</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>污水管网、泵站、化粪池、隔油池</t>
+        </is>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t>城口县东安及河鱼片区污水管网建设项目(一期)招标计划表 重庆市工程建设项目招标计划表 项 名 目 称城口县东安及河鱼片区污水管网建设项目（一期） 招标 法人 或招 标人城口县生态环境局 名称 （盖 网 章） 项目 批准 文件 及文 号 主 建 内 要 设 容 在 污 城 水 口 处 县 理 东 站 安 1座 镇 ， 等 改 片 建 区 后 新 设 建 计 污 规 水 模 管 20 网 0m 29 3 . / 0 d 0 。 km，其中新建dn110污水管5.80km，dn160污水管2.75km，dn200污水管0.57km，DN300污水干管4.36km，D 务 N400污水干管8.12km，DN200压力管7.4km,以及建设配套泵站2座,化粪池56座，隔油池32座。改扩建 序号 招标项目名称 招标内容 招标方式 招标文件计划发布时间 拟交易场所 合同预估金额(万元) 备注 招 项 标 目1 城 建 口 设 县 项 东 目 安 （ 及 一 河 期 鱼 ） 片区污水管网 工程施工 公开招标 2026-09 城 易 口 中 县 心 公共资源交 3400.00 本 暂 为 计 定 准 划 ， 。 表 最 所 终 列 以 招 实 标 际 项 招 目 标 信 时 息 的 均 信 为 息 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3074602.html 商 cqdingjiu 2026.08.21 10:07:01 道 管 国 中</t>
@@ -4414,9 +5602,13 @@
         </is>
       </c>
       <c r="O71" t="n">
-        <v>0</v>
-      </c>
-      <c r="P71" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4449,16 +5641,24 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路长4000米，包括道路、综合管网等基础配套设施等。</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等</t>
+        </is>
+      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t>阀门产业园(管网改造)项目招标公告 阀门产业园（管网改造）项目招标公告 1.招标条件 本招标项目 阀门产业园（管网改造）项目已由垫江县发展和改革委员会以垫江发改委发【2022】459 号（批文 名称及编号）批准建设，项目业主为 垫江县丹香建设有限公司，建设资金来自 自筹资金 （资金来源）， 项目出资比例为 100% ，招标人为 垫江县丹香建设有限公司。项目已具备招标条件，现对该项目的施工进 行公开招标，评标办法采用经评审的最低投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 重庆市垫江县高新区县城组团 2.2 项目概况与建设规模： 场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路 务 长4000米，包括道路、综合管网等基础配套设施等。 2.3 本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元 商 2.4 招标范围： 包括土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等。具体详见施工图和 工程量清单。 道 2.5 工期要求：建设工期180日历天 缺陷责任期要求：24个月 管 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 国 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 中 4.1.1 本次招标要求投标人具备的资质条件： 具备建设行政主管部门颁发的有效的市政公用工程施工总承包叁 级及以上资质 ； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标 不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （垫江县）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（垫江县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资 源交易监督网、重庆市公共资源交易网（垫江县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 4.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）本项目招标公告网页下方“我要 提问”栏提出疑问，提问时间从本公告发布至2026-08-24 09:00:00前。 4.3招标人应于2026-08-24 23:59:59前在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-18 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 垫江县丹香建设有限公司 代理机构: 重庆博钰大数据科技有限公司 地 址: 地 址: 重庆市垫江县桂溪街道南内街88号 网 邮 编: 邮 编: 项目负责人: 熊老师 项目负责人: 郭威 电 话: 023-74630098 电 话: 023-74692498 务 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 商 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 道 2026年08月18日 信息来源:https://www.chinapipe.net/project/d3074578.html cqdingjiu 2026.08.21 10:07:02 管 国 中</t>
@@ -4470,9 +5670,13 @@
         </is>
       </c>
       <c r="O72" t="n">
-        <v>0</v>
-      </c>
-      <c r="P72" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>重庆, 管网改造, 投资金额, 产品种类</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improve Chongqing district recognition
</commit_message>
<xml_diff>
--- a/site/matches.xlsx
+++ b/site/matches.xlsx
@@ -606,8 +606,16 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>璧山区</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>璧山区</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。</t>
@@ -826,8 +834,16 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(二标段)，包括田块整治、灌溉与排水、田间道路、地力提升和其他工程。</t>
@@ -1350,8 +1366,16 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>新建50m³蓄水池4口、取水池2座；新建50m³/d-100m³/d水厂2座；改造100m³/d-300m³/d水厂5座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设施。</t>
@@ -2154,8 +2178,16 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
           <t>本项目主要涉及室外蒸汽管道φ219x6mm的安装，管道材质为20#，地上敷设，蒸汽管道运行压力1.08MPa，管道设计压力1.2MPa。蒸汽管道系统包括从锅炉房分汽缸到6#和8#车间分汽缸的所有蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温工作。还包括钢结构桁架工程的采购、运输、制作、安装、防腐工作，以及管道附件及控制系统的采购、运输、安装、接线等工作。此外，还需要进行调试与验收，确保蒸汽管道系统能够正常使用并备案。</t>
@@ -2222,8 +2254,16 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>巴南区</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>巴南区</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>完成重庆国际生物城配套公寓项目（民用1020户）天然气表后管道定制化服务。（含安装燃气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个，其它配套管件及辅材，墙体管道暗埋等）</t>
@@ -2426,8 +2466,16 @@
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>永川区</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>永川区</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>蒸汽管道改造</t>
@@ -2646,8 +2694,16 @@
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>大渡口区</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>大渡口区</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr">
         <is>
           <t>重庆市大渡口区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防护工程施工劳务招标。</t>
@@ -3458,8 +3514,16 @@
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>北碚区</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>北碚区</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供水管网68.5km及其附属设施。</t>
@@ -3678,8 +3742,16 @@
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>涪陵区</t>
+        </is>
+      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>整治De315原水管长1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。</t>
@@ -4118,8 +4190,16 @@
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>石柱土家族自治县</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>石柱土家族自治县</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
           <t>本次修复选择开挖换管：开挖约80米，2孔110波纹管、2孔蜂窝管，新建两通信手控井。</t>
@@ -5082,8 +5162,16 @@
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>大渡口区</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>大渡口区</t>
+        </is>
+      </c>
       <c r="J64" t="inlineStr">
         <is>
           <t>安装部分包括材料验收、运输及履带式挖掘机及人工布管、管道管件安装、新旧管道的碰口、安装DN400直埋球阀1座、管道和商焊口的除锈及防腐、管道下沟后15KV电火花检测、管道的清管、强度及严密性试验、警示带敷设和线路标志桩（砖）安装、监检手续等。土建部分包括清表、扫线、平整场地、沟槽、基坑、阀井砌筑、回填土方、余方弃置、人工开挖人行道（花台）、公路及路面恢复、其他线缆穿跨越工道程施工、交通组织、水工保护等。</t>
@@ -5150,8 +5238,16 @@
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>石柱土家族自治县</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>石柱土家族自治县</t>
+        </is>
+      </c>
       <c r="J65" t="inlineStr">
         <is>
           <t>2026-2027年度用户供水管道安装及管网抢（维）修服务</t>

</xml_diff>

<commit_message>
Apply plastic pipe scoring rule
</commit_message>
<xml_diff>
--- a/site/matches.xlsx
+++ b/site/matches.xlsx
@@ -566,11 +566,11 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>重庆, 管材, 询比采购</t>
+          <t>塑料管不计匹配分</t>
         </is>
       </c>
     </row>
@@ -4294,11 +4294,11 @@
         </is>
       </c>
       <c r="O52" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标</t>
+          <t>塑料管不计匹配分</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 改造, 配水主支管道, 更换配水主管网, 抗菌耐磨涂塑钢管, PE管, 泵站改造, 集成泵站, 蓄水池整治, 测控井</t>
+          <t>重庆, 管材招标, 改造, 配水主支管道, 更换配水主管网, 抗菌耐磨涂塑钢管, 泵站改造, 集成泵站, 蓄水池整治, 测控井</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>涪陵区, 珍溪镇, 农村供水, 提升工程, PE管, 衬塑钢管, 水泵, 不锈钢水箱, 减压阀, 排污阀</t>
+          <t>涪陵区, 珍溪镇, 农村供水, 提升工程, 衬塑钢管, 水泵, 不锈钢水箱, 减压阀, 排污阀</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 雨水管网, 高密度聚乙烯, HDPE, 钢筋混凝土管</t>
+          <t>重庆, 管材, 招标, 雨水管网, 高密度聚乙烯, 钢筋混凝土管</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add positive match workbook download
</commit_message>
<xml_diff>
--- a/site/matches.xlsx
+++ b/site/matches.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>PDF来源网页链接</t>
+          <t>产品用量</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
@@ -560,11 +560,7 @@
           <t>中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管 材询比采购公告 中铁十一局集团有限公司建安分公司招标采购中心就中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房 及配套综合交通枢纽工程CQZSG-2标段项目经理部管材组织询比采购，诚邀有意向的合格供应商参与报价。 一、项目概况及询比采购内容 1.1项目概况 网 （1）新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程位于重庆市中心渝中区中部，具体位置为菜园 坝立交桥以西，龙家湾隧道以东，菜袁路以北，王家坡以南。正在建设的地铁18号线贴临站房北侧，地铁26/27 号线从站区地下通过。项目共划分为4个施工标段，CQZSG-1标段：为国铁站房、地铁站台区域；站北路密不可 分的边坡及场坪工程，包含土石方工程和边坡支护工程，不含机电工程，由中铁建设承建。CQZSG-2标段：为 务 枢纽配套工程，地铁区间、西广场、成都局剩余还建，由中铁十一局承建。CQZSG-3标段：地铁区间、CTC、 站场、东广场，由中铁建工承建。CQZSG-4标段：人防车库、铁路自营车场、综合开发生产配套房屋等，由中 铁二局承建。 （2）标段概况：我方负责新建重庆至黔江铁路重庆站站商房及配套综合交通枢纽工程CQZSG-2标段全部施工内容 （简称B区），主要包含：（1）B区投影范围内盖板以下27号线、26号线明挖区间基坑支护、土石方、区间主体 结构及配套防水、综合接地工程（不含砌筑墙体、装饰装修和机电安装工程），以及承轨层以下市政排水 涵DK1+196（196m）和行包通道；（2）轨道交通26号线暗挖隧道预留工程，其中26左线487m，26号右线408m； （3）站北路E、F、H连接匝道工程，其中E匝道道247m、F匝道285.5m、H匝道174m；（4）B区盖板及以上还建房 屋，其中西侧盖板约3.56万㎡，还建房屋等总建筑面积约3.50万㎡。 1.2询比内容 详见拟采购货物一览表 管 二、供应商资格要求 2.1供应商必须是“中国铁建云链平台”注册并通过审核的供应商。 2.2本次询比采购不接受国被列入“《2026年中国铁建合作方警示名录》、《中铁十一局集团有限公司不良行为供 应商名录》、《JD采购网失信名单》（此项核查针对JMRH项目）”中的供应商,不接受近一年内在铁路建设工程 网公布有违法行为记录及物资供应不良记录、被中国铁路总公司限制投标或已清退出铁路市场的供货商（此项 核查针对铁路站房项目），不接受在铁建云链平台被标记的不良行为供应商。 中 2.3供应商在报价时，如是法定代表人签字的需提供法定代表人身份证复印件、如是法人授权代理人签字的需提 供授权委托书及被授权人身份证复印件。 2.4询比响应供应商需提供营业执照复印件。 2.5其它要求：提供样品、每批次货物必须附符合规范要求的出厂质量检验报告、型式检验报告及合格证或吊牌 等质量证明文件，甲方凭此报告检验质量。 2.6袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠像胶带，另配堵头。 三、拟采购物资及相关要求 3.1拟采购物资一览表 交 序 物资 型号 单 项目 货 交货日 数量 备注 号 名称 规格 位 名称 地 期 址 重 直 庆 径6:0mm 市 包含车 PVC 批次交 壁 渝 丝、黑 1 （袖 米 7100 货与零 厚4:-45.mm 中 色胶布、 阀管） 星交货 单节 新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程 区 管筛、 （具体 长4m CQZSG-2 标段项目经理部 菜 管箍、 以项目 园 堵头等 通知为 坝 一切相 准） 直 网 重 关费用 2 PE管 米 7100 径2:5mm 庆 站 合计 14200 务 3.2技术规格书： 按询比文件第二章项目技术规格书执行 商 3.3结算和付款 3.3.1采购物资报价规则： 道 固定价格。 3.3.2付款方式 （1）货款支付方式：支付方式包管括但不限于银行转账、银行汇票、银行本票、支票、银行承兑汇票、商业承兑 汇票、财务公司票据、供应链票据、其他数字化信用凭证，票据贴息费用由 供货单位 承担。 （2）付款周期：本合同无预付款。甲方在收到乙方提交的合规增值税专用发票，并经税务机关认证通过后次月 支付乙方上月供应期所国供合格物资70%货款，全部货物供应完毕后三个月内付至95%，剩余货款暂时扣留作为质 量保证金，供货完毕后，由乙方提交结算确认单，经甲方审核通过后做最终结算，待所有物资验收合格后12个月 内无息付清。 （3）逾期付款约定：如甲方付款逾期，双方秉持“长期合作，友好往来”原则，在逾期付款行为发生后一年内 中 乙方不向甲方收取逾期付款利息。若一年甲方仍未支付款项，需向乙方支付逾期付款利息，逾期付款利息起算 时间为全部款项到期之日一年后至付清之日，逾期利息的利率为合同订立时中国人民银行授权全国银行间同业 拆借中心公布的一年期贷款市场报价利率(LPR)1倍。 3.4拟采购物资相关的要求 3.4.1本次询比为整体采购，询比响应供应商报价时须写明单价、到站价和运距，报价包含货物制造、运输、装卸、 售后服务等交付采购人使用前所有可能发生的费用，收到报价后不再增补任何费用。 3.4.2交货期：按照采购人规定的期限内分批次运抵交付。 3.4.3供货地点：甲方指定的甲方所属 中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通 枢纽工程CQZSG-2标段项目施工现场。 3.4.4询比响应供应商必须保证产品的质量及售后服务。询比响应供应商提供的货物制造标准及技术规范等，必须 符合最新相关国家标准、部颁标准相关标准和规范的要求，进场提供相关检验检测报告。 3.4.5采购方在确定成交供应商后有权对成交产品的结构、规格做适当调整，调整内容将以工作联系函形式提前发 至供应商。 3.4.6售后服务：本批采购货物若在验收阶段出现不符合规格或质量标准，供应商必须接受退货要求，并在采购人 规定期限内等量补运合格产品，若未按时交付影响采购人使用，供应商必须承担由此给采购单位造成的后续经 济损失。 3.4.7报价方不得虚报各项技术指标，所供货物若不能符合技术要求，成交供应商必须接受全额退还货款，并承担 由此给采购单位造成的经济损失。 3.4.8验收方法及标准 （1）验收依据：询比采购文件、厂家货物技术标准说明及国家有关的质量标准规定，均为验收依据。 （2）货物验收：货物运抵采购人指定交货处后由双方对照采购清单及技术要求进行验收。 （3）其它要求：每批次货物必须附符合规范要求的出厂质量检验报告、型式检验报告及合格证或吊牌等质量证 明文件，甲方凭此报告检验质量。 网 （4）2.6袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠像胶带，另配堵头。 四、报价文件递交 务 4.1此次报价供应商需制作电子报价文件，在递交截止时间前线上递交报价文件。 4.2报价文件递交截止时间：2026年08月24日15时00分。 商 4.3报价文件递交地点：中国铁建云链平台（www.crccep.cn），供应商须登录该平台，在报价文件递交截止时间 前完成所有报价文件资料的上传。 五、发布公告的媒介 道 本次询比公告发布媒体:中国招标投标公共服务平台(www.cebpubservice.com)、中国铁建云链平台（www.crccep.cn） 上同时发布。 管 六、联系方式 1.采购组织单位：中铁十一局集团有限公司建安分公司招标采购中心 地 址：湖北省武汉市国武昌区丁字桥路47号 联 系 人：张先生 联系电话：027-87258521 中 电子邮件：2454774350@qq.com 2.采购人：中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程 CQZSG-2 标段项 目经理部 地 址：重庆市渝中区菜袁路59号 联 系 人：金先生 联系电话：16607273445 电子邮件：2285445503@qq.com 2026年08月21日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3077066.html cqdingjiu 2026.08.21 10:06:40</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3077066.html</t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>0</v>
       </c>
@@ -636,11 +632,7 @@
           <t>璧山项目钢筋混凝土管询价公告 本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用 地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行 建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉 泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含 市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范 围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期 实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。 网 登录地 mhem&amp;cNh6e0&amp;ce2C2m3s1e71=a64so0d9FAe=0903%e08005206E%6772dm6=%82he29&amp;=cI8p9eeyAs%7t?E%5lB%1iB%a1DetE%c9eweNAi%1iotvB%n/9cE%7.cBe9%ccAiE%p.E%s9%/29址/A%2:：psE%7tAhtD%B8%E%6B%7B%7E%5%78D9%E%5C9%F%9E%7AE%A%1E%9%78%78E%8B%4AD%N&amp;8E%6m657optUa3%6=6290%e3ni51B%5917E%443d6=E%862B%I8eAc%A1iD&amp;88no%tE%4BA%A%4E%7AC%AC%E%4BA%C8%E%8%88AA%E%5A8%A%1E%5B%7A%5E%7A%8B8%E%5B%1%08E%6C9%%98E%9%99%09E%5%58AC%E%5F%8B%8E%8A%5BF%E%9%38A%8EF%BC%%88E%5B9%BD%E%9%99%58EF%BC%%98E%6%59B%0E%5AD%%79E%7BB%F%8E%6B%5E8%E%4BA%A%7E%4B%8A9%E%5B9%AD%E%5C8%BA%E%9%58D8%E%5A%5%79E%9A%1B%9E%7B9%AE%EF%BC%%88E%8A%5BF%E%7%98%78E%5C8%BA%EF%BC%%98E%9A%1B%9E%7B9%AE%E%7=BgB&amp;upC%a=sod&amp;euF%pN=8Flk&amp;cmsusheaE%c7=te%0a9m%6he=8tT&amp;cpS7eeyeE%s9sha%&amp;3c2845d5=pur5A6I&amp;8optUni 信息来源:https://www.chinapipe.net/project/d3077008.html 务 cqdingjiu 2026.08.21 10:06:40 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3077008.html</t>
-        </is>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
         <v>70</v>
       </c>
@@ -712,11 +704,7 @@
           <t>中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目(二期)临水临电材料采购公告 物资采购 【招标公告】中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目(二期)临水临电材料采购 招标编号：cscec2026081900001246027 项目：重庆市第四人民医院科学城院区建设项目（二期） 发布时间：2026-08-20 17:52:30 报名截止：None 区域：重庆市市辖区沙坪坝区 招标品类：其他类 招标（资格预审）公告 网 中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料采购 采 购 文 件 务 采 购 人： 中国建筑第七工程局有限公司 日 期： 2026年8月 商 目 录 一、响应须知 道 二、评审办法 三、响应注意事项 管 四、响应文件的上传 五．响应文件 六、物资设备合同 国 一、响应须知 【公司总部供应链中心业务监督电话：17516461564】 中 1、工程概况： 工程名称：临水临电材料采购 采购名称： 中国建筑第七工程局有限公司重庆区域暨重庆市第四人民医院科学城院区建设项目 (二期)临水临电 材料采购 采购编号： cscec2026081900001246027 项目地址： 重庆市 工程内容：重庆市第四人民医院科学城院区建设项目 (二期)建筑总用地面积15214.5平方米；总建筑面积65020平 方米，其中住院楼22229.9平方米，实验教学楼8103.6平方米，院内生活楼5830.59平方米，高压氧舱315.53平方米， 地下车库28540.38平方米，以及给排水工程、强电工程、弱电工程、消防工程、暖通工程、总图工程等。为参考。 （说明：描述本工程概况）。最终工程规模及内容以上级部门及采购人确定为准。 采购概算金额：135万元（含税）【采购概算金额视为最高采购限价，响应人响应报价高于最高采购限价的，作 无效响应处理】。 2、采购范围及相关要求： （1）资格审查方式： 资格后审 （2）采购联系人：项目联系人： 修经理 ，电话： 17838218888 ，地址：重庆市 公司联系人： 苟经理 ，电话： 19828530610 ，地址：四川省青白江国际贸易产业园10幢 （3）采购内容： 临水临电材料 （4）工程价款支付： 月结方式，即每月20日结算（遇节假日顺延），次月25日前（结算日后35日历天内），乙 方提供与结算等额增值税专用发票后，支付至前月结算额的70%（遇节假日顺延），最终结算办理完毕6个月后 付至最终结算价款的 97%，剩余3%质保金在质保期满后30日内无息支付。（质保期自全部货物供货完毕且验收 合格日起1年计算）（支付工程款时均应扣除根据采购合同应予扣除的其它金额。） 网 3、响应方式： （1）响应保证金缴纳方式 务 响应保证金采用保证金现金或购买保证金保险（二选一）两种支付方式，支付成功后点击页面【去响应】按钮， 响应人方可正常响应。 方式一：保证金现金缴纳： 商 1、本次采购的响应保证金为/元。 2、保证金收款账户信息请参见云筑网保证金支付页面信息。 道 页面显示账户只对公办理，不接受个人汇款，响应人以响应人基本账户或对公账号转账；响应人转账时务必备注 “交易识别码”（具体操作详见附件《供应商保证金操作手册》或可拨打云筑客服电话：4006-818-555） 方式二：保证金保险缴纳： 管 1、保证金保险可替代保证金，购买后无需再缴纳保证金，响应人可通过“云筑网”购买，响应保险费不退 还；(具体操作详见云筑网上传附件《供应商保证金操作手册》） 2、如发生扣除保证金国情况，保险公司按照保险合同约定向采购单位赔偿相关款项后，保险公司代位取得向响应 单位追偿的权利，响应单位应在规定时间内向保险公司支付相应追偿款。 以下情况可免缴本采购项响应保证金： 中 ①工程局A级分供商。 发生以下情况，响应保证金不予退还： ①响应截止后响应人撤销响应文件的，采购人可以不退还响应保证金。 ②成交人无正当理由不与采购人订立合同，在签订合同时向采购人提出附加条件，或者不按照采购文件要求提 交履约保证金的，取消其成交资格。 （2）采购文件领取事宜：响应人根据采购公告内容领取采购文件，然后根据采购文件要求，进行响应，一经报 价即认为响应人对采购文件已作出实质性响应。 （3）采购文件的澄清与修改 ①采购文件的答疑：如响应人发现采购文件有不清楚的地方或对内容有疑问，要求澄清和解答的，均应在距响 应截止时间2天前向采购人提出答疑，采购人应解答响应人提出的问题。 ②采购人允许响应人在响应截止日期之前对云筑网响应进行修改，但必须在响应截止时间之前完成云筑网响应， 逾期未响应的，则视为无效响应。 （4）（4）响应文件递交事宜 采用云筑网电子响应。 4、评审： （1）评审方法：本次采购拟选出 1 名成交人，区段划分：（如选2个及以上，应明确划分各成交人分供范围及工 程量，成交人按照最终排名顺序享有优先选择权）。采用经评审的（原则上应选择合理低价法），在响应文件 能够满足采购文件实质性要求的响应人中，评审出响应价格合理低价的响应人，但响应价格低于其成本的除外， 具体由采购评审小组在评审会上商定。 （2）响应人有下列情形之一的，取消成交资格： ①成交人在成交后拒签合同； 网 ②成交人未按约定缴纳履约保证金。 采购人： 中国建筑第七工程局有限公司 务 采购时间：2026年8月 二、评 审 办 法 （一）、评审依据 商 1、采购文件 2、响应文件 道 3、评审办法 （二）、评审小组 管 1、评审小组成员：（评审小组应由5人及以上单数评审专家组成，项目负责人必须参与评审。与分供商存在利害 关系的应回避。） 2、小组成员负责根据国评审办法及标准开展评审工作。 3、与响应人有利害关系的，不得进入评审小组。 （三）、评审原则 中 （1）采取经评审的合理低价法：从满足采购文件实质性要求的响应人中，选择合理报价中最低者（不合理低价 除外）为成交分供商。 （四）、初步评审 有效分供商（资审通过并参与有效报价的分供商）数量不少于N（拟选分供商数量）+2家。（询比采购和竞价采 购要求，其他采购方式参照采购管理办法，下同） 出现以下情形的，响应无效。 1、未按要求缴纳响应保证金的。 2、未按要求完成线上响应的。 3、未响应采购文件的实质性要求和条件的。 4、响应人提供虚假资料、隐瞒误导采购的。 5、响应人以他人名义响应或者以其他方式弄虚作假，骗取成交的。 6、响应人ip重复、涉嫌弄虚作假或串通交易行为的。 7、采购文件或法律规定的其它情形。 （五）、详细评审 1、评审：以云筑网填报数据为准。 2、排名：对进入详细评审的响应人响应报价进行汇总后，按响应报价由低到高进行综合排名。 若出现响应人响应报价相同时，按其年度供应商考评评级高低优先排序，若仍相同，可再选用以下进行情况排序 （根据情况自行排序）。 网 ①近三年工抵房金额； ②具有绿色节能环保材料设备； 务 ③云筑网显示的该响应人响应时间等。 1）、采购概算金额（见采购公告）视为最高采购限价，响应人响应报价高于采购概算金额的，作无效响应处理。 响应人响应报价低于成本的，经评审小组评审确定后，作无效响应处理。 商 2）、在评审过程中，评审小组可以要求响应人对所提交的响应文件中含义不明确、表述不一致或者有明显笔误、 文字和计算错误的内容作出必要的澄清、说明或者补正，该澄清、说明和补正属于响应文件的组成部分，须经 采购授权代表书面署名确认，不得改变响应文件的实质性内容，且须经评审小组一致同意。评审小组不接受响 应人主动提出的澄清、说明或补正。 道 3）、经以上评审，有效响应人数量仍须满足“有效分供商（资审通过并参与有效报价的分供商）数量不少于N （拟选分供商数量）+2家”，否则本次采购按废止处理（成交单位数量为“N”）。 管 4）、废止后重新发起采购，需经调查核实后，视具体调查核实结果决定是否准予原响应人参与新发起的采购响 应。 （六）、确定成交候选单位 国 多轮次公开竞争报价：（说明：如需要(应视采购标的物及响应报价情况)进行多轮次公开竞争报价的，应按详细 评审的排名顺序确定一定比例(首轮最高价不得进入二次报价)的有效响应人进行后续轮次报价，总轮次不超过3轮 （竞价采购）。 中 报价规则：响应人提交的首轮报价作为后续报价基准；后续轮次总报价不得高于前轮报价，若设置参考价，单 项报价不得高于参考单价。否则该轮报价无效；最终轮次报价提交后不得撤回或修改（以系统记录为准）。 晋级规则：每轮报价截止后，采购人按报价从低到高排序；出现相同报价时，依次比较：（1）资源库等级；（2） （参考上述第五条第2点，以优质优价为原则，优先选用具备相应能力的本级及上级A级分供商） 成交机制：最终按末轮有效报价的从低到高排序；当最低报价出现多家时，可自主决定成交人。 最终按照排名顺序拟定有效响应人作为成交候选单位，具体成交候选单位数量由评审小组根据采购文件确定。 成交候选单位经审批后作为最终成交单位。 成交候选人放弃成交、因不可抗力不能履行合同、不按照采购文件要求提交履约保证金，或者被查实存在影响 成交结果的违法行为等情形，不符合成交条件的，采购人可以按照评审小组提出的成交候选人名单排序依次确 定其他成交候选人为成交人，也可以重新采购。 （七）、其他事项 1、因响应人原因造成其自身未响应采购要求及未能成交等情况，由响应人自行承担相应责任及损失，与采购人 无关。 2、本采购文件中的合同范本即实际签约合同范本，双方均不允许以任何理由更改合同内容。 三、响应注意事项 1、若响应人对采购文件中之任何内容有不理解之处，须立即联系采购人，以便在响应截止日期之前能予以解释。 2、采购人不保证一定要接受最低价成交，不论响应结果如何响应人的响应文件均不退回，且不对未成交单位做 任何解释。 3、响应人在响应之前，对本采购项的分包条件均已了解，响应即认为已详细了解。 4、采购人对响应人进行考察时，响应人应提供便利条件。 5、本次采购的最终解释权在采购人。 网 四、响应文件的上传 1需上传的响应附件（未上传视为不响应采购文件）有： 务 1.1.《响应函》 1.2.《响应承诺函》 1.3.法定代表人身份证明（格式）； 商 1.4.授权委托书（格式）（若若为法定代表人响应则可不提供）； 1.5.报价清单明细（盖章版） 道 1.6金融工具支付方式及优惠措施 1.7.响应保证金汇款凭证扫描件或免缴证明（云筑网平台缴纳的无须提供）（若需） 管 六、响应文件格式 一、封面（格式） 国 中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料采购响应文件 响应内容：临水临电材料采购 中 （编号：cscec2026081900001246027） 响应人：（盖章） 法定代表人 或授权代理人（签字盖章）： 响 应 函 致：中国建筑第七工程局有限公司 1、经勘察了本工程现场,并仔细研究了响应须知、合同协议条款、合同条件、采购图纸、工程规范、地质勘察报 告、工程量清单、响应答疑、及其他有关采购文件后，我公司愿以我公司云筑网所上传的含税综合单价，并按 采购文件所要求的条件承包在规定工期内完成重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料的施 工、竣工并补充其任何缺陷。 2、我公司保证本工程质量必须：达到符合工程所需材料质量验收标准、设计、合同及有关工程施工及验收规范 的要求标准。 3、一旦我公司的云筑网响应内容被接纳，我公司将在收到成交通知书后按贵公司的要求开始施工，我公司保证 于承诺的工期内或双方议定的工期内完成并交付本合同中规定的整项工程。 4、我公司同意在本区段的正式建设工程施工合同签署之前，云筑网响应将始终对我公司具有约束力，并可随时 被贵公司接受。 5、我公司知道：云筑网报价及云筑网响应的其他部分构成我公司向贵公司的要约，贵公司如发出成交通知书则 成交通知书及云筑网响应、采购文件将构成约束我们双方的合同，如果我公司在接到成交通知书后，没有按贵 公司要求的时间签署正式合同或坚持提出附加条件，那么我公司同意贵公司有权另选成交单位并向我公司追讨 有关损失。 6、我公司知道，贵公司并无义务必须接受所收到的价格最低的或其他任何响应书。 7、云筑网响应内容已考虑了贵公司向我公司发出的关于采购文件的相关答疑，网补充通知（如有的话） 8、云筑网响应效力优先于同时提交的任何响应文件的其他组成部分。 响应人： （盖章） 务 日 期： 年 月 日 响应承诺书 商 致：中国建筑第七工程局有限公司 我系有幸参与贵公司 重庆市第四人民医院科学城院区建设项目 (二期)临水临电材料的响应，我公司经研究决定， 在此郑重承诺： 道 1、我公司在响应过程中已完全了解并掌握了采购内容、合同条件及施工现场等情况。确保云筑网响应报价操作 为本公司自己操作，如响应后发生非本公司操作的情形，本公司承担相应违约责任。 管 2、我公司已经详细阅读该采购文件所有内容，充分领会并完全接受采购文件所述响应人应尽的实质性的权利与 义务。我公司保证不会对采购文件产生不利于双方友好合作关系和将增加贵公司采购范围内经济支出的重大误 解。 3、我公司确认，贵公国司发出的采购文件所有内容为不可割裂的整体。 4、我公司保证成交后不会对成交价格提出任何异议，更不会以任何理由要求贵公司针对成交范围的价款要求额 外补偿。不会以不了解采购文件、合同文件为由或曲解、片面理解采购文件、合同文件或割裂采购文件、合同 文件，断章取义，向贵公司提出任何补偿要求。 中 5、在本合同的履约过程中，如因我公司的供货或质量原因导致贵司损失，我公司保证承担因此而给贵公司带来 的所有经济上的损失。 6、我公司将本工程作为重点项目对待，保证不会出现供货能力不能满足施工需要的现象。为满足本工程业主及 贵公司在质量、进度、安全、环保上的要求，我公司将采取一切措施保证物资设备生产、供应、租赁，运输等 均满足贵公司的要求，并保证不会因此而向贵公司提出增加任何补偿要求。 7、我公司承诺无论本工程最终的成本状况如何，将不会违背合同基本原则而向贵公司要求增加或补偿合同文件 约定以外的任何费用。 8、我公司认为，贵公司可以就物资设备采购数量或租赁时长进行调整，并且此种调整不构成我公司的索赔理由。 响应人：（盖章） 法定代表人或 其授权代理人：（签字或盖章） 日 期： 年 月 日 响应人名称：【全称】 单位性质： 地 址： 成立时间：年月日 经营期限： 姓名：性别：年龄：职务：系（响应人名称）的法定代表人。 网 特此证明。 响应人：（盖单位章） 务 年月日 授权委托书 商 本人（姓名）系（响应人名称）的法定代表人，现委托（姓名）为我方代理人。代理人根据授权，以我方名义 签署、澄清、说明、补正、递交、撤回、修改中国建筑第七工程局有限公司重庆市第四人民医院科学城院区建 设项目 (二期)临水临电材料采购（采购项目名称）响应文件、签订合同和处理有关事宜，其法律后果由我方承担。 道 委托期限：本授权书于年月日签字生效，至本次采购期结束为止。授权期限内无特殊情况不变更合法授权代理 人。 代理人无权转委托。 管 特此声明。 响应人：（盖章） 国 法定代表人：（签字） 身份证号： 中 授权代理人：（签字） 身份证号： 联系方式： 日期： 年 月 日 备注：法定代表人和委托代理人必须在授权书上亲笔签名，不得使用印章、签名章或其他电子制版签名,同时附 法定代表人和授权代理人身份证复印件（正反面，加盖公章） 报价清单明细 不 含 含 不含 计量单 税 税 含税 备 序号 材料名称 规格型号 数量 税 税合 税额 位 率 单 合价 注 单 价 价 价 1 镀锌钢管 DN100*4.0 米 500 2 镀锌钢管 DN150*4.5 米 250 3 镀锌钢管 DN65*3.25 米 650 4 镀锌钢管 DN50*3.25 米 800 5 PE管 DN100*1.6MPA 米 450 6 PPR管 DN50*1.6MPA 米 400 7 闸阀 DN100 个 22 8 闸阀 DN250 个 10 9 截止阀 DN50 个 42 网 10 截止阀 DN25 个 60 11 蝶阀 DN100 个 6 12 消防箱 800×1000×250mm 台 20 务 功率30kw,扬程144m，流 13 加压泵（变频控制） 台 1 量55m/h 14 橡塑保温材料 DN100*20mm 米 620 商 15 橡塑保温材料 DN150*30mm 米 280 16 橡塑保温材料 DN65*20mm 米 700 17 压线钳 CO-1000 个 1 道 18 污水泵 380V4KW=25米 台 12 19 污水泵 380V5KW=30米 台 7 20 热熔机 63-160 台 1 管 21 电工胶布 / 卷 200 22 高压自粘带 / 卷 120 23 水泵控制箱 / 个 8 国 24 PE聚乙烯管 DE110*1.6MPA m 560 25 PE聚乙烯管 DE75*1.6MPA m 420 26 PE聚乙烯管 DE63*1.6MPA m 480 中 27 PE聚乙烯管 DE32*1.6MPA m 750 28 PE球阀 DN25 个 6 29 PE球阀 DN50 个 6 30 PE球阀 DN100 个 5 31 镀锌桥架 200*100*1.2mm 米 1200 32 PVC排水管 DE300*5.0 m 180 33 PVC排水管 DE200*5.0 m 380 34 PVC排水管 DE160*4.0 m 486 35 PVC排水管 De110*4.0 米 560 36 PVC排水管 DE75*3.0 m 420 37 PVC排水管 DE50*2.0 m 660 38 PVC排水管 DE32*2.0 m 380 39 PPR给水管 De90*1.6MPA 米 440 40 PPR给水管 DE75*1.6MPA 米 360 41 PPR给水管 DE63*1.6MPA 米 450 42 PPR给水管 De50*1.6MPA 米 435 43 PPR给水管 De40*1.6MPA 米 315 44 PPR给水管 DE32*1.6MPA 米 520 45 PPR给水管 De25*1.6MPA 米 680 46 PPR给水管 De20*1.6MPA 米 370 47 橡塑保温板 平板×20mm m 15 48 橡塑保温板 平板×30mm m 28 49 保温胶 3公斤/桶 桶 25 网 50 PPR给水管接头 De75 个 30 51 PPR给水管弯头 De75 个 20 52 PPR给水管三通 De75 个 22 务 53 PPR给水管接头 De63 个 20 54 PPR给水管弯头 De63 个 15 55 PPR给水管三通 De63 个 15 商 56 PPR给水管接头 De50 个 17 57 PPR给水管弯头 De50 个 22 58 PPR给水管三通 De50 个 17 道 59 PPR给水管接头 De40 个 14 60 PPR给水管弯头 De40 个 22 61 PPR给水管三通 De40 个 17 管 62 PPR给水管接头 De32 个 14 63 PPR给水管弯头 De32 个 14 64 PPR给水管三通 De32 个 17 国 65 PPR给水管接头 De25 个 22 66 PPR给水管弯头 De25 个 17 67 PPR给水管三通 De25 个 14 中 68 PPR给水管接头 De20 个 25 69 PPR给水管弯头 De20 个 17 70 PPR给水管三通 De20 个 22 71 PPR内丝直接 De25 个 17 72 PPR内丝直接 De20 个 84 73 球墨铸铁井盖 700*800*40T 套 22 74 球墨铸铁井盖 1000*1000*20T 套 20 75 球墨铸铁雨箅子 400*600*30 块 1750 76 球墨铸铁雨箅子 350*500*30 块 1200 77 高分子成品排水沟 300*300*1000 米 850 78 高压洗车机 380v/3KW 套 5 79 高压洗车机 380v/5.5KW 套 3 80 HDPE双壁波纹管 DN300 米 360 81 HDPE双壁波纹管 DN200 米 410 82 HDPE双壁波纹管 DN400 米 340 83 HDPE双壁波纹管 DN800 米 260 84 玻璃钢化粪池 20m 个 1 85 玻璃钢化粪池 50m 个 1 86 不锈钢消防水箱 12m 个 1 87 一级配电柜 2000*1200*500*630A 台 1 88 二级配电柜 800*600*210*250A 台 8 89 铜芯电缆线 YC3*16+2*10 米 60 90 铜芯电缆线 YC3*10+2*6 米 70 网 91 铜芯电缆线 YC3*6+2*4 米 70 92 铜芯电缆线 YC3*10 米 100 93 铜芯电缆线 YC3*6 米 100 务 94 铜芯电缆线 YC3*4 米 100 95 铜芯电缆线 YC3*2.5+2*1.5 米 100 96 聚录乙烯铝芯电缆 YJLV-22-4*185+1*95 米 50 商 97 聚录乙烯铝芯电缆 YJLY-4*25+1*16 米 90 98 聚录乙烯铝芯电缆 YJLY-4*35+1*16 米 100 99 聚录乙烯铝芯电缆 YJY-4*50+1*25 米 90 道 100 聚录乙烯铝芯电缆 YJLY-4*70+1*35 米 72 101 网线 Cat5e 米 100 102 铜芯电线 BV-2.5 米 400 管 103 铜芯电线 BV-4 米 300 104 铜芯电线 BV-6 米 200 105 铝芯电缆线 YJLV3*10 米 100 国 106 透明塑壳断路器 3P32A 米 34 107 透明塑壳断路器 3P63A 米 28 108 透明塑壳断路器 4P100A 米 26 中 109 透明塑壳断路器 4P160A 米 22 110 透明塑壳断路器 4P250A 米 20 111 透明塑壳断路器 4P400A 米 8 112 低压铝芯电缆 YJLV-4*300+1 米 20 113 低压铝芯电缆 YJLV-4*150+1 米 50 114 铝芯铠装电缆 YJLV-22-4*95+1*50 米 60 115 铜铝线鼻 300mm2 个 20 116 铜铝线鼻 150mm2 个 36 117 铜铝线鼻 95mm2 个 24 118 铜铝线鼻 50mm2 个 20 合计 0.00 0.00 0.00 1、综合单价：包括但不限于材料费、保险费、风险费、包装费、装车费、过桥过路费、管理费、检验费、技术 指导费、货到工地负责卸货堆入至指定地点等所有费用。本合同单价一次包死，在合同履行过程中不再做任何 调整。本合同的总价为暂估价，用方有权调整合同中材料计划或材料数量，材料数量和规格的调整，不影响本 合同单价及其他条款的执行。 2、计量方式：查看检测报告合格证，以实际验收通过数量计量。 3、付款比例：月结方式，即每月20日结算（遇节假日顺延），次月25日前（结算日后35日历天内），乙方提供 与结算等额增值税专用发票后，支付前月结算额的70%（遇节假日顺延）；供货完毕，验收合格，材料相关资料 （包括不限于合格证、质检报告等）移交甲方，且最终结算办理完毕6个月后付至最终结算价款的 97%；剩余3% 质保金在质保期满后30日内无息支付。质保期自全部货物供货完毕且竣工验收合格日起1年计算，支付工程款时 均应扣除根据采购合同应予扣除的其它金额。 4、付款方式： （1）现金支付:采用现金转账的模式支付； （2）非现金支付:包括不限于(1)金融工具支付:银行承兑汇票，商业承兑汇票，网应付账款保理，银行信用证，中 建财务公司承兑汇票。(2)工抵房支付。 5、响应报价表中所列数量的变动，丝毫不会降低或影响合同条款的效力。 务 6、整个合同执行期内，若遇市场价格下行，甲方有权做出价格调整，乙方应接受并重新签订补充协议确认价格。 若乙方无法接受新的低价，甲方有权重新选择其他能够响应该价格的供应商进行供货，乙方无条件同意。 响应人（加盖公章）： 商 法定代表人或授权代理人（签字）： 日 期：年月 道 金融工具支付方式及优惠措施 管 1、金融工具支付： 可接受金融工具支付比例累计为%，其中： ① 可接受的国银行承兑汇票比例%；贴息响应人自行承担。 ② 可接受的商业承兑汇票比例%；贴息响应人自行承担。 金融支付 ③ 可接受的应付账款保理比例 %；贴息响应人自行承担。 中④ 可接受的银行信用证比例%；贴息响应人自行承担。 ⑤ 可接受的中建财务公司承兑汇票比例为%；贴息响应人自行承担。 2、资产支付 资产支付 可接受比例为合同额的%。 3、优惠付款比例：按按照采购文件的付款比例，我方可优惠%。 4、如响应人提供其他由于采购条件的承诺，请逐项列示。 响应人（加盖公章）： 法定代表人或授权代理人（签字）： 日 期：年月 响应保证金汇款凭证扫描件或免缴证明（若需） 响应人（加盖公章）： 法定代表人或授权代理人（签字）： 日 期：年月 六、物资设备采购合同 合同编号：______________________ 物资采购与供应合同 （通用） 项目名称：【 重庆市第四人民医院科学城院区建设项目 (二期) 】 网 甲 方：【 】 乙 方：【 】 务 签订时间：【 】 签订地点：【 】 商 目录 1. 工程概况及供货范围 道 2. 企业性质 3. 合同价款 2 管 4. 质量要求 5. 供货时间及地点 6. 交货与验收 国 7. 结算方式及时间 8. 支付 中 9. 发票 10. 双方责任 11. 不可抗力 12. 权利瑕疵 13. 保密 14. 违约与赔偿 15. 联络与送达 16. 争议解决 17. 补充条款 18. 其他 物资采购与供应合同 甲方（买受人）：【中建七局安装工程有限公司 】 乙方（出卖人）：【 】 根据《中华人民共和国民法典》及有关规定，为明确双方权利、义务和责任，经双方协商一致，就甲方承包的 【高新LIVE（咸阳高新区租赁住房）建设项目】工程所用【 水电管材】采购与供应事宜签订本合同条款，愿共 同遵守。 1. 网 1.1 工程名称：【高新LIVE（咸阳高新区租赁住房）建设项目 】 1.2 工程地点：【陕西省咸阳市星火大道】 务 本合同供货范围为：【高新LIVE（咸阳高新区租赁住房）建设项目 】的【水电管材】供应（以下简称为“本合 同标的物”）。 1.3本合同标的物的数量为暂定量，乙方按附件1《计划采商购与供应物资清单》所列品种和规格供货，最终以经甲 方验收合格的实际数量为准。 2. 企业性质 道 乙方企业规模：大型 □中型 □小型 □微型企业 以上企业规模由乙方根据（1）工信部官网：“中小企业规模类型测试网址https://baosong.miit.gov.cn/ScaleTest。 （2）工信部微信小程序：“中小企业规模类型自测”两种渠道自测确定。 管 乙方应保证其企业规模的真实性。如乙方提供信息不实，经甲方查证后，将按照《中国建筑股份有限公司分供 商资源管理办法》中的《不良行为分供商禁用处理标准》第19项对乙方严格实施禁用管理。 合同价款 国 3.1 本合同采用第【 】种价格形式： （1）固定综合单价包干，价格不可调整。 中 3.2 本合同价款为各项货款之和，合同价款（含增值税）暂定：（大写）【 】（￥【 】元），其中不含税价款为 （大写）【 】（￥【 】元），增值税为（大写）【 】（￥【 】元），税率为【 】%。最终甲乙双方以实际验收 的数量结算。 3.3 本合同约定的不含税价款不因国家税率变化而变化，在合同履行期间，如遇国家的税率调整，则价税合计的 合同价款或货款相应调整，以开具发票时间为准。 3.4 本合同不含税价款仅指不包含增值税，除增值税外的其他全部税费（包括但不限于城市建设维护税、教育费 附加及地方教育费附加、个人所得税、合同印花税、企业所得税、车船使用税以及国家和地方规定的所有税费） 均包含在不含税价款中。 3.5 本合同标的物的计价、结算和支付货币均为人民币。 3.6 本合同标的物的计量单位为中华人民共和国法定公制计量单位（除技术规范标准另有规定外）。 3.7 本合同标的物的不含税单价，指运抵本工程施工现场甲方指定交货地点的综合单价，包括但不限于货物费、 加工费、包装费、人工搬运费（由乙方自行协调，甲方只进行指定场地和材料验收工作）、运输费、出厂检测费 （包括但不限于到场后的第三方检测费用）、装卸费、码放费、现场倒运费用，保险费、仓储费、驻厂监造费、 运输造成的道路污染的清理及维修费用、除增值税以外的税金、乙方合理的利润、管理费、市场价格波动带来 的风险、向有关部门缴纳的各项费用以及政策性文件所规定的各项应有费用等乙方履行本合同规定义务的全部 价款与费税。除本合同第3.1条约定的因素外，不含税单价不因政府政策变动、市场环境改变、税率调整等而调 整。 3.8 除合同条款另有约定外，本合同标的物的不含税单价已包含专利、专有技术以及技术秘密的使用费。 质量要求 4.1 乙方应在交货同时向甲方提供本合同标的物制造商出具的书面质量保证书。 4.2 本合同所采购与供应的物资，应符合现行中华人民共和国国家标准及行业或地方标准，行业标准或地方标准 高于国家标准的，执行行业标准或地方标准。各项技术性能指标经本工程所在地具有相应检测资质的专业机构 或单位检测中心检验必须符合相关标准要求。合同执行过程中，若出现新的国家标准、行业标准、地方标准， 则以更新后的标准为准。 网 4.3 乙方的物资供应与管理应符合国家有关环保法律、法规和甲方ISO14001环境体系及OHSMS18001职业安全健康 管理体系标准。 4.4 本合同标的物的质量保证期为最后一批货物验收合格之日起满【180】日。 务 4.5在合同履行期及质量保证期内，乙方无条件地向甲方提供缺陷产品的免费维修、更换等服务。针对甲方提出 的书面要求，乙方必须在3日内给予书面答复。如有必要，乙方在3日内指派专人到现场解决，因此产生的所有费 用均由乙方承担。 商 4.6 如缺陷产品经乙方进行免费维修和更换后仍无法达到甲方要求的质量标准时，甲方有权终止合同。终止合同 后，乙方需向甲方赔偿由于乙方问题造成的损失及其连带损失。如乙方借故推脱或拒绝甲方提出的维修、更换 等服务请求，甲方有权自行采购同等货物替代或委托第三方维修，实际发生的更换等或维修费用，从应支付给 乙方的任一期货款中扣除，并保留进一步索赔道的权利，乙方不得提出异议。维修或更换物资的质量保证期相应 延长6个月。 4.7 如因乙方产品质量导致工程出现质量问题，由此给甲方造成的一切损失由乙方承担。 管 4.8 其他质量要求：/。 供货时间及地点 5.1 供货方式：□按批次国供货 □一次性供货 5.2 通知方式：供货时间及数量以甲方书面通知为准，甲方可以选择通过电子邮件、微信、QQ等方式将物资采购 订单发送至乙方。紧急情况下，甲方可口头通知乙方发货，手续后补，乙方应予以确认。 中 5.3 供货地点：乙方负责送货至施工现场，卸至甲方指定的卸货地点【高新LIVE（咸阳高新区租赁住房）建设项 目】。乙方不得雇佣甲方在班人员及设备装卸货物。运输、装卸过程中发生的安全事故责任，乙方自行承担。 5.4 根据工程项目施工需要，甲方对所采购物资的数量和送货时间如有变更，应及时书面通知乙方，乙方按变更 后的数量和送货时间供货，货物单价不因货物数量和送货时间的变更而变化。 5.5 乙方应确保已经知悉货物运输的交通状况、交货卸车环境以及政府的交通管制政策措施，不得以此等理由要 求增加费用、减免责任、提出索赔、要求延长或变更供货期限。 交货与验收 6.1交货 6.1.1 除另有规定和协议要求外，乙方提供的全部货物须采用国家、企业、行业标准要求包装，具有足够的强度 及安全起吊标识，保证货物能够经受多次搬运、装卸、长途及短途运输的要求，并采取良好的防潮、防震、防 腐蚀、防爆及防止其它损坏的必要保措施。包装物的回收按以下第【 2】项方式执行：（1）不回收；（2）包装 物由乙方在交货时回收；（3）其它方式：【 /】。 6.1.2 装箱单应注明货物的名称、规格、型号、数量、质量、生产商、发货地、供货人、收货人、交货地、承运 人等，并在显著位置标明装卸警示标志。 6.1.3 乙方运抵甲方指定现场的物资，交货单据上应详细列明当次供应物资的名称、品牌、产地、生产厂家、规 格型号、计量单位、数量。 6.1.4 乙方应向甲方提交本合同标的物的技术文件，包括材质报告（物资质量检验报告）和出厂检验报告（合格 证），以及按照工程竣工验收规定及甲方要求，提供所有相关符合要求的资料。 6.1.5 乙方在首次供货前需提供样品，乙方须在样品和样品资料上加盖单位公章，样品经双方指定人员签字确认 后予以封存，在提交文件上注明与合同文件约定不同之处。 6.2.1 乙方须随货提供载有数量、规格等内容的送货单，否则，甲方有权对本批次货物不予验收确认，由此导致 的违约责任由乙方承担。乙方送货到交货地点后，甲方指定验收人员对产品的规格、尺寸偏差、外观、数量及 质量证明资料等进行查验。若产品的以上各项符合合同约定，则双方人员共同在收领单上签字确认。 6.2.2 甲乙双方在交货现场以 【 点数】方式进行数量验收。乙方应对在甲方工地网现场的验收数据进行确认。 6.2.3 进行数量验收的同时，甲方可以按照封存样品标准进行尺寸、外观质量验收，尺寸和外观质量符合要求方 可卸车，否则不得卸车。 务 6.2.4 外观质量符合要求的， 甲方可打开包装进行质量、性能检验或及时按规定取样送本工程所在地具有相应检 测资质的专业机构或单位进行检测。抽检未发现不合格产品不视为乙方供应产品全部合格，甲方有权随时将乙 方所供货物送到有检测资质的第三方进行检测。如检测合格，检测费用由甲方承担；如检测不合格，甲方可全 部退货，检测费用由乙方承担，并承担由此给甲方造成的一切损失。 商 6.2.5 甲方及工程监理（业主）的收货验收仅作为感观合格的依据，不能免除乙方对货物品牌真实性、内在质量 及使用功能所负的责任。如甲方、本工程建设单位或监理单位提出异议，乙方需参照有关标准规范，结合现场 情况解决。 道 6.2.6 若发现不合格产品，乙方必须及时（接到甲方通知后【 3】小时内），从甲方项目现场运走不合格品，甲方 不负有保管义务，不对不合格产品的损毁灭失承担人和责任，若超过【 12】小时乙方仍未运走的，甲方收取场 地租赁费（根据货物合理确定）【 1.0】万元/天，且不合格品的储存、装卸、运输等所有相关费用及风险由乙方 承担。 管 6.2.7 如因乙方产品问题造成甲方工期、质量、劳务等损失，全部责任均由乙方承担。乙方对甲方所提出的质量 问题有不同意见的，双方可送至双方共同选定的具有法定资质的检测机构检测，所产生的费用及责任由责任方 承担。 国 6.2.8 本合同的标的物所有权自【卸货完毕且经甲方验收合格】起转移。 结算方式及时间 中 7.1 过程结算：甲乙双方按以下第【 1】条约定的时间办理过程结算。 （1）每月20日结算（遇节假日顺延），每季度最后一个月的25日后支付当期货款额的70%（遇节假日顺延，乙 方提供与结算等额增值税专用发票），供货完毕，验收合格，材料相关资料（包括不限于合格证、质检报告等） 移交甲方，且最终结算办理完毕6个月后付至最终结算价款的 97%，余款3%（不计息）待质保期满无质量问题后 无息付清。（质保期为供货完毕且验收合格后2年）（支付工程款时均应扣除根据采购合同应予扣除的其它金额。 ）； （2）按节点结算，具体结算节点为：【 】。 7.2 最终结算：全部供货完毕后【 6个月后】日内，乙方应向甲方提供完整的结算资料，甲方在收到完整的结算 资料后【 5 】日内进行审核。 7.3 结算依据：包括但不限于物资采购与供应合同、乙方合法等额有效增值税发票（含税务机关代开）、产品合 格报告、项目授权人员验收单、送货单等有效材料。 7.4 乙方未按照约定的期限和甲方要求提供结算资料，或未委派专人与甲方办理结算，或提供的结算资料不齐全、 提供虚假资料的，经甲方催告后10个工作日内，乙方仍未按要求提供结算资料的，甲方有权不予办理结算并暂停 支付材料款，同时甲方可根据本合同、现有结算资料及乙方实际履约情况单方办理结算，确定结算价格，结算 对甲乙双方具有法律约束力。 支付 支付/√不支付预付款 8.1.1 预付款金额（或占合同价款的比例）：【 /】。 8.1.2 预付款的支付时间：【 /】，在乙方提交等额银行保函及增值税专用发票后，甲方向乙方支付预付款。 8.1.3 扣回预付款的时间、比例：【 /】。 8.1.4 乙方提交的银行保函有效期至预付款抵扣完为止，若预付款保函到期日前，预付款无法抵扣完毕，则乙方 应于预付款保函到期日前不少于10日及时办理保函延期，否则甲方有权暂停支付未抵扣完部分的货款。 网 / 8.2.1 货款支付，按以下第【 3】条约定的时间和比例支付。 务 （1）月度付款：甲方在次月的25日支付上月月度结算货款的【 / 】%。双方办理完毕最终结算后【 / 】（条款说 明：建议不超过60日，如超过60日，应当按照行业规范、交易习惯合理约定付款期限并及时支付款项）个日历天 内付至总结算货款（且不超含税合同价款）的【 / 】%。余款【 /】%作为质保金，在质保期届满后28日内付清； 或由乙方提供等同余款金额的质保保函（仅接受金融机构出具的无条件见索即付保函，质保保函格式以开函金 融机构标准格式为准），则双方办理完毕最终结算后【 /商】（条款说明：建议不超过60日，如超过60日，应当按 照行业规范、交易习惯合理约定付款期限并及时支付款项）个日历天内付清。 （2）节点付款：按节点支付（条款说明：此处需具体罗列每个付款节点及各节点对应的付款比例，节点结算完 成后约定支付期限应在60日内，如超过60日，道应当按照行业规范、交易习惯合理约定付款期限并及时支付款项）， 余款【 /】作为质保金，在质保期满后28日内付清，或由乙方提供等同余款金额的质保保函（仅接受金融机构出 具的无条件见索即付保函，质保保函格式以开函金融机构标准格式为准），则在最后一个付款节点付清。每次 付款前乙方应提供结算值【100%】的发票，否则甲方可拒绝付款。 管 （3）其他支付方式【每月20日结算（遇节假日顺延），每季度最后一个月的25日后支付当期货款额的70%（遇 节假日顺延，乙方提供与结算等额增值税专用发票），供货完毕，验收合格，材料相关资料（包括不限于合格 证、质检报告等）移交甲方，且最终结算办理完毕6个月后付至最终结算价款的 97%，余款3%（不计息）待质保 期满无质量问题后无息付清。（质保期为供货完毕且验收合格后2年）（支付工程款时均应扣除根据采购合同应 予扣除的其它金额。）国】 （4）甲方依合同约定确认的进度款仅为中期付款依据，不作为竣工结算的依据，且不视为对因变更调整的合同 价款、索赔的价款或费用以及其他约定的追加合同价款的确认。 中 8.2.2 甲乙双方协商一致同意本合同采用【银行转账支票、网银转账、银行承兑汇票、银行保理、商业承兑汇票、 国内信用证、应收账款电子凭证、抵房抵款及其他】常规支付方式的付款方式。付款过程中产生的贴息费用及 手续费由【乙方】承担。乙方委托专职收款人办理收付款业务，收款人必须取得授权 8.3 乙方指定以下帐户为收款帐户，甲方所有款项均需通过该帐户支付。如乙方变更收款帐户，应提前十五天以 上书面通知甲方，否则造成资金的损失由乙方自行承担，与甲方无关。 账户名：【 】 开户行：【 】 账 号：【 】 发票 9.1 乙方在向甲方请款时，应根据甲方确认的应支付金额开具合法、有效、完整、准确的增值税（请勾选：□专 用□普通）发票，计税方法为【□一般计税方法 □简易计税方法】，双方发票信息如下： 名 称 纳税人身份 □一般纳税人 □小规模纳税人（请勾选） 甲方 纳税人识别号 地 址、电 话 开户行及账号 名 称 纳税人身份 □一般纳税人 □小规模纳税人（请勾选） 网 纳税人识别号 乙方 地 址、电 话 开户行及账号 务 联 行 号 该开户行为乙方在税务局已备案的乙方单位账户。 9.2 任何一方如上述信息发生变更，应提前10日以书面方商式通知另一方。如一方未按本合同规定通知而使另一方 遭受损失的，应予以赔偿。 9.3 每次乙方在甲方付款前必须提供符合国家现行税法规定的合法有效等额增值税发票，甲乙双方一致确认提供 发票为主合同义务而非附随义务，若乙方未按要求提供发票，甲方有权暂停付款。乙方应在开票之日起7天内将 道 发票送达甲方指定人员【 刘磊】，甲方指定人员签收发票的日期为发票的送达日期。 9.4 乙方开具的增值税专用发票应保证信息完整、内容规范，如乙方未提供发票或提供的发票不合规、不及时、 无法认证，甲方有权拒绝付款，且不视为甲方付款逾期，乙方无权要求甲方支付利息、违约金或赔偿损失，也 管 不得以此为由中止履行合同约定的义务。 9.5若乙方由一般纳税人身份变为小规模纳税人身份的，或者计税方法发生变化的，或者政策法规等规范性文件 发生变化的，并导致甲方可抵扣的进项税额减少或被税务机关要求补缴税款的，则减少的进项税额或补缴的税 款应由乙方承担，甲方国有权从将支付的任何一笔款项中扣除。 9.6 增值税税率变化：合同执行过程中如果遇到国家税务政策调整，增值税税率发生变化的，按新的税率执行， 不含税价不变，仅调整增值税税率的原则进行相应调整。 中 若乙方提供的发票不符合要求的，发包人有权拒收增值税发票，并有权暂停支付相应款项，乙方不得以此为由 中止履行合同的义务。如因乙方不能按期提供发票或提供的发票不符合要求而导致付款延期的，由其自行承担 后果，发包人不承担任何责任。 9.8若乙方迟延提供发票的，每日应按暂定合同总价的0.05%向甲方支付违约金，但迟延违约金累计支付不超过90 日；若乙方迟延提供发票超过90日且已跨年的，视为乙方未提供发票，乙方除应支付前述迟延违约金外，还应另 行向甲方支付以下款项： （1）相当于合同暂定总价1%的违约金； （2）甲方因未收到发票所产生的税款损失， 损失金额按以下公式计算：赔偿损失金额=未提供发票对应的增值税税额*（1+增值税附加税率）+未提供发票金额 *甲方企业所得税税率。 9.9乙方保证开具的发票已经依法足额纳税，支付每笔款项前，乙方需提供发票对应税期的增值税纳税申报表和 完税证明。 9.10乙方承诺其提供的发票真实合法，若发包人认证后出现走逃失联、被列为异常纳税人等违规行为，导致发包 人不能认证抵扣或者认证抵扣后被税务机关要求进项转出情形，应在72小时内补开合规发票，否则按以下方法计 算应赔偿发包人损失，应赔偿损失金额=进项转出税额*（1+增值税附率)+不合规发票金额*发包人企业所得税税 率，逾期未赔偿的，甲方有权从结算金额或者履约保证金中扣除。 9.11乙方主张已开具发票的，应提供：①税务系统发票开具记录 ；②采购方签收凭证或者发票邮寄物流凭证。无 法完整提供两项证据的视为未开票。 10.双方责任 10.1 双方现场代表 10.1.1甲方现场代表为【 】，其职务为【 】 ，其授权签署文件的范围为：【签发监管项目的各类文函、工程变更 指令、索赔文件的报出、违约处罚决定文件等】。 10.1.2甲方收货代表：【 】，联系电话【 】。甲方指定收货代表仅有对乙方送货单中货物的数量及乙方提供的单 据是否齐全子以确认的权利，对货物单价、质量、货款以及总结算单没有确认的权利。 10.1.3乙方应将物资按合同约定时间运至甲方指定地点，并经甲方指定收货代表和甲方工程项目所属其他1人及以 上在甲方指定的收领单上签字验收确认后有效。 网 10.1.4 甲方未经授权的任何人员和项目印章均无权从事下列行为：【（1）签订本合同的补充协议或签署其他合 同类文件，包括但不限于采购合同、分包合同、租赁合同；（2）签署任何借贷、担保性质的文件，包括但不限 于借条、保函、保证书、承诺书；（3）签署代他人清偿债务的文件，签署任何放弃债权的文件；（4）签署任何 对总承包合同进行修改和补充的文件;（5）收取现金及任何款项；（6）签署合同价款的变更、结算及支付确认 务 文件；（7）签署任何劳动关系确认文件、工资发放承诺文件。】 10.1.5 甲方授权人员的职权/职责范围、授权签署文件范围均不可转授权，任何形式的转授权、代签行为，甲方均 不予认可且不承担任何法律责任。 商 10.1.6 乙方确认已完全明白和理解甲方对甲方人员及项目印章的上述授权范围，超出甲方授权范围的行为属于无 权代理行为，对甲方无效，甲方不承担任何法律责任。乙方应谨慎审查相关文件的签署主体资格和权限，对于 无权代理人签署的相关文件，乙方应及时与甲方核实。 道 10.1.7 乙方现场代表为【 】，其职务为【 】，其授权范围为：【全面代表乙方履行本合同，并有权代表乙方签署、 确认履约过程中形成的工程变更、价款确认、经济索赔、违约处罚决定及物资丢失损坏赔偿文件；签署确权文 件及结算书；签收甲方发出的各类文函、工程变更及其他文件等。】 管 10.1.8 双方更换各自代表时，应及时书面通知对方，以确保物资顺利交接。 10.1.9 甲方禁止项目部及任何人员以甲方、甲方分公司、甲方项目部的名义对外借款或者支取任何款项，如乙方 或乙方有关人员以任何形式将款项出借或支付或返还给甲方项目部及任何人员，则不论该等款项是否实际用于 甲方工程，均与甲方无国关，该行为均属于乙方与相关人员个人之间的经济关系，乙方无权向甲方主张任何权利。 10.1.10 未经甲方书面授权不得擅自与建设方及有关部门发生工作上的联系，严禁在对外任何事务中签署甲方单 位名称或带有甲方简称中任何“【中国建筑】”“【中建】”“【中建XX局】”“【XX局】”等字样的落款， 每发现一次中乙方承担2万元的违约金并赔偿所有直接或间接损失。 10.2卫生、环境与安全保护 10.2.1 甲乙双方须贯彻执行国家、地方政府相关部门发布的有关卫生法律、法规，以及甲方发布的规章制度，积 极配合政府部门的检查，对于提出的要求按所属责任立刻整改，确保瘟疫和传染疾病防控的管理落实到位。 10.2.2 乙方保证在运输和卸货过程中应采取相应的环保措施，符合国家环保要求。车辆在进入项目现场要保证不 沾泥土和脏物，车辆出入项目现场必须在项目大门内现场洗车。乙方在卸货过程中保证噪声不超过以下标准 （白天小于或等于【 】dB、夜间小于或等于【 】dB）。乙方保证乙方人员以及车辆进入本工地现场，应遵守现 场的一切卫生环保、文明施工的规定，因违反环保要求所造成的一切罚款由乙方承担。 10.2.3 甲乙双方必须贯彻执行国家和政府、行业主管部门颁布实施的有关安全生产的法律、法规及有关规定。乙 方车辆及人员进出工地现场时必须接受甲方安全检查。乙方因供货造成安全生产责任事故的，责任由乙方承担。 乙方必须对自身出入工地现场的人员进行安全交底，并为其配备安全防护用品，因乙方原因造成的各种人员伤 害及经济损失由乙方自行承担，并赔偿甲方及其它方因此造成的一切损失。 10.3 售后服务 10.3.1 如所供货物为专业性较高的产品，乙方应免费为甲方或工程业主提供操作及维修人员的培训服务，培训内 容应包括：基本原理、操作使用、维修保养等。 10.3.2 对于工程中的剩余或未使用到的货物在不严重影响外观、质量和功能的情况下甲方有权退货，退货原则上 以合同约定的含税单价为准，确因商品特殊的（比如定制等），价格由双方协商，协商不一致的，按照附件1 《计划采购与供应物资清单》中的含税单价（考虑甲方已支付费用、乙方承担运费等情况下，原则上不低于【 】%）【 】%退货，退货数量以实际数量为准。 不可抗力 11.1 不可抗力是指合同当事人在签订合同时不可预见，在合同履行过程中不可避免且不能克服的自然灾害和社会 性突发事件，包括地震、海啸、瘟疫、骚乱、戒严、暴动、战争等情形。 11.2 不可抗力事件发生后，乙方应立即通知甲方现场代表并迅速采取措施，尽量减少损失，并在24小时内向甲方 通报受害情况，提供必要证明。不可抗力持续发生，乙方应每日报告一次受害情况，直到不可抗力结束。甲方 应对受害处理提供必要的条件，并负责处理工作的组织、指挥。不可抗力发生后网，乙方未采取有效措施控制灾 害而发生的损失由乙方承担。 11.3 不可抗力引起的后果，由甲乙双方应各自承担其人员伤亡及财产损失，履行合同的期限相应延长。 务 不可抗力发生后，双方均应采取措施尽量避免和减少损失的扩大，任何一方没有采取有效措施导致损失扩大的， 应对扩大的损失承担责任。 因一方迟延履行合同义务，在迟延履行期间遭遇不可抗力的，不能免除迟延履行方的违约责任。 商 11.4 因单次不可抗力导致合同无法履行连续超过【30】天或累计超过【60】天的，甲方有权解除合同。合同解除 后，双方应就合同履行情况及结算与付款等善后事宜达成补充协议。 权利瑕疵 道 12.1 涉及到知识产权（专利权）标记的产品，乙方应提供知识产权（或专利权）及其权属的有效证明材料。乙方 承诺其提供的物资不侵犯他人的知识产权（或专利权），若乙方提供物资侵犯他人知识产权（或专利权）导致 他人向甲方索赔的，乙方承担由此给甲方造成的一切损失，包括但不限于甲方处理此纠纷发生的律师费、诉讼 管 费、仲裁费、差旅费等一切损失。此外，乙方应向甲方支付合同价款【5】%的违约金。甲方针对上述一切损失 有权从乙方结算货款中扣除或依法追索。 12.2 乙方所供物资应不存在任何权属纠纷及抵押、查封等权利限制情形，如乙方所供物资存在权属纠纷或任何权 利限制情形导致甲方遭国受损失，乙方应赔偿甲方全部损失。 保密 13.1 除法律规定或合同另有约定外，未经乙方同意，甲方不得将乙方提供的技术秘密及声明需要保密的资料信息 中 等商业秘密泄露给第三方。 13.2 除法律规定或合同条款另有约定外，未经甲方书面同意，乙方不得将甲方提供的图纸、文件以及声明需要保 密的资料信息等商业秘密泄露给第三方。 13.3 任何一方违反上述约定，应负责赔偿守约方因此造成的一切损失。 违约与赔偿14.1甲方应按照合同约定及时向乙方支付合同价款，若因甲方资金不到位，乙方同意给予甲方【 30 】 日的宽限期，宽限期内不视为甲方违约。超过宽限期仍未支付的，乙方可向甲方主张自宽限期结束后的违约金； 违约金以逾期支付的价款为基数，自宽限期结束之日起至甲方支付逾期价款之日止，按照中国人民银行同期活 期存款利率向乙方计付，向乙方计付，逾期支付违约金的上限为逾期支付金额的【 / 】%（不超过3%）。在我方 支付逾期付款利息后，分供商不可就此向我方再主张逾期付款的违约责任。（条款说明：乙方为中小企业时， 甲方前述条款支付期限+本条宽限期整体不得超过60日）。14.2 除本合同中规定的不可抗力外，其他不论任何原 因，乙方若不能按约定期限足额足量送至甲方指定现场存货地点，甲方向乙方收取逾期运达物资货款（含增值 税）每日【3】％的违约金，自逾期之日起计算至乙方实际送达之日止，延迟或供货不足超过【3】日时，甲方有 权单方面终止合同。14.3 未经甲方书面同意自行停止供应本合同约定的货物，均视为乙方违约，乙方除承担因此 给甲方造成的一切损失外，乙方另支付合同价款的【5】%作为违约金。 14.4若乙方提供的货物为非合同约定的厂家或品牌的产品，或提供的是假冒他人品牌的产品，甲方有权立即终止 合同，乙方必须支付合同价款【2】倍的违约金给甲方，如乙方所供产品已安装至工程项目，则乙方除承担违约 金外，还必须承担拆除、工程维修、工作面清理和重新安装产生的所有费用等，如违约金不足以弥补因此给甲 方造成的所有损失，包括一切直接损失和间接损失，则超出部分，甲方有权向乙方追偿。乙方提供的货物为合 同约定的厂家及品牌产品，但货物质量不合格或不符合约定的技术要求时，可由乙方负责更换质量合格和符合 约定技术要求的产品，同时承担合同价款【5】%的违约金，并承担因违约造成的各项损失，甲方也可直接要求 解除合同，乙方承担因此给甲方造成的所有损失。乙方提供的合同标的物因品牌、质量等原因导致甲方被项目 业主或总包方罚款或追究违约责任，乙方应向甲方相应承担赔偿责任。 14.5 本合同履行过程中，如果乙方不能按时交货，应在交货前48小时内以书面形式通报甲方，甲方视情况确定是 否同意变更供货时间。如甲方不同意变更供货时间，可自行采购部分或全部货物。甲方在自行采购和接收该违 约部分货物时实际发生的所有额外费用及因此给甲方造成的损失，从甲方应支付给乙方的任一期货款中扣除， 甲方同时保留进一步索赔的权利。 14.6甲方提出索赔通知后，乙方应在【28】日内答复，如果在【28】日内未答复，视为乙方已接受该索赔，同时 甲方保留进一步要求赔偿的权利。 网 14.7 乙方在进出场时乙方不得私自运送甲方现场物资出场，一经发现，乙方向甲方支付所涉及物资原值【2】倍 的违约金，情节严重的交由司法机关处理。 务 14.8 由于乙方自身原因（如：不按约定开立银行账户、未及时提交报量资料或不按合同配合甲方进行款项支付 等），导致货款或工程款延期支付，甲方不承担延期付款利息及违约金，乙方不得因此停止供货；乙方擅自停 供的视为乙方违约，乙方承担因此给甲方造成的所有责任及损失。 14.9 如果出现合同为可调价合同，甲乙双方调价达不成一致商情形；或者出现合同为不可调价合同，乙方提出调价， 甲乙双方达不成一致情形，则甲方有权选择其他供应商，甲方不承担任何违约责任。 14.10 若乙方因14.5和14.9款原因停止供货，或未完成全部供货、或主张解除合同等不履行合同的情形，乙方剩余 款项的支付不适用本合同8.2条款，甲乙双方应道就剩余款项的支付签订书面补充协议，重新明确支付条款，甲方 不承担任何违约责任。 14.11 其他违约与赔偿要求：【 /】。 管 联络与送达 甲方：收件人【 】，联系电话【 】，电子邮箱【 】，地址【 】。 乙方：收件人【 】，联国系电话【 】，电子邮箱【 】，地址【 】。 15.2 一方通过电子邮箱发送文件的，文件到达对方邮箱即视为送达，送达时间为电子邮件到达对方邮箱地址时间； 一方通过信函邮寄送达的，则信函寄出后的第三个工作日或收件人实际签收日（以先到的时间为准）视为送达； 一方选择直中接送达的，则递交时视为送达。 15.3 邮件邮寄至上述地址被拒收或无人签收，亦视为已经送达，由此增加的费用和（或）延误的期限由拒绝接收 一方承担。 15.4 双方承诺，因本协议的履行或争议解决，上述联系人和联系方式为有效的联系方式，各项通知均应当向上述 联系人、联系方式送达。在诉讼、仲裁中，上述联系人、联系方式亦为有效的送达地址，向上述地址的送达即 为有效送达，即使发生拒收、退信等事件。 上述联系信息发生变更的，变更方应当即时通知对方；在对方收到变更通知之前，对方当事人或者仲裁、司法 机构已经向原联系人、联系方式进行的通知，视为有效通知。 争议解决 16.1 因本合同引起或与之相关的任何争议、纠纷或权利主张，则必须先行向对方发出书面和解申请书，并告知对 方争议、纠纷或权利主张之事实及依据、联系人及联系方式，在对方收到上述通知之日起 3 个月为双方和解期限。 在和解期限内，若双方达成和解协议的，双方的权利义务按照和解协议履行；若未达成和解协议的，任何一方 采用下列第【 】种争议解决方式，并自行承担本方发生的律师费、差旅费、保函费等相关费用∶ （1）向仲裁委员会申请仲裁 周口仲裁委员会（开庭地点：郑州） 郑州仲裁委员会 武汉仲裁委员会 北京仲裁委员会 上海仲裁委员会 中国国际经济贸易仲裁委员会 R成都仲裁委 （2）向【 】人民法院提起诉讼。 网 1.因本合同引起的或与本合同有关的任何争议，如仲裁委员会，则按照其仲裁规则进行仲裁。仲裁裁决是终局的， 对双方均有约束力。 务 2.双方承诺：任何一方向仲裁委员会申请仲裁的，双方均自愿放弃向对方主张仲裁费用和实际发生的其他费用， 包括但不限于鉴定费用、评估费用、审计费用等；双方均自愿放弃向对方主张补偿因办理案件支出的合理费用， 包括但不限于律师费、保全费、差旅费、公证费等。 3.双方约定：仲裁案件无论标的额大小、复杂程度如何，商均适用普通程序，即由三名仲裁员组成仲裁庭审理，以 确保案件公正审理。 4.调解期限：争议应先行和解协商解决，设定3-6个月和解期（可根据情况调整），且和解期限不计入仲裁审理 期限。任何一方若未履行上述和解程序而直接道提请至争议解决机构的，则需要向对方承担签约合同价【10】%的 违约金；如一方出现上述情形，另一方提起反诉或反请求，则提起反诉或反请求的一方不承担违约金。 17.禁止债权转让条款甲乙双方确认，若发生下列任一情形，即视为乙方重大违约，乙方需向甲方支付合同总价 （建议10%） %的违约金，且甲方有权视违约程度单方解除本合同，同时乙方应赔偿甲方因此遭受的全部损失 管 （包括但不限于直接损失、间接损失、维权产生的律师费、诉讼费、保全费等）。具体情形如下： （1）未经甲 方事先书面同意，乙方擅自将其在本合同项下对甲方享有的全部或部分债权进行转让、质押或以其他方式处分 给任何第三方的； （2）因乙方与乙方债权人存在债务纠纷，导致该乙方债权人以甲方为被告或被申请人提起代 位权诉讼、仲裁或采取其他司法/仲裁手段的； （3）未经甲方事先书面同意，乙方以自身名义或委托任何第三 方，就本合同相关事项国对甲方的关联单位（包括但不限于业主单位、建设单位、 发包方）提起代位权诉讼、仲 裁或采取其他司法/仲裁手段的； （4）其他性质同上述条款规定的情形。18.补充条款 /】 中 其他 19.1 本合同采用下列第【 2 】种签订方式： （1）本合同自双方签字并盖章后生效，一式【叁】份，甲方执 【贰】份，乙方执【壹】份，每份具有同等法律 效力。 （2）本合同采用电子签章签署生效。根据《中华人民共和国民法典》、《电子签名法》等相关法律、法规，双 方一致认可在【 】平台（网址：【 】）使用电子印章签署合同为其真实意思表示，且确保在该平台注册时，使 用的企业信息和个人相关信息真实有效，并且自觉遵守国家法律法规和甲方在该平台的合同签约流程。甲乙双 方使用电子签章方式签署的合同，只有通过验证生效的电子原件具有法律效力，未经电子印章服务平台公司提 供书面证明材料的电子合同打印版不能作为法律依据。如因乙方使用不当给甲方造成损失，乙方愿自行承担由 此造成的全部经济损失和法律责任。 19.2未尽事宜经双方协商一致后，可签订补充协议，与本合同具有同等法律效力。 19.3对于因本合同产生的任何争议或投诉，乙方可通过【 】（条款说明：根据各公司情况填写投诉平台或者联系 方式）进行提交。甲方将在收到乙方的投诉后，对乙方的投诉进行初步审查，并尽快与乙方取得联系以进一步 了解详情。因不可抗力或第三方原因导致无法按时处理投诉的情况，甲方将尽快通知乙方，并尽力协调解决问 题。 19.4本合同条款（包括但不���于免责条款、责任限制条款等）均经双方充分协商，双方已就全部条款内容达成一 致意见，不存在单方预先拟定且未予协商的情形。 附件： 附件1：《计划采购与供应物资清单》 附件2：《法人授权委托书》 附件3：《廉政合同书》 （以下无正文） 甲 方：【盖章】 乙 方：【盖章】 网 法定代表人：【签字】 法定代表人：【签字】 委托代理人：【签字】 委托代理人：【签字】 务 地 址：【 】 地 址：【 】 电 话：【 】 电 话：【 】 商 电子信箱：【 】 电子信箱：【 】 附件1 道 计划采购与供应物资清单 人民币：元 管 计量 暂定 单价 暂定含税 序号 物资名称 规格型号 品牌/产地 生产厂家 备注 单位 数量 不含税单价 增值税 含税单价 货款金额 价税合计 暂定合同价款人民币大写： 国 以上数量为暂定项目，最终以双方签字确认的采购结算单为准 中 附件2 中国建筑 项目管理表格 表格编号 法人授权委托书 CSCEC-WZ-HN003 （甲方）： 本授权委托书声明：本的法定代表人，授权委托我公司的 为我公司代理人，代表我公司与贵公司工程对涉及投标报价，物资合同、补充协议的签订、履行，物资结算、收款等业务进行签字确认，由在上述授权范围签字的所有文书，我公 司均予认可，由此产生的一切经济法律责任由我公司承担。 代理期限为前述代理人对上述业务发生第一次签字确认之日起至本工程结算完成之日止。代理人无转委托权。 特此委托。 代理人（签字/按指纹）：身份证号码： （供应商）法定代表人签字： （供应商盖章）： 日期： 附件3 廉政合同书 甲方：【 】 乙方：【 】 为确保甲方对业主的承诺，高效、优质共同完成施工任务，争创优质工程，保证合同双方能够高效廉洁地履行， 维护双方合法权益，经双方协商，特订立如下廉政合同书。 第一条 甲乙双方的权利和义务 1.甲乙双方应本着“公开、公平、公正、诚信、透明”的原则开展工作，自觉遵守党和国家、工程项目所在省、 市、区工程建设有关法律法规以及廉政建设的各项规定。 2.甲乙双方应建立健全廉政教育制度，开展经常性教育活动，积极宣贯“合规诚信 自律清正”的廉洁从业核心理 念，加强廉政教育。 3.加强相互监督，发现对方有违反廉政合同书规定的行为，应及时提醒对方纠正。 第二条 甲方的责任 网 甲方工作人员不得有以下行为： （1）为乙方多结算工程量、多签证、多付工程款等，并向乙方索要或接受贿赂、回扣、礼金、有价证券（卡）、 务 贵重物品和好处费等; （2）在乙方报销任何应由甲方或个人支付的费用; （3）参加有可能影响公正执行公务的超标准宴请和娱乐商、健身等活动; （4）接受乙方提供的通讯工具、交通工具和高档办公用品; （5）要求、暗示或接受乙方为个人住房装修道、婚丧嫁娶、配偶子女工作的安排以及出国（境）、旅游提供的方 便; （6）向乙方介绍或推荐配偶、子女、亲属参与的工程施工合同有关的设备、材料、工程分包、劳务等; 管 （7）向乙方推荐分包单位或要求乙方购买合同规定以外的材料、机具设备等; （8）因乙方拒绝本人的不合理要求，而故意刁难乙方。 第三条 乙方的责任 国 乙方应当通过正常途径开展业务，不得有以下行为： （1）为多结算工程量、多签证、多收工程款等，向甲方及其管理人员行贿或馈赠礼金、有价证券（卡）、贵重 中 礼品; （2）为甲方及其工作人员报销应由甲方单位或个人支付的任何费用; （3）安排甲方人员参加超标准宴请、娱乐活动及带有黄、赌性质的娱乐活动; （4）为甲方人员购置或提供通讯工具、交通工具和高档办公用品等; （5）乙方向甲方工作人员及其家属或者亲友介绍从事与甲乙双方工程有关的工程分包及材料设备、周转工具的 供应、租赁等经营活动。 第四条 违约责任 1.如甲方工作人员有违反本廉政合同书的行为，由甲方纪委查处，追究相应的党纪、政务责任，涉嫌犯罪的，移 交司法机关追究刑事责任；对实名举报的，甲方要立即调查，并采取有效措施保障乙方的合法权益，防止报复 事件发生。 2.如乙方单位或个人有违反本廉政合同书的行为，甲方视情节对乙方处以合同额0.5%—1%的罚款，情节较重并给 甲方造成损失的，乙方另需赔偿甲方直接经济损失，并取消乙方工程分包资格。 第五条 甲方接受举报的途径 1. 受理电话：【 】 2. 受理地址：【 】 3. 受理部门：【 】 4. 受理邮箱：【 】 第六条 本廉政合同书作为采购合同的一部分，具有同等法律效力，本协议与采购合同同日生效，至甲乙双方工 程合同履约完止。 甲方： 乙方： 网 法定代表人： 法定代表人： 授权委托人： 授权委托人： 务 签订时间： 年 月 日 请查看报价网 商 址：https://xy.yzw.cn/sj/bid-detail?tenderId=&amp;source=3&amp;tenderCode=cscec2026081900001246027&amp;tenantId=cscec 信息来源:https://www.chinapipe.net/project/d3076919.html cqdingjiu 2026.08.21 10:06:42 道 管 国 中</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076919.html</t>
-        </is>
-      </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>0</v>
       </c>
@@ -788,11 +776,7 @@
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 务 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 商 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎道石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 管 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟262m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混国凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 中 2.3 本项目工程总投资金额：约3140万元； 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 网 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 务 2.7 其他： / 商 3.政府采购工程 道 3.1 是否属于政府采购工程：是 □否 管 3.2 是否专门面向中小企业预留：是 国 专门面向中小企业预留的实施方式： 中 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要网提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 务 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 商 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 道 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 管 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 国 开户银行: 开户银行: 账 号: 账 号: 中 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005499 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421353 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891814619 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001038 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00385 信息来源:https://www.chinapipe.net/project/d3076880.html cqdingjiu 2026.08.21 10:06:45</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076880.html</t>
-        </is>
-      </c>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
         <v>90</v>
       </c>
@@ -864,11 +848,7 @@
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(二标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 务 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 商 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟2道62m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 2.3 本项目工程总投资金额：约3140万元； 管 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）施工图所示范围的所 有内容为准，详见发布国的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分中： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 网 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 务 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （忠县）下载招标文件、工程量清单、电子图纸等资料。商参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（忠县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源 交易监督网、重庆市公共资源交易网（忠县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数字证 书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的，责任 自负。 道 5.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提 问”栏提出疑问，提问时间从本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 管 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 中忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 忠县发展和改革委员会 电 话: 023-54450483 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421361 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00386 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005423 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891832091 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001039 信息来源:https://www.chinapipe.net/project/d3076879.html 网 cqdingjiu 2026.08.21 10:06:45 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076879.html</t>
-        </is>
-      </c>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
         <v>0</v>
       </c>
@@ -940,11 +920,7 @@
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(一标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）已由 忠县发展和改革委 员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来 自 业主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具 备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 务 2.项目概况与招标范围 商 2.1 建设地点： 忠县马灌镇、三汇镇、永丰镇。 道 2.2 项目概况与建设规模：忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）：田块整治 工程：水田整治50.67亩、水田区域撂荒地整治79亩、旱地区域撂荒地整治62.83亩；灌溉与排水工程：新 建200m蓄水池5座、新建500m蓄水池1座、泵站1座；田间道路工程：新建2.5m混凝土生产路12325m、改 建2.5m混凝土生产路8549m、新建2.5m泥结碎石生产路1223m、新建3.0m混凝土生产路576m、改建3.0m混凝土生 管 产路648m、改建3.0m混凝土生产路（拆除原1.5m宽路）266m、改建3.5m混凝土机耕路1662m；地力提升工程：施 有机肥136.48亩；其他工程：公示牌1座、工号牌213块。 国 2.3 本项目工程总投资金额：约3140万元； 中 本次招标项目合同估算金额：一标段1167万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 网 方式一：本项目整体面向中小企业。 务 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 商 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 道 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 管 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 国 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 中 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及CA数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-10 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 网 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 务 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段） 商 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082000104 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005469 道 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421379 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00387 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891884496 管 信息来源:https://www.chinapipe.net/project/d3076876.html cqdingjiu 2026.08.21 10:06:46 国 中</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076876.html</t>
-        </is>
-      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
         <v>95</v>
       </c>
@@ -1016,11 +992,7 @@
           <t>永川区农村供水管网巩固提升改造工程(东部片区)答疑补遗文件 永川区农村供水管网巩固提升改造工程（东部片区） 补遗文件（01） 各潜在投标人： 现将“永川区农村供水管网巩固提升改造工程（东部片区）”招标文件补遗通知如下，本次发布的补遗文件中 的所有内容与招标文件具有同等法律效力，如与招标文件、答疑补遗文件（01）网不一致时，以本补遗文件为准。 请各潜在投标人自行下载本补遗文件，不管下载与否，都视为全部知晓其全部内容。 一、本招标项目招标文件第二章投标人须知前附表第1.4.1项第1条第（3）款中“具备建设行政主管部门颁发的有 效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由建设行政主管部门颁发的有效的安全生产 务 考核合格证书。”修改为： “（3）具备建设行政主管部门颁发的有效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由水 行政主管部门颁发的有效的安全生产考核合格证书”。 商 二、本招标项目招标文件第二章投标人须知前附表第1.4.1项中第3条“业绩要求”修改为： “投标人自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成过1个单项合同 输配水管网长度不少于100km的水利工程施工道业绩。 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 管 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 三、本招标项目招标文国件第二章投标人须知前附表第1.4.1项中第5条中的“5.3项目经理业绩要求”修改为： “投标人拟派的项目经理自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成 过1个单项合同输配水管网长度不少于100km的水利工程施工业绩，并在该业绩中担任项目经理。 中 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 四、本招标项目的投标文件递交的截止时间（投标截止时间）调整为2026年9月4日9时30分（北京时间），开标 时间及投标保证金递交截止时间相应顺延。 招标人：重庆市永川区惠永水务有限公司 招标代理机构：重庆永川政鑫综合能源有限公司 2026年8月20日 信息来源:https://www.chinapipe.net/project/d3076870.html cqdingjiu 2026.08.21 10:06:46</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076870.html</t>
-        </is>
-      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
         <v>80</v>
       </c>
@@ -1092,11 +1064,7 @@
           <t>长寿区海棠、石堰、龙河片区污水管网建设项目(二期)招标公告 长寿区海棠、石堰、龙河片区污水管网建设项目（二期）招标公告 1.招标条件 本招标项目长寿区海棠、石堰、龙河片区污水管网建设项目已由重庆市长寿区发展和改革委员会以长改发投 〔2024〕169号文批准建设，项目业主为重庆市长寿区住房和城乡建设服务中心，建设资金来自财政资金，项目 出资比例为100%，招标人为重庆长寿乡村建设集团有限公司。项目已具备招标条件，现对该项目的施工进行公 开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：长寿区海棠镇、龙河镇、新市街道、云台镇。 2.2 项目概况与建设规模：新改建及修复DN300mm-DN1200mm排水管道20.187公里，其中新改建管道15.21公里， 务 修复管道4.977公里，Ⅲ、Ⅳ级结构性及功能性缺陷修复453处。 2.3 本次招标项目合同估算金额：4139.45万元。 2.4 招标范围：详见招标人提供的本工程的施工图图纸、图商说、设计变更以及工程量清单所明确的全部工程内容。 2.5 工期要求：270日历天。 缺陷责任期要求：24个月。 道 3.政府采购工程 3.投标人资格要求 管 3.1 本次招标要求投标人须具备以下条件： 3.1.1 本次招标要求投标人具备的资质条件：建设行政主管部门颁发的有效的市政公用工程施工总承包三级及以 上资质； 国 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 中 3.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（长寿区） （https://www.cqggzy.com/changshouweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需 在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网 导航栏“主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登 记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn）和重庆市公共资源交易网（长寿区） （https://www.cqggzy.com/changshouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公 告发布至2026-08-25 15:00:00前。 4.3招标人应于2026-08-28 18:00:00前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn）和重庆市公共资源交 易网（长寿区）（https://www.cqggzy.com/changshouweb/）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-14 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn）和重庆市公共资源交易网（长寿区） （https://www.cqggzy.com/changshouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源 交易监督网上发布。] 7.联系方式 招 标 人: 重庆长寿乡村建设集团有限公司 代理机构: 中新创达咨询有限公司 地 址: 重庆市长寿区桃源大道3号一号商务楼5-6楼 地 址: 邮 编: 邮 编: 项目负责人: 刘老师 项目负责人: 钟亮 网 电 话: 023-40233279 电 话: 19132912275 传 真: 传 真: 电子邮箱: 电子邮箱务: 开户银行: 开户银行: 账 号: 账 号: 商 监督部门: 重庆市长寿区发展和改革委员会 电 话: 023-40245080 2026年08月20日 长寿区海棠、石堰、龙河片区污水管网建设道项目（二期） 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公 中国农业银行股份有限公司重庆自由贸易 312601010400083780000033561 司 管试验区分行 重庆联合产权交易所集团股份有限公 中国建设银行股份有限公司重庆渝中支行 6232813760003317764 司 重庆联合产权交易所集国团股份有限公 重庆银行股份有限公司七星岗支行 15010202900420146632392 司 信息来源:https://www.chinapipe.net/project/d3076848.html cqdingjiu 20中26.08.21 10:06:46</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076848.html</t>
-        </is>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
         <v>0</v>
       </c>
@@ -1168,11 +1136,7 @@
           <t>中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部刺丝滚笼、塑钢模板、泄水管询价采购公告 中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 刺丝滚笼、塑钢模板、泄水管询价采购公告 询价编号： ZT1105-XJ-2026-590 尊敬的 各潜 在供应商 : 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与 中铁十一局集团有限公司重庆至万州高铁站 前 1标项目经理部 ZT1105-XJ-2026-590， 刺丝滚笼、塑钢模板、泄水管 的报价。 一、 项目概况 务 渝万高铁站前 1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~ D1K47+550.4，正线长度 33.01km，中标造 价 31.73 亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁 301 孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负 责DK0+000~DK57+136段小型构件预制。合同工期54.7月商，开工日期为2022年11月01日，竣工日期为2027 年04 月30日。 二、 询价内容 道 本次 计划对刺丝滚笼、塑钢模板、泄水管 进行询价，询价内容如下： 询价物资一览表 管 计 序 物资 量 包件号 规格型号 数量 备注 号 名称 单 位 国 刺丝 1 GL-01 2.5mm 6m0.5m 米 6500 半径 ≥225mm，包括刀片刺绳、挂丝、连接卡、支架 滚笼 防护 中 栅栏 2 GL-01 用立 50X30X765X2.5mm 套 500 含抱箍、螺栓等配件 柱支 架 平 塑钢 3 MB-01 350X300mm 方 19.2 400*400,1个挡水沿，配固定手柄 模板 米 平 塑钢 4 MB-01 350X300mm 方 19.2 400*400,2个挡水沿，配固定手柄 模板 米 平 塑钢 5 MB-01 300X300mm 方 75.6 2个挡水沿，配固定手柄 模板 米 平 塑钢 6 MB-01 300X300mm 方 75.6 1个挡水沿，配固定手柄 模板 米 7 SSG-01 管篦 PVC250X200x10mm 个 220 材质硬聚氯乙烯 PVC，详见附图 PVC 8 SSG-01 泄水 135X38mm 块 220 材质硬聚氯乙烯 PVC，详见附图 管盖 U型 9 SSG-01 125mm 个 900 详见附图 管卡 UPV 材质硬聚氯乙烯 PVC，两端接头采用阴阳螺纹连接详见 10 SSG-01 C排 125X8mm螺纹 米 2870 附图 水管 UPV 11 SSG-01 C弯 DN125X8mm90° 个 240 材质硬聚氯乙烯 PVC，详见附图 管 UPV 网 125X125X110mm弹性密 12 SSG-01 C三 个 120 材质硬聚氯乙烯 PVC，详见附图 封圈异径斜三通 通 无压 埋地 务 排污 排水 用硬 13 SSG-01 DN125 个 150 材质硬聚氯乙烯 PVC，详见附图 聚氯 商 乙烯 管 T 型接 头 道 合 计 管 说明： 1. 表中数量为计划数量，实际 采购 过程中可能有所调整，最终结算按照实际 采购 数量结算。 2.收货地点：中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部 三、 技术质量 及报价国 要求 1. 此次 询价物资 各项技术性能要 符合 甲方 的要求，质量满足甲方项目部正常使用的要求，保证 产品 的质量合 格。 具体要求或图纸见询价文件技术规格书。 。 中 2 .报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、 结算及付款方式 每个月 15 日为双方价款结算日期（即上月 16 日至当月 15 日内），结算前双方要在对帐确认单上签字认可，乙 方按双方确认的金额开具增值税专用发票，并自发票开具之日起 7日内传递给甲方。甲乙双方在增值税专用发票 传递过程中必须留取相应的交接签证手续。自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发 票认证完成之日起第6个月，支付至本次结算金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内， 累计支付总额不超结算总金额的75%，剩余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理 末次结算后第二年，支付金额应大于等于尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总 额的15%；办理末次结算后第四年，全部付清）。 五、 报价 人资格要求 1.营业范围要求：在中华人民共和国境内依法注册，具有询价物资生产或供应经验的生产商或代理商，并且具有 合法有效的营业执照。 2.生产能力要求： 生产商须具备 询价 物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定 。 代理商需出具制造厂出具签字盖章的授权函。 3.财务能力要求：报价人为增值税一般纳税人或小规模纳税人，有依法纳税的良好记录。 4.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8月至今） 国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；每种物资全指标技术参数性能满足 国家和行业最新标准的各项规定。 5.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年8月至今）企业或企业法定代表人有人民法院生效判决、裁定 认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接受 通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合作 方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 6.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★7 .下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、 报价人需要提供的资料 1. 营业执照复印件、 法人身份证复印件、 开户许可证、商授权委托书 、 报价表 和报价人资格要求中所需的证明资 料， 所有资料需加盖公司鲜章。 2. 产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、 询价 报名截止 时间 管 有意参加本次询价采购的报价人 须在铁建云链平台 （ https:// www.crccep. cn） 完成供应商注册，并 于 202 6 年 8 月 20 日 9时 00 分 至 202 6 年 8 月 24 日 9时 00 分在网上 完成报名工作。 八、 询价 截止 时间 国 凡有意参加本次询价采购的报价人，请于 202 6 年 8 月 24 日 14 时 00分 前 提交报价。截止时间前未完成 报价 文 件传输的，视为放弃 报价 。 供应商报价必须严格按照《 报价表 》格式进行报价。 中 九、 联系方式 采购 组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村 71号 联系人：胡先生 联系电话： 13983336494 （提供平台服务支持） 采购人名称：中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 地址： 重庆市万州区双河口街道檬兴路万州现代综合物流中心信息交易大厅（中铁十一局） 联系人： 唐大伟 联系电话： 18323391938（提供采购服务支持、保证金退还） 中铁十一局集团有限公司物资设备集中采购管理中心 第五分中心 2026 年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076805.html cqdingjiu 2026.08.21 10:06:47 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076805.html</t>
-        </is>
-      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
         <v>85</v>
       </c>
@@ -1244,11 +1208,7 @@
           <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 1.招标条件 本招标项目 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 已由 垫江县发展和 改革委员会 以 垫江发改委发〔2026〕20号 文批准建设，项目业主为 垫江县太平镇人民政府，建设资金来 自 大中型后扶资金及自筹资金 ，项目出资比例为 100% ，招标人为垫江县太平镇人民政府。项目已具备招 标条件，现对本项目施工进行公开招标，评标办法采用经评审的最低投标价法。网 务 2.项目概况与招标范围 商 2.1 建设地点：垫江县太平镇桂花村 道 2.2 项目概况与建设规模：主要为河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m， 化粪池2座；产业基地水肥一体化改造45亩等。 管 2.3 本项目工程总投资金额：642.89万元 国 本次招标项目合同估算金额：约5014864.52元 中 2.4 招标范围：本工程施工图纸所含全部的施工内容，具体以招标人发布的工程量清单为准。 2.5 工期要求：工期为360日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：□是 否，因专门面向中小企业预留无法确保充分供应、充分竞争，根据 《政府采购促进中小企业发展管理办法》第六条第(三)“按本办法规定预留采购份额无法确保充分供应、充分竞 争，或者存在可能影响政府采购目标实现的情形”的规定，本项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 网 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的水利水电工程施工总承包三级 务 及以上资质。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相商应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 道 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 管 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com国/dianjiangweb/)、重庆市公共资源交易监督网下载招标文件、工程量清单、电子图纸等资 料。参与投标的投标人需在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共 资源交易监督网完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督网导航栏“主体信息”页面中“市场主体信息 登记”、“中CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流 程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督 网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-24 17:00:00前。 5.3招标人应于2026-08-28 17:00:00前在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重 庆市公共资源交易监督网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交 易监督网发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 垫江县太平镇人民政府 代理机构: 重庆皓辰建设工程咨询有限公司 重庆市渝北区金开大道1228号大雅金开国际1 地 址: 重庆市垫江县太平镇牡丹路191号 地 址: 栋9-2 邮 编: 邮 编: 项目负责人: 余老师 项目负责人: 雷雨得 电 话: 13996889839 电 话: 023-86018770 18580880860 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 网 2026年08月19日 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 务 户名 开户行 投标保证金账号 垫江县公共资源交易中心 中国农业银行重庆垫江支行 316301010400077950000005966 垫江县公共资源交易中心 中国银行重庆垫江支行 111616885778VA00139 商 垫江县公共资源交易中心 重庆农村商业银行垫江支行 2501010120010009065000128 垫江县公共资源交易中心 工商银行重庆垫江支行营业部 9558853100016843371 垫江县公共资源交易中心 重庆银行垫江支行 820101040000584-101195 道 附件：垫江县2026年度大中型水库移民后期扶持项目-.zip https://www.cqggzy.com/trade/014001/dac54522-3264-4eac-ae47-f434567ce374?categoryNum=014001001007 信息来源:https://www.chinapipe.net管/project/d3076788.html cqdingjiu 2026.08.21 10:06:47 国 中</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076788.html</t>
-        </is>
-      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
         <v>85</v>
       </c>
@@ -1320,11 +1280,7 @@
           <t>万州区新田等6个镇乡农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区新田等6个镇乡农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建水厂1座（新建2000m3茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管 主要建设内容 径DN20~DN250，管材为涂塑钢管。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 备注 称 式 发布时间 所 额(万元) 商 万州区新田 万州区新田 重庆市万 招标项目 等6个镇乡农 等6个镇乡农 公开招 州区公共 1 村饮水质量提 2026-08 5000.00 村饮水质量 标 资源交易 升项目道施工总 提升项目 中心 承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076721.html 管 cqdingjiu 2026.08.21 10:06:48 国 中</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076721.html</t>
-        </is>
-      </c>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="n">
         <v>80</v>
       </c>
@@ -1396,11 +1352,7 @@
           <t>万州区大周等4个镇乡街道农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区大周等4个镇乡街道农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建50m3蓄水池4口、取水池2座；新建50m3/d-100m3/d水厂2座；改造100m3/d-300m3/d水厂5 主要建设内容 座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设 施。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 商 备注 称 式 发布时间 所 额(万元) 万州区大周 万州区大周 重庆市万 招标项目 等4个镇乡街 等4个镇乡街 公开招 州区公共 1 道农村饮水 道农村饮道水质 2026-08 3000.00 标 资源交易 质量提升项 量提升项目施 中心 目 工总承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3076720.html cqdingjiu 2026.08.21 10:06:49 国 中</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076720.html</t>
-        </is>
-      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
         <v>80</v>
       </c>
@@ -1464,11 +1416,7 @@
           <t>二航科工新燕尾山项目纤维编绕拉挤电缆保护套管采购询价通知公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目询比采购 公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目已具备采 购条件，现公开邀请供应商参加询比采购活动。 网 1. 采购项目简介 1.1 采购项目名称：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机 电工程项目。 务 1.2采购方案编号：FA00000674478。 1.3 采购人：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程 项目经理部。 商 1.4 采购代理机构：中交二航局科工（武汉）有限公司。 1.5 采购项目资金：企业自筹。 道 1.6 采购项目概况：新燕尾山隧道工程位于重庆市内环吉庆隧道北侧，四横线分流道鹿角隧道南侧，西接白居 寺大桥，东接内环快速路，并向东延伸接渝黔复线高速，其所在的道路系统呈东西布置，为主城区南部片区重 要干道。本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目 管 全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程 包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。 2.采购范围及相关要求 国 2.1 采购范围：纤维编绕拉挤电缆保护套管（BWFRP100/2.0，79158米）。 2.2 交货期：以甲方实际订单要求为准。 中 2.3 交货地点：重庆市巴南区新燕尾山项目甲方指定位置。 2.4 物资质量标准：满足国家法律法规、标准、规范、设计参数及技术规格书要求。 3.供应商资格要求 3.1 供应商应依法设立且满足如下要求： （1）资质要求：在中华人民共和国境内依法注册，具有独立法人资格、具有采购物资生产或供应经验的企业， 并且具有合法、有效的“三证合一”的营业执照,代理商需提供制造商授权委托书。 （2）财务要求：必须是经税务部门注册登记核准的一般纳税人，有依法纳税的良好记录，提供近三年的财务报 告。 （3）业绩要求：同类产品销售业绩不少于2个，并具备与本招标项目需求相适应的供货能力。 （4）信誉要求：本项目投标截止期前未被“信用中国”、“中国政府采购网”、中国交建物资采购管理信息系 统网站列入失信被执行人、违法案件当事人、违法失信行为记录名单。 （5）其他要求：提供运输方案及生产周期。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他： / 。 4.供应商报名 4.1有意参加询比采购活动的单位，请于2026年 8 月 20 日 11 时 00 分至2026 网 年 8 月 25 日 11 时 00 分（北京时间、下同），登录“中交招采网”（网 址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 务 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 商 5. 供应商报价 5.1 报价结束（递交响应文件截止）时间：2026年 8 月 25 日 11 时 00 分。 道 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的 电子响应文件，采购人将拒收。 5.3电子采购的供应商报价文件由线上电子报价表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 管 子报价表的数据为准。 6. 开标 6.1开标时间：与报价结国束时间相同。 6.2开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标，现场开标地点/。 7. 发布公告的媒介 中 本询比采购公告在中交招采网上发布。 8. 评审办法 本项目评审办法采用 经评审的最低价法 。 9. 合同主要条款 9.1 付款条件：无预付款，到货后办理结算，双方办理完结算手续、卖方提供符合合同要求的正式发票给买方 后60天，买方支付该批材料价值80%的货款，完工结算后支付至97%，剩余3%为质保金，质保期2年，两年后供 应方申请返还3%（无息）；银行转账、承兑、18个月供应链金融混合支付方式。 9.2履约保证金的递交： （1）□不要求递交 （2）要求递交 保证金金额：2万元 ； 保证金形式：银行转账、银行保函等电子保函；其他形式：无 。 10. 成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”（网址：https://zjzcw.iccec.cn）发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联 系4006765885中标服务费请按7咨询。 10.1收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； 务 （3）在1000万元（含）至3000万元之间的，每次收取1000元； （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 10.2支付流程 （1）通知推送：中标结果发布后，系统自动道推送缴费通知（含应缴金额及支付链接）； （2）费用查询：供应商登录“中交招采网-服务管理”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网- 服务管理－发票下载”模块获取。 11.监督机构 国 监督机构名称：中交二航局科工（武汉）有限公司纪委监察部 举报电话：中027-82796466 举报邮箱：sneb_kggs@ccccltd.cn 12.其他 投标保证金采用银行转账形式的需转至中交二航局科工（武汉）有限公司账户（账 号：42001186108053006379-0006开户行：建行武汉长江支行，行号：105521000053），并备注二航科工燕尾山机 电照明项目纤维编绕管投标保证金。 13.联系方式 采购 人：中交二航局科工（武汉）有限公司 采购代理机构：中交二航局科工（武汉）有限公司 地 址：武汉市新洲区双柳街星谷大道158号地 址：武汉市新洲区双柳街星谷大道158号 邮政编码：430400 邮政编 码：430400 联系人：李鑫 联系人：毕明 月 电 话：18186145302 电 话：17853118573 电子邮件：18186145302@ccccltd.cn 电子邮件：bimingyue@ccccltd.cn 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076715.html cqdingjiu 2026.08.21 10:06:50 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076715.html</t>
-        </is>
-      </c>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
         <v>90</v>
       </c>
@@ -1540,11 +1488,7 @@
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告 重庆巴南天然气有限责任公司 重庆国际生物城配套公寓项目天然气表后管道安装工程 变更公 告 公告编号： RQBGGG202608200006 本公司于2026年08月19日发布的重庆国际生物城配套公寓项目天然气表后管道安装工程公告（编 号：RQCGXY202608170010），现做出如下变更： 网 1、对采购文件第一卷“采购需求“中墙体管道暗埋的具体内容进行明确。墙体管道暗埋应包含墙体开槽，输送 用不锈钢波纹管及钢制槽板的安装，墙体恢复，暗埋管道视频记录。 2、对由响应供应商提供的钢制槽板的规格进行明确。钢制槽板为U型开口槽，采用热镀锌Q235B钢板，钢板厚度 务 不得小于1.2mm，尺寸不得小于U40*30*1.2（宽40mm,高30mm,壁厚1.2mm热镀锌） 3、对由响应供应商提供的F型不锈钢三通，材质可以选用黄铜进行替代。 4、采购文件第二卷“技术规范及要求“中增加T/CECS633-2019 《燃气用户工程不锈钢波纹软管技术规程》。 以上内容在合同中也同步进行调整。 商 除上述变更外，原公告其余内容仍有效。 道 重庆巴南天然气有限责任公司 管 2026-08-20 信息来源:https://www.chinapipe.net/project/d3076704.html cqdingjiu 2026.08.21 10:国06:50 中</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076704.html</t>
-        </is>
-      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
         <v>80</v>
       </c>
@@ -1616,11 +1560,7 @@
           <t>合川区中南片区污水管网工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 合川区中南片区污水管网工程（一期） 名称 招标 网 法人 或招 标人 重庆市合川区住房和城乡建设委员会 名称 （盖 务 章） 项目 批准 文件 合川发改投〔2025〕19 号 商 及文 号 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新 主要 建D300排水管道38米；紫外光修复 D300-D道800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 建设 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42 内容 米；完成 D300-D1000管道清障189米、清淤2627米。 拟 招 招标文 合同预 招标 管 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 国 重 庆 市 合川 合 招标 区中 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300- 川 项目 中 南片 D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 公 区 区污 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 开 公 1 2026-09 1708.44 水管 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米， 招 共 网工程 不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清 标 资 （一 淤2627米。 源 期） 交 易 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076543.html cqdingjiu 2026.08.21 10:06:50</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076543.html</t>
-        </is>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
         <v>90</v>
       </c>
@@ -1684,11 +1624,7 @@
           <t>重庆市自来水有限公司球墨铸铁管及管件2026-2027(2年)采购项目(第二次)答疑补遗文件 重庆市自来水有限公司球墨铸铁管及管件2026-2027（2年）采购项目（第二次）答疑 提问1：样品20CM长含承口吗？如果含承口20CM那就太短，标识LOGO无法体现完整建议≥20CM 答1：球墨铸铁管样品含承口，样品长度≥20CM 网 务 招标人：重庆市自来水有限公司 招标代理机构：重庆水务集团公用工程咨询有限公司 商 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d30道76446.html cqdingjiu 2026.08.21 10:06:50 管 国 中</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076446.html</t>
-        </is>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
         <v>80</v>
       </c>
@@ -1760,11 +1696,7 @@
           <t>大足区中心城区和龙水镇市政公共排水设施运维(材料)更正一号公告 一、更正项 更正项 更正子项 更正前内容 更正后内容 网上投标 网上投标截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 递交投标响应文件 线下递交投标（响应）文件开始时间 2026-08-20 14:30:00 2026-08-25 14:30:00 递交投标响应文件 线下递交投标（响应）文件截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 网 开标 开标时间 2026-08-20 15:00:00 2026-08-25 15:00:00 招标采购（附件） 附件 务 二、补遗更正说明 清单限价重新做调整，开标时间已更正，详见更正文件内容 商 三、联系方式 采购执行方： 道 单位名称：重庆誉双项目管理有限公司 联系人：陈老师 联系电话：13996336872 采购需求方： 管 单位名称：重庆市大足区茂泰市政工程有限公司 联系人：谢老师 联系电话：18523539371 信息来源:https://www.chinapipe.net/project/d3076319.html 国 cqdingjiu 2026.08.21 10:06:50 中</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076319.html</t>
-        </is>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
         <v>80</v>
       </c>
@@ -1836,11 +1768,7 @@
           <t>璧山区2026年大路街道三台村智慧设施农业建设项目招标计划表 重庆市工程建设项目招标计划表 项目 璧山区2026年大路街道三台村智慧设施农业建设项目 名称 招标 法人 或招 网 标人 中农良品（重庆）生态农业有限公司 名称 （盖 章） 项目 批准 务 文件 及文 号 主要 1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流 建设 装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6. 内容 都市农文旅配套建设1000平方米。 商 招 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 道 璧 山 区2026 重 年 庆 大 市 路 公 招标 街 管 共 项目 道 资 三 公 源 台 项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米； 2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、 开 交 1 村 二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套； 3.项目后勤及仓储配套（含装修）5000平方米； 4.土方回填及场地平整53000平 2026-09 9182.25 招 易 智 方米； 5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米； 6.都市农文旅配套建设1000平方米。 标 中 慧 心 设 国 璧 施 山 农 分 业 中 建 心 设 项 目 中 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076777.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076777.html</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
         <v>80</v>
       </c>
@@ -1912,11 +1840,7 @@
           <t>长寿区江南街道污水处理厂更新改造工程项目公告 长寿区江南街道污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目长寿区江南街道污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源为企业 自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：长寿区江南街道污水处理厂更新改造工程包括但不限于以下内容新建混凝池-三沉池；还建格栅池； 厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统；原斜管沉淀池改 造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰）。拆除原有污泥池，新增临时污泥储罐 务 并还建污泥池；污泥堆场临时改建及恢复；实施技改期间的临时排放工程；进行基础的自控改造。 2.2 比选范围：长寿区江南街道污水处理厂更新改造工程施工图范围中的所有工作内容，包括但不限于土建工 程、设备及安装工程、工艺管道工程、电气工程、临排工程等内容，具体以比选人提供的图纸、技术规范、设 备需求清单、答疑资料、澄清资料、其他补遗资料等相关商内容为准。 2.3 建设地点：重庆市长寿区江南街道。 2.4 工期：110日历天（实际开工日期以监理工道程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 3. 参选人资格要求 管 3.1 本次比选要求参选人具备以下条件： （1）独立法人资格； （2）建设行政主管部国门颁发的有效的市政公用工程施工总承包二级及以上资质； 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 中 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月 27 日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务 大厦5楼。 5.2 比选截止时间：2026年8月 27 日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 网 联系人：曹老师 电话：023-71618725 务 代理机构：重庆招标采购（集团）有限责任公司 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 商 联系人：高老师 电话：023-67706841 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 管 信息来源:https://www.chinapipe.net/project/d3076456.html cqdingjiu 2026.08.21 10:06:51 国 中</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076456.html</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
         <v>90</v>
       </c>
@@ -1988,11 +1912,7 @@
           <t>潼南区新胜镇、双江镇污水处理厂更新改造工程项目项目公告 潼南区新胜镇、双江镇污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目潼南区新胜镇、双江镇污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源 为企业自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：潼南区新胜镇污水处理厂更新改造工程，主要建设内容为新增200m?/d一体化污水处理设备基础； 更新现有污水处理系统设备，提高现有沉淀池二沉池、三沉池液位；升级处理系统（干化池改建为污泥池，新 增叠螺脱水机，改建污泥堆场及雨棚）；新建风机房－配电室防尘防渗地坪。潼南区双江镇污水处理厂更新改 务 造工程，主要建设内容为将原有斜管沉淀池改建为好氧池，新建3座竖流沉淀池，配套安装相关设备；更新污水 处理系统中老旧及故障设备；新建储药加药区与一体化危废储存间，完善污水处理配套设施。 2.2 比选范围：潼南区新胜镇、双江镇污水处理厂更新改造工程施工图范围中的工作内容（一体化设备采购及 相关安装工作除外），包括但不限于土建工程、附属工程商（包括但不限于绿化工程、工艺管线工程、电气及自 控工程、临排清淤工程等）、一体化污水处理设备基础、标准化建设、配套设备材料采购及安装工程等内容， 其中一体化设备采购及相关安装工作不在本次比选范围内；具体以比选人提供的图纸、技术规范、工程量清单、 答疑资料、澄清资料、其他补遗资料等相关内容为准。 道 2.3 建设地点：潼南区新胜镇、双江镇。 2.4 工期：120日历天（实际开工日期以监理工程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 管 3. 参选人资格要求 3.1 本次比选要求参选人具备以下条件： 国 （1）独立法人资格； （2）建设行政主管部门颁发的有效的市政公用工程施工总承包二级及以上资质； 中 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月27日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务大厦5 楼。 5.2 比选截止时间：2026年8月27日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 网 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 务 联系人：陈老师 电话：023-42756696 商 代理机构：重庆招标采购（集团）有限责任公司 道 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 联系人：高老师 管 电话：023-67706841 重庆水务电子商务平台国咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3076454.html cqdingjiu 2026.08.21 10:06:51 中</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076454.html</t>
-        </is>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
         <v>90</v>
       </c>
@@ -2056,11 +1976,7 @@
           <t>重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 采购需求单位(全称) 重庆医科大学附属第二医院总务科 项目名称 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程 项目内容 给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源 采购预算 409674.71元 网 拟采购供应商全称 东部自来水分公司 配套业务用房第二市政水源从重庆水资源产业股份有限公司东部自来水分公司管辖范围 单一来源采购理由 的管网具体接入，属于市政管网施工，具有特殊要求。 务 公示时间 2026年8月19日-2026年8月25日 联系人及联系电话 刘老师 023-63693215 注：1.以上陈述是否真实，欢迎社会各界监督，公示时间商至少5个工作日； 2.公示期内无异议的，采购管理处将进行该项目采购；有异议请将意见反映采购人。 信息来源:https://www.chinapipe.net/project/d30道76334.html cqdingjiu 2026.08.21 10:06:51 管 国 中</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076334.html</t>
-        </is>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
         <v>80</v>
       </c>
@@ -2132,11 +2048,7 @@
           <t>中铁二院工程集团有限责任公司G319黔江区正阳至城西段改建工程管线探测工作线上询价采购公告 中铁二院工程集团有限责任公司G319黔江区正阳至城西 段改建工程管线探测工作线上询价采购 ZTEYCQ-XJ-2026-019 网 采购单位: 中铁二院工程集团有限责任公司 发布时间: 2026-08-19 16:10 报价截止时间: 务 2026-08-21 17:00 招标方联系人: 杨先生 招标方联系电话: 商 13883021521 招标方邮箱: 监督方联系人: 李先生 道 监督方联系电话: 15823237919 监督方邮箱: 保证金: 0元 管 结算与发票信息: 详情 交货信息: 详情 国 其他说明事项: 标的明细 流水号：询2026081900304 中 计量单 技术标准及要 序号 标的名称 数量 交货期 送货地址 位 求 G319黔江区正阳至城西段 合同签订后5天内完成 西南区-重庆市-市辖 1 1 项 详见询价文件 改建工程管线探测工作 本项目服务内容。 区-黔江区-项目地点 信息来源:https://www.chinapipe.net/project/d3076309.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076309.html</t>
-        </is>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
         <v>80</v>
       </c>
@@ -2208,11 +2120,7 @@
           <t>乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 1.招标条件 本招标项目乌江涪陵榨菜绿色智能化生产基地(一期)已由重庆市涪陵区发展和改革委员会以重庆市企业投资项目 备案证2020-500102-13-03-000003 批准建设，项目业主为重庆市涪陵榨菜集团股份有限公司，建设资金来自企业 自筹，项目出资比例为100% ，招标人为重庆市涪陵榨菜集团股份有限公司。项目已具备招标条件，现对乌江 涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 2.1 建设地点： 重庆市涪陵区马鞍街道人和社区 。 网 2.2 项目概况与建设规模：建筑面积约369384.27㎡。本项目蒸汽管道主要为室外蒸汽管道φ219x6mm，管道材质： 20#地上敷设，由14#锅炉房分汽缸分别接至6#和8#智能化车间分汽缸，蒸汽管道运行压力1.08MPa，管道设计压 力1.2MPa。 务 2.3 本次招标项目合同估算金额：580.643717万元。 2.4 招标范围： 商 （1）蒸汽管道系统本体：从锅炉房分汽缸后（含分气缸阀门）至6#车间、8#车间分气缸处，所有蒸汽管道、管 件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温（含保温层及保 护层）工作。 道 （2）钢结构桁架工程：负责本项目范围内所有钢结构架空桁架（管廊）的采购、运输、制作、安装、防腐工作。 （3）管道附件及控制系统：负责本工程范围内所有阀门、压力表、温度表、流量计、电动/气动执行机构以及配 套仪表电缆、桥架、保护管的采购、运输、安装、接线。负责与DCS/PLC系统接口的接线与联动调试。 管 （4）调试与验收：组织并确保整个蒸汽管道系统（含分气缸后段末端管道、桁架及其安全附件）通过项目所在 地特种设备安全监察管理部门实施的安装监督检验。负责报检、配合现场检验、整改、出具深化图纸并由设计 单位审核盖章、特种设备法定报检取证的全部费用，包括但不限于：施工前办理安装告知，设计院盖章审核， 施工中接受并通过安装国监督检验，最终负责取得《压力管道安装监督检验证书》与《特种设备使用登记证》， 确保蒸汽管道投入使用并备案，提交全套法定检验报告。 （5）土建工作部分 中 1）管架和桁架基础的施工，包括但不限于钢结构桁架的混凝土独立基础的土方开挖、浇筑、养护及回填恢复。 2）管道穿墙/板孔洞的开挖、封堵与修复。 3）室内外地面的开挖（包括但不限于疏水井、沟槽开挖、通行地沟、设备基础开挖）与恢复（包括但不限于土 方回填、渣土弃运、地面硬化）。 4）桁架及设备接地线的施工，包括但不限于接地极制作、接地干线敷设，并与厂区主接地网可靠连接，接地电 阻测试合格。 具体详见施工图、招标文件、工程量清单、答疑补遗等资料。 2.5 工期要求： 60 日历天 缺陷责任期要求： 24 个月 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：投标人应同时具备以下(1)、(2)项资质： （1）具备建设行政主管部门颁发的有效的建筑工程施工总承包二级及以上资质； （2）具备有效的《中华人民共和国特种设备生产许可证》（许可子项目：工业管道安装GC2级及以上）。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 网 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 务 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（涪陵区） （https://www.cqggzy.com/fulingweb/）下载招标文件、工程商量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网（涪陵区道）（https://www.cqggzy.com/fulingweb/）本项目招标公告网页下 方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-23 17:00:00前。 4.3招标人应于2026-08-24 18:00:00前在重庆市公共资源交易网（涪陵区）（https://www.cqggzy.com/fulingweb/）发 布澄清。 5.投标文件递交的内容 管 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-09 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（涪陵区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 中重庆市涪陵榨菜集团股份有限公司 代理机构: 中招国际招标有限公司 重庆两江新区黄山大道中段53号5-1（双 地 址: 重庆市涪陵区江北街道办事处二渡村一组 地 址: 鱼座A栋5楼） 邮 编: 408000 邮 编: 项目负责人: 徐老师 项目负责人: 寿云凤 电 话: 13212467016 电 话: 023-68881331-9032 传 真: 传 真: 电子邮箱: bsd2me@126.com 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市涪陵区发展和改革委员会 电 话: 023-72203687 2026年08月19日 乌江 涪陵 榨菜 绿色 智能 化生 产基地 (一 期)6#、 8#车 网 间蒸 汽管 道安 装工 务 程 中 中 国 国 重 银 重 商民 重 庆 行 庆 生 庆 涪 股 涪 银 涪 陵 份 陵 行 陵 重 投 公 有 道公 股 公 庆 标 共 限 共 份 共 银 开 保 户 资 公 资 有 资 行 户 证 110292140553VA00154 9902001860445897 430102029007791845-275 名 源 司 源 限 源 涪 行 金 交 重 交 公 交 陵 账 管 易 庆 易 司 易 支 号 有 涪 有 重 有 行 限 陵 限 庆 限 公 马 公 涪 公 国 司 鞍 司 陵 司 支 支 行 行 中 信息来源:https://www.chinapipe.net/project/d3076300.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076300.html</t>
-        </is>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
         <v>95</v>
       </c>
@@ -2284,11 +2192,7 @@
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程询比采购公告 采购公告 公告编号： RQXYGG202608190057 一、采购项目基本情况 采购人：重庆巴南天然气有限责任公司 网 采购项目编号：RQCGXY202608170010 采购项目名称：重庆国际生物城配套公寓项目天然气表后管道安装工程 务 采购内容和范围：完成重庆国际生物城配套公寓项目 （民用1020户）天然气表后管道定制化服务。（含安装燃 气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个， 其它配套管件及辅材，墙体管道暗埋等） 二、供应商资格要求 商 1. 资质要求:资质要求： 1.响应供应商为中华人民共和国境内合法注册的独立法人或其他组织，具有独立承担民事责任能力，具有独立订 立合同的权利。 道 2.响应供应商应具备市政公用工程施工总承包三级及以上资质、具备有效的安全生产许可证。 3.响应供应商应为本项目配备项目负责人一名，持有市政公用工程或机电工程专业二级建造师及以上资质，且为 本单位在职人员并提供社保证明。 4.响应供应商应为本项目配备专职安全员一名，持有安全生产考核合格C证，且为本单位在职人员并提供社保证 管 明。 5.项目负责人及专职安全员社保证明期限须包含2026年5月至2026年7月。提供的社保证明，须体现上述人员的姓 名、身份证号（或社保号）、单位名称、本单位参保时间（或起始参保时间），并带有社保部门公章或社保部 门的有效电子印章。 2. 信用要求:6.信用要求国： （1）响应供应商（含联合体响应的成员单位）未被“国家企业信用信息公示系统” 网站（www.gsxt.gov.cn）列 入严重违法失信企业名单（如：提供网站查询界面截图）； （2）响应供应商（含联合体响应的成员单位）未被 “信用中国”网站（www.creditchina.gov.cn）列入严重失信 主体名单（中如：提供网站查询界面截图）。 三、采购文件的获取 采购文件在 华润守正采购交易平台 发布，不再另行线下提供纸质采购文件，凡有意参与者请自行登录守正平台 查看和下载采购文件。 四、响应文件的提交 响应文件提交 / 报价截止时间： 2026-08-25 08:00:00 （北京时间，若有变化另行通知）。 响应文件提交 / 报价方式：在响应文件提交 / 报价截止时间前，通过 华润守正采购交易平台 提交电子响应文件或 报价，逾期提交将被拒收。 五、采购人联系方式 联系人：何俊 电话：15178855716 邮箱：1460553040@qq.com 六、采购明细 行号 采购内容 需求数量 单位 补充说明 1 重庆国际生物城配套公寓项目天然气表后管道定制化服务 1 元/次 具体内容详见采购文件 七、答疑澄清、通知 答疑澄清、通知等文件一经在 华润守正采购交易平台 发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注 华润守正采购交易平台 发布的相关信息，并及时查阅和处理。 八、服务费交纳 网 本项目向成交人收取服务费,供应商收到预成交通知书和服务费交款通知书10日内,向平台运营方(华润守正招标有 限公司)支付服务费,经确认无误后由采购人发送成交通知书。平台运营方在收到服务费后向成交人开具服务费发 票。 收费标准：项目总成交金额＜50万元的采购项目，免收服务费。项目总成交金额≥50万元的采购项目，按成交金 务 额的0.15%向成交人收取（金额四舍五入，精确到分）。单项目总收费封顶100000元。其他说明：（1）总价采购， 收费基数为成交金额；单价、费率采购，收费基数为预算金额。（2）单项目存在多个成交人情形的，按总成交 金额计算收费总额，各成交人按成交比例分摊；项目总成交金额50万以上，但单个成交人成交金额少于50万仍按 比例收取服务费。 商 退款说明：成交通知书发布后,平台提供相关服务已完成,成交人已交纳服务费不予退还。 多成交人服务费收取示例： 以某项目总成交金额100万为例,A、B、C多成交人情形,总服务费为0.15万, 供应商A成交金额为50万,A服务费为0.075万; 供应商B成交金额为30万,B服务费为0.045万; 道 供应商C成交金额为20万,C服务费为0.03万。 九、其它事项 管 1.本公告在 华润守正采购交易平台 ( https://www.szecp.com.cn/ )上公开发布。 2.本项目采购通过守正平台线上进行，供应商需注册 华润守正采购交易平台 ，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 国 3.如对采购项目有异议，请登录 华润守正采购交易平台 ,通过异议菜单提出。 2026年08月19日 中 信息来源:https://www.chinapipe.net/project/d3076125.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076125.html</t>
-        </is>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="n">
         <v>80</v>
       </c>
@@ -2352,11 +2256,7 @@
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)非金属管道管件阀门采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）非金属管道管件阀门采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约 330 万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采 购”包括不限于非金属管道管件阀门所含设计、制造、试验、出厂检验、防腐、运输（含保护、包装及运输、 货到现场车板交货）、保险（交货验收前）、指导安装、调试、备件及专用工具、税费、技术资料和图纸及质 保期内的各种备品、备件的供应及相关的技术服务、产品质量证明书及原材料检测报告等。（详见“第五章货 物需求一览中表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 2.6 交货期： 2.6.1合同签订后3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向买方提交完整的技术资料，以供设计院开展相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）投标人具备有效的《中华人民共和国特种设备生产许可证》压力管道管子-B级及以上资质、压力管道管 件B2级及以上资质； （3）投标人具备塑料管道管子、管件的型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4. 招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年 8 月19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 网 5.投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月10 日上午09时30分，地点在重庆市公共资源交易中心开标厅（地 址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见一、二楼大厅显示屏。 务 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 商 本次招标公告在中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 道 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 管 联 系 人：张先生 电 话：023-40717888 国 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区五里店五简路2号重庆咨询大厦A栋20楼2001室 中 项目负责人：彭文婷 电 话： 023-67703002 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购 户名 开户行 投标保证金账号 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000631258 支行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303372 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630010400 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000002549 贸易试验区分行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835014652 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146619529 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764260665 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020038958 信息来源:https://www.chinapipe.net/project/d3076119.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076119.html</t>
-        </is>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
         <v>85</v>
       </c>
@@ -2420,11 +2320,7 @@
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)衬氟管道及管件采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）衬氟管道及管件采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约225万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）衬氟管道及管件采购一批” 包括但不限于制造、涂漆、包装、运输、配合验收工作、检验检测、产品质量证明书等。（详见“第五章货物 （材料）需求一览表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 中 2.6 交货期： 2.6.1合同签订后 3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向招标方提交完整的技术资料，以供设计院开展设备相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）具备有效的《中华人民共和国特种设备生产许可证》-压力管道元件制造-元件组合装置。 （3）具有防腐管道元件特种设备型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4、招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年8 月 19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 5、投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月 10 日上午09时30分，地点在重庆市公共资源交易中心开标厅 （地址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见网一、二楼大厅显示屏。 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 务 本次招标公告在 中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 商 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 道 联 系 人：张先生 电 话：023-40717888 管 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区国五里店五简路2号重庆咨询大厦A栋20楼2001室 项目负责人：彭文婷 电 话： 023-67703002 中 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630011190 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835003139 坝支行 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000000834 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146638621 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051302432 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000620855 支行 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020013554 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764235261 信息来源:https://www.chinapipe.net/project/d3076111.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076111.html</t>
-        </is>
-      </c>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
         <v>85</v>
       </c>
@@ -2496,11 +2392,7 @@
           <t>重庆市益康环保工程有限公司永川分公司蒸汽管道改造项目询价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3076108.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076108.html</t>
-        </is>
-      </c>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="n">
         <v>60</v>
       </c>
@@ -2572,11 +2464,7 @@
           <t>南岸区融侨大道、江南大道片区2023年排水管网改造项目(三标段)招标计划表 重庆市工程建设项目招标计划表 项目名 南岸区融侨大道、江南大道片区 2023年排水管网改造项目（三标段） 称 网 招标法 人或招 重庆市南岸区城市建设发展（集团）有限公司 标人名称 （盖章） 务 项目批 准文件 南岸发改〔2024〕304《南岸区融侨大道、江南大道片区2023年排水管网改造项目总投资概算的批复》 及文号 主要建 包括改造市政混接点194个，改造管网8582米，商管径d300~d1500;缺陷管网开挖修复1355米，管 设内容 径d300~d600;非开挖修复8679米，管径d300~d1200。 招标文件 拟交 合同预估 招标内 招标 序号 招标项目名称 计划发布 易场 金额(万 备注 道容 方式 时间 所 元) 51处雨 污混错 重庆 招标项 接点位 管 市公 目 改 南岸区融侨大道、江南大道片区 2023年排 公开 共资 1 造，1082 2026-08 6600.00 水管网改造项目（三标段） 招标 源交 个管网 易中 三四级 国 心 缺陷修 复。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 中 信息来源:https://www.chinapipe.net/project/d3076097.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076097.html</t>
-        </is>
-      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
         <v>80</v>
       </c>
@@ -2648,11 +2536,7 @@
           <t>中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购公告 永川三教水厂项目 已具备采购条件，现公开邀请供应商参加询比采购活动。 1.采购项目简介 1.1 采购项目名称：中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购。 1.2 采购方案编号：FA00000663117。 网 1.3 采购人：中交一公局重庆工程有限公司。 1.4 采购代理机构：/。 务 1.5 采购项目资金：已落实 1.6 采购项目概况： 商 永川三教水厂项目：项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建 净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、 综合楼、生产建（构）筑物以及附属建筑物等。项目合同额1.7亿元，工期450天。 道 项目地址：重庆市永川区。 2.采购范围及相关要求 管 2.1 采购范围：钢筋混凝土排水管。 2.2 交货期：2026年9月-2026年12月。 2.3 交货地点：重庆市永国川区项目指定地点。 2.4 物资质量标准：满足《混凝土和钢筋混凝土排水管》（GB/T 11836-2023）的相关要求。 3.供应商资格要求 中 3.1 供应商应依法设立且满足如下要求： （1）资质要求：本次询比采购要求供应商须是在中华人民共和国境内依法注册，具有合法有效的营业执照、税 务登记、组织机构代码等证件，具有独立法人资格、具有采购物资生产经营范围的生产商或代理商（销售商）。 （2）财务要求：供应商必须是经税务部门注册登记核准的纳税人，有依法纳税的良好记录。 （3）业绩要求：无。 （4）信誉要求：无不良履约记录、未列入工程所在地质量监督部门和中国交建、中交一公局集团企业黑名单。 因质量原因被交通部质监站通报，正在进行整改的生产厂家和产品不得参与投标。生产商或代理商（销售商） 具有良好的社会信誉，近3年内没有与骗取合同有关的犯罪或严重违法行为而引起的诉讼和仲裁；近3年不曾在合 同中严重违约或被逐；财产未被接管或冻结，企业未处于禁止或取消投标状态；在最高人民法院、信用中国 （www.creditchina.gov.cn）或各级信用信息共享平台查询拟入库单位无不良行为记录。 （5）其他要求：无。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他：无。 4.供应商报名 4.1 有意参加询比采购活动的单位，请于2026年8月19日15时00分至2026年8月26日17时00分（北京时间，下同，法 定公休日、节假日不休），登录“中交招采网”（网址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 网 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 务 5.供应商报价 5.1 报价结束（递交响应文件截止）时间为2026年8月26日17时00分。 商 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的电 子响应文件，采购人将拒收。 5.3电子采购的供应商响应文件由线上电子报价道表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 子报价表的数据为准。 6.开标 管 6.1 开标时间：与报价结束时间相同。 6.2 开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标。 国 7.发布公告的媒介 本询比采购公告在 “中交招采网” 上发布。 中 8.评审办法 本项目评审办法采用 经评审的最低价法 。 9.合同主要条款 9.1 付款条件：按月结算，上月11日至本月10日为一个结算对账期，乙方必须按照甲方要求开具合规的增值税专 用发票，无发票不予付款。结算完成后1个月内支付已结算金额的70%，剩余30%货款在结算完成后3个月内支付。 付款方式为银行转账，甲方有权采用票据支付或者供应链支付的方式支付货款，因此产生的费用包含在综合单 价中，乙方不得因此调价和索赔。如遇业主支付不及时，乙方应予理解。 9.2 履约保证金的递交： （1）R不要求递交 （2）要求递交，保证金金额：/，保证金形式：/，其他形式：/ 。 10.监督机构 监督机构名称： 中交一公局重庆工程有限公司审计部 11.成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联系400-676-5885，中标服务费请按7咨询。 11.1 收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； （3）在1000万元（含）至3000万元之间的，每次收取1000元； 务 （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 11.2 支付流程 （1）通知推送：中标结果发布后，系统自动推送缴费通知（含应缴金额及支付链接）； 道 （2）费用查询：供应商登录“中交招采网—供应商协同—服务费”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网— 供应商协同—服务费—发票查询”模块获取。 12.其他 国 / 。 13.联系方式 中 采 购 人：中交一公局重庆工程有限公司 地 址：重庆市江北区创富路5号 邮 编：361021 联 系 人：汪仁宽 电 话：13527572392 电子邮件：1176245792@qq.com 项目联系人及电话： 序号 项目名称 联系人 联系电话 1 永川三教水厂项目 高博 17788661005 中交一公局重庆工程有限公司 2026年8月19日 物资信息 序号 设备物资名称 设备物资说明 税率 单位 网 1 钢筋混凝土排水管 2000mm Ⅲ级 承插口 13% 米 信息来源:https://www.chinapipe.net/project/d3076078.html 务 cqdingjiu 2026.08.21 10:06:52 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3076078.html</t>
-        </is>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" t="n">
         <v>90</v>
       </c>
@@ -2724,11 +2608,7 @@
           <t>中国铁路成都局集团有限公司重庆市大渡口区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防护工程施 工劳务招标招标公告 重庆市大渡口区萤石及配套企业 35 千伏专用变电站项目穿越渝贵等铁路防护工程施工劳务招标公告 招标编号：DXNZBCQ-GC-2026-13 1. 招标条件 本建设项目重庆市大渡口区萤石及配套企业 35 千伏专用变电站项目穿越渝贵等网铁路防护工程施工劳务招标已由 《中国铁路成都局集团有限公司关于重庆市大渡 口 区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防 护工程施工图设计的复函》（科信技审〔2025 〕115号）批准建设，建设单位为重庆建桥置业有限公司，建设资 金使用外委资金，项 目出资比例为100%，资金已落实。招标人为中国铁路成都局集团有限公司重庆工务段。本 项目已具备法定招标条件，现进行公开招标，特邀请有意向的投标人参加投标。 务 2. 项目概况与招标范围 2.1 项目概况 商 2.1.1建设地点：渝贵线K38+838、南疏Ⅰ线K10+808、川黔线K1+622、川黔线K3+781、兴珞上行线K38+619、兴珞 下行线K38+635、小西线K1+633、南疏Ⅱ线K11+257。 2.1.2建设规模：重庆市大渡 口区萤石及配套企道业35千伏专用变电站项目穿越渝贵等铁 路防护工程，本项目工分为5个交叉工点。工点一采用明挖直埋方式下穿渝贵铁路新白沙沱长江多线特大桥第14孔 （渝贵线K38+838）；工点二采用顶进套管方式下穿南疏 Ⅰ 线K10+808（ 已停用）、川黔线K3+781（ 已停用 ）； 工点三采用明挖直埋方式下穿兴珞线陈家湾双线特大桥（上行线K38+619、下行线K38+635）；工点四采用顶进 管 套管方式下穿。 2.2 招标范围：重庆市大渡口区萤石及配套企业35千伏专用变电站项目穿越渝贵等铁路防护工程施工劳务招标。 即涉铁部分第第三章桥涵，第六章通信、信号、信息及灾害监测，第十章大型临时设施和过渡工程，第十一章 其他费用中的安全生产国费以及非涉铁部分。 2.3标段划分：本项目施工招标划分为1个标段。 2.4计划工期：240日历天，计划开工日期：2026年10月8日，计划竣工日期：2027年6月4日。 中 2.5 其他说明：___/___。 3. 投标人资格要求 3.1本次招标要求投标人为在中华人民共和国境内合法注册的独立法人，具备有效的营业执照、施工企业资质和 安全生产许可证等，并在人员、设备、资金等方面具备相应的施工能力。资格要求如下： 3.1.1 标段编号：全标段 （1）资质要求：施工劳务企业资质。 （2）业绩要求：近3年内完成过铁路营业线类似项目业绩。 （3）项目负责人要求:具有工程师及以上职称，2 年及以上类似铁路营业线项目管理工作经验， 良好的职业道德， 且未在其他在建工程项目任职。 （4）本标段不接受联合体投标申请。 （投标人资格要求详见招标公告附件） 3.2 各投标人可就上述标段中的 1 个标段进行投标。 3.3投标人未在“信用中国”网站（www.creditchina.gov.cn）中被列入失信被执行人名单，投标人未在国家企业信 用信息公示系统（www.gsxt.gov.cn）中被列入严重违法失信企业名单，投标人未被列入铁路工程建设失信行 为“黑名单”，投标人及其法定代表人、拟委派的项目经理在近3年不曾有行贿犯罪记录； 其他信誉要求：未被取消或暂停投标资格、不存在辖内失信的情形、不存在最近一期国铁集团施工企业评价为D 级且在整改期内的情形。 4. 招标文件的获取 4.1凡有意参加投标者，请于2026年08月20日00时00分至2026年08月25日00时00，在重庆龙头寺旅游集散中心（重 庆市两江新区天宫殿街道昆仑大道56号附1号5楼办公室）持单位介绍信获取招标网文件。 4.2招标文件每套售价0元，售后不退。 4.3其他：凡有意参加投标者可通过网上登记获取招标文件，将获取招标文件材料扫描件（PDF格式）发送 务 至dxncq_bgs@163.com邮箱登记，由招标代理人通过电子邮件方式向有意参加投标者发送招标文件。 5. 投标文件的递交 5.1投标文件递交时间为2026年09 月10 日08时30分至2026年商09月10 日09时00分，递交比选申请文件的截止时间（比 选截止时间，下同）为2026年09月10日09时00分，地点为重庆龙头寺旅游集散中心（重庆市两江新区天宫殿街道 昆仑大道56号附1号5楼开标室）。 5.2逾期送达的或者未送达指定地点或者不按照道招标文件要求密封的投标文件，招标代理人不予受理。 6. 发布公告的媒介 本次招标公告在国铁采购平台（https://cg.95306.cn）发布。 管 7. 联系方式 招 标 人：中国铁路成都局集团有限公司 招标代理机构：成都大西南铁路监理 国 重庆工务段 有限公司 地 址：重庆市九龙坡区黄桷坪街道铁 地 址：成都市金牛区站西桥西街305 中 路3村161号 号府河路苑9栋14楼 邮 编： / 邮 编：610081 法定代表人： 法定代表人 或其委托代理人： 或其委托代理人： 联 系 人： 任女士 联 系 人：汤女士 电 话： 17393148353 电 话：023-61896910 传 真： / 传 真： / 电子邮箱： / 电子邮箱：dxncq_bgs@163.com 网 址： / 网 址： / 开户银行： / 开户银行： / 账 号： / 账 号： / 2026年08月19日 附件： 获取招标文件信息表 申请人名称： （加盖公章） 项目名称：（按公告名称填写） 获取招标文件起止时间：（按照公告时间填写） 项目编号：（按照公告填写） 单位名称 经办人 联系电话 电子邮箱 标段 资料提交时间 备注 网 注：须附经办人介绍信、身份证复印件、单位营业执照复印件。 信息来源:https://www.chinapipe.net/project/d3075989.html cqdingjiu 2026.08.21 10:06:53 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075989.html</t>
-        </is>
-      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
         <v>0</v>
       </c>
@@ -2800,11 +2680,7 @@
           <t>长江流域云阳青龙段污水管网一体化建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 长江流域云阳青龙段污水管网一体化建设项目 招标法人或 招标人名称 云阳县青江环境综合整治有限公司 网 （盖章） 项目批准文 云阳发改资环【2025】55号 件及文号 务 主要建设内 新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。 容 招标方 招标文件计 拟交易场 合同预估金额 序号 招标项目名称 招标内容 备注 式 划发布时间 所 (万元) 商 长江流域云阳 新建污水管网55.5千米， 重庆市公 青龙段污水管 其中DN200管网12千 公开招 共资源交 1 网一体化建设 米、DN300管网24千 2026-08 9100.00 标 易中心云 项目EPC总承 米、DN40道0管网19.5千 招标项目 阳分中心 包 米等。 新建污水管网55.5千米， 长江流域云阳 重庆市公 其中DN200管网12千 青龙段污水管 公开招 共资源交 2 管米、DN300管网24千 2026-08 140.00 网一体化建设 标 易中心云 米、DN400管网19.5千 项目监理 阳分中心 米等监理。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 国 信息来源:https://www.chinapipe.net/project/d3075867.html cqdingjiu 2026.08.21 10:06:53 中</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075867.html</t>
-        </is>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="n">
         <v>80</v>
       </c>
@@ -2868,11 +2744,7 @@
           <t>中国电建水电四局华中公司重庆轨道交通17号线一期5标项目雨污水排水迁改工程施工劳务分包采购项目公开询 比采购公告 询比采购公告 采购编号： PC-0104-26J6-FP0895 一、采购条件 受中国水利水电第四工程局有限公司重庆轨道交通17号线一期5标项目委托，中水电四局华中（武汉）工程有限 公司以公开询比方式采购重庆轨道交通17号线一期5标雨污水排水迁改工程项目网，建设资金来源已落实。目前项 目已具备采购条件，现进行公开询比采购。 二、项目概况、采购范围 务 1、项目概况：重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3 站5 区间的土建）：高龙大道 站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子 站区间、石家院子站～终点区间、7/17号线联络线区间。 2、采购范围： 商 （1）雨污水排水迁改工程 （2）工程招标范围工作内容：17号线一期5标道中高龙大道站、斑竹林站及高斑竖井位于城市既有道路下方，设计 采用明挖法施工。为保证市政排水管网的正常使用，在明挖施工前需对既有管网进行临时迁改，车站结构施工 后进行恢复。施工PE钢带管长度2387米、B型排水管长度2799m、钢筋混凝土管127米，检查井239座劳务部分。 （3）施工内容详见工程量清单，以及为完成此项工程而做的一切工作。 管 3、计划工期:计划开工日期：2026年9月25日（具体时间以采购人通知为准），计划完工日期：2027年 12 月25 日； 合同工期总日历天数为457天。 4、质量要求：符合《国给水排水管道工程施工及验收规范》（GB 50268）、《混凝土结构工程施工质量验收规范》 （GB 50204）、《城镇道路工程施工与质量验收规范》（CJJ 1-2008）以及项目所在地最新的相关法规、标准和 图集。工程质量全面达到设计要求和标准，其中：验收合格率 100%，优良率达 90%以上，工程综合验收质量评 定达优良标准。 中 5、付款方式：采用银行转账/支票支付工程价款，月度结算完成具备付款条件后30天内工程进度款支付比例约定 为扣除各项保证金及费用后应付价款不低于65%；清算完成并签订《退场协议》后30天内工程进度款支付比例约 定为扣除各项保证金及费用后应付价款不低于80%；清算完成并签订《退场协议》后一年内工程进度款支付比例 约定为扣除响应人缺陷责任等相关费用后应付价款不低于90%；清算完成并签订《退场协议》，办理完成保证金 退还手续后两年内，工程进度款支付比例约定为扣除响应人缺陷责任等相关费用后应付价款的100%。 6、其他：无。 三、响应人资格要求 响应人必须满足以下全部资格要求： （1）资质要求：施工劳务不分等级 （2）主要人员要求:授权委托人（如有）及项目经理、专职安全员应提供社保和劳动合同。其中劳动合同至少提 供首、末两页，并且包含有关人员的详细信息;社保证明应提供响应截止时间前三个月的社保缴纳记录。 （3）安全三类人员要求:应提供企业主要负责人安全A证、项目经理B证、专职安全员C证。 （4）响应人具有良好的银行资信和商业信誉，没有处于被责令停业，财产被接管、冻结、破产状态。 （5）响应人应具有 雨污水排水迁改 工程的施工业绩，在近 5年内(2021年7月-2026年7月内签订)的施工合同不少 于 1 个，且签订单项合同金额均在 100 万元以上（应附成交通知书和（或）合同扫描件）。 （6）其它要求:无。 （7）本次采购不接受联合体响应。 四、采购文件的获取 凡满足本公告规定资格要求并有意参加的响应人，请于2026年8月22日10时00分前在中国电建采购招标数智化平台 （https://bid.powerchina.cn/bidweb/#/login，以下简称“数智化平台”）获取采购文件，采购文件免费提供。 五、响应文件的递交 1、响应文件递交的截止时间（响应截止时间，下同）为2026年8月26日10时30分网（北京时间），响应人应在截止 时间前通过数智化平台递交电子响应文件。 2、本次采购将通过数智化平台全程在线开展，电子响应文件的加密、提交等流程须响应人在线进行操作。响应 人须提前办理数字证书用于在线递交响应文件，办理方式详见数智化平台首页，并严格按照要求进行在线操作， 务 因操作流程失误造成的递交失败将由响应人自行承担后果。 3、开启由“数智化平台”在响应截止时间后自动对响应文件进行解密，响应人及时关注开启结果。 4、响应截止时间如有变动，采购人将及时通知已获取采商购文件的响应人。 六、发布公告的媒介 本次询比采购公告同时在中国电建阳光采购网道（https://bid-zb.powerchina.cn）上发布。 七、评审办法 采用综合评估法。 管 八、联系方式 采 购 人： 中水电四局华中（武汉）工程有限公司 国 地 址： 湖北省武汉市江岸区塔子湖东路健美街30号立城中心商务楼13、14层 邮 编： 430014 中 联 系 人： 王飞 电 话： 15827222587 电子邮箱： 107830343@qq.com 九、提出异议的渠道和方式 单位名称： 中水电四局华中（武汉）工程有限公司 电 话： 17708178186 电子邮箱： sjhzgsjw@163.com 十、纪检监督机构 响应人或者其他利害关系人认为本次采购活动存在违规违纪行为的，可以书面形式向中国水利水电第四工程局 有限公司中水电四局华中（武汉）工程有限公司纪委办公室（联系方式：17708178186）提出投诉。 2026年8月 19 日 报价网址:https://bid.powerchina.cn/notice/detail?id=2409510708 信息来源:https://www.chinapipe.net/project/d3075750.html cqdingjiu 2026.08.21 10:06:53 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075750.html</t>
-        </is>
-      </c>
+      <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
         <v>85</v>
       </c>
@@ -2944,11 +2816,7 @@
           <t>万州区2026年超长期特别国债高标准农田建设项目拟进行预制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜的 信息公告 1.采购条件 1.1本项目万州区2026年超长期特别国债高标准农田建设项目工程已由 重庆市万州路桥建设有限公司承建，项目 业主为重庆市万州区农业技术与机械推广中心，代建业主为重庆市万州区农业发展有限公司，建设资金为国债 资金，项目出资比例为 100% ，承包人为重庆市万州路桥建设有限公司。项目已具备施工条件，现对该项目的预 制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜发布信息公告。 网 2.项目概况与采购范围 2.1建设地点：重庆市万州区走马镇、瀼渡镇、罗田镇、余家镇、高梁镇、分水镇、柱山乡等7个镇乡。 务 2.2本项目材料采购拟进行比选情况如下： 罗田镇谷山片区材料采购费暂定金额约： 17.5万元； 余家镇桥亭片区材料采购费暂定金额约： 17.99万元； 商 柱山乡山田片区材料采购费暂定金额约： 26.32 万元； 走马镇凉风片区材料采购费暂定金额约： 15.道66万元； 瀼渡镇高村片区材料采购费暂定金额约： 17.72 万元； 分水镇大冲片区材料采购费暂定金额约： 47.12 万元； 管 高梁镇茨坪片区材料采购费暂定金额约： 10.7万元； （以上片区片区金额为暂定金额，最终比选限价金额以比选文件为准）。 国 2.3计划采购周期： 以合同签订为准 日历天。 2.4采购范围：本项目各片区所包含的预制钢筋砼管、成品混凝土仿木栏杆等材料。 中 3.供应商资格要求 3.1本次材料采购要求供应商具备独立企业法人，具有本次所需材料生产能力的厂家或经销商等，其经营范围和 权限应满足本次所需材料的要求，并依法取得国家行政主管部门颁发的有效工商营业执照(建筑材料销售或水泥 制品制造、水泥制品销售等相关营业资格），所提供产品必须满足各项检测要求，达到国家现行标准规定的合 格标准。具有良好的商业信誉和充分的供应保障能力，具备相应售后服务能力。要求竞选人为一般纳税人，可 开具13%税率增值税专用发票，提供一般纳税人认定证明。 3.2本次供应商单位优先选择万州本地企业。 3.3本次 不接受 联合体竞选。 4. 报名要求 4.1报名时间：2026年8月 19日9:00起至 8月21日17:00止。 4.2报名地点：重庆市万州路桥建设有限公司经营部（重庆市万州区天城东路278号）。 4.3报名时，须提交有效的营业执照(有效工商营业执照((建筑材料销售或水泥制品制造、水泥制品销售等相关营 业资格）)，前述证书均为复印件并加盖单位公章。法定代表人参加报名的不需要授权委托书，只需要提供法定 代表人身份证明；非法定代表人参加报名的除提供法定代表人身份证明外还须提供授权委托书、委托代理人身 份证明。 4.4 本项目材料采购需提前报名。经资格预审合格后，通知资格预审合格的供应商，到承包人单位领取相关文件。 4.5本项目材料采购设七个片区进行比选，为保证比选公平、公正、有效，规定同一参选单位报名片区上限为2个， 且最终仅限中选一个片区。 5.联系方式 承包人：重庆市万州路桥建设有限公司 地 址：重庆市万州区天城东路278号 网 联系人： 张红娟 电 话：15923491915 务 邮 箱： 商 重庆市万州路桥建设有限公司 2026年8月19日 道 信息来源:https://www.chinapipe.net/project/d3075512.html cqdingjiu 2026.08.21 10:06:53 管 国 中</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075512.html</t>
-        </is>
-      </c>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" t="n">
         <v>80</v>
       </c>
@@ -3020,11 +2888,7 @@
           <t>中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水 管道)招标采购流标公告 发布单位：中国铁建/中铁十一局/六公司 发布时间：2026-08-19 10:40:49 投标截至时间：2026-08-18 10:00:00 内容： 各投标人： 网 中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资（污水 管道）公开招标采购（采购编号： CR1106-JC-2026-26-02）评标工作，已于北京时间2026年08月18日10:00整，在 铁建云链（https://www.crccep.com）线上平台公开开标。评审委员会根据招标文件载明的评审办法完成评审工作， 现将评审结果公示如下： 务 一、招标公告发布日期及媒体 招标公告发布日期：2026年07月27日至2026年08月01日 商 招标公告媒体：铁建云链（https://www.crccep.com） 二、拟中标信息 道 公开招标采购编号：CR1106-JC-2026-26-02 包件号：WSGD-01 序号 供应商名称 推荐排序 管 1 无 1 国 以上包件有效投标不足三家，本次招标做流标处理。 三、公示时间 中 自2026年08月19日始，至2026年08月22日止。在公示期间，所有竞标人和其他利害关系人如对公示的评审结果有 异议，可以向相关监督部门举报，逾期将不再受理。举报人必须由其法定代表人或者授权代表签字并盖章，其 他组织或者个人举报的，必须由其主要负责人或者本人签字，并附有效身份证明复印件。举报人如实反映情况 受法律保护。 公示期满，如无异议，即时生效。 监督竞诉受理部门： 中铁十一局集团第六工程有限公司招采中心 联系电话：18671041790 信息来源:https://www.chinapipe.net/project/d3075461.html cqdingjiu 2026.08.21 10:06:53</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075461.html</t>
-        </is>
-      </c>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" t="n">
         <v>80</v>
       </c>
@@ -3088,11 +2952,7 @@
           <t>协同创新区-四期房建三标段镀锌管件物资竞价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3075420.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075420.html</t>
-        </is>
-      </c>
+      <c r="N36" t="inlineStr"/>
       <c r="O36" t="n">
         <v>60</v>
       </c>
@@ -3164,11 +3024,7 @@
           <t>长江一级支流溉澜溪流域(新华水库混流箱涵)污水收集效能提升工程(渝北区)施工答疑补遗文件 长江一级支流溉澜溪流域（新华水库混流箱涵）污水收集效能提升工程（渝北区）施工答疑文件 各潜在投标人： 现将“长江一级支流溉澜溪流域（新华水库混流箱涵）污水收集效能提升工程（渝北区）施工”公开招标项目 答疑文件发布。本答疑文件是在招标文件的基础上作出的澄清、说明或补正，与招标文件具有同等法律效力， 若相关内容与原招标文件不一致时，一律以本答疑文件内容为准。 网 一、答疑部分： 问题一：1、我公司于2026年进行了优势合并整合，现准备使用合并前公司项目业绩作为本次我司投标的投标人 业绩证明，并提供上级主管单位出具的相关吸收合并文件或两家公司签订的吸收合并协议，请问是否可视为满 务 足招标业绩要求？ 2、我单位为中型企业，其控股股东为大企业，但我单位不属于大企业的分支机构，也不存在与大企业的负责人 为同一人的情形。鉴于此种情况，我单位应提供《中小企业声明函（工程类）》还是《中小企业承担合同份额 承诺函》？ 商 回复：1. 满足，但还需满足招标文件对业绩的其他要求。最终由评标委员会根据投标人提供的证明材料并结合 招标文件要求进行评审； 道 2. 贵司其控股股东为大企业，故需提供中小企业承担合同份额承诺函。 问题二：本项目有无业主专家参与评标？ 管 回复：该项目评标委员会由招标人按法律法规及相关规定依法组建。 问题三：请明确是否有业主专家 是否异地评标 回复：1. 该项目评标委国员会由招标人按法律法规及相关规定依法组建。 2.本项目是异地评标。 问题四：1、财务报告可以不提供财务报表附注吗? 中 2、投标函附录中，工期、分包、工程质量、缺陷责任期等要求可以统一填写"达到招标文件要求"吗? 3、招标文件第八章投标文件格式中(二)承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要提供其 他格式之外的其他承诺? 4、是否有业代专家参与评标，不要模糊的回答什么依法组建评标委员会。请明确回复有或者没有。 5、本项目是否异地评标？ 6、业绩竣工验收证明材料中有单位盖的项目部章是否认可呢？ 回复：1. 可以不提供财务报表附注。 2. 可以统一填写"达到招标文件要求"。 3. 投标人自行核实招标文件要求提供的承诺要求，如有需要，还需补充提供招标文件第八章投标文件格式中 （二）承诺部分之外的其他承诺。 4. 该项目评标委员会由招标人按法律法规及相关规定依法组建。 5. 本项目是异地评标。 6. 不认可。 问题五：请问**公司现在被人民法院列为被执行人且有1000多万股权冻结到2028年，因为不能履行保函的见索即 付，拒绝赔付。 相关业主方在招标文件补遗通知中直接将**公司列入担保公司回避名单，拒绝**公司所出具的保函。由此可 见**公司的信用资质、履约能力、根本无能力是存在很大问题的。请问以**公司目前的被执行和不履行投标担保 责任的情况是否符合招标文件的要求? 回复：纸质投标保函的开立人应当是具有相应资格的银行、保险机构、融资担保公司，其信用资质、履约能力、 担保能力、赔付流程、安全保密等应符合工程保函业务条件。纸质投标保函应合网法合规，符合招投标行政监督 部门、行业主管部门和金融监管部门的相关规定，满足招标文件约定要求。投标人应选择在渝依法设立总部或 者设有分支机构的金融机构开具纸质投标保函。投标人对所提交的纸质投标保函的真实性、合法性、有效性负 责。以纸质投标保函形式交纳投标保证金是否符合招标文件要求，由评标委员会评标时，根据招标文件要求进 行独立评审，并作出相应评审判断。 务 问题六：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 回复：经核实，招标文件（PDF签章版）中投标文件格式商与重庆市电子招投标系统投标文件制作软件中格式一致。 可能因重庆市电子招投标系统投标文件制作软件中的格式页边距与招标文件（PDF签章版）不一致的原因导致格 式显示不一致，该情形不影响投标人编制投标文件。若重庆市电子招投标系统投标文件制作软件导出的投标文 件格式与招标文件（PDF签章版）的投标文件格式不一致，以重庆市电子招投标系统投标文件制作软件导出的投 标文件格式为准。 道 问题七：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖 章，请问需要提供联合体协议书吗？ 管 回复：若投标人提供的公司业绩为epc业绩，且合同协议书或工程竣工验收合格的证明材料或业主证明能证明该 投标人承担的工作为施工任务的，则不需要提供联合体协议书；若投标人提供的公司业绩为epc业绩，但合同协 议书或工程竣工验收合格的证明材料或业主证明不能证明该投标人承担的工作为施工任务的，则需要提供联合 体协议书。 国 问题八：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可 以不填(空白)，对此有无要求？ 回复：投标中文件中下划线上、空格处、表格中无需要填写或无法填写内容的，填“/”或“无”均可。 问题九：公园施工业绩符合吗？ 回复：公园概念太宽泛，无法判定该施工业绩是否属市政工程，请投标人自行核实，并按招标文件要求提供施 工业绩证明材料，其是否满足要求应由评标委员会根据证明材料具体内容进行判定。 问题十：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需 要提供其他格式之外的其他承诺？ 回复：投标人自行核实招标文件要求提供的承诺要求，如有需要，还需补充提供招标文件第八章投标文件格式中 （二）承诺部分之外的其他承诺。 问题十一：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收， 请问我公司业绩满足业绩要求吗？ 回复：不满足。 问题十二：可以用自己做的材料购买协议、劳务协议、设备租赁协议作为低价说明证明材料吗？ 回复：投标人投标总报价低于招标文件规定的对应的异常低价警戒线的，应提供报价合理性说明，并提供必要 的证明材料。证明材料由投标人自行提供，但提供的说明不得降低或者改变原设计方案、技术工艺、施工标准， 不得影响项目的质量、安全、工期、结算等正常履约。 问题十三：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 回复：按照招标文件要求“提供：会计师事务所或审计机构出具的合法有效的财务审计报告及财务报表，财务 报表须至少包括现金流量表、资产负债表、利润表”。 问题十四：业绩要求的竣工时间是指竣工验收时间吗？ 回复：本项目业绩要求所指竣工时间，即为工程竣工验收合格证明载明的竣工验收时间。 问题十五：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知 书发出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面网通知相关金融机构本项目准 予提前注销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 回复：纸质投标保函原件上未加盖“正本”字样的，不因此否决投标，但投标人应确保提交的保函为唯一正本。 若因保函真伪问题导致的一切不利后果由投标人自行承担。 务 问题十六：燃气管道安装施工业绩满足吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 商 问题十七：请问招标人是否委派业主专家参与评标吗？ 回复：该项目评标委员会由招标人按法律法规及相关规定依法组建。 道 问题十八：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 回复：根据招标文件“投标人的工程量清单单项报价不得为零报价（招标人提供的工程量清单单项最高限价中 金额为零的除外）或者负数报价”，招标人提供的工程量清单单项最高限价中金额为零的，该项清单综合单价 管 报价可以为0。 问题十九：自来水厂或者净水厂施工业绩满足业绩要求吗？ 回复：满足，但还需满国足招标文件对业绩的其他要求。 问题二十：财务报告可以不提供财务报表附注吗？ 回复：可以不提供财务报表附注。 中 问题二十一：老旧小区室外环境改造施工业绩符合吗？ 回复：不满足。 问题二十二：有人提出一个无关问题。 回复：无关问题不予回复。 问题二十三：任一清单的综合单价低于警戒线，就要提供说明吗？ 回复：本招标项目单项报价未设置异常低价警戒线。 问题二十四：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 问题二十五：本项目是异地评标吗？ 回复：本项目是异地评标。 问题二十六：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、 注册证及在本单位注册的证明文件替代？ 回复：不满足。 问题二十七：污水处理厂提标改造施工业绩满足吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 问题二十八：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 回复：可以填“达到招标文件的要求”。 问题二十九：财政部 国务院国资委 金融监管总局2023年9月14日发布的《关于加网强审计报告查验工作的通知》 中要求会计师事务所应当按照规定将其承办《中华人民共和国注册会计师法》第十四条规定审计业务出具的报告 （以下简称审计报告）上传注册会计师行业统一监管平台（以下简称统一监管平台）并申请赋码。本项目投标 人提供的财务报告需要赋码和提供深度查询截图吗？ 务 回复：投标人提供的财务报告不需要赋码和提供深度查询截图。 问题三十：有人提出一个无关问题。 回复：无关问题不予回复。 商 问题三十一：我公司业绩合同金额3600万元及以上，但是竣工报告业绩金额小于3600万元，请问是否满足业绩要 求？ 道 回复：按招标文件执行。“当上述业绩证明材料中针对同一指标存在不一致时，以工程竣工验收合格的证明材 料为准”。 问题三十二：专业分包业绩满足业绩要求吗？ 管 回复：专业分包业绩可满足业绩要求，但还需满足招标文件对业绩的其他要求。 问题三十三：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养 老保险证明材料复印件国递交吗？ 回复：不需要。 问题三十四：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要 中 求”吗？ 回复：可以统一填写“达到招标文件要求”。 问题三十五：市政桥梁施工业绩满足业绩要求吗？ 回复：满足，但还需满足招标文件对业绩的其他要求。 问题三十六：有人提出一个无关问题。 回复：无关问题不予回复。 问题三十七：本项目委派业主专家吗？ 回复：该项目评标委员会由招标人按法律法规及相关规定依法组建。 特别提示：本通知与招标文件具有同等法律效力，若招标文件与本通知不一致时，一律以本通知为准。 招标人：重庆水务环境控股集团管网有限公司 招标代理机构：重庆市工程管理有限公司 2026年8月19日 信息来源:https://www.chinapipe.net/project/d3075975.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075975.html</t>
-        </is>
-      </c>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="n">
         <v>0</v>
       </c>
@@ -3240,11 +3096,7 @@
           <t>中化重庆涪陵化工搬迁后污水处理厂建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 中化重庆涪陵化工搬迁后污水处理厂建设项目 招标法人或 招标人名称 重庆市涪陵交通旅游建设投资集团有限公司 网 （盖章） 项目批准文 涪发改委发[2019] 505号 件及文号 务 主要建设内 新建一体化提升泵站及管道约5000m，投资约800万元。 容 招标 招标 招标文件计 拟交易 合同预估 序号 招标项目名称 备注 内容 方式 划发布时间 场所 金额(万元) 商 本招标计划与2026年5 月25日发布的招标项目 中化重庆涪陵 重庆市 名称为“中化重庆涪陵 招标项目 化工搬迁后污 涪陵区 公道开 化工搬迁后污水处理厂 1 水处理厂建设 施工 2026-09 公共资 800.00 招标 建设项目（场外连接管 项目（场外干 源交易 网）”的招标计划，除 管部分） 中心 招标项目名称调整外， 其余内容完全一致。 管 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075591.html cqdingjiu 2026.08.21 10:国06:54 中</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075591.html</t>
-        </is>
-      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="n">
         <v>80</v>
       </c>
@@ -3316,11 +3168,7 @@
           <t>綦江区污水处理厂设施设备更新改造工程(二期)招标公告 1.招标条件 本招标项目 綦江区污水处理厂设施设备更新改造工程（二期） 已由 重庆市綦江区发展和改革委员会 以 重庆市企业投资备案证（项目代码：2502-500110-04-01-844057） 批准建设，项目业主为 重庆南州城市管 理服务有限公司 ，建设资金来自 上级补助和业主自筹 ，项目出资比例为 100% ，招标人为 重庆南州 城市管理服务有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审的最低 投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 綦江区 2.2 项目概况与建设规模：对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造， 务 包括配电柜、风机、污水提升泵、在线监测等设备更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污 水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。 2.3 本项目工程总投资金额： 约1327.40万元 商 2.4 招标范围： 本项目设计施工图和招标文件、答疑、补遗、工程量清单等资料所涉及的全部内容。 2.5 工期要求： 180日历天 道 缺陷责任期要求： 24个月 2.6 标段划分（如有）： / 管 2.7 其他： / 3.政府采购工程 国 3.1 是否属于政府采购工程：否 4.投标人资格要求 中 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（綦江区） （https://www.cqggzy.com/qijiangweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（綦江区）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间 从本公告发布至2026-08-22 18:00:00前。 5.3招标人应于2026-09-11 18:00:00前在重庆市公共资源交易网（綦江区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（綦江区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆南州城市管理服务有限公司 代理机构: 永卓国际工程技术有限公司 地 址: 重庆市綦江区红星美凯龙生活广场3幢19-3 地 址: 两江新区网泰山大道东段98号2幢10-12号 邮 编: 邮 编: 项目负责人: 赵老师 项目负责人: 廖淼 电 话: 023-48690537 电 话: 务023-60391733 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 商开户银行: 账 号: 账 号: 监督部门: 道 电 话: 2026年08月18日 綦江区污水处理厂设施设备更新改造工程（二期） 管 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051287453 中国农业银行股份有限公司重庆自由贸 重庆联合产权交易所集国团股份有限公司 312601010400083780000031123 易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146631326 信息来源:https://www.chinapipe.net/project/d3075589.html 中 cqdingjiu 2026.08.21 10:06:54</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075589.html</t>
-        </is>
-      </c>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" t="n">
         <v>90</v>
       </c>
@@ -3392,11 +3240,7 @@
           <t>南岸区峡口、迎龙片区农村供水保障提升工程招标计划表 重庆市工程建设项目招标计划表 项目 南岸区峡口、迎龙片区农村供水保障提升工程 名称 招标 网 法人 或招 标人 重庆市江南城市建设发展（集团）有限公司 名称 务 （盖 章） 项目 批准 商 文件 南岸发改﹝2026﹞156号 及文 号 本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体 主要 化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统， 建设 对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平 内容 台。概算批复工程建安费2975.27万元。 管 拟 招 招标文 合同预 招标 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 国 所 南岸 重 区峡 庆 口、 中 市 迎龙 朱家岩水厂升级改造工程：对全厂老旧设备进行设备更新；对全 公 片区 公 厂进行智慧化改造，增加高级工艺控制系统；对厂区建筑和构筑 共 农村 开 1 物修缮；优化加药系统投加模式，增加精确加药系统；对全厂部 2026-08 资 1600.00 供水 招 分老旧管道进行更换；金属防腐工程，对金属设备和管道的防锈 源 保障 标 刷漆工作。 交 提升 招标 易 工程 项目 中 （一 心 标段） 南岸 重 区峡 庆 口、 市 迎龙 公 片区 管网工程：延伸、改造峡口镇、迎龙镇等4个乡镇 46 公里 公 共 农村 DN40~DN300 配水主支管，36公里 DN20入户管道，新建3座一体 开 2 2026-08 资 1300.00 供水 化智慧加压泵房，入户水表改造 1752 户，并配套建设监测计量 招 源 保障 基础设施。 标 交 提升 易 工程 中 （二 心 标段） 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075572.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075572.html</t>
-        </is>
-      </c>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="n">
         <v>90</v>
       </c>
@@ -3468,11 +3312,7 @@
           <t>北碚区东阳天府片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区东阳天府片区农村供水提升工程 招标法人或招 标人名称（盖 重庆北碚文旅产业发展有限公司 网 章） 项目批准文件 及文号 务 工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水 主要建设内容 管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网 附属设施。 招标项目名 招标内 招标方 招标文件计划 拟交易场 合同预估金 序号 商 备注 称 容 式 发布时间 所 额(万元) 北碚区东阳 招标项目 重庆市公 天府片区农 施工招 公开招 1 2026-08 共资源交 8457.00 村供水提升 标 道标 易中心 工程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075569.html 管 cqdingjiu 2026.08.21 10:06:55 国 中</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075569.html</t>
-        </is>
-      </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="n">
         <v>80</v>
       </c>
@@ -3544,11 +3384,7 @@
           <t>北碚区澄江片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区澄江片区农村供水提升工程 招标法人或招标 重庆北碚文旅产业发展有限公司 人名称（盖章） 网 项目批准文件及 文号 改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供 主要建设内容 务 水管网68.5km及其附属设施。 招标项目名 招标文件计划 合同预估金 序号 招标内容 招标方式 拟交易场所 备注 称 发布时间 额(万元) 招标项目 北碚区澄江 商重庆市公共 1 片区农村供 施工招标 公开招标 2026-08 资源交易中 8741.00 水提升工程 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 道 信息来源:https://www.chinapipe.net/project/d3075568.html cqdingjiu 2026.08.21 10:06:55 管 国 中</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075568.html</t>
-        </is>
-      </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="n">
         <v>80</v>
       </c>
@@ -3620,11 +3456,7 @@
           <t>涪陵区江东街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区江东街道农村供水保障能力提升工程（二期） 名称 招标 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 项目 网 批准 文件 涪陵发改〔2026〕471号 及文 号 主要 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 建设 以及配套电气工程。 务 内容 招 标 合 文 同 招 件 预 招标 标 招标方 计 拟交易 备 序号 招标项目名商称 估 项目 内 式 划 场所 注 金额 容 发 (万 布 元) 时 间 重 道 庆 市 涪 陵 公 区 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 开 公 1 涪陵区江东街道农村供水保障能力提升工程（二期） 2026-09 3137.22 管以及配套电气工程。 招 共 标 资 源 交 易 中 心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075558.html cqdingjiu 2026.08.21 10:06:55 中</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075558.html</t>
-        </is>
-      </c>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" t="n">
         <v>80</v>
       </c>
@@ -3696,11 +3528,7 @@
           <t>涪陵区龙桥街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 涪陵区龙桥街道农村供水保障能力 项目名称 提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水 名称（盖 有限公司 章） 网 项目批准 文件及文 涪陵发改〔2026〕466号 号 改造荣桂水厂老化、破损、生锈的 务 输水管道7.36公里。马武水厂增设 废水回收及污泥浓缩系统1套。荣 桂水厂增设废水回收及污泥浓缩系 主要建设 统1套。新建配水管道总长0.74公里； 商 内容 改造配水管道总长139.42公里。新 建1座微型集成泵房及改造1座泵 站(原牌坊泵站)。新增管网监测设 施40套。 道 招标 合同 招 文件 预估 标 招标方 拟交易 备 招标项目 序号 招标项目名称 计划 金 内 式 场所 注 管 发布 额(万 容 时间 元) 改造荣桂水厂老化、 破损、生锈的输水管 国 道7.36公里。马武水厂 增设废水回收及污泥 重庆 浓缩系统1套。荣桂水 市涪 厂增设废水回收及污 公 陵区 中 涪陵区龙桥街道农村供水保障能力 泥浓缩系统1套。新建 开 1 2026-09 公共 3236.36 提升工程 配水管道总长0.74公里； 招 资源 改造配水管道总 标 交易 长139.42公里。新建1 中心 座微型集成泵房及改 造1座泵站(原牌坊泵 站)。新增管网监测设 施40套。 本计划表所列招标项目信息均为暂 备注 定，最终以实际招标时的信 信息来源:https://www.chinapipe.net/project/d3075556.html cqdingjiu 2026.08.21 10:06:55</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075556.html</t>
-        </is>
-      </c>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="n">
         <v>90</v>
       </c>
@@ -3772,11 +3600,7 @@
           <t>涪陵区百胜镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区百胜镇农村供水保障能力提升工程 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕465号 及文 号 务 主要 建设整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。 内容 招 拟 标 招招标文 合同预 交 序项 标件计划 估金 备 招标内容 易 号目 方发布时 额(万 注 场 名 商 式间 所 元) 称 涪 陵 区 重 百 庆 胜 市 招标 镇 涪 项目 农 道 陵 村 公 区 供整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1开 公 1 2026-09 1489.90 水套及配套电气工程。 招 共 保 标 资 障 源 能 交 力 易 提 中 管 升 心 工 程 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075553.html 国 cqdingjiu 2026.08.21 10:06:55 中</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075553.html</t>
-        </is>
-      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="n">
         <v>80</v>
       </c>
@@ -3848,11 +3672,7 @@
           <t>涪陵区清溪镇农村供水保障能力提升工程招标计划 重庆市工程建设项目招标计划表 项目名称 涪陵区清溪镇农村供水保障能力提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕467号 务 号 对清溪水厂原取水口进行改造。改造清溪水厂输水管道长6.38公里。清溪水厂新建3000m3/d集成水 主要建设 厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04 内容 公里。四合村泵站增加1套备用加压泵。新商增管网监测设施35套。 招标项目 招标方 招标文件计 拟交易场 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 所 (万元) 对清溪水厂原道取水口进行 改造。改造清溪水厂输水 管道长6.38公里。清溪水厂 涪陵区清 新建3000m3/d集成水厂1套， 重庆市涪 招标项目 溪镇农村 增设废水回收及污泥浓缩 公开招 陵区公共 管 1 供水保障 2026-09 2888.89 系统1套。新建配水管道总 标 资源交易 能力提升 长2.46公里。改造配水管道 中心 工程 总长145.04公里。四合村泵 站增加1套备用加压泵。新 国 增管网监测设施35套。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075552.html 中 cqdingjiu 2026.08.21 10:06:55</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075552.html</t>
-        </is>
-      </c>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" t="n">
         <v>80</v>
       </c>
@@ -3924,11 +3744,7 @@
           <t>涪陵区珍溪镇农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区珍溪镇农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕476号 及文号 (一)改造11000m3/d(旺水垭6000m3/d和二水厂5000m3/d)原水处理系统及辅助设施，主要有加氯系统、 加药系统、清水池、絮凝池、重力无阀滤池、商污水处理回收池、二水厂泵房设备等及其他辅助设施。 主要建 (二)更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪 设内容 湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km， 新建应急泵站至百汇大桥配水管9km：百汇至观将泵站4.5km；共计37.3km。 道 招标项目 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 场所 (万元) (一)改造11000m3/d(旺水 垭6000m3/d和二水厂5000m3/d) 管 原水处理系统及辅助设施，主 要有加氯系统、加药系统、清 水池、絮凝池、重力无阀滤池、 污水处理回收池、二水厂泵房 涪陵国区珍 设备等及其他辅助设施。(二) 重庆市 招标项 溪镇农村 更换旺水垭水厂至张家塘配水 涪陵区 目 供水保障 公开招 1 管13.5km，张家塘至滴水配水 2026-09 公共资 3427.27 能力提升 标 管长3.3km，全长16.8km；滴水 源交易 中工程（一 至洪湖配水管长0.3km；更换八 中心 期） 一水库至旺水垭水厂引水 管1.7km，更换珍溪二水厂至珍 溪大桥配水管5km，新建应急 泵站至百汇大桥配水管9km： 百汇至观将泵站4.5km；共 计37.3km。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075551.html cqdingjiu 2026.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075551.html</t>
-        </is>
-      </c>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" t="n">
         <v>80</v>
       </c>
@@ -4000,11 +3816,7 @@
           <t>涪陵区武陵山镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区武陵山镇农村供水保障能力提升工程 名称 招标 网 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 务 （盖 章） 项目 批准 商 文件 涪陵发改〔2026〕468号 及文 号 主要 道 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高位水箱4座（总容积 354立方米），武 建设 陵山水厂新建废水处理系统1套及配套电气工程等。 内容 招 管 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 国 称 涪 陵 区 中 重 武 庆 陵 市 山 招标 涪 镇 项目 陵 农 公 区 村 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高 开 公 1 供 位水箱4座（总容积 354立方米），武陵山水厂新建废水处理系统1套 2026-09 1861.77 招 共 水 及配套电气工程等。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075549.html cqdingjiu 2026.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075549.html</t>
-        </is>
-      </c>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" t="n">
         <v>80</v>
       </c>
@@ -4076,11 +3888,7 @@
           <t>涪陵区江东街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区江东街道农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕470 号 及文号 主要建 建设配水管网总长 34.80km，新建加压泵站 2 座、改造已成泵站 2 座、新建加氯加药间 1 座、新建高位 设内容 水箱 7 座、新建计量监测设施以及配套电气工程商。 招 招标文件 拟交 合同预估 序 招标项 标 备 招标内容 计划发布 易场 金额(万 号 目名称 方 注 道 时间 所 元) 式 涪陵区 重庆 招标项 江东街 市涪 目 建设配水管网总长 34.80km，新建加压泵站 2 座、 公 道农村 陵区 管 改造已成泵站 2 座、新建加氯加药间 1 座、新建高 开 1 供水保 2026-09 公共 3503.77 位水箱 7 座、新建计量监测设施以及配套电气工 招 障能力 资源 程。 标 提升工程 交易 （一期） 中心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075548.html cqdingjiu 20中26.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075548.html</t>
-        </is>
-      </c>
+      <c r="N49" t="inlineStr"/>
       <c r="O49" t="n">
         <v>90</v>
       </c>
@@ -4144,11 +3952,7 @@
           <t>中国电建水电五局二公司重庆轨道交通17号线一期7标内外涂环氧消防复合钢管管件采购项目公开竞价采购(二次 挂网)变更公告(一) 详见附件。 信息来源:https://www.chinapipe.net/project/d3075376.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075376.html</t>
-        </is>
-      </c>
+      <c r="N50" t="inlineStr"/>
       <c r="O50" t="n">
         <v>60</v>
       </c>
@@ -4220,11 +4024,7 @@
           <t>2026年石柱分公司黄水镇黄连大道通信管道建设招标公告 ZB_ZHAOBIAOGONGGAO_START 本询比项目为 2026年石柱分公司黄水镇黄连大道通信管道建设 （标段 编号： CQBBFA202604170051 ），采购人为 中国电信股份有限公司石柱分公司 ，采购代理机构为 。项目 资金已落实。 具备采购条件，现进行公开询比，特邀请有意向的且具有提供标的物能力的潜在供应商（以下简 称供应商）参加询比响应。 1.项目概况与采购内容 1.1项目概况： 2026年石柱分公司黄水黄连大道通信管道修复项目主要针对黄水网黄连大道受损通信管道进行修 复80米 本次集中询比合同有效期为： 2026.9-2026.12 1.2采购内容 及标包划分情况： 务 1.2.1 本次询比的规模、货物名称、数量及主要技术参数、交货期及交货地点具体如下：黄水镇黄连大道80米通 信管道修复。 序号 标包名称 产品名称 规格型号 数量 交货地点 交货期 商 2026年石柱分公司黄水 黄水镇黄连 1 镇黄连大道通信管道建 管道建设 新建2孔110波纹管、 新建2孔蜂窝管 80 2026.12.20 大道 设 道 本项目 不划分标包 。 ${ } ${ 本项目允许供应商同时成交的最多标包数为 0 个。 } 本项目将按照最新的《中国电信供应商不良行为管 理规则》执行供应商不良行为处理结果，请重点关注处理结果适用的供应商主体、被处理产品、处理范围、禁 限期、处理措施等关键内容，请务必登录中国电信阳光采购网（https://caigou.chinatelecom.com.cn）查阅《中国 管 电信供应商不良行为管理规则》。 本项目根据《中国电信供应商不良行为管理规则》选择适用备选处理措施 （但涉及生产安全责任事故的处理结果不适用备选措施）。 1.2.2成交供应商数量： 1 个，每个成交供应商对应的份额如下 ： [请在此处自行编辑与采购方案相同的成交原则] 国 ${ 1.2.2成交供应商数量如下： [ 请在此处自行编辑与采购方案相同的有效供应商及成交供应商数量原则相关表格 ] 每个成交供应商对应的份额如下: [请在此处自行编辑与采购方案相同的份额分配原则] } 1.3本项目 设置最高 响应限价 。 设置最高响应限价，最高响应限价为不含税31000元人民币/计算方法，供应商响应报价高于最高 响应限价的，其响应将被否决 供应商响应报价高于最高响应限价的，其响应 将被否决。 ${ } 2.供应商中资格要求 2.1供应商基本资格要求 2.1.1 供应商 应为 中华人民共和国境内 法律上和财务上独立的法人或依法登记注册的其他组织，合法运作并 独立于采购人和采购代理机构。 供应商应具有良好的银行资信和商业信誉。法人下属不具备法人资格的分支机 构参与响应的，应提供所属法人针对本项目或覆盖本项目的经营事项的有效授权。 2.1.2 供应商 的法定代表人或负责人为同一人或者存在控股、管理关系的不同 供应商 ，不得参加同一标包响应或 者未划分标包的同一询比项目响应。 ${ 2.1.3 } ${ 2.1.3 } 2.1.4 本次询比 不接受 联合体响应。 ${如 供应商 为联合体，应满足下列要求： （1） 联合体各方必须按询比文件提供的格式签订联合体协议书，明确联合体牵头人和各方的权利义务； （2）由同一 专业的单位组成的联合体，按照资质等级较低的单位确定资质等级； （3）联合体各方不得再以自己名义单独或 加入其他联合体在同一标包或者未划分标包的同一询比项目中响应。 ${ （4） 。} } 2.1.5 本次询比 不接受代理商响应。 ${ （1）产品制造商注册地在中华人民共和国境外（与中华人民共和国有正常贸易与往来的国家或地区）及香港、 澳门、台湾地区且必须使用代理商响应和签订销售合同的；（2）产品制造商为注册地在中华人民共和国境内的 外资企业（包括香港、澳门、台湾地区资本）或者由外国投资者（包括香港、澳门、台湾地区）享有绝对控制权 （最大或最多表决权）的企业且必须使用代理商响应和签订销售合同的。代理商响应的，应满足下列要求 ： } ${ （1） ${ （2） 供应商与产品制造商 的代理合作关系迄今为止应已持续 0 年（含）以上。 } ${ （3） } } ${ 2.1.6 与供应商有产品代工制造关系的制造商不得参加同一标包响应或者未划分标包的同一询比项目响 应。 } 2.1.7 供应商须提供2022年1月1日至本项目发布公告之日的同类项目（通信管道施工类）证明材料， 合同累计金额不低于3万元（含税） 2.2供应商不得存在下列情形之一 （1） 为采购人不具有独立法人资格的附属机构（单位）； （2） 被依法暂停或取消 投标/ 响应资格的； （3） 被责令停产停业、暂扣或者吊销许可证、暂扣或者吊销执照； （4） 进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （5） 在最近三年内（自 2022年04月01日 起）被相关行业主管部门或司法机关认定有骗取 中标/成交 、严重 违约、重大工程质量或者安全问题的； 网 （6） 在最近五年内（自 2022年06月01日 起）被判处单位行贿罪，且行贿行为与采购活动相关的（以“中国 裁判文书网”的生效判决为准）； （7） 在最近五年内（自 2022年06月01日 起）被判处合同诈骗罪的（以“中国裁判文书网”的生效判决为 务 准）； （8） 被最高人民法院在“信用中国”网站（www.creditchina.gov.cn）或各级信用信息共享平台中列入失信被执 行人名单，已执行完毕或不再执行的除外； 商 （9） 为本询比项目提供过设计、编制技术规范和其他文件的咨询服务 ； （10） 为本工程项目的相关监理人，或者与本工程项目的相关监理人存在隶属关系或者其他利害关系； 道 （11） 为本询比项目的代建人 ； （12） 为本询比项目的采购代理机构 ； 管 （13） 与本询比项目的监理人或代建人或采购代理机构同为一个法定代表人 ； （14） 与本询比项目的监理人或代建人或采购代理机构存在控股或参股关系 ； （15） 被工商行政管理国机关在国家企业信用信息公示系统中列入严重违法失信企业名单的； （16） 中国电信在职员工违规担任供应商法定代表人并参与采购活动的； （17） 中国电信集团有限公司/中国电信股份有限公司中层及以上管理人员违反有关领导人员配偶、子女及其配 中 偶经商办企业行为管理规定，其配偶、子女及其配偶经商办企业参与采购活动的； （18） 中国电信领导人员离职或退休后三年内违反《国有企业领导人员廉洁从业若干规定》等相关规定任职、 投资入股的私营企业、外资企业和中介机构，参与其原任职单位采购活动的； ${ （19） } （19） 其他按照中国电信供应商不良行为处理结果及《中国电信供应商不良行为管理规则》的结 果执行规则，应对供应商及其响应产品在本项目中执行禁止采购处理措施的； （20） 法律法规、询比文件限定的其他情形。 ${ 供应商 是代理商的，本条所指的 供应商 也包括其所代理的制造商。 } ${ 联合体响应的，联合体成员均不得 存在上述任一情形。 } 2.3产品资格要求 2.3.1 产品 应是来自中华人民共和国 ${或是与中华人民共和国有正常贸易与往来的国家或地区} 的 成熟稳定的 产品 。 ${ 2.3.2 产品 。 } ${ 2.3.3 产品 。 } ${ 2.3.4 。 } ${ 2.3.5 。 } 2.3.6 产品应符合中国电信相关技术要求， 并满足以下关键技术指标： （1） 序号 技术指标 具体要求 1 开挖深度 埋深≥0.8m（道路≥1.2m） 2 施工规格 本次修复选择开挖换管：开挖约80米，2孔110波纹管、2孔蜂窝管，新建两通信手控井 ${ 2.3.7 产品 业绩要求： 。 } ${ 2.3.8 。 } ${ 2.4 产品制造商资格要求 2.4.1 制造商应提供合法有效的登记 （或注册）证明文件，应具有良好的银行资信和商业信誉。 } ${ 2.4.2 } ${ 2.4.2 } ${ 2.4.3 } ${ 2.4.4 } ${ 2.4.5 } ${ 2.5现场考察 } ${ 2.6评价检测 } 2.7 法律法规规定的其他要求。 3.资格审查方法 本项目将进行资格后审，资格审查标准和内容见询比文件第三章“评审办法”，凡未通过资格后审的供应商， 其响应将被否决 。 网 4.询比文件的获取 4.1询比文件获取时间: 2026年08月25日 00时00分00秒 至 2026年09月01日 00时00分00秒 （北京时间，下同）。 4.2询比文件获取方式：登录“中国电信阳光采购网（https://caigou.c务hinatelecom.com.cn）”后，通过“招投标-采 购文件领取”模块或通过“电子采购入口”跳转中国电信电子采购系统，进入本项目进行询比文件登记申领， 未在系统注册的供应商须先进行注册，注册方法详见本公告“ 7 供应商注册”。 4.3询比文件费用： 本项目不收取文件费用。 ${每套售价商 0 元人民币，售后不退。支付要求： } 5.响应文件的递交 5.1响应文件递交截止时间（即响应截止时间）为： 2026年09月02日 00时00分00秒 道 5.2 电子响应文件的提交方式：登录中国电信阳光采购网（https://caigou.chinatelecom.com.cn）后，通过“招投 标-我的项目”模块或通过“电子采购入口”跳转中国电信电子采购系统，选择本项目进行响应文件提交，供应 商应在响应文件提交截止时间之前通过电子采购系统完成加密电子响应文件的上传。供应商未在电子采购系统 进行询比文件申领登记或电子响应管文件未按照要求加密的，将无法通过电子采购系统提交电子响应文件 。 5.3 本项目将于响应文件提交截止同一时间通过中国电信电子采购系统开启响应文件， 采购人/采购代理机构 邀 请响应供应商的法定代表人或者其委托代理人准时参加 。 国 ${ 6.样品的递交 6.1样品递交的时间、地点：于 递交至 。 } 7. 供应商注册 7.1 中国电信阳光采购网注册 未注册过的潜在供应商，须通过中国电信阳光采购网（https://caigou.chinatelecom.com.cn）首页“立即注册”模 中 块完成注册后，方可申领本项目询比文件。 7.2 CA证书办理 参加询比响应的潜在供应商须提前办理CA证书，并确保CA证书在使用时有效。CA证书办理流程详见中国电信 阳光采购网首页“操作指引-CA办理”。 7.3 技术支撑联系方式 服务热线：4000111884 服务邮箱：zb_support@chinatelecom.cn（电子采购系统技术支撑） ctsc@chinatelecom.cn（CA证书办理技术支撑） 8. 发布公告的媒介 本询比公告在 中国电信阳光采购网（https://caigou.chinatelecom.com.cn） 、中国招标投标公共服务平台 （http://www.cebpubservice.com/） 上发布，其他媒介转载无效。 9. 联系及异议接收方式 9.1 联系方式 采 购 人: 中国电信股份有限公司石柱分公司 采购代理机构: 地 址： 重庆市石柱县城南路6号 地 址： 无 邮 编： 邮 编： 无 联 系 人： 马卫平 联 系 人： 无 电 话： 17365204567 电 话： 无 电子邮件： 17365204567@189.cn 电子邮件： 无 网 址： www.chinatelecom.com.cn或“/” 网 址： 无 网 开户银行： 无 账 号： 无 9.2 异议接收方式 务 登录中国电信阳光采购网（https://caigou.chinatelecom.com.cn）后，通过“招投标-采购异议-提出异议”模块提出。 采购代理机构： 商 2026年08月25日 信息来源:https://www.chinapipe.net/project/d30道75344.html cqdingjiu 2026.08.21 10:06:56 管 国 中</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075344.html</t>
-        </is>
-      </c>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" t="n">
         <v>0</v>
       </c>
@@ -4288,11 +4088,7 @@
           <t>重庆站站房CQZSG-4标项目蓝色PVC袖阀管(外径60mm)询价采购公告 ZTEJWZ-JZ-2026-询027（一） 采购单位:重庆站站房CQZSG-4标段项目经理部 发布时间:2026-08-18 19:06 报价截止时间:2026-08-21 10:00 招标方联系人:刘健 网 招标方联系电话:13540650091 招标方邮箱: 务 监督方联系人:纪委 监督方联系电话:028-87653066 商 监督方邮箱: 保证金:0.0元 道 结算与发票信息: 结算方式：上月21日至本月的20日为一个结算周期，当月20日为本月的结算截止日期。结算时根据甲方检验合格 及双方共同签认的凭证计算当月实际收货数量。 管 支付条件：结算完成后，甲方在收到乙方开具的正式的增值税专用发票后第1个月支付该批物资结算金额的70%， 第12个月支付20%，剩余10%在第18-24月内按月均衡支付。 发票种类：增值税专用国发票 发票抬头：中铁二局集团有限公司 税号：9151中0100MA61RKR7X3 其他要求： 交货信息: 交货方式:点数验收 收货人:刘健 收货人联系方式:13540650091 其他说明事项: 流水号：询2026081800458 交 标的 规格 计量 标的编号 数量 技术标准及要求 货 送货地址 名称 型号 单位 期 蓝色PVC袖阀管，外 西南区-重庆市-市辖区-渝中区-重 袖阀 径60mm，壁 庆市菜园坝立交以西，龙家湾隧道 0950999183764 - 23188.0 米 管 厚4.5-5mm PVC管，承压 以东，菜袁路以北，王家坡以南的 不小于5MPa,节长4m 地块内，原重庆站。 报价网址:http://www.crecgec.com 信息来源:https://www.chinapipe.net/project/d3075317.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075317.html</t>
-        </is>
-      </c>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" t="n">
         <v>0</v>
       </c>
@@ -4364,11 +4160,7 @@
           <t>涪陵区蔺市街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（一期） 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕474号 及文 号 主要 务 建设新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。 内容 拟 招招标文 合同预 招标 交 序 标件计划 估金 备 项目招标内容 易 号 方发布时 额(万 注 名称 场 式间 元) 所 商 重 庆 涪陵 市 区蔺 招标 市街 涪 项目 道农 陵 公 区 村供 新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收 开 公 1 水保 2026-09 3611.91 及污泥浓缩处理系统。 招 共 障能 道 标 资 力提 源 升工程 交 （一 易 期） 中 心 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075278.html 管 cqdingjiu 2026.08.21 10:06:57 国 中</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075278.html</t>
-        </is>
-      </c>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" t="n">
         <v>80</v>
       </c>
@@ -4440,11 +4232,7 @@
           <t>涪陵区李渡街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区李渡街道农村供水保障能力提升工程 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕469号 及文 号 商 主要 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套 建设 附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建测控井78座。 内容 招 拟 标 道 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 管 涪 陵 区 重 李 庆 渡 市 街 国 招标 涪 道 项目 陵 农 公 区 村 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂 开 公 1 供 塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建 2026-09 2372.74 招 共 水中测控井78座。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075277.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075277.html</t>
-        </is>
-      </c>
+      <c r="N54" t="inlineStr"/>
       <c r="O54" t="n">
         <v>80</v>
       </c>
@@ -4516,11 +4304,7 @@
           <t>涪陵区珍溪镇农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目名称 涪陵区珍溪镇农村供水保障能力提升工程（二期） 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕477号 务 号 (一)本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管 主要建设 有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵 内容 站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水 箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。 招标项目名 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 称 式 划发布时间 场所 (万元) 道 (一)本项目对珍溪镇23个 村(社区)安装配水管网660km 及配套附属设施，其 中：1.De160~De40的PE管 管 有232km；2.连接各村社 涪陵区珍溪 重庆市 的De32~De20的PE管有381km； 招标项目 镇农村供水 涪陵区 3.219~32的衬塑钢 公开招 1 保障能力提 2026-09 公共资 2182.77 管47km。(二)购置安装泵 标 升工国程（二 源交易 站14座(一用一备共计28台水 期） 中心 泵)，其中新建泵站10座、更 换泵站4座及配套电力设施; 新建不锈钢水箱2座等。(三) 中 购置安装(0~25kg)减压阀61 个;排污阀(25kg）3个。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075275.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075275.html</t>
-        </is>
-      </c>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" t="n">
         <v>90</v>
       </c>
@@ -4592,11 +4376,7 @@
           <t>涪陵区蔺市街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（二期） 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕475号 及文 号 商 主要 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 105.307km（dn20-dn40PE 建设 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座；新建测控井 52座。 内容 拟 招 招标文 合同预 招标 交 序 道 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 重 庆 涪陵 管 市 区蔺 涪 招标 市街 陵 项目 道农 公 区 村供 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 开 公 1 水保 105.307km（dn20-dn40PE 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座； 2026-09 2652.89 国 招 共 障能 新建测控井 52座。 标 资 力提 源 升工程 交 （二 易 期） 中 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075274.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075274.html</t>
-        </is>
-      </c>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" t="n">
         <v>80</v>
       </c>
@@ -4660,11 +4440,7 @@
           <t>重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目项目公告 重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称）比选公告 1.比选条件 本比选项目重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称），比选人为重庆市排 网 水有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。中标后合同与重庆市豪洋水务 建设管理有限公司签订。现对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 2.项目概况与比选范围 务 2.1 建设地点：重庆市巴南区 2.2 项目概况：本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1,该管道为自流管道， 位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道 为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现 象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水 厂的正常收水及运行，需对该段管道进行改造。 道 2.3 比选范围：拆除现状管道为DN600混凝土管，同时需拆除并新建9座检查井。 2.4 工期要求：30日历天，以甲方通知进场时间为准。 管 2.5缺陷责任期要求：24个月 3.投标人资格要求 国 3.1 本次比选要求投标人须具备以下条件： 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质。 中 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 项内容。 3.2 本次比选接受不联合体投标。 4.比选文件的获取 4.1 投标人于2026年8月 18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子 版，以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都 视为投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的 一切后果由投标人自行负责。各投标单位应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行供应商注册，填写相关信息，审批过后成为 平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价、递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，将被否决投标。 4.4 比选文件每份售价800元，售后不退。投标单位在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标 文件。 5.投标文件的递交 5.1 电子投标文件递交时间：2026年8月24日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月24日14时00分至14时30分（北京时间），地点：重庆水务招标采购中心 （重庆市两江新区嘉华路36号重庆水务大厦5楼）。 5.3 投标截止时间：2026年 8月24日14时30分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆市排水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝中区长江滨江路126号 地 址：重庆市两江新区嘉华路36号重庆水务大厦 道 联 系 人： 黄老师 联 系 人： 黄晓华 电 话： 023-67767416 电 话： 18523396416 管 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3075272.html 国 cqdingjiu 2026.08.21 10:06:57 中</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075272.html</t>
-        </is>
-      </c>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
         <v>90</v>
       </c>
@@ -4736,11 +4512,7 @@
           <t>重庆市潼南城区老旧供水管网改造工程招标计划 重庆市工程建设项目招标计划表 项目名称 重庆市潼南城区老旧供水管网改造工程 招标法人或招 标人名称（盖 重庆市潼南自来水有限公司 网 章） 项目批准文件 及文号 务 主要建设内容 改建潼南城区输水主管网约39.63km及配套相应阀门阀件等 招标方 招标文件计 拟交易场 合同预估 序号 招标项目名称 招标内容 备注 式 划发布时间 所 金额(万元) 对城区供水管网上商 重庆市潼南城 老旧阀门阀件、设 区老旧供水管 重庆市潼 招标项目 施设备进行更换， 网改造工程 公开招 南区公共 1 保障供水管网稳定 2026-09 918.00 （城区配套阀 标 资源交易 运行合道理增设部分 门阀件改造工 中心 计量及压力监控、 程） 水质监控等。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3075266.html cqdingjiu 2026.08.21 10:06:58 国 中</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075266.html</t>
-        </is>
-      </c>
+      <c r="N58" t="inlineStr"/>
       <c r="O58" t="n">
         <v>80</v>
       </c>
@@ -4812,11 +4584,7 @@
           <t>关于为【重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购】公开选取【工程设计】 机构的公告 我单位在重庆市网上中介超市公开选取工程设计中介服务机构，现将相关事项公告如下： 该项目为直接选取项目，由采购人从报名的中介服务机构中直接选定一家中介服务机构进行项目服务。 项目 重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购 名称 网 采购 重庆市开州区河堰镇人民政府 人 投资 审批 否 务 项目 是否 破产 商 业务 否 服务 项目 采购 道 所需 中介 其他 服务 事项 管 所需 服务 工程设计 类型 项目实施地点为国河堰镇清泉社区，项目建设内容为：硬化2米宽生产便道5.5千米，100方防旱池1口，50方 服务 蓄水池1口，标准自动化育苗大棚1个，蔬菜小棚20个，水源处理设施1套，水肥一体化配套设施1套，新 内容 建50平方米设备管理房，完善蔬菜基地配套设施等。工程总投资335万元。选取此项目设计单位（含预算 编制服务）。 中 中介 机构 资质（资格）要求 要求 资质 （资 1、报名单位提供有效的营业执照，资质证书（资质丙级或丙级以上），具备从事项目设计服务工作； 2、 格） 具有独立承担民事责任的能力； 3、具有良好的商业信誉和健全的财务会计制度； 4、具有履行合同所必 要求 需的专业技术能力； 5、有依法缴纳税收和社会保障资金的良好记录。 说明 其他 要求 无 说明 服务 时限 无要求，按照合同双方自行约定 说明 服务 3.1%费率 金额 金额 按文件要求执行 说明 选取 直接选取 方式 需规 避机 构 规避 原因 选取 2026-08-20 16:00:00 （选取时间到达后不接受报名，建议中介机构至少在选取开始半小时前完成报名。） 时间 采购 人业 网 务咨 重庆市开州区河堰镇人民政府（18716685679） 询电 话 采购 务 需求 26清泉社区项目设计服务采购说明.pdf 书下 载 商 2026-08-18 信息来源:https://www.chinapipe.net/project/d3075198.html 道 cqdingjiu 2026.08.21 10:06:58 管 国 中</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075198.html</t>
-        </is>
-      </c>
+      <c r="N59" t="inlineStr"/>
       <c r="O59" t="n">
         <v>90</v>
       </c>
@@ -4888,11 +4656,7 @@
           <t>重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目招标公告 1.招标条件 本招标项目重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目已由重庆市开州区发展和改革委员会以开州 发改审〔2026〕357号批准建设，项目业主为重庆市开州区长沙镇人民政府，建设资金来自开州区2026年中央和 市级提前批财政衔接推进乡村振兴补助资金，项目出资比例为 100% ，招标人为重庆市开州区长沙镇人民 政府。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：开州区长沙镇桔香村 2.2 项目概况与建设规模：1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输 线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米， 务 周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。 2.3 本项目工程总投资金额： 500万元 本次招标项目合同估算金额： 446.278921万元 商 2.4 招标范围：招标人发布的由重庆中煜华资工程技术有限公司设计的《重庆市开州区2026年长沙镇桔香村柑橘 基地改造提升项目》施工图及图纸说明、招标文件(含补遗)及工程量清单、答疑资料、澄清资料范围内所涉及的 工作内容，具体以招标人发布的工程量清单及道施工图为准。 2.5 工期要求： 150日历天 缺陷责任期要求： 12个月 管 2.6 标段划分（如有）： / 2.7 其他： / 国 3.政府采购工程 3.1 是否属于政府采购工程：是 中 3.2 是否专门面向中小企业预留：否，按照《政府采购促进中小企业发展管理办法》第六条第(三)“按照本办法 规定预留采购份额 无法确保充分供应、充分竞争，或者存在可能影响政府采购目标实现的情形”的规定，故本 项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包叁级及以 上资质或市政公用工程施工总承包叁级及以上资质或水利水电工程施工总承包叁级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）下载招 标文件、工程量清单、电子图纸等资料。参与投标的投标人需在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）完成市 场主体信息登记以及CA数字证书办理，办理方式请参见 重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、 重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）导航栏“主体信息”页面中“市场主 体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完 成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告 发布至2026-08-21 17:00:00前。 5.3招标人应于2026-08-25 23:59:59前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源 交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）发布澄清。 6.投标文件递交的内容 网 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-21 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 务 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交 易监督网上发布。] 商 8.联系方式 招 标 人: 重庆市开州区长沙镇人民政府 代理机构: 重庆毅仁建设项目管理有限公司 重庆市开州区文峰街道天鹅湖社区富厚街158号附10 地 址: 重庆市开州区长沙镇山花街1号 地 址: 道号 邮 编: 邮 编: 项目负责人: 丁敬余 项目负责人: 谭毅 电 话: 15826368887 管电 话: 13452653126 传 真: 传 真: 电子邮箱: 1415705480@qq.com 电子邮箱: 开户银行: 国 开户银行: 账 号: 账 号: 监督部门:中重庆市开州区公共资源交易管理局 电 话: 023-52218977 2026年08月17日 重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目 户名 开户行 投标保证金账号 重庆市开州区公共资源交易中心 重庆农村商业银行股份有限公司开州支行 3401010120010012772000200 中国农业银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 314401010400104500000006031 业部 中国工商银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 9558853100005824176 业部 重庆市开州区公共资源交易中心 重庆银行股份有限公司开州支行 680101040007547-100984 重庆市开州区公共资源交易中心 中国银行股份有限公司重庆开州支行 108865555576VA00149 信息来源:https://www.chinapipe.net/project/d3075199.html cqdingjiu 2026.08.21 10:06:58</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3075199.html</t>
-        </is>
-      </c>
+      <c r="N60" t="inlineStr"/>
       <c r="O60" t="n">
         <v>90</v>
       </c>
@@ -4964,11 +4728,7 @@
           <t>万盛城区老旧供水管网更新改造工程答疑及补遗(一) 万盛城区老旧供水管网更新改造工程 答疑及补遗（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程答疑及补遗（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。? 问题2：本项目是否采用异地评标方式？ 答：是 。 商 问题3：本项目是否有业主代表，如有，请明确业主代表数量。 答：是，本项目评标委员会共7人，其中在重道庆市综合评标专家库随机抽取5人，招标人代表2人 。 问题4：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 答：可以。 管 问题5：污水处理厂提标改造及附属管道施工业绩满足吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 国 问题6：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可以 不填(空白)，对此有无要求？ 答：无要求。? 中 问题7：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖章， 请问需要提供联合体协议书吗？ 。 答： 根据招标文件第二章“投标人须知前附表”1.4.1 第3条业绩要求中：“注：（2）投标人提供的业绩为联 合体业绩的，其在该业绩中的工作分工应与本项目承担的工作一致。”要求，故需要提供联合体协议书。 问题8：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要求”吗？ 答：填写“达到招标文件的要求”或按照招标文件相关条款填写具体内容均可 。 问题9：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 答：投标人的工程量清单单项报价不得为零报价(招标人提供的工程量清单单项最高限价中金额为零的除外)或者 负数报价，否则由评标委员会作否决投标处理。 问题10：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知书发 出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面通知相关金融机构本项目准予提前注 销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 答：需要。但不将加盖正本作为评审因素。 问题11：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收，请 问我公司业绩满足业绩要求吗？ 答：不满足。? 问题12：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 答：可以 。 问题13：业绩要求的竣工时间是指竣工验收时间吗？ 答：是的。 网 问题14：重庆市电子招投标系统投标文件-报价部分“己标价工程量清单”-“投标总价”页面招标人名称需要填 写吗？ 务 答：由投标人自行决定是否填写，是否填写不作为评审因素。 问题15：请问招标人是否委派业主专家参与评标吗？ 答：是，本项目评标委员会共7人，其中在重庆市综合评商标专家库随机抽取5人，招标人代表2人。 问题16：自来水厂或者净水厂含管道施工业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需道满足招标文件要求。? 问题17：有没有人行贿专家，有的话我们就不参加了。 答：本项目评标委员会由招标人按法律法规及相关规定依法组建。 管 问题18：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要 提供其他格式之外的其他承诺？ 答：请各潜在投标人仔国细阅读招标文件，并按招标文件要求提供相应承诺。 问题19：财务报告可以不提供财务报表附注吗？ 答：可以。 中 问题20：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题21：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、注册证 及在本单位注册的证明文件替代？ 答：退休证等材料不能替代养老保险证明，按招标文件执行。? 问题22：本项目是异地评标吗？ 答：是。 问题23：现在除了没有警戒线和技术方案的低价项目评标专家不被围猎，哪个项目不围猎评标专家，请问招标人 如何保证公平？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题24：没有低价警戒线怎么保证中高价呢？ 答：本项目未设置低价警戒线，通过综合评估法对各潜在投标人进行评审。分值由技术、商务、报价组成，综 合实力优良的投标人合理中高价可依靠综合得分优势参与竞争，同时招标文件履约追责条款约束投标人理性报 价，保障合理报价竞争环境。 问题25：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养老保险 证明材料复印件递交吗？ 答：现场递交纸质保函原件的人员不作要求 。 问题26：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 网 答：电子投标系统中锁定不可修改的格式（如封面、投标函）直接填空即可，其他投标文件格式以加盖公章的 招标文件PDF文件为准。? 问题27：专业分包业绩满足业绩要求吗？ 务 答：不满足。 问题28： 市政道路包含给水管网施工业绩满足业绩要求吗？ 商 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题29：技术负责人在资格审查部分中提供了工程类高级及以上职称证后，在商务部分中再提供工程类高级及以 上职称证可以加分吗？ 道 答：可以。 问题30：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 管 全是万盛的公司中的！业主、专家全是你们自己人吧？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 国 二、补遗 1、本次重新发布本项目的工程量清单，在《重庆市公共资源交易网》(綦江区) （https://www.cqggzy.com/qijiangweb/）网上发布，请投标人自行下载。 中 招 标 人：重庆市万盛经济技术开发区城市管理局 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 信息来源:https://www.chinapipe.net/project/d3074975.html cqdingjiu 2026.08.21 10:06:58</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074975.html</t>
-        </is>
-      </c>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" t="n">
         <v>80</v>
       </c>
@@ -5040,11 +4800,7 @@
           <t>重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 1.招标条件 本招标项目 重庆市巴南区土桥片区内涝积水整治工程已由重庆市巴南区发展和改革委员会以巴南发改审 发[2025]33号文批准建设，项目业主为重庆市巴南区住房和城乡建设委员会，代建业主为重庆市巴南公路建设有 限公司，建设资金来自区级财政资金统筹，项目出资比例为 100%，招标人为重庆市巴南公路建设有限公司。 项目已具备招标条件，现对该工程的勘察设计进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 2.1 建设地点：重庆市巴南区花溪街道、李家沱街道 务 2.2 项目概况与建设规模：为解决片区内涝问题，在李家沱街道、花溪街道改建 d400-d800 雨水管网 9665m，管材 采用高密度聚乙烯(HDPE)缠绕结构壁管 B型管；改建 d1商000-d1400雨水管网 664m，管材采用高密度聚乙 烯(HDPE)缠绕结构壁管 B 型管、III 级钢筋混凝土管；改建 d1500-d2000 雨水管网 426m，管材采用III 级钢筋混凝 土管;改建 d2100-d2600 雨水管网 1000m，管材采用 III 级钢筋混凝土管；修复雨水管网 5345m，增加智能感知设 备6 套。 道 2.3 本项目工程总投资金额：13477.10万元 管 本次招标项目工程费估算金额：11061.83万元 国 本次招标项目勘察设计合同估算金额：334.544万元 中 2.4 招标范围：主要包括勘察、施工图设计（包含高边坡、深基坑）和相应阶段的勘察工作，以及提供施工现场 全过程技术服务，并配合业主办理相关手续等，具体范围为： （1）勘察部分：完成本项目范围内的勘察工作，包括但不限于排水管网排查、1:500地形图测量、地质钻勘、管 线内窥、物探、综合管线测量，市政管网错混接点测量及调查等工作，解决区域地下空间臭气问题，勘察成果 需达到重庆市城市建成区排水管网排查技术导则的要求，并配合业主完成对应的成果审查等事宜。 （2）设计部分：包括不限于完成本项目的施工图设计、施工期间交通组织设计、桥梁（涉轨）安全论证方案及 施工期间至竣工验收阶段，质量保修阶段的设计配合服务，配合办理施工图审查相关手续及竣工验收阶段、质 量保修阶段的设计服务等工作以及协助招标人完成各项审批手续办理等工作。 2.5 勘察设计服务期限：30日历天 2.6 标段划分（如有）：/ 2.7 其他：/ 3.政府采购工程 3.投标人资格要求 3.1 本次招标要求投标人须具备以下条件： 网 3.1.1 本次招标要求投标人具备的资质条件： 务 投标人应同时具有建设行政主管部门颁发的下列勘察和设计两类资质： 商 I、投标人应具备下列勘察资质之一： 道 ①工程勘察综合甲级资质。 管 ②工程勘察专业类（岩土工程）专业甲级资质和工程勘察专业类（工程测量）甲级资质； 国 II、投标人应具备下列设计资质之一： 中 ①工程设计综合甲级资质； ②工程设计市政行业甲级资质； ③工程设计市政行业(燃气工程、轨道交通工程除外)甲级资质； ④工程设计市政行业(排水工程)甲级资质。 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的勘察设计能力，详见招标文件第二章投标人须知 前附表第1.4.1项内容。 3.2 本次招标接受联合体投标。联合体投标的，应满足下列要求：联合体组成单位数量不超过2家，由负责设计 任务的单位作为联合体牵头人。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件及其附件、澄 清、修改、补充通知、最高限价通知等资料。参与投标的投标人需在重庆市公共网资源交易网完成市场主体信息 登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息 登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程 电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 务 布至2026-08-23 12:00:00前。 4.3招标人应于2026-08-26 17:00:00前在重庆市公共资源交易网发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-24 09:30，投标人应当在投标截止时间前，通过互 商 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督道网、重庆市公共资源交易网、重庆市公共资源交易网（巴南区） 发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 重庆市巴南公路建设有限公司 代理机构: 重庆云远项目管理有限公司 管 地 址: 重庆市巴南区龙洲大道265号 地 址: 重庆市九龙坡区渝隆大厦28楼 邮 编: 邮 编: 项目负责人: 牟老师 项目负责人: 李强 国 电 话: 023-66238079 电 话: 023-68434996 传 真: 传 真: 电子邮箱: 电子邮箱: 中 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 2026年08月18日 重庆市巴南区土桥片区内涝积水整治工程勘察设计 户名 开户行 投标保证金账号 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000001675 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051304894 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020041267 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764210157 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000682897 支行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835000509 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146639123 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630018252 信息来源:https://www.chinapipe.net/project/d3074953.html cqdingjiu 2026.08.21 10:06:58 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074953.html</t>
-        </is>
-      </c>
+      <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
         <v>95</v>
       </c>
@@ -5116,11 +4872,7 @@
           <t>重庆管道公司2026年涪陵压气站管道、设备防腐项目-非招标公告 公告发布时间: 2026年08月18日09时02分19秒 一、概述 1.2.1项目概况：涪陵作业区涪陵压气站空压机、阀门等设备、消防泵房消防管道、循环水管道油漆出现锈蚀情况， 为保证设施安全运行，对站场设备、消防管道及附属钢结构进行打磨除锈、油漆防腐。 二、采购项目与标段 交货期限: 开工之日起90日内完工 网 质保期限(月): 标段 序号 标段名称 标段描述 编号 重庆管道公司2026年涪陵 涪陵作业区涪陵压气站空压务机、阀门等设备、消防泵房消防管道、循 1 1 压气站管道、设备防腐项 环水管道油漆出现锈蚀情况，为保证设施安全运行，对站场设备、消 目 防管道及附属钢结构进行打磨除锈、油漆防腐。 三、供应商资格要求 商 *1、响应人资质要求（1）响应人必须是依照中华人民共和国法律在国内注册，具备合格有效的营业执照的法人、 其他组织；与采购人存在利害关系可能影响询比采购公正性的法人、其他组织或者个人，不得参加响应。单位 负责人为同一人或者存在控股、管理关系的不同单位，不得参加同一标段响应或者未划分标段的同一询比项目 响应。（2）响应人须具备防水防腐保温工程专业承包二级及以上资质。*2、信誉要求响应人在响应文件提交截 止当日不存在以下情况：（1）响应人被“国道家企业信用信息公示系统”网站（www.gsxt.gov.cn）列入严重违法 失信企业名单（响应文件提交截止时间前已移出的除外）。（2）响应人被“信用中国”网站 （www.creditchina.gov.cn）列入严重失信主体名单（响应文件提交截止时间前已移出的除外）。（3）响应人或其 法定代表人、负责人、拟委任的项目经理被“中国执行信息公开网”（http://zxgk.court.gov.cn/shixin/）列入失信 被执行人名单（响应文件提交截止时间前已移出的除外），响应文件中需提供有效身份证号供查询。（4）响应 管 人、拟委任的项目经理被“全国建筑市场监管公共服务平台”网站（https://jzsc.mohurd.gov.cn/home）列入黑名单 （响应文件提交截止时间前已移出的除外）。上述（1）-（4）条以评审当日评审小组从官网查询信息为准。（5） 被国家管网集团或西南管道公司暂停、取消投标资格或业务承揽资格。（6）法律、行政法规规定的其他不允许 参与投标的情况。 国 四、询比文件的获取 4.1 有意向参加项目者，于2026年08月20日09时05分22秒前，登录数字供应链平台进行项目报名。 中 4.2 报名成功后于2026年08月18日09时01分42秒至2026年08月24日09时05分22秒，登录数字供应链平台进行项目下 载询比文件。 五、响应文件的递交 5.1 请于2026年08月24日11时00分00秒前，登录数字供应链平台递交项目响应文件。 5.2 逾期将无法进行递交响应文件，采购人将不予受理。 5.3 供应商在递交响应文件前，应按照有关规定提供人民币0万元项目保证金。 六、响应文件的开启 6.1 响应文件的开启时间2026年08月24日11时06分00秒 6.1 响应文件的开启地点供应链系统上 七、采购人信息 地址： 邮编： 联系人：舒建华 联系电话：18581824001 电子邮件：shujh@pipechina.com.cn 传真： 开户银行： 账户名： 账号： 信息来源:https://www.chinapipe.net/project/d3074904.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074904.html</t>
-        </is>
-      </c>
+      <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
         <v>0</v>
       </c>
@@ -5192,11 +4944,7 @@
           <t>重庆燃气集团股份有限公司输配分公司大渡口调压站至二郎调压站次高压燃气管线工程(大渡口段)公告 采购 公告 公告编号： RQXYGG202608130064 一、采购项目基本情况 网 采购人：重庆燃气集团股份有限公司输配分公司 采购项目编号：RQCGXY202608130040 务 采购项目名称：大渡口调压站至二郎调压站次高压燃气管线工程（大渡口段） 采购内容或范围：安装部分： ①材料验收（甲供材料：阀门、管材、弯头、标志桩等）、运输及履带式挖掘机及人工布管； ②管道管件安装， 新旧管道的碰口；③安装DN400直埋球阀1座； ④管道和商焊口的除锈及防腐； ⑤管道下沟后15KV电火花检测； ⑥管道的清管，强度及严密性试验；⑦警示带敷设和线路标志桩（砖）安装； ⑧监检手续等。 土建部分： ①清表； ②扫线、平整场地； ③沟槽、基坑、阀井砌筑； ④回填土方； ⑤余方弃置； ⑥人工开挖人行道（花 台），公路及路面恢复； ⑦其他线缆穿跨越工道程施工，交通组织； ⑧水工保护等。 （具体内容详见施工图纸和 工程量清单） 公告发布时间 ：2026-08-18 14:39:10 管 二、采购人联系方式 联系人：王瑶 电话：023-67502265 国 邮箱：wangyao232@crcgas.com 三、采购明细 中 行号 采购内容 需求数量 单位 补充说明 拟邀请单位 大渡口调压站至二郎调压站次高压燃气管线 重庆燃气安装工程有限责任公 1 1 项目 无 工程(大渡口段) 司 四、服务费交纳 本项目不收取服务费。 五、 其他 事项 1.本公告在华润守正 采购交易 平 台（ https://www.szecp.com.cn/ ）上公开 发布。 2. 本项目采购通过守正平台线上进行，供应商需注册华润守正 采购交易 平台，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 3 .答疑澄清、通知等文件一经在华润守正 采购交易 平台发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注华润守正 采购交易 平台发布的相关信息，并及时查阅和处理。 4 .若有参与意向 ， 请于 2026-08-22 00:00:00前联系采购人 （联系方式见公示内容）反馈。 5 .若有异议 ， 请于 2026-08-22 00:00:00前提出异议 。 信息来源:https://www.chinapipe.net/project/d3074793.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074793.html</t>
-        </is>
-      </c>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" t="n">
         <v>80</v>
       </c>
@@ -5268,11 +5016,7 @@
           <t>石柱公司2026-2027年度用户供水管道安装及管网抢(维)修工程(第二次)项目公告 石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（比选公告 1.比选条件 本比选项目石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（项目名称），比选人 为重庆石柱水利水电实业开发有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。现 对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 建设地点：比选人指定地点 务 2.2 项目概况与建设规模：2026-2027年度用户供水管道安装及管网抢（维）修服务 2.3 本次比选项目合同估算金额：约280万元 商 2.4 比选范围：完成石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程包括公司供水范围内用户 各类管道及管件安装、水表安装及更换、阀门安装等、并完成配套土建工程、零星签证等工程量清单所列项目、 管网抢维修和公司所属生产单元零星项目，具体内容详见第五章 工程量清单。 道 2.5 工期要求：1年 缺陷责任期要求：24个月 管 3.投标人资格要求 3.1 本次比选要求投标人须具备以下条件： 国 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质； 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 中 项内容。 3.2 本次比选不接受联合体投标。 4.比选文件的获取 4.1 投标人于2026年08月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价1000 元，售后不退。投标人在递交纸质投标文件时支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年08月24日10时00分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年08月24日09时30分至10时00分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼）。 5.3 投标截止时间：2026年08月24日10时00分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆石柱水利水电实业开发有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市石柱土家族自治县都督大道11号 地 址：重庆市两江新区嘉华路36号重庆水务大厦1018 联 系 人：王老师 联 系 人：颜老师 道 电 话：13658292968 电 话：023-67901915 重庆水务电子商务平台咨询电话：管023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074720.html cqdingjiu 2026.08.21 10:06:59 国 中</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074720.html</t>
-        </is>
-      </c>
+      <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
         <v>90</v>
       </c>
@@ -5336,11 +5080,7 @@
           <t>万盛城区老旧供水管网更新改造工程(甲供材料)答疑(一) 万盛城区老旧供水管网更新改造工程（甲供材料） 答疑（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程（甲供材料）答疑（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。 问题2：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 全是万盛的公司中的！业主、专家全是你们自己人吧？ 商 答：本项目招标文件严格按照《重庆市工程建设项目货物采购招标文件示范文本（2026年版）》编制，且本项目 评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题3：3PE管道部分壁厚是多少呢？ 道 答：本项目采购的3PE防腐钢管的管道部分壁厚须符合国标标准并达到设计要求。 招 标 人：重庆市万盛经济技术开发区城市管理局 管 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 国 信息来源:https://www.chinapipe.net/project/d3074712.html cqdingjiu 2026.08.21 10:06:59 中</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074712.html</t>
-        </is>
-      </c>
+      <c r="N66" t="inlineStr"/>
       <c r="O66" t="n">
         <v>80</v>
       </c>
@@ -5404,11 +5144,7 @@
           <t>重庆中法供水2026年普通防腐钢管及管件采购项目(第三次)项目公告 重庆中法供水2026年普通防腐钢管及管件采购项目（第三次）比选公告 1.比选条件 本比选项目重庆中法供水2026年普通防腐钢管及管件采购项目（第三次），比选人为重庆中法供水有限公司，比 选项目资金来自企业自筹，出资比例为100%，项目已具备比选条件。现对本项目进行公开比选，诚邀有兴趣的 潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 普通防腐钢管及管件采购清单： 务 序号 存货编码 材料名称 规格型号 单位 数量 最高单价限价（元） 1 10400177 钢高频焊管 D89*4 5 米 61.92 2 10400181 钢高频焊管 D108*5 300 米 88.89 商 3 10400182 钢高频焊管 D159*5 5 米 132.18 4 10400206 钢高频焊管 D159*6 5 米 152.13 5 10400290 钢螺旋焊管 DN219*6 5 米 196.68 道 6 10400291 钢螺旋焊管 DN219*8 5 米 244.80 7 10400292 钢螺旋焊管 DN325*8 5 米 361.28 8 10400293 钢螺旋焊管 DN377*8 5 米 423.12 管 9 10400294 钢螺旋焊管 DN426*8 5 米 475.89 10 10400295 钢螺旋焊管 DN426*10 5 米 574.29 11 10400297 钢螺旋焊管 DN529*8 5 米 595.76 国 12 10400298 钢螺旋焊管 DN529*10 5 米 718.91 13 10400299 钢螺旋焊管 DN630*10 5 米 861.50 14 10400300 钢螺旋焊管 DN720*10 5 米 987.95 中 15 10400301 钢螺旋焊管 DN820*10 5 米 1133.08 16 10400302 钢螺旋焊管 DN920*10 5 米 1279.51 17 10400304 钢螺旋焊管 DN1020*10 5 米 1424.64 18 10400305 钢螺旋焊管 DN1020*12 5 米 1652.24 19 10400306 钢螺旋焊管 DN1220*10 5 米 1709.70 20 10400307 钢螺旋焊管 DN1220*12 5 米 1982.83 21 10400308 钢螺旋焊管 DN1420*12 5 米 2375.96 22 10400309 钢螺旋焊管 DN1420*14 5 米 2697.83 23 10400332 钢螺旋焊管 DN1120*10 5 米 1574.96 24 10400342 钢螺旋焊管 DN1020*14 5 米 1879.02 25 10400322 钢螺旋焊管（特加强） DN820*10 5 米 1133.08 26 10200490 钢套筒 D159*500cm 5 个 159.00 27 10200491 钢套筒 D219*500cm 5 个 240.00 28 10200492 钢套筒 D273*500cm 5 个 300.00 29 10200493 钢套筒 D325*500cm 5 个 361.00 30 10200494 钢套筒 D377*500cm 5 个 436.00 31 10200495 钢套筒 D426*500cm 5 个 482.00 32 10200589 钢套筒 D159*1000cm 5 个 226.00 33 10200590 钢套筒 D219*1000cm 5 个 1627.00 34 10200591 钢套筒 D273*1000cm 5 个 2501.00 35 10200592 钢套筒 D325*1000cm 5 个 488.00 36 10200593 钢套筒 D377*1000cm 5 个 591.00 网 37 10200598 钢套筒 D426*1000cm 5 个 833.00 38 10200155 钢制标准接头 D108 5 个 91.00 39 10200156 钢制标准接头 D159 5 个 160.06 务 40 10200157 钢制标准接头 D219 5 个 319.41 41 10200158 钢制标准接头 D273 5 个 396.63 42 10200159 钢制标准接头 D325 5 个 475.96 商 43 10200160 钢制标准接头 D426 5 个 619.87 44 10200161 钢制标准接头 D529 5 个 779.22 45 10200162 钢制标准接头 D630 5 个 1068.44 道 46 10200163 钢制标准接头 D720 5 个 1214.46 47 10200164 钢制标准接头 D820 5 个 1428.34 48 10200165 钢制标准接头 D920 5 个 1600.14 管 49 10200169 钢制标准接头 D1220 5 个 2297.57 50 10200170 钢制标准接头 D1420 5 个 3027.02 51 10200171 钢制标准接头 D1020 5 个 2194.19 国 52 10300309 钢制大小头 DN65*DN50 5 个 14.74 53 10200667 钢制渐缩 D108＞57 3 个 21.06 54 10200668 钢制渐缩 D108＞89 3 个 26.00 中 55 10200695 钢制渐缩 D159＞108 3 个 40.72 56 10200671 钢制渐缩 D219＞159 3 个 68.09 57 10200672 钢制渐缩 D219＞108 3 个 80.03 58 10201605 钢制渐缩 219*125 3 个 75.82 59 10200694 钢制渐缩 D273＞108 3 个 129.87 60 10200673 钢制渐缩 D273＞159 3 个 94.07 61 10200674 钢制渐缩 D273＞219 3 个 84.94 62 10200675 钢制渐缩 D325＞108 3 个 184.63 63 10200676 钢制渐缩 D325＞159 3 个 143.91 64 10200680 钢制渐缩 D325＞219 3 个 131.98 65 10200677 钢制渐缩 D325＞273 3 个 124.25 66 10200684 钢制渐缩 D426＞325 3 个 285.01 67 10200685 钢制渐缩 D529＞325 3 个 617.76 68 10200679 钢制渐缩 D529＞426 3 个 547.56 69 10200659 钢制渐缩 D630＞325 3 个 756.00 70 10200687 钢制渐缩 D630＞426 3 个 728.00 71 10201539 钢制渐缩 D630＞529 3 个 722.00 72 10200690 钢制渐缩 D720＞630 3 个 848.00 73 10200691 钢制渐缩 D720＞529 3 个 842.00 74 10200682 钢制渐缩 D820＞720 3 个 913.00 75 10200692 钢制渐缩 D920＞720 3 个 1053.00 76 10201519 钢制渐缩 D920*820 3 个 1064.00 77 10200652 钢制渐缩 D1020＞820 3 个 1305.00 网 78 10200693 钢制渐缩 D1020＞920 3 个 1322.00 79 10201738 钢制渐缩 1220*820 3 个 1806.00 80 10201507 钢制渐缩 1220＞1020 3 个 1834.00 务 81 10201624 钢制三盘三通 D108⊥108 3 个 224.64 82 10200371 钢制三盘三通 DN200⊥100 3 个 435.24 83 10200373 钢制三盘三通 DN200⊥200 3 个 599.51 商 84 10201531 钢制三通 108*108 3 个 58.97 85 10200285 钢制三通 219*108 3 个 187.43 86 10201341 钢制双盘短管 89*400mm 3 个 139.00 道 87 10201342 钢制双盘短管 89*800mm 3 个 178.31 88 10201340 钢制双盘短管 108*300mm 3 个 158.65 89 10201299 钢制双盘短管 DN108*500mm 3 个 185.33 管 90 10201300 钢制双盘短管 DN108*1000mm 3 个 258.34 91 10201301 钢制双盘短管 DN108*1500mm 3 个 329.94 92 10201332 钢制双盘短管 159*300mm 3 个 251.32 国 93 10201339 钢制双盘短管 159*750mm 3 个 348.19 94 10201303 钢制双盘短管 DN159*1000mm 3 个 402.95 95 10201304 钢制双盘短管 DN159*1500mm 3 个 508.25 中 96 10201305 钢制双盘短管 DN219*500mm 3 个 463.32 97 10201306 钢制双盘短管 DN219*1000mm 3 个 672.52 98 10201307 钢制双盘短管 DN219*1500mm 3 个 876.00 99 10201312 钢制双盘短管 DN219*750mm 3 个 581.26 100 10201338 钢制双盘短管 273*1250mm 3 个 1010.88 101 10201458 钢制双盘渐缩 108*57 3 个 109.51 102 10201469 钢制双盘渐缩 108*89 3 个 117.94 103 10201514 钢制双盘渐缩 159*108 3 个 185.33 104 10201748 钢制双盘渐缩 200*80 3 个 294.84 105 10201462 钢制双盘渐缩 219*108 3 个 256.93 106 10201513 钢制双盘渐缩 219*159 3 个 280.80 107 10201465 钢制双盘渐缩 D273＞108 3 个 339.77 108 10201467 钢制双盘渐缩 D273＞219 3 个 388.91 109 10201770 钢制双盘渐缩 D273＞159 3 个 365.04 110 10201461 钢制双盘渐缩 325*219 3 个 477.36 111 10301108 钢制弯头 89*90° 3 个 28.78 112 10200702 钢制弯头 D108×90° 100 个 43.52 113 10200701 钢制弯头 D159×90° 3 个 84.24 114 10200705 钢制弯头 D219*90° 3 个 231.66 115 10200706 钢制弯头 D273*90° 3 个 300.46 116 10200709 钢制弯头 D325*90° 3 个 418.39 117 10200711 钢制弯头 D426*90° 3 个 744.12 118 10200712 钢制弯头 D529*90° 3 个 1352.05 网 119 10200764 钢制弯头 D570*90° 3 个 1474.20 120 10200714 钢制弯头 D630*90° 3 个 1535.98 121 10200715 钢制弯头 D720*90° 3 个 1742.36 务 122 10200717 钢制弯头 DN720*90°*12mm 3 个 1989.47 123 10200720 钢制弯头 D920*90° 3 个 2935.30 124 10200722 钢制弯头 D820*90° 3 个 2325.23 商 125 10200762 钢制弯头 D1020*90° 3 个 4829.55 126 10200723 钢制弯头 D1220*90° 3 个 6039.80 127 10200724 钢制弯头 D1420*90° 3 个 8297.00 道 注：管材按照米数进行报价，管件按照件数进行报价。 2.2 供货数量、时间和批次：根据工程实际进度与比选人的要求进行供货，以实际供货量为准，供货时间达到商 务条款的规定。 管 2.3 交货地点：比选人指定的施工现场。 2.4 供货期：两年。 国 3.投标人资格要求 3.1 本次比选允许投标人以投标货物的下列身份参加投标： 中 ?制造商 3.1.1 投标人为制造商应符合以下要求： 投标人必须是依法设立的，并在中国注册的，具有独立法人地位的企业。 【提供有效的营业执照】 3.2 投标人2025年的年度财务状况不亏损。 【提供由会计师事务所或审计机构出具的无保留意见的财务审计报告及会计报表，财务报表至少包括现金流量 表、资产负债表、利润表】 3.3 投标产品的制造商须通过质量ISO9001、环境ISO14001、职业健康体系ISO45001认证。 【提供有效的证书】 3.4 投标人须提供2023年1月1日至投标截止日止（以合同签订时间为准）,签订的30万元及以上的钢管及管件产品 购销合同至少1个。 【提供采购合同、不低于前述金额50％的发票，合同与发票的项目名称须一致】 注：①若投标人开具的发票上未能体现具体项目，需附上税务出具的发票清单（清单上需显示采购项目为钢管 及管件产品）。 ②若提供的合同为年度合同未体现具体金额，但实际供货金额达到30万元及以上，应提供与该合同对应的30万元 及以上的钢管及管件产品发票作为佐证。 3.5 投标人须为所投投标产品制造商，此次所提供的普通防腐钢管及管件必须是自己工厂所制造的产品，不得外 购他人产品。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函及工商部门出具的本产品商标或品牌证明文件】 3.6 投标产品过水部分涉及的涂料须提供行政主管部门出具的有效的“卫生许可网批件”及卫生疾控中心出具的卫 生检测报告。 【提供行政主管部门出具的有效的“卫生许可批件”及卫生疾控中心出具的卫生检测报告】 务 3.5 根据本次采购清单及技术规范的要求，投标人须承诺具备相关的技术手段和措施、保证产品设计使用寿命 20 年以上。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 商 3.6 投标人须承诺保证5年内不得停产同型号的投标产品。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 道 3.7 办事机构和库房【比选人有权对中标人的办事机构及库房进行实地核查，若发现与提供资料不符，将视为提 供虚假资料，按相关规定取消其中标资格，其投标保证金不予退还。】 投标人承诺：收到中标通知书后30日内提供租赁合同或产权证明，并提供重庆库房卫星定位图片。 管 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 【卫星定位图片：手机打开地图，搜索该地址、进行标注，然后截图或者电脑打开地图（地图软件不限），搜 索该地址、选择卫星模国式、进行标注、然后截图均可。】 3.8 符合第五章“技术要求”普通防腐钢管及管件技术要求。 【根据技术要求提供技术响应表，并根据技术条款要求提供对应的检测报告等。】 中 3.9 售后服务承诺【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】： 1）货物交付及付款方式要求，满足第四部分合同协议书第3条及第10条；供货单位应确保产品的及时供应，承诺 因产品供应不及时造成的一切损失均由供货单位负责赔偿。 2）有完整的售后服务方案、培训计划并在合同签订后为比选人免费提供培训服务。 3）售后服务承诺书，满足第四部分合同协议书第11条；承诺质保期后提供2年及以上定期免费巡查、保养计划。 4）承诺接到分派的工单1小时内联系用户约定维修时间，在24小时内处理完毕工单，且让用户满意。若工单超时、 未在规定时间内告知比选人维修时间或工单处理未让用户满意造成返单的，按比选人制度进行处罚。 3.10 投标人承诺不得存在下列情形之一： 1）被人民法院列入失信被执行人名单且在被执行期内； 2）被国家、重庆市（含市或任意区县）有关行政部门行政处罚，且在处罚期限内； 3）投标截止日前两年内（指2024年1月1日至投标截止日止），投标人或其法定代表人被人民法院判定犯行贿罪 的； 4）投标截止日前五年内（指2021年1月1日至投标截止日止），投标人与重庆中法供水有限公司有违约情况或终 止合同情况的。 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 3.11 投标截止日前五年内（指2021年1月1日至投标截止日止），投标人无在我司因产品及服务等对公司生产、经 营、安全造成不良影响的记录；若投标人出现过供水通报事项，因产品质量问题对生产、安全造成影响，存在 合同违约等问题，不予参加本次项目投标。 【按照第六章 三、资格审查部分“无不良记录承诺函”提供承诺函，若经验证承诺函不属实，将对中标人作否 决投标处理。】 网 3.12 投标样品要求： 3.12.1 投标人需提供以下规格型号数量的样品： 务 【①钢螺旋焊管 DN219*8 壹件 ②钢制弯头 D108*90°壹件】，提供的样品应满足第五章技术要求规定。样品为 投标人免费提供，管材样品不低于20CM，不计入采购清单内。 3.12.2 投标样品同投标文件一并递交。每件样品上分别标明样品的投标人、生产厂家、品牌、名称、规格、型号等 （格式自拟），投标样品必须密封装箱，且在密封包装外商贴样品一览表（格式自拟），注明提供样品的投标人、 生产厂家、品牌、名称、规格、型号、数量等。 3.12.3 投标人的样品在开标当日递交至样品区（样品区地点：开标当日咨询比选代理机构），中标人的投标样品 不退还，其余投标人的样品在中标公示期满后道5个工作日内退还，如不领取，投标样品按废品处理。 3.12.4 上述对投标样品的密封和标识要求是为便于评标，请投标人积极配合，未按上述要求对投标样品进行密封 和标识的，不作否决投标处理，但由此造成的其他后果由投标人自行承担。 管 3.13 若投标人违反重庆中法供水有限公司《供应商负面清单管理办法》规定且在处罚期内的，按否决投标处理 （评标委员会根据比选公告后附“供应商负面清单”进行评审）。 3.14 本次比选不接受联合体投标。 国 特别说明： （1） 本比选文件要求提供的所有检测报告须为近2年内的检测报告（2024年1月1日-投标截止日），此要求不包 括卫生许可批件及其检测报告。 中 （2） 上述所须提交的相关证明材料复印件均应加盖投标单位法人章并装入投标文件资格审查部分中。上述有一 条不满足则投标文件由评标委员会作否决投标处理。 （3） 比选人有权对投标人提供的以上资料进行核实，若发现存在弄虚作假，取消其投标、中标资格，投标人承 担因此造成的相关责任并赔偿相应损失。 4.比选文件的获取 4.1 投标人于2026年8月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价 500 元，售后不退。投标人在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年8月26日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月26日14时00分至14时30分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼。导航：重庆水务大厦东门）。 5.3 投标截止时间：2026年8月26日14时30分（北京时间）。 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 网 6.发布公告的媒介 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 务 7.联系方式 比 选 人：重庆中法供水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝北区悦来镇悦来水厂 地 址：重庆市两商江新区嘉华路36号重庆水务大厦10楼1018 联 系 人：陈老师 联 系 人：周洲 电 话：023-67585971 电 话：18602396399 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074673.html 管 cqdingjiu 2026.08.21 10:06:59 国 中</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074673.html</t>
-        </is>
-      </c>
+      <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
         <v>0</v>
       </c>
@@ -5480,11 +5216,7 @@
           <t>南岸区茶园片区乡镇老旧供水管网更新改造工程更正公告 南岸区茶园片区乡镇老旧供水管网更新改造工程更正公 告 发布日期： 2026年8月18日 网 首次公示日期： 2026年8月14日 更正日期： 2026年8月18日 采购人名称： 重庆市江南城市建设发展（集团）有限公司务 采购人地址： 重庆市南岸区米兰路51号电子信息标准化厂房2号楼 联系人： 赵老师 商 电话： 023-62820331 采购代理机构名称： 重庆多杰数字科技咨询服务有限公司 采购代理机构地址： 重庆市重庆市经开区重庆市经开区长生桥镇江峡路8号13-1幢1楼 道 经办人名称： 李佩奇、戴沛轩、李倩 联系电话： 023-67648437 本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展 更正事项： 水土保持监管测工作。 https://www.gec123.com/notices/detail/1665701682723590144 信息来源:https://www.c国hinapipe.net/project/d3074669.html cqdingjiu 2026.08.21 10:07:01 中</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074669.html</t>
-        </is>
-      </c>
+      <c r="N68" t="inlineStr"/>
       <c r="O68" t="n">
         <v>80</v>
       </c>
@@ -5548,11 +5280,7 @@
           <t>中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部排水钢管询价采购公告 中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 排水钢管询价采购公告 询价编号：ZT1105-XJ-2026-561-1 尊敬的各潜在供应商: 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与中铁十一局集团有限公司宜涪高铁重庆段站 前3标项目经理ZT1105-XJ-2026-561-1，排水钢管材料的报价。 一、项目概况 务 中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治（县）。合同金额28.01亿元，合同工期73个月， 开工日期：2024年12月，竣工日期：2030年12月。主要工程：新方斗山隧道(10660m)、石板坡隧道(4148m)、城北 隧道(3228m)、刘家坪隧道(2077m);刘家店子1号大桥工程(224.096m)、刘家店子2号大桥(232.099m)、城北大 桥(330.241m)、冉家湾大桥(355.245m),采用移动模架和支商架法现浇施工，其中24米移动模架施工6孔；32米支架法 施工5孔，移动模架施工28孔;正线铺无砟道床43.808Km。 二、询价内容 道 本次计划对排水钢管、GG-01材料进行询价，询价内容如下： 询价物资一览表 管 序号 包件号 物资名称 规格型号 计量单位 数量 备注 1 GG-01 排水钢管 Φ200*6m 米 3000 Q235B，壁厚6mm 合计 3000 国 说明：1.表中数量为计划数量，实际采购过程中可能有所调整，最终结算按照实际采购数量结算。 2.收货地点：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 中 三、技术质量及报价要求 1. 此次排水钢管、GG-01各项技术性能：Q235B 碳素结构钢无缝钢管，符合 GB/T8163 标准。质量需满足甲方项 目部正常使用的要求，保证产品的质量合格，满足试验室检测所有要求，详见技术规格书。 2.报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、结算及付款方式 自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发票认证完成之日起第6个月，支付至本次结算 金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内，累计支付总额不超结算总金额的75%，剩 余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理末次结算后第二年，支付金额应大于等于 尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总额的15%；办理末次结算后第四年，全部 付清）。 五、报价人资格要求 1.营业范围要求：在中华人民共和国境内依法注册、符合项目经营范围，具有询价物资生产或供应经验 的生产商或代理商，并且具有合法有效的营业执照。 2.生产能力要求：生产商须具备询价物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定。代 理商需出具制造厂出具签字盖章的授权函。 3.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8 月至今）国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；需满足排水钢管的相关所 有要求。 4.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年12月至今）企业或企业法定代表人有人民法院生效判决、裁 定认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接 受通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合 作方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 5.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★6.下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、报价人需要提供的资料 1.营业执照复印件、法人身份证复印件、开户许可证、授商权委托书、报价表和报价人资格要求中所需的证明资料， 所有资料需加盖公司鲜章。 2.生产厂家资质，产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、询价报名截止时间 管 有意参加本次询价采购的报价人须在铁建云链平台（https://www.crccep.cn）完成供应商注册，并于2026年8月18 日9时00分至2026年8月21日9时00分在网上完成报名工作。 八、询价截止时间 国 凡有意参加本次询价采购的报价人，请于 2026年8月21日14时00分 前提交报价。截止时间前未完成报价文件传 输的，视为放弃报价。 供应商报价必须严格按照《报价表》格式进行报价。 中 九、联系方式 采购组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村71号 采购人名称：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 地址：重庆市石柱土家族自治县金彰工业园区C区中铁十一局项目部 联系人：罗先生 联系电话：18580400001（提供采购服务支持） 中铁十一局集团有限公司 物资设备集中采购管理中心第五分中心 2026年8月18日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3074654.html cqdingjiu 2026.08.21 10:07:01 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074654.html</t>
-        </is>
-      </c>
+      <c r="N69" t="inlineStr"/>
       <c r="O69" t="n">
         <v>90</v>
       </c>
@@ -5616,11 +5344,7 @@
           <t>中铁建设集团(重庆)建设有限公司重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热 交换机组采购竞价补遗公告二 各 投标单位 ： 根据参加报名的潜在投标单位数量不满足招标方充分竞价要求的情况，此次重庆协同创新区供冷供热能源站及 配套系统工程冷却塔、分集水器、水板式热交换机组采购竞价资格预审报名截止日期将延期至 8月19日（周三） 上午9:00。 特此说明。 网 中铁建设集团（重庆）建设有限公司 2026年8月17日 务 信息来源:https://www.chinapipe.net/project/d3074650.html cqdingjiu 2026.08.21 10:07:01 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074650.html</t>
-        </is>
-      </c>
+      <c r="N70" t="inlineStr"/>
       <c r="O70" t="n">
         <v>80</v>
       </c>
@@ -5692,11 +5416,7 @@
           <t>城口县东安及河鱼片区污水管网建设项目(一期)招标计划表 重庆市工程建设项目招标计划表 项 名 目 称城口县东安及河鱼片区污水管网建设项目（一期） 招标 法人 或招 标人城口县生态环境局 名称 （盖 网 章） 项目 批准 文件 及文 号 主 建 内 要 设 容 在 污 城 水 口 处 县 理 东 站 安 1座 镇 ， 等 改 片 建 区 后 新 设 建 计 污 规 水 模 管 20 网 0m 29 3 . / 0 d 0 。 km，其中新建dn110污水管5.80km，dn160污水管2.75km，dn200污水管0.57km，DN300污水干管4.36km，D 务 N400污水干管8.12km，DN200压力管7.4km,以及建设配套泵站2座,化粪池56座，隔油池32座。改扩建 序号 招标项目名称 招标内容 招标方式 招标文件计划发布时间 拟交易场所 合同预估金额(万元) 备注 招 项 标 目1 城 建 口 设 县 项 东 目 安 （ 及 一 河 期 鱼 ） 片区污水管网 工程施工 公开招标 2026-09 城 易 口 中 县 心 公共资源交 3400.00 本 暂 为 计 定 准 划 ， 。 表 最 所 终 列 以 招 实 标 际 项 招 目 标 信 时 息 的 均 信 为 息 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3074602.html 商 cqdingjiu 2026.08.21 10:07:01 道 管 国 中</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074602.html</t>
-        </is>
-      </c>
+      <c r="N71" t="inlineStr"/>
       <c r="O71" t="n">
         <v>90</v>
       </c>
@@ -5760,11 +5480,7 @@
           <t>阀门产业园(管网改造)项目招标公告 阀门产业园（管网改造）项目招标公告 1.招标条件 本招标项目 阀门产业园（管网改造）项目已由垫江县发展和改革委员会以垫江发改委发【2022】459 号（批文 名称及编号）批准建设，项目业主为 垫江县丹香建设有限公司，建设资金来自 自筹资金 （资金来源）， 项目出资比例为 100% ，招标人为 垫江县丹香建设有限公司。项目已具备招标条件，现对该项目的施工进 行公开招标，评标办法采用经评审的最低投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 重庆市垫江县高新区县城组团 2.2 项目概况与建设规模： 场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路 务 长4000米，包括道路、综合管网等基础配套设施等。 2.3 本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元 商 2.4 招标范围： 包括土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等。具体详见施工图和 工程量清单。 道 2.5 工期要求：建设工期180日历天 缺陷责任期要求：24个月 管 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 国 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 中 4.1.1 本次招标要求投标人具备的资质条件： 具备建设行政主管部门颁发的有效的市政公用工程施工总承包叁 级及以上资质 ； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标 不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （垫江县）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（垫江县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资 源交易监督网、重庆市公共资源交易网（垫江县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 4.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）本项目招标公告网页下方“我要 提问”栏提出疑问，提问时间从本公告发布至2026-08-24 09:00:00前。 4.3招标人应于2026-08-24 23:59:59前在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-18 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 垫江县丹香建设有限公司 代理机构: 重庆博钰大数据科技有限公司 地 址: 地 址: 重庆市垫江县桂溪街道南内街88号 网 邮 编: 邮 编: 项目负责人: 熊老师 项目负责人: 郭威 电 话: 023-74630098 电 话: 023-74692498 务 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 商 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 道 2026年08月18日 信息来源:https://www.chinapipe.net/project/d3074578.html cqdingjiu 2026.08.21 10:07:02 管 国 中</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>https://www.chinapipe.net/project/d3074578.html</t>
-        </is>
-      </c>
+      <c r="N72" t="inlineStr"/>
       <c r="O72" t="n">
         <v>90</v>
       </c>

</xml_diff>